<commit_message>
ended 5 steps of calculation, fixed some bugs
</commit_message>
<xml_diff>
--- a/расчет_ступеней.xlsx
+++ b/расчет_ступеней.xlsx
@@ -413,271 +413,381 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA13"/>
+  <dimension ref="A1:BW13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>c_a_отн</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>c_a_отн_i_plus_1</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Kh</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>η_ад_полн</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>d1_отн</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ρ1</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>U_k1</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Hт_отн</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>T1_полн</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>P1_полн</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Hт</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>L_z</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>H_ад</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>ΔT_полн</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>T3_полн</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>T1_полн_i_plus_1</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>π_полн</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>P3_полн</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>P1_полн_i_plus_1</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>a_кр_1</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>a_кр_3</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>r_ср1_отн</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
           <t>c_u1_отн</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>α_1</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>c_a1</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>λ_1</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>q_1</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>F_1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>c_a3_отн</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>c_a3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>λ_3_отн</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>q_3_отн</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>F_3_отн</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>D_вт3</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>d3_отн</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>r_ср3_отн</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>c_3u_отн</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>α_3_отн</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>λ_3</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>q_3</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>F_3</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>r_ср2_отн</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>c_u2_отн</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>β_1</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>c_a2_отн</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>β_2</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>α_2</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>ε_рк</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>α_3</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>ε_на</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>c_1</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>ρ3</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>W_1</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>c_a2</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>W_2</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>c_2</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>τ_1</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>T_1</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>a_1</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>M_w1</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>λ_c2</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>T2_полн</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>τ_2</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>T_2</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="BM1" t="inlineStr">
         <is>
           <t>a_2</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="BN1" t="inlineStr">
         <is>
           <t>M_c2_ср</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="BO1" t="inlineStr">
         <is>
           <t>D_вт1</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="BP1" t="inlineStr">
         <is>
           <t>h_рк</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="BQ1" t="inlineStr">
         <is>
           <t>d2_отн</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="BR1" t="inlineStr">
         <is>
           <t>D_ср_1</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="BS1" t="inlineStr">
         <is>
           <t>D_ср_2</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="BT1" t="inlineStr">
         <is>
           <t>D_ср_3</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="BU1" t="inlineStr">
         <is>
           <t>D_вт2</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BV1" t="inlineStr">
         <is>
           <t>h_на</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BW1" t="inlineStr">
         <is>
           <t>h_на_3</t>
         </is>
@@ -685,1933 +795,2725 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0.4375</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.884203297941869</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1.066429875635743</v>
+      </c>
+      <c r="G2" t="n">
+        <v>334.9958456714842</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.3244400050544849</v>
+      </c>
+      <c r="I2" t="n">
+        <v>288</v>
+      </c>
+      <c r="J2" t="n">
+        <v>100674.7651178944</v>
+      </c>
+      <c r="K2" t="n">
+        <v>36409.37652649458</v>
+      </c>
+      <c r="L2" t="n">
+        <v>36045.28276122964</v>
+      </c>
+      <c r="M2" t="n">
+        <v>31871.35789272645</v>
+      </c>
+      <c r="N2" t="n">
+        <v>35.83030095549666</v>
+      </c>
+      <c r="O2" t="n">
+        <v>323.8303009554967</v>
+      </c>
+      <c r="P2" t="n">
+        <v>323.8303009554967</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>1.440908707022073</v>
+      </c>
+      <c r="R2" t="n">
+        <v>145063.1456357761</v>
+      </c>
+      <c r="S2" t="n">
+        <v>145063.1456357761</v>
+      </c>
+      <c r="T2" t="n">
+        <v>310.7513475433373</v>
+      </c>
+      <c r="U2" t="n">
+        <v>329.5152498904687</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.7615773105863909</v>
+      </c>
+      <c r="W2" t="n">
         <v>0.1677833565897216</v>
       </c>
-      <c r="B2" t="n">
+      <c r="X2" t="n">
         <v>1.064577496794081</v>
       </c>
-      <c r="C2" t="n">
+      <c r="Y2" t="n">
         <v>150.7481305521679</v>
       </c>
-      <c r="D2" t="n">
+      <c r="Z2" t="n">
         <v>0.5546733681375342</v>
       </c>
-      <c r="E2" t="n">
+      <c r="AA2" t="n">
         <v>0.7670768900816778</v>
       </c>
-      <c r="F2" t="n">
+      <c r="AB2" t="n">
         <v>0.3651710357190851</v>
       </c>
-      <c r="G2" t="n">
+      <c r="AC2" t="n">
         <v>0.4375</v>
       </c>
-      <c r="H2" t="n">
+      <c r="AD2" t="n">
         <v>146.5606824812743</v>
       </c>
-      <c r="I2" t="n">
+      <c r="AE2" t="n">
         <v>0.5085578472919455</v>
       </c>
-      <c r="J2" t="n">
+      <c r="AF2" t="n">
         <v>0.7185450194326043</v>
       </c>
-      <c r="K2" t="n">
+      <c r="AG2" t="n">
         <v>0.2868846230922911</v>
       </c>
-      <c r="L2" t="n">
+      <c r="AH2" t="n">
         <v>0.4226367409601864</v>
       </c>
-      <c r="M2" t="n">
+      <c r="AI2" t="n">
         <v>0.5681001461244793</v>
       </c>
-      <c r="N2" t="n">
+      <c r="AJ2" t="n">
         <v>0.8132458964011607</v>
       </c>
-      <c r="O2" t="n">
+      <c r="AK2" t="n">
         <v>0.2029970421339847</v>
       </c>
-      <c r="P2" t="n">
+      <c r="AL2" t="n">
         <v>1.128936317318384</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="AM2" t="n">
         <v>0.4903225573137425</v>
       </c>
-      <c r="R2" t="n">
+      <c r="AN2" t="n">
         <v>0.7002124444906179</v>
       </c>
-      <c r="S2" t="n">
+      <c r="AO2" t="n">
         <v>0.2943956776214189</v>
       </c>
-      <c r="T2" t="n">
+      <c r="AP2" t="n">
         <v>0.7874116034937758</v>
       </c>
-      <c r="U2" t="n">
+      <c r="AQ2" t="n">
         <v>0.5743120885198095</v>
       </c>
-      <c r="V2" t="n">
+      <c r="AR2" t="n">
         <v>0.6484989891376707</v>
       </c>
-      <c r="W2" t="n">
+      <c r="AS2" t="n">
         <v>0.44375</v>
       </c>
-      <c r="X2" t="n">
+      <c r="AT2" t="n">
         <v>1.123094102388967</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="AU2" t="n">
         <v>0.657848686446533</v>
       </c>
-      <c r="Z2" t="n">
+      <c r="AV2" t="n">
         <v>0.474595113251296</v>
       </c>
-      <c r="AA2" t="n">
+      <c r="AW2" t="n">
         <v>1.136366747647551</v>
       </c>
-      <c r="AB2" t="n">
+      <c r="AX2" t="n">
         <v>0.4785180612010175</v>
       </c>
-      <c r="AC2" t="n">
+      <c r="AY2" t="n">
         <v>160.8856583832313</v>
       </c>
-      <c r="AD2" t="n">
+      <c r="AZ2" t="n">
         <v>1.407189122308089</v>
       </c>
-      <c r="AE2" t="n">
+      <c r="BA2" t="n">
         <v>249.586801734187</v>
       </c>
-      <c r="AF2" t="n">
+      <c r="BB2" t="n">
         <v>148.6544065167211</v>
       </c>
-      <c r="AG2" t="n">
+      <c r="BC2" t="n">
         <v>164.9069462237893</v>
       </c>
-      <c r="AH2" t="n">
+      <c r="BD2" t="n">
         <v>243.1313991612655</v>
       </c>
-      <c r="AI2" t="n">
+      <c r="BE2" t="n">
         <v>0.9487229091131606</v>
       </c>
-      <c r="AJ2" t="n">
+      <c r="BF2" t="n">
         <v>273.2321978245902</v>
       </c>
-      <c r="AK2" t="n">
+      <c r="BG2" t="n">
         <v>331.5685556814791</v>
       </c>
-      <c r="AL2" t="n">
+      <c r="BH2" t="n">
         <v>0.7527456915243563</v>
       </c>
-      <c r="AM2" t="n">
+      <c r="BI2" t="n">
         <v>0.7378456664511966</v>
       </c>
-      <c r="AN2" t="n">
+      <c r="BJ2" t="n">
         <v>323.8303009554967</v>
       </c>
-      <c r="AO2" t="n">
+      <c r="BK2" t="n">
         <v>0.9092639620831983</v>
       </c>
-      <c r="AP2" t="n">
+      <c r="BL2" t="n">
         <v>644.7761790602917</v>
       </c>
-      <c r="AQ2" t="n">
+      <c r="BM2" t="n">
         <v>509.3448177872226</v>
       </c>
-      <c r="AR2" t="n">
+      <c r="BN2" t="n">
         <v>0.477341460383392</v>
       </c>
-      <c r="AS2" t="n">
+      <c r="BO2" t="n">
         <v>0.2975790404866964</v>
       </c>
-      <c r="AT2" t="n">
+      <c r="BP2" t="n">
         <v>0.2231842803650222</v>
       </c>
-      <c r="AU2" t="n">
+      <c r="BQ2" t="n">
         <v>0.4899327164348984</v>
       </c>
-      <c r="AV2" t="n">
+      <c r="BR2" t="n">
         <v>0.5665736133518423</v>
       </c>
-      <c r="AW2" t="n">
+      <c r="BS2" t="n">
         <v>0.585792973589422</v>
       </c>
-      <c r="AX2" t="n">
+      <c r="BT2" t="n">
         <v>0.6050123338270017</v>
       </c>
-      <c r="AY2" t="n">
+      <c r="BU2" t="n">
         <v>0.3644842691493443</v>
       </c>
-      <c r="AZ2" t="n">
+      <c r="BV2" t="n">
         <v>0.1897316660336983</v>
       </c>
-      <c r="BA2" t="n">
+      <c r="BW2" t="n">
         <v>0.1606554301282772</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
+        <v>0.4375</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0.425</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.8813910730500205</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.066429875635743</v>
+      </c>
+      <c r="G3" t="n">
+        <v>334.9958456714842</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.3311958650192543</v>
+      </c>
+      <c r="I3" t="n">
+        <v>323.8303009554967</v>
+      </c>
+      <c r="J3" t="n">
+        <v>145063.1456357761</v>
+      </c>
+      <c r="K3" t="n">
+        <v>37167.53410689608</v>
+      </c>
+      <c r="L3" t="n">
+        <v>36424.18342475816</v>
+      </c>
+      <c r="M3" t="n">
+        <v>32103.95011371837</v>
+      </c>
+      <c r="N3" t="n">
+        <v>36.20694177411348</v>
+      </c>
+      <c r="O3" t="n">
+        <v>360.0372427296102</v>
+      </c>
+      <c r="P3" t="n">
+        <v>360.0372427296102</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>1.389521025919508</v>
+      </c>
+      <c r="R3" t="n">
+        <v>201568.2909469347</v>
+      </c>
+      <c r="S3" t="n">
+        <v>201568.2909469347</v>
+      </c>
+      <c r="T3" t="n">
+        <v>329.5152498904687</v>
+      </c>
+      <c r="U3" t="n">
+        <v>347.448539336746</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.7615773105863909</v>
+      </c>
+      <c r="W3" t="n">
         <v>0.1633479172253532</v>
       </c>
-      <c r="B3" t="n">
+      <c r="X3" t="n">
         <v>1.064577496794081</v>
       </c>
-      <c r="C3" t="n">
+      <c r="Y3" t="n">
         <v>146.5606824812743</v>
       </c>
-      <c r="D3" t="n">
+      <c r="Z3" t="n">
         <v>0.5085578472919455</v>
       </c>
-      <c r="E3" t="n">
+      <c r="AA3" t="n">
         <v>0.7185450194326043</v>
       </c>
-      <c r="F3" t="n">
+      <c r="AB3" t="n">
         <v>0.2868846230922911</v>
       </c>
-      <c r="G3" t="n">
+      <c r="AC3" t="n">
         <v>0.425</v>
       </c>
-      <c r="H3" t="n">
+      <c r="AD3" t="n">
         <v>142.3732344103808</v>
       </c>
-      <c r="I3" t="n">
+      <c r="AE3" t="n">
         <v>0.468528766832469</v>
       </c>
-      <c r="J3" t="n">
+      <c r="AF3" t="n">
         <v>0.6733194447626319</v>
       </c>
-      <c r="K3" t="n">
+      <c r="AG3" t="n">
         <v>0.2323217907867172</v>
       </c>
-      <c r="L3" t="n">
+      <c r="AH3" t="n">
         <v>0.506480008400635</v>
       </c>
-      <c r="M3" t="n">
+      <c r="AI3" t="n">
         <v>0.6808006472126222</v>
       </c>
-      <c r="N3" t="n">
+      <c r="AJ3" t="n">
         <v>0.8554208090890487</v>
       </c>
-      <c r="O3" t="n">
+      <c r="AK3" t="n">
         <v>0.2304275261048039</v>
       </c>
-      <c r="P3" t="n">
+      <c r="AL3" t="n">
         <v>1.073179621665038</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="AM3" t="n">
         <v>0.4661209080755683</v>
       </c>
-      <c r="R3" t="n">
+      <c r="AN3" t="n">
         <v>0.6707463493850978</v>
       </c>
-      <c r="S3" t="n">
+      <c r="AO3" t="n">
         <v>0.233213016100909</v>
       </c>
-      <c r="T3" t="n">
+      <c r="AP3" t="n">
         <v>0.8084990598377197</v>
       </c>
-      <c r="U3" t="n">
+      <c r="AQ3" t="n">
         <v>0.5635107758827498</v>
       </c>
-      <c r="V3" t="n">
+      <c r="AR3" t="n">
         <v>0.6314414656442968</v>
       </c>
-      <c r="W3" t="n">
+      <c r="AS3" t="n">
         <v>0.43125</v>
       </c>
-      <c r="X3" t="n">
+      <c r="AT3" t="n">
         <v>1.054171527737041</v>
       </c>
-      <c r="Y3" t="n">
+      <c r="AU3" t="n">
         <v>0.6532160462166496</v>
       </c>
-      <c r="Z3" t="n">
+      <c r="AV3" t="n">
         <v>0.4227300620927443</v>
       </c>
-      <c r="AA3" t="n">
+      <c r="AW3" t="n">
         <v>1.07397490693721</v>
       </c>
-      <c r="AB3" t="n">
+      <c r="AX3" t="n">
         <v>0.4207588607205606</v>
       </c>
-      <c r="AC3" t="n">
+      <c r="AY3" t="n">
         <v>156.4429853478237</v>
       </c>
-      <c r="AD3" t="n">
+      <c r="AZ3" t="n">
         <v>1.776406807110386</v>
       </c>
-      <c r="AE3" t="n">
+      <c r="BA3" t="n">
         <v>248.2779526487107</v>
       </c>
-      <c r="AF3" t="n">
+      <c r="BB3" t="n">
         <v>144.4669584458276</v>
       </c>
-      <c r="AG3" t="n">
+      <c r="BC3" t="n">
         <v>166.1511251787695</v>
       </c>
-      <c r="AH3" t="n">
+      <c r="BD3" t="n">
         <v>237.7104076639635</v>
       </c>
-      <c r="AI3" t="n">
+      <c r="BE3" t="n">
         <v>0.9568948193262971</v>
       </c>
-      <c r="AJ3" t="n">
+      <c r="BF3" t="n">
         <v>309.8715373251904</v>
       </c>
-      <c r="AK3" t="n">
+      <c r="BG3" t="n">
         <v>353.1004272981889</v>
       </c>
-      <c r="AL3" t="n">
+      <c r="BH3" t="n">
         <v>0.7031369362774604</v>
       </c>
-      <c r="AM3" t="n">
+      <c r="BI3" t="n">
         <v>0.6841600431469231</v>
       </c>
-      <c r="AN3" t="n">
+      <c r="BJ3" t="n">
         <v>360.0372427296102</v>
       </c>
-      <c r="AO3" t="n">
+      <c r="BK3" t="n">
         <v>0.9219875058935334</v>
       </c>
-      <c r="AP3" t="n">
+      <c r="BL3" t="n">
         <v>653.7986833101451</v>
       </c>
-      <c r="AQ3" t="n">
+      <c r="BM3" t="n">
         <v>512.8961280967814</v>
       </c>
-      <c r="AR3" t="n">
+      <c r="BN3" t="n">
         <v>0.4634669568398624</v>
       </c>
-      <c r="AS3" t="n">
+      <c r="BO3" t="n">
         <v>0.2975790404866964</v>
       </c>
-      <c r="AT3" t="n">
+      <c r="BP3" t="n">
         <v>0.2231842803650222</v>
       </c>
-      <c r="AU3" t="n">
+      <c r="BQ3" t="n">
         <v>0.5543838557506463</v>
       </c>
-      <c r="AV3" t="n">
+      <c r="BR3" t="n">
         <v>0.5665736133518423</v>
       </c>
-      <c r="AW3" t="n">
+      <c r="BS3" t="n">
         <v>0.6014809361522618</v>
       </c>
-      <c r="AX3" t="n">
+      <c r="BT3" t="n">
         <v>0.6363882589526815</v>
       </c>
-      <c r="AY3" t="n">
+      <c r="BU3" t="n">
         <v>0.412432539638981</v>
       </c>
-      <c r="AZ3" t="n">
+      <c r="BV3" t="n">
         <v>0.1657575307888799</v>
       </c>
-      <c r="BA3" t="n">
+      <c r="BW3" t="n">
         <v>0.1187337964080529</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
+        <v>0.425</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0.4125</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.8776400396808992</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1.066429875635743</v>
+      </c>
+      <c r="G4" t="n">
+        <v>334.9958456714842</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.3375197589886442</v>
+      </c>
+      <c r="I4" t="n">
+        <v>360.0372427296102</v>
+      </c>
+      <c r="J4" t="n">
+        <v>201568.2909469347</v>
+      </c>
+      <c r="K4" t="n">
+        <v>37877.21550579287</v>
+      </c>
+      <c r="L4" t="n">
+        <v>36740.89904061908</v>
+      </c>
+      <c r="M4" t="n">
+        <v>32245.28409192084</v>
+      </c>
+      <c r="N4" t="n">
+        <v>36.52176843003885</v>
+      </c>
+      <c r="O4" t="n">
+        <v>396.559011159649</v>
+      </c>
+      <c r="P4" t="n">
+        <v>396.559011159649</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>1.347829621392633</v>
+      </c>
+      <c r="R4" t="n">
+        <v>271679.7132717671</v>
+      </c>
+      <c r="S4" t="n">
+        <v>271679.7132717671</v>
+      </c>
+      <c r="T4" t="n">
+        <v>347.448539336746</v>
+      </c>
+      <c r="U4" t="n">
+        <v>364.6453570825088</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.7615773105863909</v>
+      </c>
+      <c r="W4" t="n">
         <v>0.1591960774308347</v>
       </c>
-      <c r="B4" t="n">
+      <c r="X4" t="n">
         <v>1.064577496794081</v>
       </c>
-      <c r="C4" t="n">
+      <c r="Y4" t="n">
         <v>142.3732344103808</v>
       </c>
-      <c r="D4" t="n">
+      <c r="Z4" t="n">
         <v>0.468528766832469</v>
       </c>
-      <c r="E4" t="n">
+      <c r="AA4" t="n">
         <v>0.6733194447626319</v>
       </c>
-      <c r="F4" t="n">
+      <c r="AB4" t="n">
         <v>0.2323217907867172</v>
       </c>
-      <c r="G4" t="n">
+      <c r="AC4" t="n">
         <v>0.4125</v>
       </c>
-      <c r="H4" t="n">
+      <c r="AD4" t="n">
         <v>138.1857863394872</v>
       </c>
-      <c r="I4" t="n">
+      <c r="AE4" t="n">
         <v>0.4333023913326854</v>
       </c>
-      <c r="J4" t="n">
+      <c r="AF4" t="n">
         <v>0.6312866578179296</v>
       </c>
-      <c r="K4" t="n">
+      <c r="AG4" t="n">
         <v>0.1929432963141447</v>
       </c>
-      <c r="L4" t="n">
+      <c r="AH4" t="n">
         <v>0.558190666335634</v>
       </c>
-      <c r="M4" t="n">
+      <c r="AI4" t="n">
         <v>0.750309115081092</v>
       </c>
-      <c r="N4" t="n">
+      <c r="AJ4" t="n">
         <v>0.8840146401994062</v>
       </c>
-      <c r="O4" t="n">
+      <c r="AK4" t="n">
         <v>0.2478040511669324</v>
       </c>
-      <c r="P4" t="n">
+      <c r="AL4" t="n">
         <v>1.032320478025595</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="AM4" t="n">
         <v>0.4420825865074373</v>
       </c>
-      <c r="R4" t="n">
+      <c r="AN4" t="n">
         <v>0.6411568471991366</v>
       </c>
-      <c r="S4" t="n">
+      <c r="AO4" t="n">
         <v>0.1899730607426552</v>
       </c>
-      <c r="T4" t="n">
+      <c r="AP4" t="n">
         <v>0.8227959753928986</v>
       </c>
-      <c r="U4" t="n">
+      <c r="AQ4" t="n">
         <v>0.5575621335231457</v>
       </c>
-      <c r="V4" t="n">
+      <c r="AR4" t="n">
         <v>0.614429921562137</v>
       </c>
-      <c r="W4" t="n">
+      <c r="AS4" t="n">
         <v>0.41875</v>
       </c>
-      <c r="X4" t="n">
+      <c r="AT4" t="n">
         <v>1.006183457466621</v>
       </c>
-      <c r="Y4" t="n">
+      <c r="AU4" t="n">
         <v>0.6441646969371893</v>
       </c>
-      <c r="Z4" t="n">
+      <c r="AV4" t="n">
         <v>0.3917535359044838</v>
       </c>
-      <c r="AA4" t="n">
+      <c r="AW4" t="n">
         <v>1.029835022076156</v>
       </c>
-      <c r="AB4" t="n">
+      <c r="AX4" t="n">
         <v>0.3856703251389664</v>
       </c>
-      <c r="AC4" t="n">
+      <c r="AY4" t="n">
         <v>152.0336456146226</v>
       </c>
-      <c r="AD4" t="n">
+      <c r="AZ4" t="n">
         <v>2.19436222248338</v>
       </c>
-      <c r="AE4" t="n">
+      <c r="BA4" t="n">
         <v>246.9644608130197</v>
       </c>
-      <c r="AF4" t="n">
+      <c r="BB4" t="n">
         <v>140.279510374934</v>
       </c>
-      <c r="AG4" t="n">
+      <c r="BC4" t="n">
         <v>166.0513797701721</v>
       </c>
-      <c r="AH4" t="n">
+      <c r="BD4" t="n">
         <v>233.5925564032956</v>
       </c>
-      <c r="AI4" t="n">
+      <c r="BE4" t="n">
         <v>0.9634134657750744</v>
       </c>
-      <c r="AJ4" t="n">
+      <c r="BF4" t="n">
         <v>346.8647278262354</v>
       </c>
-      <c r="AK4" t="n">
+      <c r="BG4" t="n">
         <v>373.5833131821657</v>
       </c>
-      <c r="AL4" t="n">
+      <c r="BH4" t="n">
         <v>0.6610693039509383</v>
       </c>
-      <c r="AM4" t="n">
+      <c r="BI4" t="n">
         <v>0.6406020311687126</v>
       </c>
-      <c r="AN4" t="n">
+      <c r="BJ4" t="n">
         <v>396.559011159649</v>
       </c>
-      <c r="AO4" t="n">
+      <c r="BK4" t="n">
         <v>0.93160483961042</v>
       </c>
-      <c r="AP4" t="n">
+      <c r="BL4" t="n">
         <v>660.6185155539247</v>
       </c>
-      <c r="AQ4" t="n">
+      <c r="BM4" t="n">
         <v>515.5642209446628</v>
       </c>
-      <c r="AR4" t="n">
+      <c r="BN4" t="n">
         <v>0.4530813949332761</v>
       </c>
-      <c r="AS4" t="n">
+      <c r="BO4" t="n">
         <v>0.2975790404866964</v>
       </c>
-      <c r="AT4" t="n">
+      <c r="BP4" t="n">
         <v>0.2231842803650222</v>
       </c>
-      <c r="AU4" t="n">
+      <c r="BQ4" t="n">
         <v>0.5949675909202978</v>
       </c>
-      <c r="AV4" t="n">
+      <c r="BR4" t="n">
         <v>0.5665736133518423</v>
       </c>
-      <c r="AW4" t="n">
+      <c r="BS4" t="n">
         <v>0.6121170921843355</v>
       </c>
-      <c r="AX4" t="n">
+      <c r="BT4" t="n">
         <v>0.6576605710168285</v>
       </c>
-      <c r="AY4" t="n">
+      <c r="BU4" t="n">
         <v>0.4426247120668587</v>
       </c>
-      <c r="AZ4" t="n">
+      <c r="BV4" t="n">
         <v>0.1506614445749411</v>
       </c>
-      <c r="BA4" t="n">
+      <c r="BW4" t="n">
         <v>0.09287846744055345</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
+        <v>0.4125</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.8729343479869782</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1.066429875635743</v>
+      </c>
+      <c r="G5" t="n">
+        <v>334.9958456714842</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.3433570658223036</v>
+      </c>
+      <c r="I5" t="n">
+        <v>396.559011159649</v>
+      </c>
+      <c r="J5" t="n">
+        <v>271679.7132717671</v>
+      </c>
+      <c r="K5" t="n">
+        <v>38532.29101774057</v>
+      </c>
+      <c r="L5" t="n">
+        <v>36990.99937703094</v>
+      </c>
+      <c r="M5" t="n">
+        <v>32290.71392257523</v>
+      </c>
+      <c r="N5" t="n">
+        <v>36.77037711434487</v>
+      </c>
+      <c r="O5" t="n">
+        <v>433.3293882739939</v>
+      </c>
+      <c r="P5" t="n">
+        <v>433.3293882739939</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>1.313130303218921</v>
+      </c>
+      <c r="R5" t="n">
+        <v>356750.8642669851</v>
+      </c>
+      <c r="S5" t="n">
+        <v>356750.8642669851</v>
+      </c>
+      <c r="T5" t="n">
+        <v>364.6453570825088</v>
+      </c>
+      <c r="U5" t="n">
+        <v>381.1762635425639</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.7615773105863909</v>
+      </c>
+      <c r="W5" t="n">
         <v>0.1553636977416573</v>
       </c>
-      <c r="B5" t="n">
+      <c r="X5" t="n">
         <v>1.064577496794081</v>
       </c>
-      <c r="C5" t="n">
+      <c r="Y5" t="n">
         <v>138.1857863394872</v>
       </c>
-      <c r="D5" t="n">
+      <c r="Z5" t="n">
         <v>0.4333023913326854</v>
       </c>
-      <c r="E5" t="n">
+      <c r="AA5" t="n">
         <v>0.6312866578179296</v>
       </c>
-      <c r="F5" t="n">
+      <c r="AB5" t="n">
         <v>0.1929432963141447</v>
       </c>
-      <c r="G5" t="n">
+      <c r="AC5" t="n">
         <v>0.4</v>
       </c>
-      <c r="H5" t="n">
+      <c r="AD5" t="n">
         <v>133.9983382685937</v>
       </c>
-      <c r="I5" t="n">
+      <c r="AE5" t="n">
         <v>0.4019499360408819</v>
       </c>
-      <c r="J5" t="n">
+      <c r="AF5" t="n">
         <v>0.5922271443277999</v>
       </c>
-      <c r="K5" t="n">
+      <c r="AG5" t="n">
         <v>0.1637251255561614</v>
       </c>
-      <c r="L5" t="n">
+      <c r="AH5" t="n">
         <v>0.5931253835185788</v>
       </c>
-      <c r="M5" t="n">
+      <c r="AI5" t="n">
         <v>0.7972676873324286</v>
       </c>
-      <c r="N5" t="n">
+      <c r="AJ5" t="n">
         <v>0.9043328384130478</v>
       </c>
-      <c r="O5" t="n">
+      <c r="AK5" t="n">
         <v>0.2594013382727521</v>
       </c>
-      <c r="P5" t="n">
+      <c r="AL5" t="n">
         <v>0.9997621798616013</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="AM5" t="n">
         <v>0.4189892047782126</v>
       </c>
-      <c r="R5" t="n">
+      <c r="AN5" t="n">
         <v>0.6121999974112641</v>
       </c>
-      <c r="S5" t="n">
+      <c r="AO5" t="n">
         <v>0.1583836392892018</v>
       </c>
-      <c r="T5" t="n">
+      <c r="AP5" t="n">
         <v>0.8329550744997194</v>
       </c>
-      <c r="U5" t="n">
+      <c r="AQ5" t="n">
         <v>0.5542658266274929</v>
       </c>
-      <c r="V5" t="n">
+      <c r="AR5" t="n">
         <v>0.5974865025033296</v>
       </c>
-      <c r="W5" t="n">
+      <c r="AS5" t="n">
         <v>0.40625</v>
       </c>
-      <c r="X5" t="n">
+      <c r="AT5" t="n">
         <v>0.9695253360656676</v>
       </c>
-      <c r="Y5" t="n">
+      <c r="AU5" t="n">
         <v>0.6325005241171194</v>
       </c>
-      <c r="Z5" t="n">
+      <c r="AV5" t="n">
         <v>0.372038833562338</v>
       </c>
-      <c r="AA5" t="n">
+      <c r="AW5" t="n">
         <v>0.9954739554152893</v>
       </c>
-      <c r="AB5" t="n">
+      <c r="AX5" t="n">
         <v>0.3629734312981698</v>
       </c>
-      <c r="AC5" t="n">
+      <c r="AY5" t="n">
         <v>147.6621745217523</v>
       </c>
-      <c r="AD5" t="n">
+      <c r="AZ5" t="n">
         <v>2.659616017028643</v>
       </c>
-      <c r="AE5" t="n">
+      <c r="BA5" t="n">
         <v>245.6347060214273</v>
       </c>
-      <c r="AF5" t="n">
+      <c r="BB5" t="n">
         <v>136.0920623040405</v>
       </c>
-      <c r="AG5" t="n">
+      <c r="BC5" t="n">
         <v>165.0366338893982</v>
       </c>
-      <c r="AH5" t="n">
+      <c r="BD5" t="n">
         <v>230.2105659161242</v>
       </c>
-      <c r="AI5" t="n">
+      <c r="BE5" t="n">
         <v>0.9687081729442294</v>
       </c>
-      <c r="AJ5" t="n">
+      <c r="BF5" t="n">
         <v>384.1499551650339</v>
       </c>
-      <c r="AK5" t="n">
+      <c r="BG5" t="n">
         <v>393.1495592776405</v>
       </c>
-      <c r="AL5" t="n">
+      <c r="BH5" t="n">
         <v>0.6247869296171872</v>
       </c>
-      <c r="AM5" t="n">
+      <c r="BI5" t="n">
         <v>0.603947800360391</v>
       </c>
-      <c r="AN5" t="n">
+      <c r="BJ5" t="n">
         <v>433.3293882739939</v>
       </c>
-      <c r="AO5" t="n">
+      <c r="BK5" t="n">
         <v>0.9392078424066409</v>
       </c>
-      <c r="AP5" t="n">
+      <c r="BL5" t="n">
         <v>666.0099478516489</v>
       </c>
-      <c r="AQ5" t="n">
+      <c r="BM5" t="n">
         <v>517.6637543981512</v>
       </c>
-      <c r="AR5" t="n">
+      <c r="BN5" t="n">
         <v>0.4447106137144423</v>
       </c>
-      <c r="AS5" t="n">
+      <c r="BO5" t="n">
         <v>0.2975790404866964</v>
       </c>
-      <c r="AT5" t="n">
+      <c r="BP5" t="n">
         <v>0.2231842803650222</v>
       </c>
-      <c r="AU5" t="n">
+      <c r="BQ5" t="n">
         <v>0.6225980342642162</v>
       </c>
-      <c r="AV5" t="n">
+      <c r="BR5" t="n">
         <v>0.5665736133518423</v>
       </c>
-      <c r="AW5" t="n">
+      <c r="BS5" t="n">
         <v>0.619674929595378</v>
       </c>
-      <c r="AX5" t="n">
+      <c r="BT5" t="n">
         <v>0.6727762458389134</v>
       </c>
-      <c r="AY5" t="n">
+      <c r="BU5" t="n">
         <v>0.4631803141131219</v>
       </c>
-      <c r="AZ5" t="n">
+      <c r="BV5" t="n">
         <v>0.1403836435518095</v>
       </c>
-      <c r="BA5" t="n">
+      <c r="BW5" t="n">
         <v>0.07541110884908103</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0.3875</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.8672584703581266</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1.066429875635743</v>
+      </c>
+      <c r="G6" t="n">
+        <v>334.9958456714842</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.3486475855755174</v>
+      </c>
+      <c r="I6" t="n">
+        <v>433.3293882739939</v>
+      </c>
+      <c r="J6" t="n">
+        <v>356750.8642669851</v>
+      </c>
+      <c r="K6" t="n">
+        <v>39126.00487150306</v>
+      </c>
+      <c r="L6" t="n">
+        <v>37169.7046279279</v>
+      </c>
+      <c r="M6" t="n">
+        <v>32235.74117928013</v>
+      </c>
+      <c r="N6" t="n">
+        <v>36.94801652875537</v>
+      </c>
+      <c r="O6" t="n">
+        <v>470.2774048027492</v>
+      </c>
+      <c r="P6" t="n">
+        <v>470.2774048027492</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>1.28363103095909</v>
+      </c>
+      <c r="R6" t="n">
+        <v>457936.4796945766</v>
+      </c>
+      <c r="S6" t="n">
+        <v>457936.4796945766</v>
+      </c>
+      <c r="T6" t="n">
+        <v>381.1762635425639</v>
+      </c>
+      <c r="U6" t="n">
+        <v>397.0944646181332</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.7615773105863909</v>
+      </c>
+      <c r="W6" t="n">
         <v>0.1518903013578152</v>
       </c>
-      <c r="B6" t="n">
+      <c r="X6" t="n">
         <v>1.064577496794081</v>
       </c>
-      <c r="C6" t="n">
+      <c r="Y6" t="n">
         <v>133.9983382685937</v>
       </c>
-      <c r="D6" t="n">
+      <c r="Z6" t="n">
         <v>0.4019499360408819</v>
       </c>
-      <c r="E6" t="n">
+      <c r="AA6" t="n">
         <v>0.5922271443277999</v>
       </c>
-      <c r="F6" t="n">
+      <c r="AB6" t="n">
         <v>0.1637251255561614</v>
       </c>
-      <c r="G6" t="n">
+      <c r="AC6" t="n">
         <v>0.3875</v>
       </c>
-      <c r="H6" t="n">
+      <c r="AD6" t="n">
         <v>129.8108901977001</v>
       </c>
-      <c r="I6" t="n">
+      <c r="AE6" t="n">
         <v>0.3737796859822607</v>
       </c>
-      <c r="J6" t="n">
+      <c r="AF6" t="n">
         <v>0.5558891806916422</v>
       </c>
-      <c r="K6" t="n">
+      <c r="AG6" t="n">
         <v>0.1415608615306941</v>
       </c>
-      <c r="L6" t="n">
+      <c r="AH6" t="n">
         <v>0.6180530627448302</v>
       </c>
-      <c r="M6" t="n">
+      <c r="AI6" t="n">
         <v>0.8307749923973037</v>
       </c>
-      <c r="N6" t="n">
+      <c r="AJ6" t="n">
         <v>0.9192896953607008</v>
       </c>
-      <c r="O6" t="n">
+      <c r="AK6" t="n">
         <v>0.2674717268010952</v>
       </c>
-      <c r="P6" t="n">
+      <c r="AL6" t="n">
         <v>0.9720262250235825</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="AM6" t="n">
         <v>0.3972152038601151</v>
       </c>
-      <c r="R6" t="n">
+      <c r="AN6" t="n">
         <v>0.5843288480641364</v>
       </c>
-      <c r="S6" t="n">
+      <c r="AO6" t="n">
         <v>0.1346710017740956</v>
       </c>
-      <c r="T6" t="n">
+      <c r="AP6" t="n">
         <v>0.8404335029735459</v>
       </c>
-      <c r="U6" t="n">
+      <c r="AQ6" t="n">
         <v>0.5524812982168491</v>
       </c>
-      <c r="V6" t="n">
+      <c r="AR6" t="n">
         <v>0.5806335590240905</v>
       </c>
-      <c r="W6" t="n">
+      <c r="AS6" t="n">
         <v>0.39375</v>
       </c>
-      <c r="X6" t="n">
+      <c r="AT6" t="n">
         <v>0.9393663462540609</v>
       </c>
-      <c r="Y6" t="n">
+      <c r="AU6" t="n">
         <v>0.6191945916757878</v>
       </c>
-      <c r="Z6" t="n">
+      <c r="AV6" t="n">
         <v>0.3587327872299704</v>
       </c>
-      <c r="AA6" t="n">
+      <c r="AW6" t="n">
         <v>0.9666442621479878</v>
       </c>
-      <c r="AB6" t="n">
+      <c r="AX6" t="n">
         <v>0.3474496704722</v>
       </c>
-      <c r="AC6" t="n">
+      <c r="AY6" t="n">
         <v>143.3338608703159</v>
       </c>
-      <c r="AD6" t="n">
+      <c r="AZ6" t="n">
         <v>3.169793873235574</v>
       </c>
-      <c r="AE6" t="n">
+      <c r="BA6" t="n">
         <v>244.2756650661178</v>
       </c>
-      <c r="AF6" t="n">
+      <c r="BB6" t="n">
         <v>131.9046142331469</v>
       </c>
-      <c r="AG6" t="n">
+      <c r="BC6" t="n">
         <v>163.4132722977984</v>
       </c>
-      <c r="AH6" t="n">
+      <c r="BD6" t="n">
         <v>227.2730542356306</v>
       </c>
-      <c r="AI6" t="n">
+      <c r="BE6" t="n">
         <v>0.9730727081527885</v>
       </c>
-      <c r="AJ6" t="n">
+      <c r="BF6" t="n">
         <v>421.6610013699664</v>
       </c>
-      <c r="AK6" t="n">
+      <c r="BG6" t="n">
         <v>411.8974635892041</v>
       </c>
-      <c r="AL6" t="n">
+      <c r="BH6" t="n">
         <v>0.5930496947894299</v>
       </c>
-      <c r="AM6" t="n">
+      <c r="BI6" t="n">
         <v>0.572340021043074</v>
       </c>
-      <c r="AN6" t="n">
+      <c r="BJ6" t="n">
         <v>470.2774048027492</v>
       </c>
-      <c r="AO6" t="n">
+      <c r="BK6" t="n">
         <v>0.9454044833854023</v>
       </c>
-      <c r="AP6" t="n">
+      <c r="BL6" t="n">
         <v>670.4041025304953</v>
       </c>
-      <c r="AQ6" t="n">
+      <c r="BM6" t="n">
         <v>519.368650087941</v>
       </c>
-      <c r="AR6" t="n">
+      <c r="BN6" t="n">
         <v>0.437594864836659</v>
       </c>
-      <c r="AS6" t="n">
+      <c r="BO6" t="n">
         <v>0.2975790404866964</v>
       </c>
-      <c r="AT6" t="n">
+      <c r="BP6" t="n">
         <v>0.2231842803650222</v>
       </c>
-      <c r="AU6" t="n">
+      <c r="BQ6" t="n">
         <v>0.6423837994849889</v>
       </c>
-      <c r="AV6" t="n">
+      <c r="BR6" t="n">
         <v>0.5665736133518423</v>
       </c>
-      <c r="AW6" t="n">
+      <c r="BS6" t="n">
         <v>0.6252384885193522</v>
       </c>
-      <c r="AX6" t="n">
+      <c r="BT6" t="n">
         <v>0.6839033636868619</v>
       </c>
-      <c r="AY6" t="n">
+      <c r="BU6" t="n">
         <v>0.4778998866873533</v>
       </c>
-      <c r="AZ6" t="n">
+      <c r="BV6" t="n">
         <v>0.1330238572646938</v>
       </c>
-      <c r="BA6" t="n">
+      <c r="BW6" t="n">
         <v>0.06294726923595534</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
+        <v>0.3875</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.8605972014216101</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1.066429875635743</v>
+      </c>
+      <c r="G7" t="n">
+        <v>334.9958456714842</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.3533255394992114</v>
+      </c>
+      <c r="I7" t="n">
+        <v>470.2774048027492</v>
+      </c>
+      <c r="J7" t="n">
+        <v>457936.4796945766</v>
+      </c>
+      <c r="K7" t="n">
+        <v>39650.97523005291</v>
+      </c>
+      <c r="L7" t="n">
+        <v>37271.91671624973</v>
+      </c>
+      <c r="M7" t="n">
+        <v>32076.10721762385</v>
+      </c>
+      <c r="N7" t="n">
+        <v>37.04961900223631</v>
+      </c>
+      <c r="O7" t="n">
+        <v>507.3270238049855</v>
+      </c>
+      <c r="P7" t="n">
+        <v>507.3270238049855</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>1.258098598953983</v>
+      </c>
+      <c r="R7" t="n">
+        <v>576129.2435136657</v>
+      </c>
+      <c r="S7" t="n">
+        <v>576129.2435136657</v>
+      </c>
+      <c r="T7" t="n">
+        <v>397.0944646181332</v>
+      </c>
+      <c r="U7" t="n">
+        <v>412.4399969472064</v>
+      </c>
+      <c r="V7" t="n">
+        <v>0.7615773105863909</v>
+      </c>
+      <c r="W7" t="n">
         <v>0.1488190741438032</v>
       </c>
-      <c r="B7" t="n">
+      <c r="X7" t="n">
         <v>1.064577496794081</v>
       </c>
-      <c r="C7" t="n">
+      <c r="Y7" t="n">
         <v>129.8108901977001</v>
       </c>
-      <c r="D7" t="n">
+      <c r="Z7" t="n">
         <v>0.3737796859822607</v>
       </c>
-      <c r="E7" t="n">
+      <c r="AA7" t="n">
         <v>0.5558891806916422</v>
       </c>
-      <c r="F7" t="n">
+      <c r="AB7" t="n">
         <v>0.1415608615306941</v>
       </c>
-      <c r="G7" t="n">
+      <c r="AC7" t="n">
         <v>0.375</v>
       </c>
-      <c r="H7" t="n">
+      <c r="AD7" t="n">
         <v>125.6234421268066</v>
       </c>
-      <c r="I7" t="n">
+      <c r="AE7" t="n">
         <v>0.3482637835623633</v>
       </c>
-      <c r="J7" t="n">
+      <c r="AF7" t="n">
         <v>0.5220220244246978</v>
       </c>
-      <c r="K7" t="n">
+      <c r="AG7" t="n">
         <v>0.1244499868451066</v>
       </c>
-      <c r="L7" t="n">
+      <c r="AH7" t="n">
         <v>0.6365266021211494</v>
       </c>
-      <c r="M7" t="n">
+      <c r="AI7" t="n">
         <v>0.8556067673047103</v>
       </c>
-      <c r="N7" t="n">
+      <c r="AJ7" t="n">
         <v>0.9306081184520197</v>
       </c>
-      <c r="O7" t="n">
+      <c r="AK7" t="n">
         <v>0.2733222986142951</v>
       </c>
-      <c r="P7" t="n">
+      <c r="AL7" t="n">
         <v>0.94708331955606</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="AM7" t="n">
         <v>0.3769042166111551</v>
       </c>
-      <c r="R7" t="n">
+      <c r="AN7" t="n">
         <v>0.5577971839788439</v>
       </c>
-      <c r="S7" t="n">
+      <c r="AO7" t="n">
         <v>0.1164682001603178</v>
       </c>
-      <c r="T7" t="n">
+      <c r="AP7" t="n">
         <v>0.8460927145192053</v>
       </c>
-      <c r="U7" t="n">
+      <c r="AQ7" t="n">
         <v>0.5515503936407113</v>
       </c>
-      <c r="V7" t="n">
+      <c r="AR7" t="n">
         <v>0.5638932886886516</v>
       </c>
-      <c r="W7" t="n">
+      <c r="AS7" t="n">
         <v>0.38125</v>
       </c>
-      <c r="X7" t="n">
+      <c r="AT7" t="n">
         <v>0.913006188823837</v>
       </c>
-      <c r="Y7" t="n">
+      <c r="AU7" t="n">
         <v>0.6048180107391227</v>
       </c>
-      <c r="Z7" t="n">
+      <c r="AV7" t="n">
         <v>0.3491129001351854</v>
       </c>
-      <c r="AA7" t="n">
+      <c r="AW7" t="n">
         <v>0.9409630125541549</v>
       </c>
-      <c r="AB7" t="n">
+      <c r="AX7" t="n">
         <v>0.3361450018150323</v>
       </c>
-      <c r="AC7" t="n">
+      <c r="AY7" t="n">
         <v>139.0549019493772</v>
       </c>
-      <c r="AD7" t="n">
+      <c r="AZ7" t="n">
         <v>3.721602002135425</v>
       </c>
-      <c r="AE7" t="n">
+      <c r="BA7" t="n">
         <v>242.8728905954796</v>
       </c>
-      <c r="AF7" t="n">
+      <c r="BB7" t="n">
         <v>127.7171661622534</v>
       </c>
-      <c r="AG7" t="n">
+      <c r="BC7" t="n">
         <v>161.3924812349645</v>
       </c>
-      <c r="AH7" t="n">
+      <c r="BD7" t="n">
         <v>224.6120038691836</v>
       </c>
-      <c r="AI7" t="n">
+      <c r="BE7" t="n">
         <v>0.9767147910578338</v>
       </c>
-      <c r="AJ7" t="n">
+      <c r="BF7" t="n">
         <v>459.3268971711375</v>
       </c>
-      <c r="AK7" t="n">
+      <c r="BG7" t="n">
         <v>429.900884327747</v>
       </c>
-      <c r="AL7" t="n">
+      <c r="BH7" t="n">
         <v>0.5649508978686322</v>
       </c>
-      <c r="AM7" t="n">
+      <c r="BI7" t="n">
         <v>0.5445931663556255</v>
       </c>
-      <c r="AN7" t="n">
+      <c r="BJ7" t="n">
         <v>507.3270238049855</v>
       </c>
-      <c r="AO7" t="n">
+      <c r="BK7" t="n">
         <v>0.9505697138597924</v>
       </c>
-      <c r="AP7" t="n">
+      <c r="BL7" t="n">
         <v>674.066864619529</v>
       </c>
-      <c r="AQ7" t="n">
+      <c r="BM7" t="n">
         <v>520.7855063731264</v>
       </c>
-      <c r="AR7" t="n">
+      <c r="BN7" t="n">
         <v>0.4312946522522004</v>
       </c>
-      <c r="AS7" t="n">
+      <c r="BO7" t="n">
         <v>0.2975790404866964</v>
       </c>
-      <c r="AT7" t="n">
+      <c r="BP7" t="n">
         <v>0.2231842803650222</v>
       </c>
-      <c r="AU7" t="n">
+      <c r="BQ7" t="n">
         <v>0.6570736359990065</v>
       </c>
-      <c r="AV7" t="n">
+      <c r="BR7" t="n">
         <v>0.5665736133518423</v>
       </c>
-      <c r="AW7" t="n">
+      <c r="BS7" t="n">
         <v>0.6294486453735235</v>
       </c>
-      <c r="AX7" t="n">
+      <c r="BT7" t="n">
         <v>0.6923236773952047</v>
       </c>
-      <c r="AY7" t="n">
+      <c r="BU7" t="n">
         <v>0.4888283553242228</v>
       </c>
-      <c r="AZ7" t="n">
+      <c r="BV7" t="n">
         <v>0.127559622946259</v>
       </c>
-      <c r="BA7" t="n">
+      <c r="BW7" t="n">
         <v>0.05371049954779572</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.3625</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.8529356580420905</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1.066429875635743</v>
+      </c>
+      <c r="G8" t="n">
+        <v>334.9958456714842</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.3573195700399479</v>
+      </c>
+      <c r="I8" t="n">
+        <v>507.3270238049855</v>
+      </c>
+      <c r="J8" t="n">
+        <v>576129.2435136657</v>
+      </c>
+      <c r="K8" t="n">
+        <v>40099.19419057097</v>
+      </c>
+      <c r="L8" t="n">
+        <v>37693.24253913671</v>
+      </c>
+      <c r="M8" t="n">
+        <v>32149.91062885868</v>
+      </c>
+      <c r="N8" t="n">
+        <v>37.468431947452</v>
+      </c>
+      <c r="O8" t="n">
+        <v>544.7954557524375</v>
+      </c>
+      <c r="P8" t="n">
+        <v>544.7954557524375</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>1.238387978501664</v>
+      </c>
+      <c r="R8" t="n">
+        <v>713471.5292305814</v>
+      </c>
+      <c r="S8" t="n">
+        <v>713471.5292305814</v>
+      </c>
+      <c r="T8" t="n">
+        <v>412.4399969472064</v>
+      </c>
+      <c r="U8" t="n">
+        <v>427.3990130004892</v>
+      </c>
+      <c r="V8" t="n">
+        <v>0.7615773105863909</v>
+      </c>
+      <c r="W8" t="n">
         <v>0.1461968646286187</v>
       </c>
-      <c r="B8" t="n">
+      <c r="X8" t="n">
         <v>1.064577496794081</v>
       </c>
-      <c r="C8" t="n">
+      <c r="Y8" t="n">
         <v>125.6234421268066</v>
       </c>
-      <c r="D8" t="n">
+      <c r="Z8" t="n">
         <v>0.3482637835623633</v>
       </c>
-      <c r="E8" t="n">
+      <c r="AA8" t="n">
         <v>0.5220220244246978</v>
       </c>
-      <c r="F8" t="n">
+      <c r="AB8" t="n">
         <v>0.1244499868451067</v>
       </c>
-      <c r="G8" t="n">
+      <c r="AC8" t="n">
         <v>0.3625</v>
       </c>
-      <c r="H8" t="n">
+      <c r="AD8" t="n">
         <v>121.435994055913</v>
       </c>
-      <c r="I8" t="n">
+      <c r="AE8" t="n">
         <v>0.3248720262443578</v>
       </c>
-      <c r="J8" t="n">
+      <c r="AF8" t="n">
         <v>0.4902267786136445</v>
       </c>
-      <c r="K8" t="n">
+      <c r="AG8" t="n">
         <v>0.1108926247734101</v>
       </c>
-      <c r="L8" t="n">
+      <c r="AH8" t="n">
         <v>0.6507693397424607</v>
       </c>
-      <c r="M8" t="n">
+      <c r="AI8" t="n">
         <v>0.874751580189404</v>
       </c>
-      <c r="N8" t="n">
+      <c r="AJ8" t="n">
         <v>0.939465360469416</v>
       </c>
-      <c r="O8" t="n">
+      <c r="AK8" t="n">
         <v>0.2778401656135346</v>
       </c>
-      <c r="P8" t="n">
+      <c r="AL8" t="n">
         <v>0.9235220626756799</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="AM8" t="n">
         <v>0.3579847479308438</v>
       </c>
-      <c r="R8" t="n">
+      <c r="AN8" t="n">
         <v>0.532609775801597</v>
       </c>
-      <c r="S8" t="n">
+      <c r="AO8" t="n">
         <v>0.1020682245887486</v>
       </c>
-      <c r="T8" t="n">
+      <c r="AP8" t="n">
         <v>0.8505213355279034</v>
       </c>
-      <c r="U8" t="n">
+      <c r="AQ8" t="n">
         <v>0.5510264886289833</v>
       </c>
-      <c r="V8" t="n">
+      <c r="AR8" t="n">
         <v>0.5472873917189358</v>
       </c>
-      <c r="W8" t="n">
+      <c r="AS8" t="n">
         <v>0.36875</v>
       </c>
-      <c r="X8" t="n">
+      <c r="AT8" t="n">
         <v>0.8886668819554222</v>
       </c>
-      <c r="Y8" t="n">
+      <c r="AU8" t="n">
         <v>0.5897582525396874</v>
       </c>
-      <c r="Z8" t="n">
+      <c r="AV8" t="n">
         <v>0.3413794902364864</v>
       </c>
-      <c r="AA8" t="n">
+      <c r="AW8" t="n">
         <v>0.9168465296054072</v>
       </c>
-      <c r="AB8" t="n">
+      <c r="AX8" t="n">
         <v>0.3270882770657199</v>
       </c>
-      <c r="AC8" t="n">
+      <c r="AY8" t="n">
         <v>134.8326123950213</v>
       </c>
-      <c r="AD8" t="n">
+      <c r="AZ8" t="n">
         <v>4.317328488730078</v>
       </c>
-      <c r="AE8" t="n">
+      <c r="BA8" t="n">
         <v>241.4104959520961</v>
       </c>
-      <c r="AF8" t="n">
+      <c r="BB8" t="n">
         <v>123.5297180913598</v>
       </c>
-      <c r="AG8" t="n">
+      <c r="BC8" t="n">
         <v>159.1402078158146</v>
       </c>
-      <c r="AH8" t="n">
+      <c r="BD8" t="n">
         <v>222.1117834262884</v>
       </c>
-      <c r="AI8" t="n">
+      <c r="BE8" t="n">
         <v>0.9797853895098045</v>
       </c>
-      <c r="AJ8" t="n">
+      <c r="BF8" t="n">
         <v>497.0716056276176</v>
       </c>
-      <c r="AK8" t="n">
+      <c r="BG8" t="n">
         <v>447.2155310812989</v>
       </c>
-      <c r="AL8" t="n">
+      <c r="BH8" t="n">
         <v>0.5398079430926793</v>
       </c>
-      <c r="AM8" t="n">
+      <c r="BI8" t="n">
         <v>0.5196824902963315</v>
       </c>
-      <c r="AN8" t="n">
+      <c r="BJ8" t="n">
         <v>544.7954557524375</v>
       </c>
-      <c r="AO8" t="n">
+      <c r="BK8" t="n">
         <v>0.9549883515465672</v>
       </c>
-      <c r="AP8" t="n">
+      <c r="BL8" t="n">
         <v>677.2002037192149</v>
       </c>
-      <c r="AQ8" t="n">
+      <c r="BM8" t="n">
         <v>521.9945152666484</v>
       </c>
-      <c r="AR8" t="n">
+      <c r="BN8" t="n">
         <v>0.4255059716725719</v>
       </c>
-      <c r="AS8" t="n">
+      <c r="BO8" t="n">
         <v>0.2975790404866964</v>
       </c>
-      <c r="AT8" t="n">
+      <c r="BP8" t="n">
         <v>0.2231842803650222</v>
       </c>
-      <c r="AU8" t="n">
+      <c r="BQ8" t="n">
         <v>0.6684108649448608</v>
       </c>
-      <c r="AV8" t="n">
+      <c r="BR8" t="n">
         <v>0.5665736133518423</v>
       </c>
-      <c r="AW8" t="n">
+      <c r="BS8" t="n">
         <v>0.6327433073496426</v>
       </c>
-      <c r="AX8" t="n">
+      <c r="BT8" t="n">
         <v>0.6989130013474428</v>
       </c>
-      <c r="AY8" t="n">
+      <c r="BU8" t="n">
         <v>0.4972626596029361</v>
       </c>
-      <c r="AZ8" t="n">
+      <c r="BV8" t="n">
         <v>0.1233424708069024</v>
       </c>
-      <c r="BA8" t="n">
+      <c r="BW8" t="n">
         <v>0.04658913073714011</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
+        <v>0.3625</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.8442592793216259</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.066429875635743</v>
+      </c>
+      <c r="G9" t="n">
+        <v>334.9958456714842</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.3605527408399267</v>
+      </c>
+      <c r="I9" t="n">
+        <v>544.7954557524375</v>
+      </c>
+      <c r="J9" t="n">
+        <v>713471.5292305814</v>
+      </c>
+      <c r="K9" t="n">
+        <v>40462.02778444644</v>
+      </c>
+      <c r="L9" t="n">
+        <v>38034.30611737965</v>
+      </c>
+      <c r="M9" t="n">
+        <v>32110.81587215705</v>
+      </c>
+      <c r="N9" t="n">
+        <v>37.80746134928394</v>
+      </c>
+      <c r="O9" t="n">
+        <v>582.6029171017215</v>
+      </c>
+      <c r="P9" t="n">
+        <v>582.6029171017215</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>1.220524649009106</v>
+      </c>
+      <c r="R9" t="n">
+        <v>870809.5877921456</v>
+      </c>
+      <c r="S9" t="n">
+        <v>870809.5877921456</v>
+      </c>
+      <c r="T9" t="n">
+        <v>427.3990130004892</v>
+      </c>
+      <c r="U9" t="n">
+        <v>441.980495162634</v>
+      </c>
+      <c r="V9" t="n">
+        <v>0.7615773105863909</v>
+      </c>
+      <c r="W9" t="n">
         <v>0.1440741840057616</v>
       </c>
-      <c r="B9" t="n">
+      <c r="X9" t="n">
         <v>1.064577496794081</v>
       </c>
-      <c r="C9" t="n">
+      <c r="Y9" t="n">
         <v>121.435994055913</v>
       </c>
-      <c r="D9" t="n">
+      <c r="Z9" t="n">
         <v>0.3248720262443578</v>
       </c>
-      <c r="E9" t="n">
+      <c r="AA9" t="n">
         <v>0.4902267786136445</v>
       </c>
-      <c r="F9" t="n">
+      <c r="AB9" t="n">
         <v>0.1108926247734101</v>
       </c>
-      <c r="G9" t="n">
+      <c r="AC9" t="n">
         <v>0.35</v>
       </c>
-      <c r="H9" t="n">
+      <c r="AD9" t="n">
         <v>117.2485459850195</v>
       </c>
-      <c r="I9" t="n">
+      <c r="AE9" t="n">
         <v>0.3033211971446864</v>
       </c>
-      <c r="J9" t="n">
+      <c r="AF9" t="n">
         <v>0.4603395387699436</v>
       </c>
-      <c r="K9" t="n">
+      <c r="AG9" t="n">
         <v>0.100056302624151</v>
       </c>
-      <c r="L9" t="n">
+      <c r="AH9" t="n">
         <v>0.6619729934593227</v>
       </c>
-      <c r="M9" t="n">
+      <c r="AI9" t="n">
         <v>0.8898113151741506</v>
       </c>
-      <c r="N9" t="n">
+      <c r="AJ9" t="n">
         <v>0.946510479765531</v>
       </c>
-      <c r="O9" t="n">
+      <c r="AK9" t="n">
         <v>0.281528605843333</v>
       </c>
-      <c r="P9" t="n">
+      <c r="AL9" t="n">
         <v>0.9005374717254715</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="AM9" t="n">
         <v>0.3404490152611628</v>
       </c>
-      <c r="R9" t="n">
+      <c r="AN9" t="n">
         <v>0.5088534310976932</v>
       </c>
-      <c r="S9" t="n">
+      <c r="AO9" t="n">
         <v>0.09051697283767492</v>
       </c>
-      <c r="T9" t="n">
+      <c r="AP9" t="n">
         <v>0.854043895175961</v>
       </c>
-      <c r="U9" t="n">
+      <c r="AQ9" t="n">
         <v>0.5506466038529215</v>
       </c>
-      <c r="V9" t="n">
+      <c r="AR9" t="n">
         <v>0.5308367445217098</v>
       </c>
-      <c r="W9" t="n">
+      <c r="AS9" t="n">
         <v>0.35625</v>
       </c>
-      <c r="X9" t="n">
+      <c r="AT9" t="n">
         <v>0.8653500475224741</v>
       </c>
-      <c r="Y9" t="n">
+      <c r="AU9" t="n">
         <v>0.5742398709033788</v>
       </c>
-      <c r="Z9" t="n">
+      <c r="AV9" t="n">
         <v>0.3345133030007643</v>
       </c>
-      <c r="AA9" t="n">
+      <c r="AW9" t="n">
         <v>0.8933979759636368</v>
       </c>
-      <c r="AB9" t="n">
+      <c r="AX9" t="n">
         <v>0.319158105060258</v>
       </c>
-      <c r="AC9" t="n">
+      <c r="AY9" t="n">
         <v>130.6757008041521</v>
       </c>
-      <c r="AD9" t="n">
+      <c r="AZ9" t="n">
         <v>4.953187281049108</v>
       </c>
-      <c r="AE9" t="n">
+      <c r="BA9" t="n">
         <v>239.8711457535123</v>
       </c>
-      <c r="AF9" t="n">
+      <c r="BB9" t="n">
         <v>119.3422700204662</v>
       </c>
-      <c r="AG9" t="n">
+      <c r="BC9" t="n">
         <v>156.7565726515706</v>
       </c>
-      <c r="AH9" t="n">
+      <c r="BD9" t="n">
         <v>219.7035832877112</v>
       </c>
-      <c r="AI9" t="n">
+      <c r="BE9" t="n">
         <v>0.9824096944273142</v>
       </c>
-      <c r="AJ9" t="n">
+      <c r="BF9" t="n">
         <v>535.2123372111415</v>
       </c>
-      <c r="AK9" t="n">
+      <c r="BG9" t="n">
         <v>464.0560698884079</v>
       </c>
-      <c r="AL9" t="n">
+      <c r="BH9" t="n">
         <v>0.5169012137072022</v>
       </c>
-      <c r="AM9" t="n">
+      <c r="BI9" t="n">
         <v>0.4970888663466193</v>
       </c>
-      <c r="AN9" t="n">
+      <c r="BJ9" t="n">
         <v>582.6029171017215</v>
       </c>
-      <c r="AO9" t="n">
+      <c r="BK9" t="n">
         <v>0.9588171098257054</v>
       </c>
-      <c r="AP9" t="n">
+      <c r="BL9" t="n">
         <v>679.9152482351244</v>
       </c>
-      <c r="AQ9" t="n">
+      <c r="BM9" t="n">
         <v>523.0398639490919</v>
       </c>
-      <c r="AR9" t="n">
+      <c r="BN9" t="n">
         <v>0.4200513162206986</v>
       </c>
-      <c r="AS9" t="n">
+      <c r="BO9" t="n">
         <v>0.2975790404866964</v>
       </c>
-      <c r="AT9" t="n">
+      <c r="BP9" t="n">
         <v>0.2231842803650222</v>
       </c>
-      <c r="AU9" t="n">
+      <c r="BQ9" t="n">
         <v>0.6773344445505896</v>
       </c>
-      <c r="AV9" t="n">
+      <c r="BR9" t="n">
         <v>0.5665736133518423</v>
       </c>
-      <c r="AW9" t="n">
+      <c r="BS9" t="n">
         <v>0.6353639071499578</v>
       </c>
-      <c r="AX9" t="n">
+      <c r="BT9" t="n">
         <v>0.7041542009480733</v>
       </c>
-      <c r="AY9" t="n">
+      <c r="BU9" t="n">
         <v>0.5039013352448847</v>
       </c>
-      <c r="AZ9" t="n">
+      <c r="BV9" t="n">
         <v>0.1200231329859281</v>
       </c>
-      <c r="BA9" t="n">
+      <c r="BW9" t="n">
         <v>0.04098730387870908</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.3375</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.8345538265996715</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1.066429875635743</v>
+      </c>
+      <c r="G10" t="n">
+        <v>334.9958456714842</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.3629425367369873</v>
+      </c>
+      <c r="I10" t="n">
+        <v>582.6029171017215</v>
+      </c>
+      <c r="J10" t="n">
+        <v>870809.5877921456</v>
+      </c>
+      <c r="K10" t="n">
+        <v>40730.21597727716</v>
+      </c>
+      <c r="L10" t="n">
+        <v>38286.40301864053</v>
+      </c>
+      <c r="M10" t="n">
+        <v>31952.06414594367</v>
+      </c>
+      <c r="N10" t="n">
+        <v>38.05805469049754</v>
+      </c>
+      <c r="O10" t="n">
+        <v>620.660971792219</v>
+      </c>
+      <c r="P10" t="n">
+        <v>620.660971792219</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>1.204167456353411</v>
+      </c>
+      <c r="R10" t="n">
+        <v>1048600.566299831</v>
+      </c>
+      <c r="S10" t="n">
+        <v>1048600.566299831</v>
+      </c>
+      <c r="T10" t="n">
+        <v>441.980495162634</v>
+      </c>
+      <c r="U10" t="n">
+        <v>456.1881452229234</v>
+      </c>
+      <c r="V10" t="n">
+        <v>0.7615773105863909</v>
+      </c>
+      <c r="W10" t="n">
         <v>0.1425052061332324</v>
       </c>
-      <c r="B10" t="n">
+      <c r="X10" t="n">
         <v>1.064577496794081</v>
       </c>
-      <c r="C10" t="n">
+      <c r="Y10" t="n">
         <v>117.2485459850195</v>
       </c>
-      <c r="D10" t="n">
+      <c r="Z10" t="n">
         <v>0.3033211971446864</v>
       </c>
-      <c r="E10" t="n">
+      <c r="AA10" t="n">
         <v>0.4603395387699436</v>
       </c>
-      <c r="F10" t="n">
+      <c r="AB10" t="n">
         <v>0.100056302624151</v>
       </c>
-      <c r="G10" t="n">
+      <c r="AC10" t="n">
         <v>0.3375</v>
       </c>
-      <c r="H10" t="n">
+      <c r="AD10" t="n">
         <v>113.0610979141259</v>
       </c>
-      <c r="I10" t="n">
+      <c r="AE10" t="n">
         <v>0.2833789606329719</v>
       </c>
-      <c r="J10" t="n">
+      <c r="AF10" t="n">
         <v>0.4322063770688386</v>
       </c>
-      <c r="K10" t="n">
+      <c r="AG10" t="n">
         <v>0.09134516475091831</v>
       </c>
-      <c r="L10" t="n">
+      <c r="AH10" t="n">
         <v>0.6709315018399133</v>
       </c>
-      <c r="M10" t="n">
+      <c r="AI10" t="n">
         <v>0.9018531691514183</v>
       </c>
-      <c r="N10" t="n">
+      <c r="AJ10" t="n">
         <v>0.9521919813536703</v>
       </c>
-      <c r="O10" t="n">
+      <c r="AK10" t="n">
         <v>0.2847475699273967</v>
       </c>
-      <c r="P10" t="n">
+      <c r="AL10" t="n">
         <v>0.8775390029012443</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="AM10" t="n">
         <v>0.3242639972996528</v>
       </c>
-      <c r="R10" t="n">
+      <c r="AN10" t="n">
         <v>0.4865739919422437</v>
       </c>
-      <c r="S10" t="n">
+      <c r="AO10" t="n">
         <v>0.08113866210185122</v>
       </c>
-      <c r="T10" t="n">
+      <c r="AP10" t="n">
         <v>0.8568846459700306</v>
       </c>
-      <c r="U10" t="n">
+      <c r="AQ10" t="n">
         <v>0.5502155635368724</v>
       </c>
-      <c r="V10" t="n">
+      <c r="AR10" t="n">
         <v>0.5145610942928165</v>
       </c>
-      <c r="W10" t="n">
+      <c r="AS10" t="n">
         <v>0.34375</v>
       </c>
-      <c r="X10" t="n">
+      <c r="AT10" t="n">
         <v>0.8423473256617744</v>
       </c>
-      <c r="Y10" t="n">
+      <c r="AU10" t="n">
         <v>0.5584232149984406</v>
       </c>
-      <c r="Z10" t="n">
+      <c r="AV10" t="n">
         <v>0.3277862313689579</v>
       </c>
-      <c r="AA10" t="n">
+      <c r="AW10" t="n">
         <v>0.8699731692653212</v>
       </c>
-      <c r="AB10" t="n">
+      <c r="AX10" t="n">
         <v>0.3115499542668806</v>
       </c>
-      <c r="AC10" t="n">
+      <c r="AY10" t="n">
         <v>126.5946303533889</v>
       </c>
-      <c r="AD10" t="n">
+      <c r="AZ10" t="n">
         <v>5.624360949315135</v>
       </c>
-      <c r="AE10" t="n">
+      <c r="BA10" t="n">
         <v>238.2360518720631</v>
       </c>
-      <c r="AF10" t="n">
+      <c r="BB10" t="n">
         <v>115.1548219495727</v>
       </c>
-      <c r="AG10" t="n">
+      <c r="BC10" t="n">
         <v>154.3200418328142</v>
       </c>
-      <c r="AH10" t="n">
+      <c r="BD10" t="n">
         <v>217.3349232851236</v>
       </c>
-      <c r="AI10" t="n">
+      <c r="BE10" t="n">
         <v>0.9846660418937857</v>
       </c>
-      <c r="AJ10" t="n">
+      <c r="BF10" t="n">
         <v>573.6693083783255</v>
       </c>
-      <c r="AK10" t="n">
+      <c r="BG10" t="n">
         <v>480.4389481704237</v>
       </c>
-      <c r="AL10" t="n">
+      <c r="BH10" t="n">
         <v>0.4958716456675673</v>
       </c>
-      <c r="AM10" t="n">
+      <c r="BI10" t="n">
         <v>0.4764151053923584</v>
       </c>
-      <c r="AN10" t="n">
+      <c r="BJ10" t="n">
         <v>620.660971792219</v>
       </c>
-      <c r="AO10" t="n">
+      <c r="BK10" t="n">
         <v>0.9621714412256647</v>
       </c>
-      <c r="AP10" t="n">
+      <c r="BL10" t="n">
         <v>682.2938677268862</v>
       </c>
-      <c r="AQ10" t="n">
+      <c r="BM10" t="n">
         <v>523.9539680340154</v>
       </c>
-      <c r="AR10" t="n">
+      <c r="BN10" t="n">
         <v>0.4147977428257859</v>
       </c>
-      <c r="AS10" t="n">
+      <c r="BO10" t="n">
         <v>0.2975790404866964</v>
       </c>
-      <c r="AT10" t="n">
+      <c r="BP10" t="n">
         <v>0.2231842803650222</v>
       </c>
-      <c r="AU10" t="n">
+      <c r="BQ10" t="n">
         <v>0.6844724925067254</v>
       </c>
-      <c r="AV10" t="n">
+      <c r="BR10" t="n">
         <v>0.5665736133518423</v>
       </c>
-      <c r="AW10" t="n">
+      <c r="BS10" t="n">
         <v>0.6374772768888605</v>
       </c>
-      <c r="AX10" t="n">
+      <c r="BT10" t="n">
         <v>0.7083809404258787</v>
       </c>
-      <c r="AY10" t="n">
+      <c r="BU10" t="n">
         <v>0.509211668899222</v>
       </c>
-      <c r="AZ10" t="n">
+      <c r="BV10" t="n">
         <v>0.1173679661587594</v>
       </c>
-      <c r="BA10" t="n">
+      <c r="BW10" t="n">
         <v>0.03650804968841376</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
+        <v>0.3375</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.8238053834530781</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1.066429875635743</v>
+      </c>
+      <c r="G11" t="n">
+        <v>334.9958456714842</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.3644008637646071</v>
+      </c>
+      <c r="I11" t="n">
+        <v>620.660971792219</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1048600.566299831</v>
+      </c>
+      <c r="K11" t="n">
+        <v>40893.87266886935</v>
+      </c>
+      <c r="L11" t="n">
+        <v>38440.24030873719</v>
+      </c>
+      <c r="M11" t="n">
+        <v>31667.27690756771</v>
+      </c>
+      <c r="N11" t="n">
+        <v>38.21097446196539</v>
+      </c>
+      <c r="O11" t="n">
+        <v>658.8719462541844</v>
+      </c>
+      <c r="P11" t="n">
+        <v>658.8719462541844</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>1.189052302015514</v>
+      </c>
+      <c r="R11" t="n">
+        <v>1246840.917253586</v>
+      </c>
+      <c r="S11" t="n">
+        <v>1246840.917253586</v>
+      </c>
+      <c r="T11" t="n">
+        <v>456.1881452229234</v>
+      </c>
+      <c r="U11" t="n">
+        <v>470.021024613823</v>
+      </c>
+      <c r="V11" t="n">
+        <v>0.7615773105863909</v>
+      </c>
+      <c r="W11" t="n">
         <v>0.141547767533534</v>
       </c>
-      <c r="B11" t="n">
+      <c r="X11" t="n">
         <v>1.064577496794081</v>
       </c>
-      <c r="C11" t="n">
+      <c r="Y11" t="n">
         <v>113.0610979141259</v>
       </c>
-      <c r="D11" t="n">
+      <c r="Z11" t="n">
         <v>0.2833789606329719</v>
       </c>
-      <c r="E11" t="n">
+      <c r="AA11" t="n">
         <v>0.4322063770688386</v>
       </c>
-      <c r="F11" t="n">
+      <c r="AB11" t="n">
         <v>0.09134516475091832</v>
       </c>
-      <c r="G11" t="n">
+      <c r="AC11" t="n">
         <v>0.325</v>
       </c>
-      <c r="H11" t="n">
+      <c r="AD11" t="n">
         <v>108.8736498432324</v>
       </c>
-      <c r="I11" t="n">
+      <c r="AE11" t="n">
         <v>0.264852390566271</v>
       </c>
-      <c r="J11" t="n">
+      <c r="AF11" t="n">
         <v>0.4056848070423067</v>
       </c>
-      <c r="K11" t="n">
+      <c r="AG11" t="n">
         <v>0.08432577123228341</v>
       </c>
-      <c r="L11" t="n">
+      <c r="AH11" t="n">
         <v>0.6781934296933768</v>
       </c>
-      <c r="M11" t="n">
+      <c r="AI11" t="n">
         <v>0.9116145123449262</v>
       </c>
-      <c r="N11" t="n">
+      <c r="AJ11" t="n">
         <v>0.9568283595080879</v>
       </c>
-      <c r="O11" t="n">
+      <c r="AK11" t="n">
         <v>0.2877665857908671</v>
       </c>
-      <c r="P11" t="n">
+      <c r="AL11" t="n">
         <v>0.8540733970766762</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="AM11" t="n">
         <v>0.3093872915612632</v>
       </c>
-      <c r="R11" t="n">
+      <c r="AN11" t="n">
         <v>0.4657932677724579</v>
       </c>
-      <c r="S11" t="n">
+      <c r="AO11" t="n">
         <v>0.07344392158062314</v>
       </c>
-      <c r="T11" t="n">
+      <c r="AP11" t="n">
         <v>0.8592028350472394</v>
       </c>
-      <c r="U11" t="n">
+      <c r="AQ11" t="n">
         <v>0.5495796948299662</v>
       </c>
-      <c r="V11" t="n">
+      <c r="AR11" t="n">
         <v>0.4984787765891089</v>
       </c>
-      <c r="W11" t="n">
+      <c r="AS11" t="n">
         <v>0.33125</v>
       </c>
-      <c r="X11" t="n">
+      <c r="AT11" t="n">
         <v>0.8191312917860756</v>
       </c>
-      <c r="Y11" t="n">
+      <c r="AU11" t="n">
         <v>0.5424268789629988</v>
       </c>
-      <c r="Z11" t="n">
+      <c r="AV11" t="n">
         <v>0.3206525151969667</v>
       </c>
-      <c r="AA11" t="n">
+      <c r="AW11" t="n">
         <v>0.8460863486369866</v>
       </c>
-      <c r="AB11" t="n">
+      <c r="AX11" t="n">
         <v>0.3036594696739878</v>
       </c>
-      <c r="AC11" t="n">
+      <c r="AY11" t="n">
         <v>122.6020817033145</v>
       </c>
-      <c r="AD11" t="n">
+      <c r="AZ11" t="n">
         <v>6.325027396634392</v>
       </c>
-      <c r="AE11" t="n">
+      <c r="BA11" t="n">
         <v>236.4849743786179</v>
       </c>
-      <c r="AF11" t="n">
+      <c r="BB11" t="n">
         <v>110.9673738786792</v>
       </c>
-      <c r="AG11" t="n">
+      <c r="BC11" t="n">
         <v>151.8950557315864</v>
       </c>
-      <c r="AH11" t="n">
+      <c r="BD11" t="n">
         <v>214.9630528285631</v>
       </c>
-      <c r="AI11" t="n">
+      <c r="BE11" t="n">
         <v>0.9866160607784294</v>
       </c>
-      <c r="AJ11" t="n">
+      <c r="BF11" t="n">
         <v>612.3540830685511</v>
       </c>
-      <c r="AK11" t="n">
+      <c r="BG11" t="n">
         <v>496.3736383647526</v>
       </c>
-      <c r="AL11" t="n">
+      <c r="BH11" t="n">
         <v>0.4764253298335728</v>
       </c>
-      <c r="AM11" t="n">
+      <c r="BI11" t="n">
         <v>0.45734773887015</v>
       </c>
-      <c r="AN11" t="n">
+      <c r="BJ11" t="n">
         <v>658.8719462541844</v>
       </c>
-      <c r="AO11" t="n">
+      <c r="BK11" t="n">
         <v>0.9651388409583935</v>
       </c>
-      <c r="AP11" t="n">
+      <c r="BL11" t="n">
         <v>684.3981066951061</v>
       </c>
-      <c r="AQ11" t="n">
+      <c r="BM11" t="n">
         <v>524.7613002211986</v>
       </c>
-      <c r="AR11" t="n">
+      <c r="BN11" t="n">
         <v>0.4096396832959126</v>
       </c>
-      <c r="AS11" t="n">
+      <c r="BO11" t="n">
         <v>0.2975790404866964</v>
       </c>
-      <c r="AT11" t="n">
+      <c r="BP11" t="n">
         <v>0.2231842803650222</v>
       </c>
-      <c r="AU11" t="n">
+      <c r="BQ11" t="n">
         <v>0.6902601129331082</v>
       </c>
-      <c r="AV11" t="n">
+      <c r="BR11" t="n">
         <v>0.5665736133518423</v>
       </c>
-      <c r="AW11" t="n">
+      <c r="BS11" t="n">
         <v>0.6392018880920168</v>
       </c>
-      <c r="AX11" t="n">
+      <c r="BT11" t="n">
         <v>0.7118301628321914</v>
       </c>
-      <c r="AY11" t="n">
+      <c r="BU11" t="n">
         <v>0.5135173552321824</v>
       </c>
-      <c r="AZ11" t="n">
+      <c r="BV11" t="n">
         <v>0.1152151229922792</v>
       </c>
-      <c r="BA11" t="n">
+      <c r="BW11" t="n">
         <v>0.03287708576168202</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.8120003556960932</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1.066429875635743</v>
+      </c>
+      <c r="G12" t="n">
+        <v>334.9958456714842</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.3648340491519012</v>
+      </c>
+      <c r="I12" t="n">
+        <v>658.8719462541844</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1246840.917253586</v>
+      </c>
+      <c r="K12" t="n">
+        <v>40942.48569323765</v>
+      </c>
+      <c r="L12" t="n">
+        <v>38485.93655164339</v>
+      </c>
+      <c r="M12" t="n">
+        <v>31250.59416923171</v>
+      </c>
+      <c r="N12" t="n">
+        <v>38.25639816266739</v>
+      </c>
+      <c r="O12" t="n">
+        <v>697.1283444168519</v>
+      </c>
+      <c r="P12" t="n">
+        <v>697.1283444168519</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>1.174972243401005</v>
+      </c>
+      <c r="R12" t="n">
+        <v>1465003.469709612</v>
+      </c>
+      <c r="S12" t="n">
+        <v>1465003.469709612</v>
+      </c>
+      <c r="T12" t="n">
+        <v>470.021024613823</v>
+      </c>
+      <c r="U12" t="n">
+        <v>483.4740260685887</v>
+      </c>
+      <c r="V12" t="n">
+        <v>0.7615773105863909</v>
+      </c>
+      <c r="W12" t="n">
         <v>0.1412633673936713</v>
       </c>
-      <c r="B12" t="n">
+      <c r="X12" t="n">
         <v>1.064577496794081</v>
       </c>
-      <c r="C12" t="n">
+      <c r="Y12" t="n">
         <v>108.8736498432324</v>
       </c>
-      <c r="D12" t="n">
+      <c r="Z12" t="n">
         <v>0.264852390566271</v>
       </c>
-      <c r="E12" t="n">
+      <c r="AA12" t="n">
         <v>0.4056848070423067</v>
       </c>
-      <c r="F12" t="n">
+      <c r="AB12" t="n">
         <v>0.08432577123228341</v>
       </c>
-      <c r="G12" t="n">
+      <c r="AC12" t="n">
         <v>0.3125</v>
       </c>
-      <c r="H12" t="n">
+      <c r="AD12" t="n">
         <v>104.6862017723388</v>
       </c>
-      <c r="I12" t="n">
+      <c r="AE12" t="n">
         <v>0.2475795080404627</v>
       </c>
-      <c r="J12" t="n">
+      <c r="AF12" t="n">
         <v>0.3806439700063695</v>
       </c>
-      <c r="K12" t="n">
+      <c r="AG12" t="n">
         <v>0.07867891571681149</v>
       </c>
-      <c r="L12" t="n">
+      <c r="AH12" t="n">
         <v>0.6841493266339539</v>
       </c>
-      <c r="M12" t="n">
+      <c r="AI12" t="n">
         <v>0.9196203140046615</v>
       </c>
-      <c r="N12" t="n">
+      <c r="AJ12" t="n">
         <v>0.9606512171256621</v>
       </c>
-      <c r="O12" t="n">
+      <c r="AK12" t="n">
         <v>0.2907964460364127</v>
       </c>
-      <c r="P12" t="n">
+      <c r="AL12" t="n">
         <v>0.8297807583132409</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="AM12" t="n">
         <v>0.2957759736655972</v>
       </c>
-      <c r="R12" t="n">
+      <c r="AN12" t="n">
         <v>0.4465201903401176</v>
       </c>
-      <c r="S12" t="n">
+      <c r="AO12" t="n">
         <v>0.06707122204581961</v>
       </c>
-      <c r="T12" t="n">
+      <c r="AP12" t="n">
         <v>0.8611142638560265</v>
       </c>
-      <c r="U12" t="n">
+      <c r="AQ12" t="n">
         <v>0.5486113102580497</v>
       </c>
-      <c r="V12" t="n">
+      <c r="AR12" t="n">
         <v>0.4826064562566781</v>
       </c>
-      <c r="W12" t="n">
+      <c r="AS12" t="n">
         <v>0.31875</v>
       </c>
-      <c r="X12" t="n">
+      <c r="AT12" t="n">
         <v>0.7952941051769974</v>
       </c>
-      <c r="Y12" t="n">
+      <c r="AU12" t="n">
         <v>0.5263410536891099</v>
       </c>
-      <c r="Z12" t="n">
+      <c r="AV12" t="n">
         <v>0.3126876489203193</v>
       </c>
-      <c r="AA12" t="n">
+      <c r="AW12" t="n">
         <v>0.8213575967455732</v>
       </c>
-      <c r="AB12" t="n">
+      <c r="AX12" t="n">
         <v>0.2950165430564633</v>
       </c>
-      <c r="AC12" t="n">
+      <c r="AY12" t="n">
         <v>118.7135375702998</v>
       </c>
-      <c r="AD12" t="n">
+      <c r="AZ12" t="n">
         <v>7.048422847999833</v>
       </c>
-      <c r="AE12" t="n">
+      <c r="BA12" t="n">
         <v>234.596226942576</v>
       </c>
-      <c r="AF12" t="n">
+      <c r="BB12" t="n">
         <v>106.7799258077856</v>
       </c>
-      <c r="AG12" t="n">
+      <c r="BC12" t="n">
         <v>149.5371544469267</v>
       </c>
-      <c r="AH12" t="n">
+      <c r="BD12" t="n">
         <v>212.5510843845128</v>
       </c>
-      <c r="AI12" t="n">
+      <c r="BE12" t="n">
         <v>0.9883088685352219</v>
       </c>
-      <c r="AJ12" t="n">
+      <c r="BF12" t="n">
         <v>651.1689877120725</v>
       </c>
-      <c r="AK12" t="n">
+      <c r="BG12" t="n">
         <v>511.8636086848034</v>
       </c>
-      <c r="AL12" t="n">
+      <c r="BH12" t="n">
         <v>0.4583178467118498</v>
       </c>
-      <c r="AM12" t="n">
+      <c r="BI12" t="n">
         <v>0.4396328922008292</v>
       </c>
-      <c r="AN12" t="n">
+      <c r="BJ12" t="n">
         <v>697.1283444168519</v>
       </c>
-      <c r="AO12" t="n">
+      <c r="BK12" t="n">
         <v>0.967787153349189</v>
       </c>
-      <c r="AP12" t="n">
+      <c r="BL12" t="n">
         <v>686.2760748270256</v>
       </c>
-      <c r="AQ12" t="n">
+      <c r="BM12" t="n">
         <v>525.4807717389875</v>
       </c>
-      <c r="AR12" t="n">
+      <c r="BN12" t="n">
         <v>0.4044887954341541</v>
       </c>
-      <c r="AS12" t="n">
+      <c r="BO12" t="n">
         <v>0.2975790404866964</v>
       </c>
-      <c r="AT12" t="n">
+      <c r="BP12" t="n">
         <v>0.2231842803650222</v>
       </c>
-      <c r="AU12" t="n">
+      <c r="BQ12" t="n">
         <v>0.6950075904856097</v>
       </c>
-      <c r="AV12" t="n">
+      <c r="BR12" t="n">
         <v>0.5665736133518423</v>
       </c>
-      <c r="AW12" t="n">
+      <c r="BS12" t="n">
         <v>0.6406238909692106</v>
       </c>
-      <c r="AX12" t="n">
+      <c r="BT12" t="n">
         <v>0.7146741685865788</v>
       </c>
-      <c r="AY12" t="n">
+      <c r="BU12" t="n">
         <v>0.5170492297691963</v>
       </c>
-      <c r="AZ12" t="n">
+      <c r="BV12" t="n">
         <v>0.1134491857237723</v>
       </c>
-      <c r="BA12" t="n">
+      <c r="BW12" t="n">
         <v>0.02989913729139348</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.7991254713803608</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1.066429875635743</v>
+      </c>
+      <c r="G13" t="n">
+        <v>334.9958456714842</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.3641428413236223</v>
+      </c>
+      <c r="I13" t="n">
+        <v>697.1283444168519</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1465003.469709612</v>
+      </c>
+      <c r="K13" t="n">
+        <v>40864.91681860507</v>
+      </c>
+      <c r="L13" t="n">
+        <v>38413.02180948877</v>
+      </c>
+      <c r="M13" t="n">
+        <v>30696.82416065179</v>
+      </c>
+      <c r="N13" t="n">
+        <v>38.18391829969062</v>
+      </c>
+      <c r="O13" t="n">
+        <v>735.3122627165425</v>
+      </c>
+      <c r="P13" t="n">
+        <v>735.3122627165425</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>1.161763539474074</v>
+      </c>
+      <c r="R13" t="n">
+        <v>1701987.616311639</v>
+      </c>
+      <c r="S13" t="n">
+        <v>1701987.616311639</v>
+      </c>
+      <c r="T13" t="n">
+        <v>483.4740260685887</v>
+      </c>
+      <c r="U13" t="n">
+        <v>496.5382177525278</v>
+      </c>
+      <c r="V13" t="n">
+        <v>0.7615773105863909</v>
+      </c>
+      <c r="W13" t="n">
         <v>0.1417171675651513</v>
       </c>
-      <c r="B13" t="n">
+      <c r="X13" t="n">
         <v>1.064577496794081</v>
       </c>
-      <c r="C13" t="n">
+      <c r="Y13" t="n">
         <v>104.6862017723388</v>
       </c>
-      <c r="D13" t="n">
+      <c r="Z13" t="n">
         <v>0.2475795080404627</v>
       </c>
-      <c r="E13" t="n">
+      <c r="AA13" t="n">
         <v>0.3806439700063695</v>
       </c>
-      <c r="F13" t="n">
+      <c r="AB13" t="n">
         <v>0.07867891571681147</v>
       </c>
-      <c r="G13" t="n">
+      <c r="AC13" t="n">
         <v>0.3</v>
       </c>
-      <c r="H13" t="n">
+      <c r="AD13" t="n">
         <v>100.4987537014453</v>
       </c>
-      <c r="I13" t="n">
+      <c r="AE13" t="n">
         <v>0.2314229337341716</v>
       </c>
-      <c r="J13" t="n">
+      <c r="AF13" t="n">
         <v>0.356964158557928</v>
       </c>
-      <c r="K13" t="n">
+      <c r="AG13" t="n">
         <v>0.07416764671794335</v>
       </c>
-      <c r="L13" t="n">
+      <c r="AH13" t="n">
         <v>0.6890844320072977</v>
       </c>
-      <c r="M13" t="n">
+      <c r="AI13" t="n">
         <v>0.9262539873511073</v>
       </c>
-      <c r="N13" t="n">
+      <c r="AJ13" t="n">
         <v>0.9638325708036187</v>
       </c>
-      <c r="O13" t="n">
+      <c r="AK13" t="n">
         <v>0.2940089553983466</v>
       </c>
-      <c r="P13" t="n">
+      <c r="AL13" t="n">
         <v>0.8043697733634284</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="AM13" t="n">
         <v>0.2833915018027358</v>
       </c>
-      <c r="R13" t="n">
+      <c r="AN13" t="n">
         <v>0.4287582016046487</v>
       </c>
-      <c r="S13" t="n">
+      <c r="AO13" t="n">
         <v>0.0617485368298673</v>
       </c>
-      <c r="T13" t="n">
+      <c r="AP13" t="n">
         <v>0.8627049406950048</v>
       </c>
-      <c r="U13" t="n">
+      <c r="AQ13" t="n">
         <v>0.5471991620698325</v>
       </c>
-      <c r="V13" t="n">
+      <c r="AR13" t="n">
         <v>0.466958890421039</v>
       </c>
-      <c r="W13" t="n">
+      <c r="AS13" t="n">
         <v>0.30625</v>
       </c>
-      <c r="X13" t="n">
+      <c r="AT13" t="n">
         <v>0.7705127448541069</v>
       </c>
-      <c r="Y13" t="n">
+      <c r="AU13" t="n">
         <v>0.5102357395223244</v>
       </c>
-      <c r="Z13" t="n">
+      <c r="AV13" t="n">
         <v>0.3035538544330679</v>
       </c>
-      <c r="AA13" t="n">
+      <c r="AW13" t="n">
         <v>0.7954836030482841</v>
       </c>
-      <c r="AB13" t="n">
+      <c r="AX13" t="n">
         <v>0.2852478635259598</v>
       </c>
-      <c r="AC13" t="n">
+      <c r="AY13" t="n">
         <v>114.9480074251195</v>
       </c>
-      <c r="AD13" t="n">
+      <c r="AZ13" t="n">
         <v>7.786942573692805</v>
       </c>
-      <c r="AE13" t="n">
+      <c r="BA13" t="n">
         <v>232.5466861290662</v>
       </c>
-      <c r="AF13" t="n">
+      <c r="BB13" t="n">
         <v>102.5924777368921</v>
       </c>
-      <c r="AG13" t="n">
+      <c r="BC13" t="n">
         <v>147.2964805650054</v>
       </c>
-      <c r="AH13" t="n">
+      <c r="BD13" t="n">
         <v>210.0656314077421</v>
       </c>
-      <c r="AI13" t="n">
+      <c r="BE13" t="n">
         <v>0.9897840645330738</v>
       </c>
-      <c r="AJ13" t="n">
+      <c r="BF13" t="n">
         <v>690.0065262381241</v>
       </c>
-      <c r="AK13" t="n">
+      <c r="BG13" t="n">
         <v>526.9070372439256</v>
       </c>
-      <c r="AL13" t="n">
+      <c r="BH13" t="n">
         <v>0.4413429119213136</v>
       </c>
-      <c r="AM13" t="n">
+      <c r="BI13" t="n">
         <v>0.4230603484230449</v>
       </c>
-      <c r="AN13" t="n">
+      <c r="BJ13" t="n">
         <v>735.3122627165425</v>
       </c>
-      <c r="AO13" t="n">
+      <c r="BK13" t="n">
         <v>0.970169990265362</v>
       </c>
-      <c r="AP13" t="n">
+      <c r="BL13" t="n">
         <v>687.9657893062114</v>
       </c>
-      <c r="AQ13" t="n">
+      <c r="BM13" t="n">
         <v>526.127280213873</v>
       </c>
-      <c r="AR13" t="n">
+      <c r="BN13" t="n">
         <v>0.3992677044276236</v>
       </c>
-      <c r="AS13" t="n">
+      <c r="BO13" t="n">
         <v>0.2975790404866964</v>
       </c>
-      <c r="AT13" t="n">
+      <c r="BP13" t="n">
         <v>0.2231842803650222</v>
       </c>
-      <c r="AU13" t="n">
+      <c r="BQ13" t="n">
         <v>0.6989417925686972</v>
       </c>
-      <c r="AV13" t="n">
+      <c r="BR13" t="n">
         <v>0.5665736133518423</v>
       </c>
-      <c r="AW13" t="n">
+      <c r="BS13" t="n">
         <v>0.6418072711878795</v>
       </c>
-      <c r="AX13" t="n">
+      <c r="BT13" t="n">
         <v>0.7170409290239167</v>
       </c>
-      <c r="AY13" t="n">
+      <c r="BU13" t="n">
         <v>0.5199760699716112</v>
       </c>
-      <c r="AZ13" t="n">
+      <c r="BV13" t="n">
         <v>0.1119857656225648</v>
       </c>
-      <c r="BA13" t="n">
+      <c r="BW13" t="n">
         <v>0.02743158460472156</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added an optimizer to find the best compressor parameters.
</commit_message>
<xml_diff>
--- a/расчет_ступеней.xlsx
+++ b/расчет_ступеней.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BW13"/>
+  <dimension ref="A1:BW16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -795,2726 +795,3407 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.45</v>
+        <v>0.55</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4375</v>
+        <v>0.5433333333333333</v>
       </c>
       <c r="C2" t="n">
         <v>0.99</v>
       </c>
       <c r="D2" t="n">
-        <v>0.884203297941869</v>
+        <v>0.8749158980578627</v>
       </c>
       <c r="E2" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="F2" t="n">
-        <v>1.066429875635743</v>
+        <v>1.01899260985795</v>
       </c>
       <c r="G2" t="n">
-        <v>334.9958456714842</v>
+        <v>330.3561984983635</v>
       </c>
       <c r="H2" t="n">
-        <v>0.3244400050544849</v>
+        <v>0.2595630893762285</v>
       </c>
       <c r="I2" t="n">
         <v>288</v>
       </c>
       <c r="J2" t="n">
-        <v>100674.7651178944</v>
+        <v>100435.150625479</v>
       </c>
       <c r="K2" t="n">
-        <v>36409.37652649458</v>
+        <v>28327.47431431331</v>
       </c>
       <c r="L2" t="n">
-        <v>36045.28276122964</v>
+        <v>28044.19957117017</v>
       </c>
       <c r="M2" t="n">
-        <v>31871.35789272645</v>
+        <v>24536.31605312428</v>
       </c>
       <c r="N2" t="n">
-        <v>35.83030095549666</v>
+        <v>27.87693794350912</v>
       </c>
       <c r="O2" t="n">
-        <v>323.8303009554967</v>
+        <v>315.8769379435091</v>
       </c>
       <c r="P2" t="n">
-        <v>323.8303009554967</v>
+        <v>315.8769379435091</v>
       </c>
       <c r="Q2" t="n">
-        <v>1.440908707022073</v>
+        <v>1.329125860037873</v>
       </c>
       <c r="R2" t="n">
-        <v>145063.1456357761</v>
+        <v>133490.955953123</v>
       </c>
       <c r="S2" t="n">
-        <v>145063.1456357761</v>
+        <v>133490.955953123</v>
       </c>
       <c r="T2" t="n">
         <v>310.7513475433373</v>
       </c>
       <c r="U2" t="n">
-        <v>329.5152498904687</v>
+        <v>325.4436007858483</v>
       </c>
       <c r="V2" t="n">
-        <v>0.7615773105863909</v>
+        <v>0.7905694150420949</v>
       </c>
       <c r="W2" t="n">
-        <v>0.1677833565897216</v>
+        <v>0.2311225957333003</v>
       </c>
       <c r="X2" t="n">
-        <v>1.064577496794081</v>
+        <v>1.163669370778668</v>
       </c>
       <c r="Y2" t="n">
-        <v>150.7481305521679</v>
+        <v>181.6959091741</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.5546733681375342</v>
+        <v>0.6367447812769583</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.7670768900816778</v>
+        <v>0.8432463363915963</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.3651710357190851</v>
+        <v>0.3171396294850015</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.4375</v>
+        <v>0.5433333333333333</v>
       </c>
       <c r="AD2" t="n">
-        <v>146.5606824812743</v>
+        <v>179.4935345174442</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.5085578472919455</v>
+        <v>0.6006290571014145</v>
       </c>
       <c r="AF2" t="n">
-        <v>0.7185450194326043</v>
+        <v>0.8113975363946587</v>
       </c>
       <c r="AG2" t="n">
-        <v>0.2868846230922911</v>
+        <v>0.2596975787927992</v>
       </c>
       <c r="AH2" t="n">
-        <v>0.4226367409601864</v>
+        <v>0.4594760190053363</v>
       </c>
       <c r="AI2" t="n">
-        <v>0.5681001461244793</v>
+        <v>0.6262928638025335</v>
       </c>
       <c r="AJ2" t="n">
-        <v>0.8132458964011607</v>
+        <v>0.8343388853607324</v>
       </c>
       <c r="AK2" t="n">
-        <v>0.2029970421339847</v>
+        <v>0.258758555424513</v>
       </c>
       <c r="AL2" t="n">
-        <v>1.128936317318384</v>
+        <v>1.128380965431894</v>
       </c>
       <c r="AM2" t="n">
-        <v>0.4903225573137425</v>
+        <v>0.6108874765005141</v>
       </c>
       <c r="AN2" t="n">
-        <v>0.7002124444906179</v>
+        <v>0.8201830387177463</v>
       </c>
       <c r="AO2" t="n">
-        <v>0.2943956776214189</v>
+        <v>0.2569157928083544</v>
       </c>
       <c r="AP2" t="n">
-        <v>0.7874116034937758</v>
+        <v>0.8124541502014136</v>
       </c>
       <c r="AQ2" t="n">
-        <v>0.5743120885198095</v>
+        <v>0.5443772360304509</v>
       </c>
       <c r="AR2" t="n">
-        <v>0.6484989891376707</v>
+        <v>0.7768834776589806</v>
       </c>
       <c r="AS2" t="n">
-        <v>0.44375</v>
+        <v>0.5466666666666666</v>
       </c>
       <c r="AT2" t="n">
-        <v>1.123094102388967</v>
+        <v>1.114870585168517</v>
       </c>
       <c r="AU2" t="n">
-        <v>0.657848686446533</v>
+        <v>0.7874965457542674</v>
       </c>
       <c r="AV2" t="n">
-        <v>0.474595113251296</v>
+        <v>0.3379871075095369</v>
       </c>
       <c r="AW2" t="n">
-        <v>1.136366747647551</v>
+        <v>1.126334514505067</v>
       </c>
       <c r="AX2" t="n">
-        <v>0.4785180612010175</v>
+        <v>0.3388379687507993</v>
       </c>
       <c r="AY2" t="n">
-        <v>160.8856583832313</v>
+        <v>197.086657963137</v>
       </c>
       <c r="AZ2" t="n">
-        <v>1.407189122308089</v>
+        <v>1.252350556323866</v>
       </c>
       <c r="BA2" t="n">
-        <v>249.586801734187</v>
+        <v>259.1729636003568</v>
       </c>
       <c r="BB2" t="n">
-        <v>148.6544065167211</v>
+        <v>180.5947218457721</v>
       </c>
       <c r="BC2" t="n">
-        <v>164.9069462237893</v>
+        <v>201.1404516790544</v>
       </c>
       <c r="BD2" t="n">
-        <v>243.1313991612655</v>
+        <v>254.865261663562</v>
       </c>
       <c r="BE2" t="n">
-        <v>0.9487229091131606</v>
+        <v>0.9324260139194265</v>
       </c>
       <c r="BF2" t="n">
-        <v>273.2321978245902</v>
+        <v>268.5386920087948</v>
       </c>
       <c r="BG2" t="n">
-        <v>331.5685556814791</v>
+        <v>328.7084241644237</v>
       </c>
       <c r="BH2" t="n">
-        <v>0.7527456915243563</v>
+        <v>0.7884585381685123</v>
       </c>
       <c r="BI2" t="n">
-        <v>0.7378456664511966</v>
+        <v>0.7831318884382398</v>
       </c>
       <c r="BJ2" t="n">
-        <v>323.8303009554967</v>
+        <v>315.8769379435091</v>
       </c>
       <c r="BK2" t="n">
-        <v>0.9092639620831983</v>
+        <v>0.8977840742185261</v>
       </c>
       <c r="BL2" t="n">
-        <v>644.7761790602917</v>
+        <v>649.5118034080301</v>
       </c>
       <c r="BM2" t="n">
-        <v>509.3448177872226</v>
+        <v>511.2118633397067</v>
       </c>
       <c r="BN2" t="n">
-        <v>0.477341460383392</v>
+        <v>0.4985511486344378</v>
       </c>
       <c r="BO2" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.3668220137585716</v>
       </c>
       <c r="BP2" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.1834110068792858</v>
       </c>
       <c r="BQ2" t="n">
-        <v>0.4899327164348984</v>
+        <v>0.5658299146908039</v>
       </c>
       <c r="BR2" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5799965296833545</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.585792973589422</v>
+        <v>0.5960521349267831</v>
       </c>
       <c r="BT2" t="n">
-        <v>0.6050123338270017</v>
+        <v>0.6121077401702117</v>
       </c>
       <c r="BU2" t="n">
-        <v>0.3644842691493443</v>
+        <v>0.4151177375034429</v>
       </c>
       <c r="BV2" t="n">
-        <v>0.1897316660336983</v>
+        <v>0.1592631450068501</v>
       </c>
       <c r="BW2" t="n">
-        <v>0.1606554301282772</v>
+        <v>0.1370840042559034</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.4375</v>
+        <v>0.5433333333333333</v>
       </c>
       <c r="B3" t="n">
-        <v>0.425</v>
+        <v>0.5366666666666667</v>
       </c>
       <c r="C3" t="n">
         <v>0.98</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8813910730500205</v>
+        <v>0.8771926580212601</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="F3" t="n">
-        <v>1.066429875635743</v>
+        <v>1.01899260985795</v>
       </c>
       <c r="G3" t="n">
-        <v>334.9958456714842</v>
+        <v>330.3561984983635</v>
       </c>
       <c r="H3" t="n">
-        <v>0.3311958650192543</v>
+        <v>0.2643367262041065</v>
       </c>
       <c r="I3" t="n">
-        <v>323.8303009554967</v>
+        <v>315.8769379435091</v>
       </c>
       <c r="J3" t="n">
-        <v>145063.1456357761</v>
+        <v>133490.955953123</v>
       </c>
       <c r="K3" t="n">
-        <v>37167.53410689608</v>
+        <v>28848.44620963379</v>
       </c>
       <c r="L3" t="n">
-        <v>36424.18342475816</v>
+        <v>28271.47728544112</v>
       </c>
       <c r="M3" t="n">
-        <v>32103.95011371837</v>
+        <v>24799.53230620377</v>
       </c>
       <c r="N3" t="n">
-        <v>36.20694177411348</v>
+        <v>28.10286012469296</v>
       </c>
       <c r="O3" t="n">
-        <v>360.0372427296102</v>
+        <v>343.9797980682021</v>
       </c>
       <c r="P3" t="n">
-        <v>360.0372427296102</v>
+        <v>343.9797980682021</v>
       </c>
       <c r="Q3" t="n">
-        <v>1.389521025919508</v>
+        <v>1.300842391209521</v>
       </c>
       <c r="R3" t="n">
-        <v>201568.2909469347</v>
+        <v>173650.6943469054</v>
       </c>
       <c r="S3" t="n">
-        <v>201568.2909469347</v>
+        <v>173650.6943469054</v>
       </c>
       <c r="T3" t="n">
-        <v>329.5152498904687</v>
+        <v>325.4436007858483</v>
       </c>
       <c r="U3" t="n">
-        <v>347.448539336746</v>
+        <v>339.6121704124694</v>
       </c>
       <c r="V3" t="n">
-        <v>0.7615773105863909</v>
+        <v>0.7905694150420949</v>
       </c>
       <c r="W3" t="n">
-        <v>0.1633479172253532</v>
+        <v>0.2281034827135892</v>
       </c>
       <c r="X3" t="n">
-        <v>1.064577496794081</v>
+        <v>1.163669370778668</v>
       </c>
       <c r="Y3" t="n">
-        <v>146.5606824812743</v>
+        <v>179.4935345174442</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.5085578472919455</v>
+        <v>0.6006290571014145</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.7185450194326043</v>
+        <v>0.8113975363946587</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.2868846230922911</v>
+        <v>0.2596975787927993</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.425</v>
+        <v>0.5366666666666667</v>
       </c>
       <c r="AD3" t="n">
-        <v>142.3732344103808</v>
+        <v>177.2911598607885</v>
       </c>
       <c r="AE3" t="n">
-        <v>0.468528766832469</v>
+        <v>0.5685086818351996</v>
       </c>
       <c r="AF3" t="n">
-        <v>0.6733194447626319</v>
+        <v>0.7808554921734913</v>
       </c>
       <c r="AG3" t="n">
-        <v>0.2323217907867172</v>
+        <v>0.2164779885688478</v>
       </c>
       <c r="AH3" t="n">
-        <v>0.506480008400635</v>
+        <v>0.5183324998489354</v>
       </c>
       <c r="AI3" t="n">
-        <v>0.6808006472126222</v>
+        <v>0.7065177121432007</v>
       </c>
       <c r="AJ3" t="n">
-        <v>0.8554208090890487</v>
+        <v>0.8657849841537051</v>
       </c>
       <c r="AK3" t="n">
-        <v>0.2304275261048039</v>
+        <v>0.2775059382011241</v>
       </c>
       <c r="AL3" t="n">
-        <v>1.073179621665038</v>
+        <v>1.096833439915491</v>
       </c>
       <c r="AM3" t="n">
-        <v>0.4661209080755683</v>
+        <v>0.5877030380378492</v>
       </c>
       <c r="AN3" t="n">
-        <v>0.6707463493850978</v>
+        <v>0.7984193669688989</v>
       </c>
       <c r="AO3" t="n">
-        <v>0.233213016100909</v>
+        <v>0.2117158391966206</v>
       </c>
       <c r="AP3" t="n">
-        <v>0.8084990598377197</v>
+        <v>0.8281771995978999</v>
       </c>
       <c r="AQ3" t="n">
-        <v>0.5635107758827498</v>
+        <v>0.5369241791707747</v>
       </c>
       <c r="AR3" t="n">
-        <v>0.6314414656442968</v>
+        <v>0.7680978352575358</v>
       </c>
       <c r="AS3" t="n">
-        <v>0.43125</v>
+        <v>0.54</v>
       </c>
       <c r="AT3" t="n">
-        <v>1.054171527737041</v>
+        <v>1.076160684397948</v>
       </c>
       <c r="AU3" t="n">
-        <v>0.6532160462166496</v>
+        <v>0.7882542720494674</v>
       </c>
       <c r="AV3" t="n">
-        <v>0.4227300620927443</v>
+        <v>0.308062849140412</v>
       </c>
       <c r="AW3" t="n">
-        <v>1.07397490693721</v>
+        <v>1.093568951179471</v>
       </c>
       <c r="AX3" t="n">
-        <v>0.4207588607205606</v>
+        <v>0.3053146791300039</v>
       </c>
       <c r="AY3" t="n">
-        <v>156.4429853478237</v>
+        <v>194.669887641445</v>
       </c>
       <c r="AZ3" t="n">
-        <v>1.776406807110386</v>
+        <v>1.51455275775179</v>
       </c>
       <c r="BA3" t="n">
-        <v>248.2779526487107</v>
+        <v>258.3501719836211</v>
       </c>
       <c r="BB3" t="n">
-        <v>144.4669584458276</v>
+        <v>178.3923471891163</v>
       </c>
       <c r="BC3" t="n">
-        <v>166.1511251787695</v>
+        <v>202.6859317515446</v>
       </c>
       <c r="BD3" t="n">
-        <v>237.7104076639635</v>
+        <v>251.5674000292789</v>
       </c>
       <c r="BE3" t="n">
-        <v>0.9568948193262971</v>
+        <v>0.9398741226275776</v>
       </c>
       <c r="BF3" t="n">
-        <v>309.8715373251904</v>
+        <v>296.8845599079414</v>
       </c>
       <c r="BG3" t="n">
-        <v>353.1004272981889</v>
+        <v>345.6218620466004</v>
       </c>
       <c r="BH3" t="n">
-        <v>0.7031369362774604</v>
+        <v>0.7474937217622756</v>
       </c>
       <c r="BI3" t="n">
-        <v>0.6841600431469231</v>
+        <v>0.7407490718714309</v>
       </c>
       <c r="BJ3" t="n">
-        <v>360.0372427296102</v>
+        <v>343.9797980682021</v>
       </c>
       <c r="BK3" t="n">
-        <v>0.9219875058935334</v>
+        <v>0.9085484687536023</v>
       </c>
       <c r="BL3" t="n">
-        <v>653.7986833101451</v>
+        <v>657.2994235138542</v>
       </c>
       <c r="BM3" t="n">
-        <v>512.8961280967814</v>
+        <v>514.2674363062806</v>
       </c>
       <c r="BN3" t="n">
-        <v>0.4634669568398624</v>
+        <v>0.4891762189652889</v>
       </c>
       <c r="BO3" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.3668220137585716</v>
       </c>
       <c r="BP3" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.1834110068792858</v>
       </c>
       <c r="BQ3" t="n">
-        <v>0.5543838557506463</v>
+        <v>0.6097171047851944</v>
       </c>
       <c r="BR3" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5799965296833545</v>
       </c>
       <c r="BS3" t="n">
-        <v>0.6014809361522618</v>
+        <v>0.6075872562108723</v>
       </c>
       <c r="BT3" t="n">
-        <v>0.6363882589526815</v>
+        <v>0.6351779827383902</v>
       </c>
       <c r="BU3" t="n">
-        <v>0.412432539638981</v>
+        <v>0.447315312400702</v>
       </c>
       <c r="BV3" t="n">
-        <v>0.1657575307888799</v>
+        <v>0.1431643575582206</v>
       </c>
       <c r="BW3" t="n">
-        <v>0.1187337964080529</v>
+        <v>0.1076557638341039</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.425</v>
+        <v>0.5366666666666667</v>
       </c>
       <c r="B4" t="n">
-        <v>0.4125</v>
+        <v>0.53</v>
       </c>
       <c r="C4" t="n">
         <v>0.97</v>
       </c>
       <c r="D4" t="n">
-        <v>0.8776400396808992</v>
+        <v>0.8792475775053105</v>
       </c>
       <c r="E4" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="F4" t="n">
-        <v>1.066429875635743</v>
+        <v>1.01899260985795</v>
       </c>
       <c r="G4" t="n">
-        <v>334.9958456714842</v>
+        <v>330.3561984983635</v>
       </c>
       <c r="H4" t="n">
-        <v>0.3375197589886442</v>
+        <v>0.2690626901699927</v>
       </c>
       <c r="I4" t="n">
-        <v>360.0372427296102</v>
+        <v>343.9797980682021</v>
       </c>
       <c r="J4" t="n">
-        <v>201568.2909469347</v>
+        <v>173650.6943469054</v>
       </c>
       <c r="K4" t="n">
-        <v>37877.21550579287</v>
+        <v>29364.21531677354</v>
       </c>
       <c r="L4" t="n">
-        <v>36740.89904061908</v>
+        <v>28483.28885727033</v>
       </c>
       <c r="M4" t="n">
-        <v>32245.28409192084</v>
+        <v>25043.86272713894</v>
       </c>
       <c r="N4" t="n">
-        <v>36.52176843003885</v>
+        <v>28.31340840682935</v>
       </c>
       <c r="O4" t="n">
-        <v>396.559011159649</v>
+        <v>372.2932064750314</v>
       </c>
       <c r="P4" t="n">
-        <v>396.559011159649</v>
+        <v>372.2932064750314</v>
       </c>
       <c r="Q4" t="n">
-        <v>1.347829621392633</v>
+        <v>1.277053490892431</v>
       </c>
       <c r="R4" t="n">
-        <v>271679.7132717671</v>
+        <v>221761.22541161</v>
       </c>
       <c r="S4" t="n">
-        <v>271679.7132717671</v>
+        <v>221761.22541161</v>
       </c>
       <c r="T4" t="n">
-        <v>347.448539336746</v>
+        <v>339.6121704124694</v>
       </c>
       <c r="U4" t="n">
-        <v>364.6453570825088</v>
+        <v>353.3127681404651</v>
       </c>
       <c r="V4" t="n">
-        <v>0.7615773105863909</v>
+        <v>0.7905694150420949</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1591960774308347</v>
+        <v>0.2251145206591726</v>
       </c>
       <c r="X4" t="n">
-        <v>1.064577496794081</v>
+        <v>1.163669370778668</v>
       </c>
       <c r="Y4" t="n">
-        <v>142.3732344103808</v>
+        <v>177.2911598607885</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.468528766832469</v>
+        <v>0.5685086818351996</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.6733194447626319</v>
+        <v>0.7808554921734913</v>
       </c>
       <c r="AB4" t="n">
-        <v>0.2323217907867172</v>
+        <v>0.2164779885688478</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.4125</v>
+        <v>0.53</v>
       </c>
       <c r="AD4" t="n">
-        <v>138.1857863394872</v>
+        <v>175.0887852041327</v>
       </c>
       <c r="AE4" t="n">
-        <v>0.4333023913326854</v>
+        <v>0.5396749531487905</v>
       </c>
       <c r="AF4" t="n">
-        <v>0.6312866578179296</v>
+        <v>0.7517267294576299</v>
       </c>
       <c r="AG4" t="n">
-        <v>0.1929432963141447</v>
+        <v>0.1831856369214446</v>
       </c>
       <c r="AH4" t="n">
-        <v>0.558190666335634</v>
+        <v>0.5589225687416454</v>
       </c>
       <c r="AI4" t="n">
-        <v>0.750309115081092</v>
+        <v>0.7618443656294672</v>
       </c>
       <c r="AJ4" t="n">
-        <v>0.8840146401994062</v>
+        <v>0.8889338663369074</v>
       </c>
       <c r="AK4" t="n">
-        <v>0.2478040511669324</v>
+        <v>0.2904999969061935</v>
       </c>
       <c r="AL4" t="n">
-        <v>1.032320478025595</v>
+        <v>1.073200018697416</v>
       </c>
       <c r="AM4" t="n">
-        <v>0.4420825865074373</v>
+        <v>0.5651219377667424</v>
       </c>
       <c r="AN4" t="n">
-        <v>0.6411568471991366</v>
+        <v>0.7763585765325808</v>
       </c>
       <c r="AO4" t="n">
-        <v>0.1899730607426552</v>
+        <v>0.1773736310631089</v>
       </c>
       <c r="AP4" t="n">
-        <v>0.8227959753928986</v>
+        <v>0.8397516406895011</v>
       </c>
       <c r="AQ4" t="n">
-        <v>0.5575621335231457</v>
+        <v>0.5323375667571771</v>
       </c>
       <c r="AR4" t="n">
-        <v>0.614429921562137</v>
+        <v>0.7592833643790334</v>
       </c>
       <c r="AS4" t="n">
-        <v>0.41875</v>
+        <v>0.5333333333333334</v>
       </c>
       <c r="AT4" t="n">
-        <v>1.006183457466621</v>
+        <v>1.047909504026529</v>
       </c>
       <c r="AU4" t="n">
-        <v>0.6441646969371893</v>
+        <v>0.7863325665854001</v>
       </c>
       <c r="AV4" t="n">
-        <v>0.3917535359044838</v>
+        <v>0.2886261396474953</v>
       </c>
       <c r="AW4" t="n">
-        <v>1.029835022076156</v>
+        <v>1.069402867446432</v>
       </c>
       <c r="AX4" t="n">
-        <v>0.3856703251389664</v>
+        <v>0.2830703008610317</v>
       </c>
       <c r="AY4" t="n">
-        <v>152.0336456146226</v>
+        <v>192.2569931323033</v>
       </c>
       <c r="AZ4" t="n">
-        <v>2.19436222248338</v>
+        <v>1.807707852097115</v>
       </c>
       <c r="BA4" t="n">
-        <v>246.9644608130197</v>
+        <v>257.5402235089658</v>
       </c>
       <c r="BB4" t="n">
-        <v>140.279510374934</v>
+        <v>176.1899725324606</v>
       </c>
       <c r="BC4" t="n">
-        <v>166.0513797701721</v>
+        <v>203.3631160598059</v>
       </c>
       <c r="BD4" t="n">
-        <v>233.5925564032956</v>
+        <v>248.9377491918774</v>
       </c>
       <c r="BE4" t="n">
-        <v>0.9634134657750744</v>
+        <v>0.9461329797796673</v>
       </c>
       <c r="BF4" t="n">
-        <v>346.8647278262354</v>
+        <v>325.4506313302762</v>
       </c>
       <c r="BG4" t="n">
-        <v>373.5833131821657</v>
+        <v>361.8678156759038</v>
       </c>
       <c r="BH4" t="n">
-        <v>0.6610693039509383</v>
+        <v>0.7116969577079606</v>
       </c>
       <c r="BI4" t="n">
-        <v>0.6406020311687126</v>
+        <v>0.7045818086396137</v>
       </c>
       <c r="BJ4" t="n">
-        <v>396.559011159649</v>
+        <v>372.2932064750314</v>
       </c>
       <c r="BK4" t="n">
-        <v>0.93160483961042</v>
+        <v>0.9172607458223552</v>
       </c>
       <c r="BL4" t="n">
-        <v>660.6185155539247</v>
+        <v>663.6024165755675</v>
       </c>
       <c r="BM4" t="n">
-        <v>515.5642209446628</v>
+        <v>516.7272668761979</v>
       </c>
       <c r="BN4" t="n">
-        <v>0.4530813949332761</v>
+        <v>0.4817584926315107</v>
       </c>
       <c r="BO4" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.3668220137585716</v>
       </c>
       <c r="BP4" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.1834110068792858</v>
       </c>
       <c r="BQ4" t="n">
-        <v>0.5949675909202978</v>
+        <v>0.6405978739282687</v>
       </c>
       <c r="BR4" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5799965296833545</v>
       </c>
       <c r="BS4" t="n">
-        <v>0.6121170921843355</v>
+        <v>0.6160787757895745</v>
       </c>
       <c r="BT4" t="n">
-        <v>0.6576605710168285</v>
+        <v>0.6521610218957946</v>
       </c>
       <c r="BU4" t="n">
-        <v>0.4426247120668587</v>
+        <v>0.4699708042476542</v>
       </c>
       <c r="BV4" t="n">
-        <v>0.1506614445749411</v>
+        <v>0.1318366116347445</v>
       </c>
       <c r="BW4" t="n">
-        <v>0.09287846744055345</v>
+        <v>0.08736072938774891</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.4125</v>
+        <v>0.53</v>
       </c>
       <c r="B5" t="n">
-        <v>0.4</v>
+        <v>0.5233333333333333</v>
       </c>
       <c r="C5" t="n">
         <v>0.96</v>
       </c>
       <c r="D5" t="n">
-        <v>0.8729343479869782</v>
+        <v>0.8810742363872112</v>
       </c>
       <c r="E5" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="F5" t="n">
-        <v>1.066429875635743</v>
+        <v>1.01899260985795</v>
       </c>
       <c r="G5" t="n">
-        <v>334.9958456714842</v>
+        <v>330.3561984983635</v>
       </c>
       <c r="H5" t="n">
-        <v>0.3433570658223036</v>
+        <v>0.2737328478793182</v>
       </c>
       <c r="I5" t="n">
-        <v>396.559011159649</v>
+        <v>372.2932064750314</v>
       </c>
       <c r="J5" t="n">
-        <v>271679.7132717671</v>
+        <v>221761.22541161</v>
       </c>
       <c r="K5" t="n">
-        <v>38532.29101774057</v>
+        <v>29873.89399594412</v>
       </c>
       <c r="L5" t="n">
-        <v>36990.99937703094</v>
+        <v>28678.93823610635</v>
       </c>
       <c r="M5" t="n">
-        <v>32290.71392257523</v>
+        <v>25268.2736067734</v>
       </c>
       <c r="N5" t="n">
-        <v>36.77037711434487</v>
+        <v>28.50789089076178</v>
       </c>
       <c r="O5" t="n">
-        <v>433.3293882739939</v>
+        <v>400.8010973657932</v>
       </c>
       <c r="P5" t="n">
-        <v>433.3293882739939</v>
+        <v>400.8010973657932</v>
       </c>
       <c r="Q5" t="n">
-        <v>1.313130303218921</v>
+        <v>1.256726699210606</v>
       </c>
       <c r="R5" t="n">
-        <v>356750.8642669851</v>
+        <v>278693.2528244318</v>
       </c>
       <c r="S5" t="n">
-        <v>356750.8642669851</v>
+        <v>278693.2528244318</v>
       </c>
       <c r="T5" t="n">
-        <v>364.6453570825088</v>
+        <v>353.3127681404651</v>
       </c>
       <c r="U5" t="n">
-        <v>381.1762635425639</v>
+        <v>366.5905180808015</v>
       </c>
       <c r="V5" t="n">
-        <v>0.7615773105863909</v>
+        <v>0.7905694150420949</v>
       </c>
       <c r="W5" t="n">
-        <v>0.1553636977416573</v>
+        <v>0.22216085358044</v>
       </c>
       <c r="X5" t="n">
-        <v>1.064577496794081</v>
+        <v>1.163669370778668</v>
       </c>
       <c r="Y5" t="n">
-        <v>138.1857863394872</v>
+        <v>175.0887852041327</v>
       </c>
       <c r="Z5" t="n">
-        <v>0.4333023913326854</v>
+        <v>0.5396749531487905</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.6312866578179296</v>
+        <v>0.7517267294576299</v>
       </c>
       <c r="AB5" t="n">
-        <v>0.1929432963141447</v>
+        <v>0.1831856369214445</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.4</v>
+        <v>0.5233333333333333</v>
       </c>
       <c r="AD5" t="n">
-        <v>133.9983382685937</v>
+        <v>172.8864105474769</v>
       </c>
       <c r="AE5" t="n">
-        <v>0.4019499360408819</v>
+        <v>0.5135856672874103</v>
       </c>
       <c r="AF5" t="n">
-        <v>0.5922271443277999</v>
+        <v>0.7240261143390112</v>
       </c>
       <c r="AG5" t="n">
-        <v>0.1637251255561614</v>
+        <v>0.1570284104663461</v>
       </c>
       <c r="AH5" t="n">
-        <v>0.5931253835185788</v>
+        <v>0.5885102091982426</v>
       </c>
       <c r="AI5" t="n">
-        <v>0.7972676873324286</v>
+        <v>0.8021740614312992</v>
       </c>
       <c r="AJ5" t="n">
-        <v>0.9043328384130478</v>
+        <v>0.9064996483267894</v>
       </c>
       <c r="AK5" t="n">
-        <v>0.2594013382727521</v>
+        <v>0.2997257989200545</v>
       </c>
       <c r="AL5" t="n">
-        <v>0.9997621798616013</v>
+        <v>1.054667013070643</v>
       </c>
       <c r="AM5" t="n">
-        <v>0.4189892047782126</v>
+        <v>0.5434765911200543</v>
       </c>
       <c r="AN5" t="n">
-        <v>0.6121999974112641</v>
+        <v>0.754382910729652</v>
       </c>
       <c r="AO5" t="n">
-        <v>0.1583836392892018</v>
+        <v>0.1507094981258448</v>
       </c>
       <c r="AP5" t="n">
-        <v>0.8329550744997194</v>
+        <v>0.8485345316844422</v>
       </c>
       <c r="AQ5" t="n">
-        <v>0.5542658266274929</v>
+        <v>0.5295794185860807</v>
       </c>
       <c r="AR5" t="n">
-        <v>0.5974865025033296</v>
+        <v>0.7504449411331544</v>
       </c>
       <c r="AS5" t="n">
-        <v>0.40625</v>
+        <v>0.5266666666666666</v>
       </c>
       <c r="AT5" t="n">
-        <v>0.9695253360656676</v>
+        <v>1.026261321111047</v>
       </c>
       <c r="AU5" t="n">
-        <v>0.6325005241171194</v>
+        <v>0.7826405252138178</v>
       </c>
       <c r="AV5" t="n">
-        <v>0.372038833562338</v>
+        <v>0.2758163799778928</v>
       </c>
       <c r="AW5" t="n">
-        <v>0.9954739554152893</v>
+        <v>1.050673859882218</v>
       </c>
       <c r="AX5" t="n">
-        <v>0.3629734312981698</v>
+        <v>0.2680333346683998</v>
       </c>
       <c r="AY5" t="n">
-        <v>147.6621745217523</v>
+        <v>189.8486237330193</v>
       </c>
       <c r="AZ5" t="n">
-        <v>2.659616017028643</v>
+        <v>2.132563514482126</v>
       </c>
       <c r="BA5" t="n">
-        <v>245.6347060214273</v>
+        <v>256.7418819150192</v>
       </c>
       <c r="BB5" t="n">
-        <v>136.0920623040405</v>
+        <v>173.9875978758048</v>
       </c>
       <c r="BC5" t="n">
-        <v>165.0366338893982</v>
+        <v>203.4066565885848</v>
       </c>
       <c r="BD5" t="n">
-        <v>230.2105659161242</v>
+        <v>246.7369691893362</v>
       </c>
       <c r="BE5" t="n">
-        <v>0.9687081729442294</v>
+        <v>0.9514584908239752</v>
       </c>
       <c r="BF5" t="n">
-        <v>384.1499551650339</v>
+        <v>354.221532376752</v>
       </c>
       <c r="BG5" t="n">
-        <v>393.1495592776405</v>
+        <v>377.5242717589293</v>
       </c>
       <c r="BH5" t="n">
-        <v>0.6247869296171872</v>
+        <v>0.6800672198341821</v>
       </c>
       <c r="BI5" t="n">
-        <v>0.603947800360391</v>
+        <v>0.6730587863566948</v>
       </c>
       <c r="BJ5" t="n">
-        <v>433.3293882739939</v>
+        <v>400.8010973657932</v>
       </c>
       <c r="BK5" t="n">
-        <v>0.9392078424066409</v>
+        <v>0.9244986450180088</v>
       </c>
       <c r="BL5" t="n">
-        <v>666.0099478516489</v>
+        <v>668.8387546823074</v>
       </c>
       <c r="BM5" t="n">
-        <v>517.6637543981512</v>
+        <v>518.761950545694</v>
       </c>
       <c r="BN5" t="n">
-        <v>0.4447106137144423</v>
+        <v>0.4756265738645435</v>
       </c>
       <c r="BO5" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.3668220137585716</v>
       </c>
       <c r="BP5" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.1834110068792858</v>
       </c>
       <c r="BQ5" t="n">
-        <v>0.6225980342642162</v>
+        <v>0.663341317062243</v>
       </c>
       <c r="BR5" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5799965296833545</v>
       </c>
       <c r="BS5" t="n">
-        <v>0.619674929595378</v>
+        <v>0.622522291312347</v>
       </c>
       <c r="BT5" t="n">
-        <v>0.6727762458389134</v>
+        <v>0.6650480529413397</v>
       </c>
       <c r="BU5" t="n">
-        <v>0.4631803141131219</v>
+        <v>0.4866563954680702</v>
       </c>
       <c r="BV5" t="n">
-        <v>0.1403836435518095</v>
+        <v>0.1234938160245365</v>
       </c>
       <c r="BW5" t="n">
-        <v>0.07541110884908103</v>
+        <v>0.0725669091594503</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.4</v>
+        <v>0.5233333333333333</v>
       </c>
       <c r="B6" t="n">
-        <v>0.3875</v>
+        <v>0.5166666666666667</v>
       </c>
       <c r="C6" t="n">
         <v>0.95</v>
       </c>
       <c r="D6" t="n">
-        <v>0.8672584703581266</v>
+        <v>0.8826676089429577</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="F6" t="n">
-        <v>1.066429875635743</v>
+        <v>1.01899260985795</v>
       </c>
       <c r="G6" t="n">
-        <v>334.9958456714842</v>
+        <v>330.3561984983635</v>
       </c>
       <c r="H6" t="n">
-        <v>0.3486475855755174</v>
+        <v>0.2783389497856022</v>
       </c>
       <c r="I6" t="n">
-        <v>433.3293882739939</v>
+        <v>400.8010973657932</v>
       </c>
       <c r="J6" t="n">
-        <v>356750.8642669851</v>
+        <v>278693.2528244318</v>
       </c>
       <c r="K6" t="n">
-        <v>39126.00487150306</v>
+        <v>30376.58193109288</v>
       </c>
       <c r="L6" t="n">
-        <v>37169.7046279279</v>
+        <v>28857.75283453823</v>
       </c>
       <c r="M6" t="n">
-        <v>32235.74117928013</v>
+        <v>25471.80369392872</v>
       </c>
       <c r="N6" t="n">
-        <v>36.94801652875537</v>
+        <v>28.68563900053502</v>
       </c>
       <c r="O6" t="n">
-        <v>470.2774048027492</v>
+        <v>429.4867363663282</v>
       </c>
       <c r="P6" t="n">
-        <v>470.2774048027492</v>
+        <v>429.4867363663282</v>
       </c>
       <c r="Q6" t="n">
-        <v>1.28363103095909</v>
+        <v>1.239121976574034</v>
       </c>
       <c r="R6" t="n">
-        <v>457936.4796945766</v>
+        <v>345334.934297657</v>
       </c>
       <c r="S6" t="n">
-        <v>457936.4796945766</v>
+        <v>345334.934297657</v>
       </c>
       <c r="T6" t="n">
-        <v>381.1762635425639</v>
+        <v>366.5905180808015</v>
       </c>
       <c r="U6" t="n">
-        <v>397.0944646181332</v>
+        <v>379.4824142218317</v>
       </c>
       <c r="V6" t="n">
-        <v>0.7615773105863909</v>
+        <v>0.7905694150420949</v>
       </c>
       <c r="W6" t="n">
-        <v>0.1518903013578152</v>
+        <v>0.2192476989486998</v>
       </c>
       <c r="X6" t="n">
-        <v>1.064577496794081</v>
+        <v>1.163669370778668</v>
       </c>
       <c r="Y6" t="n">
-        <v>133.9983382685937</v>
+        <v>172.8864105474769</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.4019499360408819</v>
+        <v>0.5135856672874103</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.5922271443277999</v>
+        <v>0.7240261143390112</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.1637251255561614</v>
+        <v>0.1570284104663461</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.3875</v>
+        <v>0.5166666666666667</v>
       </c>
       <c r="AD6" t="n">
-        <v>129.8108901977001</v>
+        <v>170.6840358908212</v>
       </c>
       <c r="AE6" t="n">
-        <v>0.3737796859822607</v>
+        <v>0.4898177442230555</v>
       </c>
       <c r="AF6" t="n">
-        <v>0.5558891806916422</v>
+        <v>0.697718957219101</v>
       </c>
       <c r="AG6" t="n">
-        <v>0.1415608615306941</v>
+        <v>0.1361282651628454</v>
       </c>
       <c r="AH6" t="n">
-        <v>0.6180530627448302</v>
+        <v>0.6108958189145675</v>
       </c>
       <c r="AI6" t="n">
-        <v>0.8307749923973037</v>
+        <v>0.8326869653420473</v>
       </c>
       <c r="AJ6" t="n">
-        <v>0.9192896953607008</v>
+        <v>0.9201542213809998</v>
       </c>
       <c r="AK6" t="n">
-        <v>0.2674717268010952</v>
+        <v>0.3063566828539088</v>
       </c>
       <c r="AL6" t="n">
-        <v>0.9720262250235825</v>
+        <v>1.039595659752858</v>
       </c>
       <c r="AM6" t="n">
-        <v>0.3972152038601151</v>
+        <v>0.5229057101248068</v>
       </c>
       <c r="AN6" t="n">
-        <v>0.5843288480641364</v>
+        <v>0.7327403564424538</v>
       </c>
       <c r="AO6" t="n">
-        <v>0.1346710017740956</v>
+        <v>0.1296220010026499</v>
       </c>
       <c r="AP6" t="n">
-        <v>0.8404335029735459</v>
+        <v>0.8553618182115473</v>
       </c>
       <c r="AQ6" t="n">
-        <v>0.5524812982168491</v>
+        <v>0.5280449340574782</v>
       </c>
       <c r="AR6" t="n">
-        <v>0.5806335590240905</v>
+        <v>0.7415873974789472</v>
       </c>
       <c r="AS6" t="n">
-        <v>0.39375</v>
+        <v>0.52</v>
       </c>
       <c r="AT6" t="n">
-        <v>0.9393663462540609</v>
+        <v>1.008999437032235</v>
       </c>
       <c r="AU6" t="n">
-        <v>0.6191945916757878</v>
+        <v>0.7777221794859068</v>
       </c>
       <c r="AV6" t="n">
-        <v>0.3587327872299704</v>
+        <v>0.2674120395532883</v>
       </c>
       <c r="AW6" t="n">
-        <v>0.9666442621479878</v>
+        <v>1.035577946863965</v>
       </c>
       <c r="AX6" t="n">
-        <v>0.3474496704722</v>
+        <v>0.2578557673780582</v>
       </c>
       <c r="AY6" t="n">
-        <v>143.3338608703159</v>
+        <v>187.4454377846733</v>
       </c>
       <c r="AZ6" t="n">
-        <v>3.169793873235574</v>
+        <v>2.489787201375131</v>
       </c>
       <c r="BA6" t="n">
-        <v>244.2756650661178</v>
+        <v>255.9538514603378</v>
       </c>
       <c r="BB6" t="n">
-        <v>131.9046142331469</v>
+        <v>171.7852232191491</v>
       </c>
       <c r="BC6" t="n">
-        <v>163.4132722977984</v>
+        <v>202.9840166499692</v>
       </c>
       <c r="BD6" t="n">
-        <v>227.2730542356306</v>
+        <v>244.8274784943593</v>
       </c>
       <c r="BE6" t="n">
-        <v>0.9730727081527885</v>
+        <v>0.9560382937261576</v>
       </c>
       <c r="BF6" t="n">
-        <v>421.6610013699664</v>
+        <v>383.1811972491644</v>
       </c>
       <c r="BG6" t="n">
-        <v>411.8974635892041</v>
+        <v>392.653519690291</v>
       </c>
       <c r="BH6" t="n">
-        <v>0.5930496947894299</v>
+        <v>0.651856760795685</v>
       </c>
       <c r="BI6" t="n">
-        <v>0.572340021043074</v>
+        <v>0.645161591997362</v>
       </c>
       <c r="BJ6" t="n">
-        <v>470.2774048027492</v>
+        <v>429.4867363663282</v>
       </c>
       <c r="BK6" t="n">
-        <v>0.9454044833854023</v>
+        <v>0.9306277533685716</v>
       </c>
       <c r="BL6" t="n">
-        <v>670.4041025304953</v>
+        <v>673.2729258069427</v>
       </c>
       <c r="BM6" t="n">
-        <v>519.368650087941</v>
+        <v>520.4787165943305</v>
       </c>
       <c r="BN6" t="n">
-        <v>0.437594864836659</v>
+        <v>0.4703890297308387</v>
       </c>
       <c r="BO6" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.3668220137585716</v>
       </c>
       <c r="BP6" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.1834110068792858</v>
       </c>
       <c r="BQ6" t="n">
-        <v>0.6423837994849889</v>
+        <v>0.680652393008596</v>
       </c>
       <c r="BR6" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5799965296833545</v>
       </c>
       <c r="BS6" t="n">
-        <v>0.6252384885193522</v>
+        <v>0.6275310892971061</v>
       </c>
       <c r="BT6" t="n">
-        <v>0.6839033636868619</v>
+        <v>0.6750656489108576</v>
       </c>
       <c r="BU6" t="n">
-        <v>0.4778998866873533</v>
+        <v>0.4993565629460078</v>
       </c>
       <c r="BV6" t="n">
-        <v>0.1330238572646938</v>
+        <v>0.1171437322855677</v>
       </c>
       <c r="BW6" t="n">
-        <v>0.06294726923595534</v>
+        <v>0.06137410430128787</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.3875</v>
+        <v>0.5166666666666667</v>
       </c>
       <c r="B7" t="n">
-        <v>0.375</v>
+        <v>0.51</v>
       </c>
       <c r="C7" t="n">
         <v>0.9399999999999999</v>
       </c>
       <c r="D7" t="n">
-        <v>0.8605972014216101</v>
+        <v>0.8840297017740676</v>
       </c>
       <c r="E7" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="F7" t="n">
-        <v>1.066429875635743</v>
+        <v>1.01899260985795</v>
       </c>
       <c r="G7" t="n">
-        <v>334.9958456714842</v>
+        <v>330.3561984983635</v>
       </c>
       <c r="H7" t="n">
-        <v>0.3533255394992114</v>
+        <v>0.2828930011726652</v>
       </c>
       <c r="I7" t="n">
-        <v>470.2774048027492</v>
+        <v>429.4867363663282</v>
       </c>
       <c r="J7" t="n">
-        <v>457936.4796945766</v>
+        <v>345334.934297657</v>
       </c>
       <c r="K7" t="n">
-        <v>39650.97523005291</v>
+        <v>30873.58932148536</v>
       </c>
       <c r="L7" t="n">
-        <v>37271.91671624973</v>
+        <v>29021.17396219624</v>
       </c>
       <c r="M7" t="n">
-        <v>32076.10721762385</v>
+        <v>25655.57976293367</v>
       </c>
       <c r="N7" t="n">
-        <v>37.04961900223631</v>
+        <v>28.84808544949924</v>
       </c>
       <c r="O7" t="n">
-        <v>507.3270238049855</v>
+        <v>458.3348218158275</v>
       </c>
       <c r="P7" t="n">
-        <v>507.3270238049855</v>
+        <v>458.3348218158275</v>
       </c>
       <c r="Q7" t="n">
-        <v>1.258098598953983</v>
+        <v>1.223714194449077</v>
       </c>
       <c r="R7" t="n">
-        <v>576129.2435136657</v>
+        <v>422591.2609391822</v>
       </c>
       <c r="S7" t="n">
-        <v>576129.2435136657</v>
+        <v>422591.2609391822</v>
       </c>
       <c r="T7" t="n">
-        <v>397.0944646181332</v>
+        <v>379.4824142218317</v>
       </c>
       <c r="U7" t="n">
-        <v>412.4399969472064</v>
+        <v>392.0199813209105</v>
       </c>
       <c r="V7" t="n">
-        <v>0.7615773105863909</v>
+        <v>0.7905694150420949</v>
       </c>
       <c r="W7" t="n">
-        <v>0.1488190741438032</v>
+        <v>0.2163674639557862</v>
       </c>
       <c r="X7" t="n">
-        <v>1.064577496794081</v>
+        <v>1.163669370778668</v>
       </c>
       <c r="Y7" t="n">
-        <v>129.8108901977001</v>
+        <v>170.6840358908212</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.3737796859822607</v>
+        <v>0.4898177442230555</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.5558891806916422</v>
+        <v>0.697718957219101</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.1415608615306941</v>
+        <v>0.1361282651628454</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.375</v>
+        <v>0.51</v>
       </c>
       <c r="AD7" t="n">
-        <v>125.6234421268066</v>
+        <v>168.4816612341654</v>
       </c>
       <c r="AE7" t="n">
-        <v>0.3482637835623633</v>
+        <v>0.4680343173960578</v>
       </c>
       <c r="AF7" t="n">
-        <v>0.5220220244246978</v>
+        <v>0.6727435922915034</v>
       </c>
       <c r="AG7" t="n">
-        <v>0.1244499868451066</v>
+        <v>0.1191834119456657</v>
       </c>
       <c r="AH7" t="n">
-        <v>0.6365266021211494</v>
+        <v>0.6283067002390071</v>
       </c>
       <c r="AI7" t="n">
-        <v>0.8556067673047103</v>
+        <v>0.8564190215864946</v>
       </c>
       <c r="AJ7" t="n">
-        <v>0.9306081184520197</v>
+        <v>0.9309816165035615</v>
       </c>
       <c r="AK7" t="n">
-        <v>0.2733222986142951</v>
+        <v>0.3111452462475973</v>
       </c>
       <c r="AL7" t="n">
-        <v>0.94708331955606</v>
+        <v>1.026946687773078</v>
       </c>
       <c r="AM7" t="n">
-        <v>0.3769042166111551</v>
+        <v>0.503447796603768</v>
       </c>
       <c r="AN7" t="n">
-        <v>0.5577971839788439</v>
+        <v>0.7115932367921735</v>
       </c>
       <c r="AO7" t="n">
-        <v>0.1164682001603178</v>
+        <v>0.1126765581068928</v>
       </c>
       <c r="AP7" t="n">
-        <v>0.8460927145192053</v>
+        <v>0.8607755157728282</v>
       </c>
       <c r="AQ7" t="n">
-        <v>0.5515503936407113</v>
+        <v>0.5273692063357156</v>
       </c>
       <c r="AR7" t="n">
-        <v>0.5638932886886516</v>
+        <v>0.7327043540050766</v>
       </c>
       <c r="AS7" t="n">
-        <v>0.38125</v>
+        <v>0.5133333333333334</v>
       </c>
       <c r="AT7" t="n">
-        <v>0.913006188823837</v>
+        <v>0.9947777367543102</v>
       </c>
       <c r="AU7" t="n">
-        <v>0.6048180107391227</v>
+        <v>0.7719120599890752</v>
       </c>
       <c r="AV7" t="n">
-        <v>0.3491129001351854</v>
+        <v>0.2620733827492336</v>
       </c>
       <c r="AW7" t="n">
-        <v>0.9409630125541549</v>
+        <v>1.022991656980053</v>
       </c>
       <c r="AX7" t="n">
-        <v>0.3361450018150323</v>
+        <v>0.2510795969909776</v>
       </c>
       <c r="AY7" t="n">
-        <v>139.0549019493772</v>
+        <v>185.0464595122539</v>
       </c>
       <c r="AZ7" t="n">
-        <v>3.721602002135425</v>
+        <v>2.879976293973698</v>
       </c>
       <c r="BA7" t="n">
-        <v>242.8728905954796</v>
+        <v>255.1779408559948</v>
       </c>
       <c r="BB7" t="n">
-        <v>127.7171661622534</v>
+        <v>169.5828485624933</v>
       </c>
       <c r="BC7" t="n">
-        <v>161.3924812349645</v>
+        <v>202.212234884853</v>
       </c>
       <c r="BD7" t="n">
-        <v>224.6120038691836</v>
+        <v>243.1272127708831</v>
       </c>
       <c r="BE7" t="n">
-        <v>0.9767147910578338</v>
+        <v>0.9600130962407062</v>
       </c>
       <c r="BF7" t="n">
-        <v>459.3268971711375</v>
+        <v>412.3128915733546</v>
       </c>
       <c r="BG7" t="n">
-        <v>429.900884327747</v>
+        <v>407.3060459328526</v>
       </c>
       <c r="BH7" t="n">
-        <v>0.5649508978686322</v>
+        <v>0.626501726168982</v>
       </c>
       <c r="BI7" t="n">
-        <v>0.5445931663556255</v>
+        <v>0.6201908687196671</v>
       </c>
       <c r="BJ7" t="n">
-        <v>507.3270238049855</v>
+        <v>458.3348218158275</v>
       </c>
       <c r="BK7" t="n">
-        <v>0.9505697138597924</v>
+        <v>0.9358938810594575</v>
       </c>
       <c r="BL7" t="n">
-        <v>674.066864619529</v>
+        <v>677.0827640427808</v>
       </c>
       <c r="BM7" t="n">
-        <v>520.7855063731264</v>
+        <v>521.9492513073021</v>
       </c>
       <c r="BN7" t="n">
-        <v>0.4312946522522004</v>
+        <v>0.4658062295557158</v>
       </c>
       <c r="BO7" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.3668220137585716</v>
       </c>
       <c r="BP7" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.1834110068792858</v>
       </c>
       <c r="BQ7" t="n">
-        <v>0.6570736359990065</v>
+        <v>0.694167830649013</v>
       </c>
       <c r="BR7" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5799965296833545</v>
       </c>
       <c r="BS7" t="n">
-        <v>0.6294486453735235</v>
+        <v>0.6315028161797239</v>
       </c>
       <c r="BT7" t="n">
-        <v>0.6923236773952047</v>
+        <v>0.6830091026760933</v>
       </c>
       <c r="BU7" t="n">
-        <v>0.4888283553242228</v>
+        <v>0.5092720830501801</v>
       </c>
       <c r="BV7" t="n">
-        <v>0.127559622946259</v>
+        <v>0.1121859722334815</v>
       </c>
       <c r="BW7" t="n">
-        <v>0.05371049954779572</v>
+        <v>0.05266866363906803</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.375</v>
+        <v>0.51</v>
       </c>
       <c r="B8" t="n">
-        <v>0.3625</v>
+        <v>0.5033333333333334</v>
       </c>
       <c r="C8" t="n">
         <v>0.9399999999999999</v>
       </c>
       <c r="D8" t="n">
-        <v>0.8529356580420905</v>
+        <v>0.8851551928471313</v>
       </c>
       <c r="E8" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="F8" t="n">
-        <v>1.066429875635743</v>
+        <v>1.01899260985795</v>
       </c>
       <c r="G8" t="n">
-        <v>334.9958456714842</v>
+        <v>330.3561984983635</v>
       </c>
       <c r="H8" t="n">
-        <v>0.3573195700399479</v>
+        <v>0.2873857616296107</v>
       </c>
       <c r="I8" t="n">
-        <v>507.3270238049855</v>
+        <v>458.3348218158275</v>
       </c>
       <c r="J8" t="n">
-        <v>576129.2435136657</v>
+        <v>422591.2609391822</v>
       </c>
       <c r="K8" t="n">
-        <v>40099.19419057097</v>
+        <v>31363.90771286501</v>
       </c>
       <c r="L8" t="n">
-        <v>37693.24253913671</v>
+        <v>29482.07325009311</v>
       </c>
       <c r="M8" t="n">
-        <v>32149.91062885868</v>
+        <v>26096.21023321942</v>
       </c>
       <c r="N8" t="n">
-        <v>37.468431947452</v>
+        <v>29.30623583508261</v>
       </c>
       <c r="O8" t="n">
-        <v>544.7954557524375</v>
+        <v>487.6410576509101</v>
       </c>
       <c r="P8" t="n">
-        <v>544.7954557524375</v>
+        <v>487.6410576509101</v>
       </c>
       <c r="Q8" t="n">
-        <v>1.238387978501664</v>
+        <v>1.212504630046815</v>
       </c>
       <c r="R8" t="n">
-        <v>713471.5292305814</v>
+        <v>512393.8605060804</v>
       </c>
       <c r="S8" t="n">
-        <v>713471.5292305814</v>
+        <v>512393.8605060804</v>
       </c>
       <c r="T8" t="n">
-        <v>412.4399969472064</v>
+        <v>392.0199813209105</v>
       </c>
       <c r="U8" t="n">
-        <v>427.3990130004892</v>
+        <v>404.358809265175</v>
       </c>
       <c r="V8" t="n">
-        <v>0.7615773105863909</v>
+        <v>0.7905694150420949</v>
       </c>
       <c r="W8" t="n">
-        <v>0.1461968646286187</v>
+        <v>0.2135259927506889</v>
       </c>
       <c r="X8" t="n">
-        <v>1.064577496794081</v>
+        <v>1.163669370778668</v>
       </c>
       <c r="Y8" t="n">
-        <v>125.6234421268066</v>
+        <v>168.4816612341654</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.3482637835623633</v>
+        <v>0.4680343173960578</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.5220220244246978</v>
+        <v>0.6727435922915034</v>
       </c>
       <c r="AB8" t="n">
-        <v>0.1244499868451067</v>
+        <v>0.1191834119456657</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.3625</v>
+        <v>0.5033333333333334</v>
       </c>
       <c r="AD8" t="n">
-        <v>121.435994055913</v>
+        <v>166.2792865775097</v>
       </c>
       <c r="AE8" t="n">
-        <v>0.3248720262443578</v>
+        <v>0.4478210551388968</v>
       </c>
       <c r="AF8" t="n">
-        <v>0.4902267786136445</v>
+        <v>0.6488550652132633</v>
       </c>
       <c r="AG8" t="n">
-        <v>0.1108926247734101</v>
+        <v>0.1051218473812989</v>
       </c>
       <c r="AH8" t="n">
-        <v>0.6507693397424607</v>
+        <v>0.6422872546996068</v>
       </c>
       <c r="AI8" t="n">
-        <v>0.874751580189404</v>
+        <v>0.8754753403681166</v>
       </c>
       <c r="AJ8" t="n">
-        <v>0.939465360469416</v>
+        <v>0.9398023918868981</v>
       </c>
       <c r="AK8" t="n">
-        <v>0.2778401656135346</v>
+        <v>0.3146515870937543</v>
       </c>
       <c r="AL8" t="n">
-        <v>0.9235220626756799</v>
+        <v>1.015946073443035</v>
       </c>
       <c r="AM8" t="n">
-        <v>0.3579847479308438</v>
+        <v>0.484956438220453</v>
       </c>
       <c r="AN8" t="n">
-        <v>0.532609775801597</v>
+        <v>0.6908970018343493</v>
       </c>
       <c r="AO8" t="n">
-        <v>0.1020682245887486</v>
+        <v>0.0987250530206893</v>
       </c>
       <c r="AP8" t="n">
-        <v>0.8505213355279034</v>
+        <v>0.8651859034644964</v>
       </c>
       <c r="AQ8" t="n">
-        <v>0.5510264886289833</v>
+        <v>0.5272772926466498</v>
       </c>
       <c r="AR8" t="n">
-        <v>0.5472873917189358</v>
+        <v>0.7238011676951294</v>
       </c>
       <c r="AS8" t="n">
-        <v>0.36875</v>
+        <v>0.5066666666666667</v>
       </c>
       <c r="AT8" t="n">
-        <v>0.8886668819554222</v>
+        <v>0.9826149747102656</v>
       </c>
       <c r="AU8" t="n">
-        <v>0.5897582525396874</v>
+        <v>0.7654668155981543</v>
       </c>
       <c r="AV8" t="n">
-        <v>0.3413794902364864</v>
+        <v>0.2588138070151362</v>
       </c>
       <c r="AW8" t="n">
-        <v>0.9168465296054072</v>
+        <v>1.012099504766793</v>
       </c>
       <c r="AX8" t="n">
-        <v>0.3270882770657199</v>
+        <v>0.2466326891686383</v>
       </c>
       <c r="AY8" t="n">
-        <v>134.8326123950213</v>
+        <v>182.6524303501638</v>
       </c>
       <c r="AZ8" t="n">
-        <v>4.317328488730078</v>
+        <v>3.3082827805304</v>
       </c>
       <c r="BA8" t="n">
-        <v>241.4104959520961</v>
+        <v>254.4126923439285</v>
       </c>
       <c r="BB8" t="n">
-        <v>123.5297180913598</v>
+        <v>167.3804739058375</v>
       </c>
       <c r="BC8" t="n">
-        <v>159.1402078158146</v>
+        <v>201.1902719181625</v>
       </c>
       <c r="BD8" t="n">
-        <v>222.1117834262884</v>
+        <v>241.5743010493417</v>
       </c>
       <c r="BE8" t="n">
-        <v>0.9797853895098045</v>
+        <v>0.9634906462899344</v>
       </c>
       <c r="BF8" t="n">
-        <v>497.0716056276176</v>
+        <v>441.6013136885135</v>
       </c>
       <c r="BG8" t="n">
-        <v>447.2155310812989</v>
+        <v>421.5242633297759</v>
       </c>
       <c r="BH8" t="n">
-        <v>0.5398079430926793</v>
+        <v>0.6035540880475745</v>
       </c>
       <c r="BI8" t="n">
-        <v>0.5196824902963315</v>
+        <v>0.5974255921080215</v>
       </c>
       <c r="BJ8" t="n">
-        <v>544.7954557524375</v>
+        <v>487.6410576509101</v>
       </c>
       <c r="BK8" t="n">
-        <v>0.9549883515465672</v>
+        <v>0.9405137769823967</v>
       </c>
       <c r="BL8" t="n">
-        <v>677.2002037192149</v>
+        <v>680.4250787692673</v>
       </c>
       <c r="BM8" t="n">
-        <v>521.9945152666484</v>
+        <v>523.2359264171396</v>
       </c>
       <c r="BN8" t="n">
-        <v>0.4255059716725719</v>
+        <v>0.4616928785902046</v>
       </c>
       <c r="BO8" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.3668220137585716</v>
       </c>
       <c r="BP8" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.1834110068792858</v>
       </c>
       <c r="BQ8" t="n">
-        <v>0.6684108649448608</v>
+        <v>0.7050484345825851</v>
       </c>
       <c r="BR8" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5799965296833545</v>
       </c>
       <c r="BS8" t="n">
-        <v>0.6327433073496426</v>
+        <v>0.6347384707687515</v>
       </c>
       <c r="BT8" t="n">
-        <v>0.6989130013474428</v>
+        <v>0.6894804118541484</v>
       </c>
       <c r="BU8" t="n">
-        <v>0.4972626596029361</v>
+        <v>0.5172545731418249</v>
       </c>
       <c r="BV8" t="n">
-        <v>0.1233424708069024</v>
+        <v>0.1081947271876592</v>
       </c>
       <c r="BW8" t="n">
-        <v>0.04658913073714011</v>
+        <v>0.0456783864087682</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.3625</v>
+        <v>0.5033333333333334</v>
       </c>
       <c r="B9" t="n">
-        <v>0.35</v>
+        <v>0.4966666666666667</v>
       </c>
       <c r="C9" t="n">
         <v>0.9399999999999999</v>
       </c>
       <c r="D9" t="n">
-        <v>0.8442592793216259</v>
+        <v>0.886040204530712</v>
       </c>
       <c r="E9" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="F9" t="n">
-        <v>1.066429875635743</v>
+        <v>1.01899260985795</v>
       </c>
       <c r="G9" t="n">
-        <v>334.9958456714842</v>
+        <v>330.3561984983635</v>
       </c>
       <c r="H9" t="n">
-        <v>0.3605527408399267</v>
+        <v>0.2918079074728968</v>
       </c>
       <c r="I9" t="n">
-        <v>544.7954557524375</v>
+        <v>487.6410576509101</v>
       </c>
       <c r="J9" t="n">
-        <v>713471.5292305814</v>
+        <v>512393.8605060804</v>
       </c>
       <c r="K9" t="n">
-        <v>40462.02778444644</v>
+        <v>31846.519562997</v>
       </c>
       <c r="L9" t="n">
-        <v>38034.30611737965</v>
+        <v>29935.72838921718</v>
       </c>
       <c r="M9" t="n">
-        <v>32110.81587215705</v>
+        <v>26524.25890475783</v>
       </c>
       <c r="N9" t="n">
-        <v>37.80746134928394</v>
+        <v>29.75718527755187</v>
       </c>
       <c r="O9" t="n">
-        <v>582.6029171017215</v>
+        <v>517.398242928462</v>
       </c>
       <c r="P9" t="n">
-        <v>582.6029171017215</v>
+        <v>517.398242928462</v>
       </c>
       <c r="Q9" t="n">
-        <v>1.220524649009106</v>
+        <v>1.202378070080593</v>
       </c>
       <c r="R9" t="n">
-        <v>870809.5877921456</v>
+        <v>616091.1411164453</v>
       </c>
       <c r="S9" t="n">
-        <v>870809.5877921456</v>
+        <v>616091.1411164453</v>
       </c>
       <c r="T9" t="n">
-        <v>427.3990130004892</v>
+        <v>404.358809265175</v>
       </c>
       <c r="U9" t="n">
-        <v>441.980495162634</v>
+        <v>416.5136622656132</v>
       </c>
       <c r="V9" t="n">
-        <v>0.7615773105863909</v>
+        <v>0.7905694150420949</v>
       </c>
       <c r="W9" t="n">
-        <v>0.1440741840057616</v>
+        <v>0.2107291821486428</v>
       </c>
       <c r="X9" t="n">
-        <v>1.064577496794081</v>
+        <v>1.163669370778668</v>
       </c>
       <c r="Y9" t="n">
-        <v>121.435994055913</v>
+        <v>166.2792865775097</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.3248720262443578</v>
+        <v>0.4478210551388968</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.4902267786136445</v>
+        <v>0.6488550652132633</v>
       </c>
       <c r="AB9" t="n">
-        <v>0.1108926247734101</v>
+        <v>0.1051218473812989</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.35</v>
+        <v>0.4966666666666667</v>
       </c>
       <c r="AD9" t="n">
-        <v>117.2485459850195</v>
+        <v>164.0769119208539</v>
       </c>
       <c r="AE9" t="n">
-        <v>0.3033211971446864</v>
+        <v>0.4289942661294574</v>
       </c>
       <c r="AF9" t="n">
-        <v>0.4603395387699436</v>
+        <v>0.6260092288210374</v>
       </c>
       <c r="AG9" t="n">
-        <v>0.100056302624151</v>
+        <v>0.0933428901700914</v>
       </c>
       <c r="AH9" t="n">
-        <v>0.6619729934593227</v>
+        <v>0.6536884130678781</v>
       </c>
       <c r="AI9" t="n">
-        <v>0.8898113151741506</v>
+        <v>0.8910157904237872</v>
       </c>
       <c r="AJ9" t="n">
-        <v>0.946510479765531</v>
+        <v>0.9470768550610151</v>
       </c>
       <c r="AK9" t="n">
-        <v>0.281528605843333</v>
+        <v>0.3171786054504727</v>
       </c>
       <c r="AL9" t="n">
-        <v>0.9005374717254715</v>
+        <v>1.006182775046917</v>
       </c>
       <c r="AM9" t="n">
-        <v>0.3404490152611628</v>
+        <v>0.4674047518645908</v>
       </c>
       <c r="AN9" t="n">
-        <v>0.5088534310976932</v>
+        <v>0.670722061360207</v>
       </c>
       <c r="AO9" t="n">
-        <v>0.09051697283767492</v>
+        <v>0.08712030520183586</v>
       </c>
       <c r="AP9" t="n">
-        <v>0.854043895175961</v>
+        <v>0.868823135051555</v>
       </c>
       <c r="AQ9" t="n">
-        <v>0.5506466038529215</v>
+        <v>0.527614810474916</v>
       </c>
       <c r="AR9" t="n">
-        <v>0.5308367445217098</v>
+        <v>0.7148831019922585</v>
       </c>
       <c r="AS9" t="n">
-        <v>0.35625</v>
+        <v>0.5</v>
       </c>
       <c r="AT9" t="n">
-        <v>0.8653500475224741</v>
+        <v>0.9719690024117941</v>
       </c>
       <c r="AU9" t="n">
-        <v>0.5742398709033788</v>
+        <v>0.7585319039895938</v>
       </c>
       <c r="AV9" t="n">
-        <v>0.3345133030007643</v>
+        <v>0.2570859004195356</v>
       </c>
       <c r="AW9" t="n">
-        <v>0.8933979759636368</v>
+        <v>1.002466556264767</v>
       </c>
       <c r="AX9" t="n">
-        <v>0.319158105060258</v>
+        <v>0.2439346522751727</v>
       </c>
       <c r="AY9" t="n">
-        <v>130.6757008041521</v>
+        <v>180.2640997302265</v>
       </c>
       <c r="AZ9" t="n">
-        <v>4.953187281049108</v>
+        <v>3.776266265917991</v>
       </c>
       <c r="BA9" t="n">
-        <v>239.8711457535123</v>
+        <v>253.6565891408028</v>
       </c>
       <c r="BB9" t="n">
-        <v>119.3422700204662</v>
+        <v>165.1780992491818</v>
       </c>
       <c r="BC9" t="n">
-        <v>156.7565726515706</v>
+        <v>199.9741661384299</v>
       </c>
       <c r="BD9" t="n">
-        <v>219.7035832877112</v>
+        <v>240.1345068725876</v>
       </c>
       <c r="BE9" t="n">
-        <v>0.9824096944273142</v>
+        <v>0.9665760504290475</v>
       </c>
       <c r="BF9" t="n">
-        <v>535.2123372111415</v>
+        <v>471.3421675312601</v>
       </c>
       <c r="BG9" t="n">
-        <v>464.0560698884079</v>
+        <v>435.4873528908478</v>
       </c>
       <c r="BH9" t="n">
-        <v>0.5169012137072022</v>
+        <v>0.5824660290522381</v>
       </c>
       <c r="BI9" t="n">
-        <v>0.4970888663466193</v>
+        <v>0.5765345260618423</v>
       </c>
       <c r="BJ9" t="n">
-        <v>582.6029171017215</v>
+        <v>517.398242928462</v>
       </c>
       <c r="BK9" t="n">
-        <v>0.9588171098257054</v>
+        <v>0.9446013233764412</v>
       </c>
       <c r="BL9" t="n">
-        <v>679.9152482351244</v>
+        <v>683.3822593499328</v>
       </c>
       <c r="BM9" t="n">
-        <v>523.0398639490919</v>
+        <v>524.3717058271155</v>
       </c>
       <c r="BN9" t="n">
-        <v>0.4200513162206986</v>
+        <v>0.4579471092815971</v>
       </c>
       <c r="BO9" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.3668220137585716</v>
       </c>
       <c r="BP9" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.1834110068792858</v>
       </c>
       <c r="BQ9" t="n">
-        <v>0.6773344445505896</v>
+        <v>0.7139378684462849</v>
       </c>
       <c r="BR9" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5799965296833545</v>
       </c>
       <c r="BS9" t="n">
-        <v>0.6353639071499578</v>
+        <v>0.6374069039992936</v>
       </c>
       <c r="BT9" t="n">
-        <v>0.7041542009480733</v>
+        <v>0.6948172783152328</v>
       </c>
       <c r="BU9" t="n">
-        <v>0.5039013352448847</v>
+        <v>0.5237762532039368</v>
       </c>
       <c r="BV9" t="n">
-        <v>0.1200231329859281</v>
+        <v>0.1049338871566032</v>
       </c>
       <c r="BW9" t="n">
-        <v>0.04098730387870908</v>
+        <v>0.03997780722463257</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.35</v>
+        <v>0.4966666666666667</v>
       </c>
       <c r="B10" t="n">
-        <v>0.3375</v>
+        <v>0.49</v>
       </c>
       <c r="C10" t="n">
         <v>0.9399999999999999</v>
       </c>
       <c r="D10" t="n">
-        <v>0.8345538265996715</v>
+        <v>0.8866846944514155</v>
       </c>
       <c r="E10" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="F10" t="n">
-        <v>1.066429875635743</v>
+        <v>1.01899260985795</v>
       </c>
       <c r="G10" t="n">
-        <v>334.9958456714842</v>
+        <v>330.3561984983635</v>
       </c>
       <c r="H10" t="n">
-        <v>0.3629425367369873</v>
+        <v>0.2961695371069186</v>
       </c>
       <c r="I10" t="n">
-        <v>582.6029171017215</v>
+        <v>517.398242928462</v>
       </c>
       <c r="J10" t="n">
-        <v>870809.5877921456</v>
+        <v>616091.1411164453</v>
       </c>
       <c r="K10" t="n">
-        <v>40730.21597727716</v>
+        <v>32322.52696344526</v>
       </c>
       <c r="L10" t="n">
-        <v>38286.40301864053</v>
+        <v>30383.17534563854</v>
       </c>
       <c r="M10" t="n">
-        <v>31952.06414594367</v>
+        <v>26940.29654781129</v>
       </c>
       <c r="N10" t="n">
-        <v>38.05805469049754</v>
+        <v>30.20196356425303</v>
       </c>
       <c r="O10" t="n">
-        <v>620.660971792219</v>
+        <v>547.600206492715</v>
       </c>
       <c r="P10" t="n">
-        <v>620.660971792219</v>
+        <v>547.600206492715</v>
       </c>
       <c r="Q10" t="n">
-        <v>1.204167456353411</v>
+        <v>1.193179329499475</v>
       </c>
       <c r="R10" t="n">
-        <v>1048600.566299831</v>
+        <v>735107.2146678865</v>
       </c>
       <c r="S10" t="n">
-        <v>1048600.566299831</v>
+        <v>735107.2146678865</v>
       </c>
       <c r="T10" t="n">
-        <v>441.980495162634</v>
+        <v>416.5136622656132</v>
       </c>
       <c r="U10" t="n">
-        <v>456.1881452229234</v>
+        <v>428.4977820677807</v>
       </c>
       <c r="V10" t="n">
-        <v>0.7615773105863909</v>
+        <v>0.7905694150420949</v>
       </c>
       <c r="W10" t="n">
-        <v>0.1425052061332324</v>
+        <v>0.2079706453579238</v>
       </c>
       <c r="X10" t="n">
-        <v>1.064577496794081</v>
+        <v>1.163669370778668</v>
       </c>
       <c r="Y10" t="n">
-        <v>117.2485459850195</v>
+        <v>164.0769119208539</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.3033211971446864</v>
+        <v>0.4289942661294574</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.4603395387699436</v>
+        <v>0.6260092288210374</v>
       </c>
       <c r="AB10" t="n">
-        <v>0.100056302624151</v>
+        <v>0.09334289017009137</v>
       </c>
       <c r="AC10" t="n">
-        <v>0.3375</v>
+        <v>0.49</v>
       </c>
       <c r="AD10" t="n">
-        <v>113.0610979141259</v>
+        <v>161.8745372641982</v>
       </c>
       <c r="AE10" t="n">
-        <v>0.2833789606329719</v>
+        <v>0.4113989955386405</v>
       </c>
       <c r="AF10" t="n">
-        <v>0.4322063770688386</v>
+        <v>0.6041564687702409</v>
       </c>
       <c r="AG10" t="n">
-        <v>0.09134516475091831</v>
+        <v>0.08339233905144858</v>
       </c>
       <c r="AH10" t="n">
-        <v>0.6709315018399133</v>
+        <v>0.6631087135010758</v>
       </c>
       <c r="AI10" t="n">
-        <v>0.9018531691514183</v>
+        <v>0.9038562144984964</v>
       </c>
       <c r="AJ10" t="n">
-        <v>0.9521919813536703</v>
+        <v>0.9531411376306114</v>
       </c>
       <c r="AK10" t="n">
-        <v>0.2847475699273967</v>
+        <v>0.318958052214398</v>
       </c>
       <c r="AL10" t="n">
-        <v>0.8775390029012443</v>
+        <v>0.9973423395446045</v>
       </c>
       <c r="AM10" t="n">
-        <v>0.3242639972996528</v>
+        <v>0.4507561511543577</v>
       </c>
       <c r="AN10" t="n">
-        <v>0.4865739919422437</v>
+        <v>0.651117799170164</v>
       </c>
       <c r="AO10" t="n">
-        <v>0.08113866210185122</v>
+        <v>0.07737773586903117</v>
       </c>
       <c r="AP10" t="n">
-        <v>0.8568846459700306</v>
+        <v>0.8718552763363532</v>
       </c>
       <c r="AQ10" t="n">
-        <v>0.5502155635368724</v>
+        <v>0.5282812194346006</v>
       </c>
       <c r="AR10" t="n">
-        <v>0.5145610942928165</v>
+        <v>0.7059448619703695</v>
       </c>
       <c r="AS10" t="n">
-        <v>0.34375</v>
+        <v>0.4933333333333334</v>
       </c>
       <c r="AT10" t="n">
-        <v>0.8423473256617744</v>
+        <v>0.9624677305416228</v>
       </c>
       <c r="AU10" t="n">
-        <v>0.5584232149984406</v>
+        <v>0.751203012861814</v>
       </c>
       <c r="AV10" t="n">
-        <v>0.3277862313689579</v>
+        <v>0.2565228685712533</v>
       </c>
       <c r="AW10" t="n">
-        <v>0.8699731692653212</v>
+        <v>0.9937642336736436</v>
       </c>
       <c r="AX10" t="n">
-        <v>0.3115499542668806</v>
+        <v>0.2425612208118296</v>
       </c>
       <c r="AY10" t="n">
-        <v>126.5946303533889</v>
+        <v>177.8806523432204</v>
       </c>
       <c r="AZ10" t="n">
-        <v>5.624360949315135</v>
+        <v>4.285450887797291</v>
       </c>
       <c r="BA10" t="n">
-        <v>238.2360518720631</v>
+        <v>252.9111572103827</v>
       </c>
       <c r="BB10" t="n">
-        <v>115.1548219495727</v>
+        <v>162.975724592526</v>
       </c>
       <c r="BC10" t="n">
-        <v>154.3200418328142</v>
+        <v>198.6045059914631</v>
       </c>
       <c r="BD10" t="n">
-        <v>217.3349232851236</v>
+        <v>238.785798693533</v>
       </c>
       <c r="BE10" t="n">
-        <v>0.9846660418937857</v>
+        <v>0.969327319938008</v>
       </c>
       <c r="BF10" t="n">
-        <v>573.6693083783255</v>
+        <v>501.5282521584804</v>
       </c>
       <c r="BG10" t="n">
-        <v>480.4389481704237</v>
+        <v>449.2158807728041</v>
       </c>
       <c r="BH10" t="n">
-        <v>0.4958716456675673</v>
+        <v>0.563005824227072</v>
       </c>
       <c r="BI10" t="n">
-        <v>0.4764151053923584</v>
+        <v>0.5572626246540556</v>
       </c>
       <c r="BJ10" t="n">
-        <v>620.660971792219</v>
+        <v>547.600206492715</v>
       </c>
       <c r="BK10" t="n">
-        <v>0.9621714412256647</v>
+        <v>0.9482430611939455</v>
       </c>
       <c r="BL10" t="n">
-        <v>682.2938677268862</v>
+        <v>686.0169147924961</v>
       </c>
       <c r="BM10" t="n">
-        <v>523.9539680340154</v>
+        <v>525.3815431054927</v>
       </c>
       <c r="BN10" t="n">
-        <v>0.4147977428257859</v>
+        <v>0.4544997855883693</v>
       </c>
       <c r="BO10" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.3668220137585716</v>
       </c>
       <c r="BP10" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.1834110068792858</v>
       </c>
       <c r="BQ10" t="n">
-        <v>0.6844724925067254</v>
+        <v>0.721292760085028</v>
       </c>
       <c r="BR10" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5799965296833545</v>
       </c>
       <c r="BS10" t="n">
-        <v>0.6374772768888605</v>
+        <v>0.639631416343474</v>
       </c>
       <c r="BT10" t="n">
-        <v>0.7083809404258787</v>
+        <v>0.6992663030035934</v>
       </c>
       <c r="BU10" t="n">
-        <v>0.509211668899222</v>
+        <v>0.5291721255277364</v>
       </c>
       <c r="BV10" t="n">
-        <v>0.1173679661587594</v>
+        <v>0.1022359509947034</v>
       </c>
       <c r="BW10" t="n">
-        <v>0.03650804968841376</v>
+        <v>0.03526765700803369</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.3375</v>
+        <v>0.49</v>
       </c>
       <c r="B11" t="n">
-        <v>0.325</v>
+        <v>0.4833333333333333</v>
       </c>
       <c r="C11" t="n">
         <v>0.9399999999999999</v>
       </c>
       <c r="D11" t="n">
-        <v>0.8238053834530781</v>
+        <v>0.887084061455359</v>
       </c>
       <c r="E11" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="F11" t="n">
-        <v>1.066429875635743</v>
+        <v>1.01899260985795</v>
       </c>
       <c r="G11" t="n">
-        <v>334.9958456714842</v>
+        <v>330.3561984983635</v>
       </c>
       <c r="H11" t="n">
-        <v>0.3644008637646071</v>
+        <v>0.3004539467556255</v>
       </c>
       <c r="I11" t="n">
-        <v>620.660971792219</v>
+        <v>547.600206492715</v>
       </c>
       <c r="J11" t="n">
-        <v>1048600.566299831</v>
+        <v>735107.2146678865</v>
       </c>
       <c r="K11" t="n">
-        <v>40893.87266886935</v>
+        <v>32790.10694397101</v>
       </c>
       <c r="L11" t="n">
-        <v>38440.24030873719</v>
+        <v>30822.70052733275</v>
       </c>
       <c r="M11" t="n">
-        <v>31667.27690756771</v>
+        <v>27342.32636880857</v>
       </c>
       <c r="N11" t="n">
-        <v>38.21097446196539</v>
+        <v>30.63886732339239</v>
       </c>
       <c r="O11" t="n">
-        <v>658.8719462541844</v>
+        <v>578.2390738161074</v>
       </c>
       <c r="P11" t="n">
-        <v>658.8719462541844</v>
+        <v>578.2390738161074</v>
       </c>
       <c r="Q11" t="n">
-        <v>1.189052302015514</v>
+        <v>1.184763652161305</v>
       </c>
       <c r="R11" t="n">
-        <v>1246840.917253586</v>
+        <v>870928.3083800498</v>
       </c>
       <c r="S11" t="n">
-        <v>1246840.917253586</v>
+        <v>870928.3083800498</v>
       </c>
       <c r="T11" t="n">
-        <v>456.1881452229234</v>
+        <v>428.4977820677807</v>
       </c>
       <c r="U11" t="n">
-        <v>470.021024613823</v>
+        <v>440.3221110170835</v>
       </c>
       <c r="V11" t="n">
-        <v>0.7615773105863909</v>
+        <v>0.7905694150420949</v>
       </c>
       <c r="W11" t="n">
-        <v>0.141547767533534</v>
+        <v>0.2052609467741006</v>
       </c>
       <c r="X11" t="n">
-        <v>1.064577496794081</v>
+        <v>1.163669370778668</v>
       </c>
       <c r="Y11" t="n">
-        <v>113.0610979141259</v>
+        <v>161.8745372641982</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.2833789606329719</v>
+        <v>0.4113989955386405</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.4322063770688386</v>
+        <v>0.6041564687702409</v>
       </c>
       <c r="AB11" t="n">
-        <v>0.09134516475091832</v>
+        <v>0.08339233905144861</v>
       </c>
       <c r="AC11" t="n">
-        <v>0.325</v>
+        <v>0.4833333333333333</v>
       </c>
       <c r="AD11" t="n">
-        <v>108.8736498432324</v>
+        <v>159.6721626075424</v>
       </c>
       <c r="AE11" t="n">
-        <v>0.264852390566271</v>
+        <v>0.3949044052960693</v>
       </c>
       <c r="AF11" t="n">
-        <v>0.4056848070423067</v>
+        <v>0.5832461355531482</v>
       </c>
       <c r="AG11" t="n">
-        <v>0.08432577123228341</v>
+        <v>0.07492278450542181</v>
       </c>
       <c r="AH11" t="n">
-        <v>0.6781934296933768</v>
+        <v>0.6709790337886259</v>
       </c>
       <c r="AI11" t="n">
-        <v>0.9116145123449262</v>
+        <v>0.9145839243855182</v>
       </c>
       <c r="AJ11" t="n">
-        <v>0.9568283595080879</v>
+        <v>0.958244163755881</v>
       </c>
       <c r="AK11" t="n">
-        <v>0.2877665857908671</v>
+        <v>0.3201490716692275</v>
       </c>
       <c r="AL11" t="n">
-        <v>0.8540733970766762</v>
+        <v>0.9892092539638102</v>
       </c>
       <c r="AM11" t="n">
-        <v>0.3093872915612632</v>
+        <v>0.4349611283481297</v>
       </c>
       <c r="AN11" t="n">
-        <v>0.4657932677724579</v>
+        <v>0.6321077326660305</v>
       </c>
       <c r="AO11" t="n">
-        <v>0.07344392158062314</v>
+        <v>0.06913129245130799</v>
       </c>
       <c r="AP11" t="n">
-        <v>0.8592028350472394</v>
+        <v>0.874406789398988</v>
       </c>
       <c r="AQ11" t="n">
-        <v>0.5495796948299662</v>
+        <v>0.5291895934338091</v>
       </c>
       <c r="AR11" t="n">
-        <v>0.4984787765891089</v>
+        <v>0.696995567805058</v>
       </c>
       <c r="AS11" t="n">
-        <v>0.33125</v>
+        <v>0.4866666666666667</v>
       </c>
       <c r="AT11" t="n">
-        <v>0.8191312917860756</v>
+        <v>0.953822451893052</v>
       </c>
       <c r="AU11" t="n">
-        <v>0.5424268789629988</v>
+        <v>0.7435633897203713</v>
       </c>
       <c r="AV11" t="n">
-        <v>0.3206525151969667</v>
+        <v>0.256826884087994</v>
       </c>
       <c r="AW11" t="n">
-        <v>0.8460863486369866</v>
+        <v>0.9857691042117221</v>
       </c>
       <c r="AX11" t="n">
-        <v>0.3036594696739878</v>
+        <v>0.2422057144913509</v>
       </c>
       <c r="AY11" t="n">
-        <v>122.6020817033145</v>
+        <v>175.5034385862216</v>
       </c>
       <c r="AZ11" t="n">
-        <v>6.325027396634392</v>
+        <v>4.837283589515337</v>
       </c>
       <c r="BA11" t="n">
-        <v>236.4849743786179</v>
+        <v>252.1736780466167</v>
       </c>
       <c r="BB11" t="n">
-        <v>110.9673738786792</v>
+        <v>160.7733499358703</v>
       </c>
       <c r="BC11" t="n">
-        <v>151.8950557315864</v>
+        <v>197.1148144606858</v>
       </c>
       <c r="BD11" t="n">
-        <v>214.9630528285631</v>
+        <v>237.5088922511478</v>
       </c>
       <c r="BE11" t="n">
-        <v>0.9866160607784294</v>
+        <v>0.9717918110782996</v>
       </c>
       <c r="BF11" t="n">
-        <v>612.3540830685511</v>
+        <v>532.1533964144063</v>
       </c>
       <c r="BG11" t="n">
-        <v>496.3736383647526</v>
+        <v>462.7280417062494</v>
       </c>
       <c r="BH11" t="n">
-        <v>0.4764253298335728</v>
+        <v>0.5449716795134331</v>
       </c>
       <c r="BI11" t="n">
-        <v>0.45734773887015</v>
+        <v>0.5393980595308624</v>
       </c>
       <c r="BJ11" t="n">
-        <v>658.8719462541844</v>
+        <v>578.2390738161074</v>
       </c>
       <c r="BK11" t="n">
-        <v>0.9651388409583935</v>
+        <v>0.9515082888957234</v>
       </c>
       <c r="BL11" t="n">
-        <v>684.3981066951061</v>
+        <v>688.3791798337485</v>
       </c>
       <c r="BM11" t="n">
-        <v>524.7613002211986</v>
+        <v>526.2853283133655</v>
       </c>
       <c r="BN11" t="n">
-        <v>0.4096396832959126</v>
+        <v>0.4512930144040195</v>
       </c>
       <c r="BO11" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.3668220137585716</v>
       </c>
       <c r="BP11" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.1834110068792858</v>
       </c>
       <c r="BQ11" t="n">
-        <v>0.6902601129331082</v>
+        <v>0.7274437893707612</v>
       </c>
       <c r="BR11" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5799965296833545</v>
       </c>
       <c r="BS11" t="n">
-        <v>0.6392018880920168</v>
+        <v>0.6415033186630079</v>
       </c>
       <c r="BT11" t="n">
-        <v>0.7118301628321914</v>
+        <v>0.7030101076426614</v>
       </c>
       <c r="BU11" t="n">
-        <v>0.5135173552321824</v>
+        <v>0.5336847914262977</v>
       </c>
       <c r="BV11" t="n">
-        <v>0.1152151229922792</v>
+        <v>0.09997961804542277</v>
       </c>
       <c r="BW11" t="n">
-        <v>0.03287708576168202</v>
+        <v>0.03133249686425865</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0.325</v>
+        <v>0.4833333333333333</v>
       </c>
       <c r="B12" t="n">
-        <v>0.3125</v>
+        <v>0.4766666666666667</v>
       </c>
       <c r="C12" t="n">
         <v>0.9399999999999999</v>
       </c>
       <c r="D12" t="n">
-        <v>0.8120003556960932</v>
+        <v>0.8872368569202875</v>
       </c>
       <c r="E12" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="F12" t="n">
-        <v>1.066429875635743</v>
+        <v>1.01899260985795</v>
       </c>
       <c r="G12" t="n">
-        <v>334.9958456714842</v>
+        <v>330.3561984983635</v>
       </c>
       <c r="H12" t="n">
-        <v>0.3648340491519012</v>
+        <v>0.3046699184544066</v>
       </c>
       <c r="I12" t="n">
-        <v>658.8719462541844</v>
+        <v>578.2390738161074</v>
       </c>
       <c r="J12" t="n">
-        <v>1246840.917253586</v>
+        <v>870928.3083800498</v>
       </c>
       <c r="K12" t="n">
-        <v>40942.48569323765</v>
+        <v>33250.21793391992</v>
       </c>
       <c r="L12" t="n">
-        <v>38485.93655164339</v>
+        <v>31255.20485788472</v>
       </c>
       <c r="M12" t="n">
-        <v>31250.59416923171</v>
+        <v>27730.76972050935</v>
       </c>
       <c r="N12" t="n">
-        <v>38.25639816266739</v>
+        <v>31.06879210525321</v>
       </c>
       <c r="O12" t="n">
-        <v>697.1283444168519</v>
+        <v>609.3078659213606</v>
       </c>
       <c r="P12" t="n">
-        <v>697.1283444168519</v>
+        <v>609.3078659213606</v>
       </c>
       <c r="Q12" t="n">
-        <v>1.174972243401005</v>
+        <v>1.177030148064128</v>
       </c>
       <c r="R12" t="n">
-        <v>1465003.469709612</v>
+        <v>1025108.875765811</v>
       </c>
       <c r="S12" t="n">
-        <v>1465003.469709612</v>
+        <v>1025108.875765811</v>
       </c>
       <c r="T12" t="n">
-        <v>470.021024613823</v>
+        <v>440.3221110170835</v>
       </c>
       <c r="U12" t="n">
-        <v>483.4740260685887</v>
+        <v>451.9966011414602</v>
       </c>
       <c r="V12" t="n">
-        <v>0.7615773105863909</v>
+        <v>0.7905694150420949</v>
       </c>
       <c r="W12" t="n">
-        <v>0.1412633673936713</v>
+        <v>0.2025945321503091</v>
       </c>
       <c r="X12" t="n">
-        <v>1.064577496794081</v>
+        <v>1.163669370778668</v>
       </c>
       <c r="Y12" t="n">
-        <v>108.8736498432324</v>
+        <v>159.6721626075424</v>
       </c>
       <c r="Z12" t="n">
-        <v>0.264852390566271</v>
+        <v>0.3949044052960693</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.4056848070423067</v>
+        <v>0.5832461355531482</v>
       </c>
       <c r="AB12" t="n">
-        <v>0.08432577123228341</v>
+        <v>0.07492278450542178</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.3125</v>
+        <v>0.4766666666666667</v>
       </c>
       <c r="AD12" t="n">
-        <v>104.6862017723388</v>
+        <v>157.4697879508866</v>
       </c>
       <c r="AE12" t="n">
-        <v>0.2475795080404627</v>
+        <v>0.3793982636452001</v>
       </c>
       <c r="AF12" t="n">
-        <v>0.3806439700063695</v>
+        <v>0.5632271200850089</v>
       </c>
       <c r="AG12" t="n">
-        <v>0.07867891571681149</v>
+        <v>0.06766425569023406</v>
       </c>
       <c r="AH12" t="n">
-        <v>0.6841493266339539</v>
+        <v>0.6776186395344173</v>
       </c>
       <c r="AI12" t="n">
-        <v>0.9196203140046615</v>
+        <v>0.9236340978984978</v>
       </c>
       <c r="AJ12" t="n">
-        <v>0.9606512171256621</v>
+        <v>0.9625746586111572</v>
       </c>
       <c r="AK12" t="n">
-        <v>0.2907964460364127</v>
+        <v>0.3208808500673349</v>
       </c>
       <c r="AL12" t="n">
-        <v>0.8297807583132409</v>
+        <v>0.9816074212305465</v>
       </c>
       <c r="AM12" t="n">
-        <v>0.2957759736655972</v>
+        <v>0.419971480377387</v>
       </c>
       <c r="AN12" t="n">
-        <v>0.4465201903401176</v>
+        <v>0.6137058459021709</v>
       </c>
       <c r="AO12" t="n">
-        <v>0.06707122204581961</v>
+        <v>0.06209871409825427</v>
       </c>
       <c r="AP12" t="n">
-        <v>0.8611142638560265</v>
+        <v>0.8765720368266261</v>
       </c>
       <c r="AQ12" t="n">
-        <v>0.5486113102580497</v>
+        <v>0.5302872321937201</v>
       </c>
       <c r="AR12" t="n">
-        <v>0.4826064562566781</v>
+        <v>0.6880306120776167</v>
       </c>
       <c r="AS12" t="n">
-        <v>0.31875</v>
+        <v>0.48</v>
       </c>
       <c r="AT12" t="n">
-        <v>0.7952941051769974</v>
+        <v>0.9458343174188085</v>
       </c>
       <c r="AU12" t="n">
-        <v>0.5263410536891099</v>
+        <v>0.7356640262208594</v>
       </c>
       <c r="AV12" t="n">
-        <v>0.3126876489203193</v>
+        <v>0.2578037053411918</v>
       </c>
       <c r="AW12" t="n">
-        <v>0.8213575967455732</v>
+        <v>0.9783003714220208</v>
       </c>
       <c r="AX12" t="n">
-        <v>0.2950165430564633</v>
+        <v>0.2426363452011614</v>
       </c>
       <c r="AY12" t="n">
-        <v>118.7135375702998</v>
+        <v>173.1317556491292</v>
       </c>
       <c r="AZ12" t="n">
-        <v>7.048422847999833</v>
+        <v>5.433149169660529</v>
       </c>
       <c r="BA12" t="n">
-        <v>234.596226942576</v>
+        <v>251.4454667479009</v>
       </c>
       <c r="BB12" t="n">
-        <v>106.7799258077856</v>
+        <v>158.5709752792145</v>
       </c>
       <c r="BC12" t="n">
-        <v>149.5371544469267</v>
+        <v>195.528779700271</v>
       </c>
       <c r="BD12" t="n">
-        <v>212.5510843845128</v>
+        <v>236.2923483443731</v>
       </c>
       <c r="BE12" t="n">
-        <v>0.9883088685352219</v>
+        <v>0.9740084184462929</v>
       </c>
       <c r="BF12" t="n">
-        <v>651.1689877120725</v>
+        <v>563.209725771476</v>
       </c>
       <c r="BG12" t="n">
-        <v>511.8636086848034</v>
+        <v>476.038932505957</v>
       </c>
       <c r="BH12" t="n">
-        <v>0.4583178467118498</v>
+        <v>0.528203576594556</v>
       </c>
       <c r="BI12" t="n">
-        <v>0.4396328922008292</v>
+        <v>0.5227746132330348</v>
       </c>
       <c r="BJ12" t="n">
-        <v>697.1283444168519</v>
+        <v>609.3078659213606</v>
       </c>
       <c r="BK12" t="n">
-        <v>0.967787153349189</v>
+        <v>0.9544511172931751</v>
       </c>
       <c r="BL12" t="n">
-        <v>686.2760748270256</v>
+        <v>690.5082015377847</v>
       </c>
       <c r="BM12" t="n">
-        <v>525.4807717389875</v>
+        <v>527.098548632742</v>
       </c>
       <c r="BN12" t="n">
-        <v>0.4044887954341541</v>
+        <v>0.4482887478201174</v>
       </c>
       <c r="BO12" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.3668220137585716</v>
       </c>
       <c r="BP12" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.1834110068792858</v>
       </c>
       <c r="BQ12" t="n">
-        <v>0.6950075904856097</v>
+        <v>0.7326370666931614</v>
       </c>
       <c r="BR12" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5799965296833545</v>
       </c>
       <c r="BS12" t="n">
-        <v>0.6406238909692106</v>
+        <v>0.6430918395063915</v>
       </c>
       <c r="BT12" t="n">
-        <v>0.7146741685865788</v>
+        <v>0.7061871493294285</v>
       </c>
       <c r="BU12" t="n">
-        <v>0.5170492297691963</v>
+        <v>0.5374948083171168</v>
       </c>
       <c r="BV12" t="n">
-        <v>0.1134491857237723</v>
+        <v>0.09807460960001319</v>
       </c>
       <c r="BW12" t="n">
-        <v>0.02989913729139348</v>
+        <v>0.02801269399136297</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.3125</v>
+        <v>0.4766666666666667</v>
       </c>
       <c r="B13" t="n">
-        <v>0.3</v>
+        <v>0.47</v>
       </c>
       <c r="C13" t="n">
         <v>0.9399999999999999</v>
       </c>
       <c r="D13" t="n">
-        <v>0.7991254713803608</v>
+        <v>0.8871396719634219</v>
       </c>
       <c r="E13" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="F13" t="n">
-        <v>1.066429875635743</v>
+        <v>1.01899260985795</v>
       </c>
       <c r="G13" t="n">
-        <v>334.9958456714842</v>
+        <v>330.3561984983635</v>
       </c>
       <c r="H13" t="n">
-        <v>0.3641428413236223</v>
+        <v>0.3088064239835401</v>
       </c>
       <c r="I13" t="n">
-        <v>697.1283444168519</v>
+        <v>609.3078659213606</v>
       </c>
       <c r="J13" t="n">
-        <v>1465003.469709612</v>
+        <v>1025108.875765811</v>
       </c>
       <c r="K13" t="n">
-        <v>40864.91681860507</v>
+        <v>33701.65636612976</v>
       </c>
       <c r="L13" t="n">
-        <v>38413.02180948877</v>
+        <v>31679.55698416197</v>
       </c>
       <c r="M13" t="n">
-        <v>30696.82416065179</v>
+        <v>28104.19179087598</v>
       </c>
       <c r="N13" t="n">
-        <v>38.18391829969062</v>
+        <v>31.49061330433595</v>
       </c>
       <c r="O13" t="n">
-        <v>735.3122627165425</v>
+        <v>640.7984792256966</v>
       </c>
       <c r="P13" t="n">
-        <v>735.3122627165425</v>
+        <v>640.7984792256966</v>
       </c>
       <c r="Q13" t="n">
-        <v>1.161763539474074</v>
+        <v>1.169883030704616</v>
       </c>
       <c r="R13" t="n">
-        <v>1701987.616311639</v>
+        <v>1199257.478383109</v>
       </c>
       <c r="S13" t="n">
-        <v>1701987.616311639</v>
+        <v>1199257.478383109</v>
       </c>
       <c r="T13" t="n">
-        <v>483.4740260685887</v>
+        <v>451.9966011414602</v>
       </c>
       <c r="U13" t="n">
-        <v>496.5382177525278</v>
+        <v>463.5296431560511</v>
       </c>
       <c r="V13" t="n">
-        <v>0.7615773105863909</v>
+        <v>0.7905694150420949</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1417171675651513</v>
+        <v>0.1999783763451207</v>
       </c>
       <c r="X13" t="n">
-        <v>1.064577496794081</v>
+        <v>1.163669370778668</v>
       </c>
       <c r="Y13" t="n">
-        <v>104.6862017723388</v>
+        <v>157.4697879508866</v>
       </c>
       <c r="Z13" t="n">
-        <v>0.2475795080404627</v>
+        <v>0.3793982636452001</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.3806439700063695</v>
+        <v>0.5632271200850089</v>
       </c>
       <c r="AB13" t="n">
-        <v>0.07867891571681147</v>
+        <v>0.06766425569023406</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.3</v>
+        <v>0.47</v>
       </c>
       <c r="AD13" t="n">
-        <v>100.4987537014453</v>
+        <v>155.2674132942309</v>
       </c>
       <c r="AE13" t="n">
-        <v>0.2314229337341716</v>
+        <v>0.3647842428199741</v>
       </c>
       <c r="AF13" t="n">
-        <v>0.356964158557928</v>
+        <v>0.5440499571377209</v>
       </c>
       <c r="AG13" t="n">
-        <v>0.07416764671794335</v>
+        <v>0.06140503585093043</v>
       </c>
       <c r="AH13" t="n">
-        <v>0.6890844320072977</v>
+        <v>0.6832678985389423</v>
       </c>
       <c r="AI13" t="n">
-        <v>0.9262539873511073</v>
+        <v>0.9313343705002441</v>
       </c>
       <c r="AJ13" t="n">
-        <v>0.9638325708036187</v>
+        <v>0.9662773177703919</v>
       </c>
       <c r="AK13" t="n">
-        <v>0.2940089553983466</v>
+        <v>0.3212532171733763</v>
       </c>
       <c r="AL13" t="n">
-        <v>0.8043697733634284</v>
+        <v>0.9743997274875045</v>
       </c>
       <c r="AM13" t="n">
-        <v>0.2833915018027358</v>
+        <v>0.4057391306291831</v>
       </c>
       <c r="AN13" t="n">
-        <v>0.4287582016046487</v>
+        <v>0.5959162664950163</v>
       </c>
       <c r="AO13" t="n">
-        <v>0.0617485368298673</v>
+        <v>0.05606057260230587</v>
       </c>
       <c r="AP13" t="n">
-        <v>0.8627049406950048</v>
+        <v>0.8784233664062434</v>
       </c>
       <c r="AQ13" t="n">
-        <v>0.5471991620698325</v>
+        <v>0.531524125891526</v>
       </c>
       <c r="AR13" t="n">
-        <v>0.466958890421039</v>
+        <v>0.6790558969686254</v>
       </c>
       <c r="AS13" t="n">
-        <v>0.30625</v>
+        <v>0.4733333333333334</v>
       </c>
       <c r="AT13" t="n">
-        <v>0.7705127448541069</v>
+        <v>0.9383386323572477</v>
       </c>
       <c r="AU13" t="n">
-        <v>0.5102357395223244</v>
+        <v>0.7275532672972517</v>
       </c>
       <c r="AV13" t="n">
-        <v>0.3035538544330679</v>
+        <v>0.2592827353886222</v>
       </c>
       <c r="AW13" t="n">
-        <v>0.7954836030482841</v>
+        <v>0.9712183196685195</v>
       </c>
       <c r="AX13" t="n">
-        <v>0.2852478635259598</v>
+        <v>0.2436650523712678</v>
       </c>
       <c r="AY13" t="n">
-        <v>114.9480074251195</v>
+        <v>170.7665041009618</v>
       </c>
       <c r="AZ13" t="n">
-        <v>7.786942573692805</v>
+        <v>6.074326617699174</v>
       </c>
       <c r="BA13" t="n">
-        <v>232.5466861290662</v>
+        <v>250.7246603128491</v>
       </c>
       <c r="BB13" t="n">
-        <v>102.5924777368921</v>
+        <v>156.3686006225587</v>
       </c>
       <c r="BC13" t="n">
-        <v>147.2964805650054</v>
+        <v>193.8668907052053</v>
       </c>
       <c r="BD13" t="n">
-        <v>210.0656314077421</v>
+        <v>235.1250548996557</v>
       </c>
       <c r="BE13" t="n">
-        <v>0.9897840645330738</v>
+        <v>0.9760094929238345</v>
       </c>
       <c r="BF13" t="n">
-        <v>690.0065262381241</v>
+        <v>594.690261252411</v>
       </c>
       <c r="BG13" t="n">
-        <v>526.9070372439256</v>
+        <v>489.1621137389118</v>
       </c>
       <c r="BH13" t="n">
-        <v>0.4413429119213136</v>
+        <v>0.512559442505542</v>
       </c>
       <c r="BI13" t="n">
-        <v>0.4230603484230449</v>
+        <v>0.5072492307045374</v>
       </c>
       <c r="BJ13" t="n">
-        <v>735.3122627165425</v>
+        <v>640.7984792256966</v>
       </c>
       <c r="BK13" t="n">
-        <v>0.970169990265362</v>
+        <v>0.9571163696582758</v>
       </c>
       <c r="BL13" t="n">
-        <v>687.9657893062114</v>
+        <v>692.4364077957325</v>
       </c>
       <c r="BM13" t="n">
-        <v>526.127280213873</v>
+        <v>527.8339824610489</v>
       </c>
       <c r="BN13" t="n">
-        <v>0.3992677044276236</v>
+        <v>0.4454526663921389</v>
       </c>
       <c r="BO13" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.3668220137585716</v>
       </c>
       <c r="BP13" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.1834110068792858</v>
       </c>
       <c r="BQ13" t="n">
-        <v>0.6989417925686972</v>
+        <v>0.7370584924529089</v>
       </c>
       <c r="BR13" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5799965296833545</v>
       </c>
       <c r="BS13" t="n">
-        <v>0.6418072711878795</v>
+        <v>0.6444500563954436</v>
       </c>
       <c r="BT13" t="n">
-        <v>0.7170409290239167</v>
+        <v>0.7089035831075328</v>
       </c>
       <c r="BU13" t="n">
-        <v>0.5199760699716112</v>
+        <v>0.540738560918866</v>
       </c>
       <c r="BV13" t="n">
-        <v>0.1119857656225648</v>
+        <v>0.09645273329913862</v>
       </c>
       <c r="BW13" t="n">
-        <v>0.02743158460472156</v>
+        <v>0.02518806448910044</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0.4633333333333334</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.8867906223057505</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1.01899260985795</v>
+      </c>
+      <c r="G14" t="n">
+        <v>330.3561984983635</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.3128524608067445</v>
+      </c>
+      <c r="I14" t="n">
+        <v>640.7984792256966</v>
+      </c>
+      <c r="J14" t="n">
+        <v>1199257.478383109</v>
+      </c>
+      <c r="K14" t="n">
+        <v>34143.22147640612</v>
+      </c>
+      <c r="L14" t="n">
+        <v>32094.62818782175</v>
+      </c>
+      <c r="M14" t="n">
+        <v>28461.21530335013</v>
+      </c>
+      <c r="N14" t="n">
+        <v>31.90320893421645</v>
+      </c>
+      <c r="O14" t="n">
+        <v>672.701688159913</v>
+      </c>
+      <c r="P14" t="n">
+        <v>672.701688159913</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>1.16324343509115</v>
+      </c>
+      <c r="R14" t="n">
+        <v>1395028.388713118</v>
+      </c>
+      <c r="S14" t="n">
+        <v>1395028.388713118</v>
+      </c>
+      <c r="T14" t="n">
+        <v>463.5296431560511</v>
+      </c>
+      <c r="U14" t="n">
+        <v>474.9282851547367</v>
+      </c>
+      <c r="V14" t="n">
+        <v>0.7905694150420949</v>
+      </c>
+      <c r="W14" t="n">
+        <v>0.1974194379734731</v>
+      </c>
+      <c r="X14" t="n">
+        <v>1.163669370778668</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>155.2674132942309</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>0.3647842428199741</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>0.5440499571377209</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>0.06140503585093043</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>0.4633333333333334</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>153.0650386375751</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>0.3509790833065976</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>0.525667382413151</v>
+      </c>
+      <c r="AG14" t="n">
+        <v>0.05597726199730441</v>
+      </c>
+      <c r="AH14" t="n">
+        <v>0.6881105248608028</v>
+      </c>
+      <c r="AI14" t="n">
+        <v>0.9379351552680958</v>
+      </c>
+      <c r="AJ14" t="n">
+        <v>0.9694643767276306</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>0.3213353951078977</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>0.9674905209827243</v>
+      </c>
+      <c r="AM14" t="n">
+        <v>0.3922139692006276</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>0.578731489558265</v>
+      </c>
+      <c r="AO14" t="n">
+        <v>0.05084468586846386</v>
+      </c>
+      <c r="AP14" t="n">
+        <v>0.8800168958848628</v>
+      </c>
+      <c r="AQ14" t="n">
+        <v>0.532860485515865</v>
+      </c>
+      <c r="AR14" t="n">
+        <v>0.6700771141371021</v>
+      </c>
+      <c r="AS14" t="n">
+        <v>0.4666666666666667</v>
+      </c>
+      <c r="AT14" t="n">
+        <v>0.9312064177956002</v>
+      </c>
+      <c r="AU14" t="n">
+        <v>0.7192695921958087</v>
+      </c>
+      <c r="AV14" t="n">
+        <v>0.2611293036584981</v>
+      </c>
+      <c r="AW14" t="n">
+        <v>0.9644261057893925</v>
+      </c>
+      <c r="AX14" t="n">
+        <v>0.2451565135935838</v>
+      </c>
+      <c r="AY14" t="n">
+        <v>168.4085895407851</v>
+      </c>
+      <c r="AZ14" t="n">
+        <v>6.761980349845451</v>
+      </c>
+      <c r="BA14" t="n">
+        <v>250.0093488402438</v>
+      </c>
+      <c r="BB14" t="n">
+        <v>154.166225965903</v>
+      </c>
+      <c r="BC14" t="n">
+        <v>192.1456136513616</v>
+      </c>
+      <c r="BD14" t="n">
+        <v>233.9981012978615</v>
+      </c>
+      <c r="BE14" t="n">
+        <v>0.9778220760317097</v>
+      </c>
+      <c r="BF14" t="n">
+        <v>626.586899274433</v>
+      </c>
+      <c r="BG14" t="n">
+        <v>502.1090566720151</v>
+      </c>
+      <c r="BH14" t="n">
+        <v>0.4979184213431814</v>
+      </c>
+      <c r="BI14" t="n">
+        <v>0.4927019691438728</v>
+      </c>
+      <c r="BJ14" t="n">
+        <v>672.701688159913</v>
+      </c>
+      <c r="BK14" t="n">
+        <v>0.9595407949336251</v>
+      </c>
+      <c r="BL14" t="n">
+        <v>694.1903850359623</v>
+      </c>
+      <c r="BM14" t="n">
+        <v>528.5020750414039</v>
+      </c>
+      <c r="BN14" t="n">
+        <v>0.442757204462309</v>
+      </c>
+      <c r="BO14" t="n">
+        <v>0.3668220137585716</v>
+      </c>
+      <c r="BP14" t="n">
+        <v>0.1834110068792858</v>
+      </c>
+      <c r="BQ14" t="n">
+        <v>0.7408505072453273</v>
+      </c>
+      <c r="BR14" t="n">
+        <v>0.5799965296833545</v>
+      </c>
+      <c r="BS14" t="n">
+        <v>0.6456191397801052</v>
+      </c>
+      <c r="BT14" t="n">
+        <v>0.711241749876856</v>
+      </c>
+      <c r="BU14" t="n">
+        <v>0.5435205499235805</v>
+      </c>
+      <c r="BV14" t="n">
+        <v>0.09506173879678137</v>
+      </c>
+      <c r="BW14" t="n">
+        <v>0.02276675132817019</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>0.4633333333333334</v>
+      </c>
+      <c r="B15" t="n">
+        <v>0.4566666666666667</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.8861860900624504</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1.01899260985795</v>
+      </c>
+      <c r="G15" t="n">
+        <v>330.3561984983635</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.3168147406662835</v>
+      </c>
+      <c r="I15" t="n">
+        <v>672.701688159913</v>
+      </c>
+      <c r="J15" t="n">
+        <v>1395028.388713118</v>
+      </c>
+      <c r="K15" t="n">
+        <v>34575.64575220337</v>
+      </c>
+      <c r="L15" t="n">
+        <v>32501.10700707116</v>
+      </c>
+      <c r="M15" t="n">
+        <v>28802.02894129771</v>
+      </c>
+      <c r="N15" t="n">
+        <v>32.30726342651209</v>
+      </c>
+      <c r="O15" t="n">
+        <v>705.0089515864252</v>
+      </c>
+      <c r="P15" t="n">
+        <v>705.0089515864252</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>1.157054569684315</v>
+      </c>
+      <c r="R15" t="n">
+        <v>1614123.97199986</v>
+      </c>
+      <c r="S15" t="n">
+        <v>1614123.97199986</v>
+      </c>
+      <c r="T15" t="n">
+        <v>474.9282851547367</v>
+      </c>
+      <c r="U15" t="n">
+        <v>486.1990348272283</v>
+      </c>
+      <c r="V15" t="n">
+        <v>0.7905694150420949</v>
+      </c>
+      <c r="W15" t="n">
+        <v>0.1949134721568421</v>
+      </c>
+      <c r="X15" t="n">
+        <v>1.163669370778668</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>153.0650386375751</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>0.3509790833065976</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>0.525667382413151</v>
+      </c>
+      <c r="AB15" t="n">
+        <v>0.05597726199730441</v>
+      </c>
+      <c r="AC15" t="n">
+        <v>0.4566666666666667</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>150.8626639809193</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>0.3379099229908096</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>0.5080340262126917</v>
+      </c>
+      <c r="AG15" t="n">
+        <v>0.05124625064326233</v>
+      </c>
+      <c r="AH15" t="n">
+        <v>0.692289943098427</v>
+      </c>
+      <c r="AI15" t="n">
+        <v>0.9436319483732867</v>
+      </c>
+      <c r="AJ15" t="n">
+        <v>0.9722245764201718</v>
+      </c>
+      <c r="AK15" t="n">
+        <v>0.3211909139007521</v>
+      </c>
+      <c r="AL15" t="n">
+        <v>0.9607904300051596</v>
+      </c>
+      <c r="AM15" t="n">
+        <v>0.3793519973377993</v>
+      </c>
+      <c r="AN15" t="n">
+        <v>0.5621434959384141</v>
+      </c>
+      <c r="AO15" t="n">
+        <v>0.04631351110651925</v>
+      </c>
+      <c r="AP15" t="n">
+        <v>0.8813969957311334</v>
+      </c>
+      <c r="AQ15" t="n">
+        <v>0.5342738545897996</v>
+      </c>
+      <c r="AR15" t="n">
+        <v>0.6610906338160872</v>
+      </c>
+      <c r="AS15" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="AT15" t="n">
+        <v>0.9243478208701578</v>
+      </c>
+      <c r="AU15" t="n">
+        <v>0.7108350463555755</v>
+      </c>
+      <c r="AV15" t="n">
+        <v>0.2632571870540705</v>
+      </c>
+      <c r="AW15" t="n">
+        <v>0.9578337607810785</v>
+      </c>
+      <c r="AX15" t="n">
+        <v>0.246998714425503</v>
+      </c>
+      <c r="AY15" t="n">
+        <v>166.0574920583078</v>
+      </c>
+      <c r="AZ15" t="n">
+        <v>7.497165624283808</v>
+      </c>
+      <c r="BA15" t="n">
+        <v>249.3004942251385</v>
+      </c>
+      <c r="BB15" t="n">
+        <v>151.9638513092472</v>
+      </c>
+      <c r="BC15" t="n">
+        <v>190.3764767522471</v>
+      </c>
+      <c r="BD15" t="n">
+        <v>232.9066379252696</v>
+      </c>
+      <c r="BE15" t="n">
+        <v>0.97946894718021</v>
+      </c>
+      <c r="BF15" t="n">
+        <v>658.89041426834</v>
+      </c>
+      <c r="BG15" t="n">
+        <v>514.8894513242714</v>
+      </c>
+      <c r="BH15" t="n">
+        <v>0.4841825630413469</v>
+      </c>
+      <c r="BI15" t="n">
+        <v>0.4790355826354806</v>
+      </c>
+      <c r="BJ15" t="n">
+        <v>705.0089515864252</v>
+      </c>
+      <c r="BK15" t="n">
+        <v>0.9617541517615142</v>
+      </c>
+      <c r="BL15" t="n">
+        <v>695.7916624768873</v>
+      </c>
+      <c r="BM15" t="n">
+        <v>529.1112674232144</v>
+      </c>
+      <c r="BN15" t="n">
+        <v>0.4401846119428358</v>
+      </c>
+      <c r="BO15" t="n">
+        <v>0.3668220137585716</v>
+      </c>
+      <c r="BP15" t="n">
+        <v>0.1834110068792858</v>
+      </c>
+      <c r="BQ15" t="n">
+        <v>0.7441245380766146</v>
+      </c>
+      <c r="BR15" t="n">
+        <v>0.5799965296833545</v>
+      </c>
+      <c r="BS15" t="n">
+        <v>0.646631641789699</v>
+      </c>
+      <c r="BT15" t="n">
+        <v>0.7132667538960434</v>
+      </c>
+      <c r="BU15" t="n">
+        <v>0.5459225230888614</v>
+      </c>
+      <c r="BV15" t="n">
+        <v>0.09386075221414092</v>
+      </c>
+      <c r="BW15" t="n">
+        <v>0.02067704220935812</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>0.4566666666666667</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.8853238625511552</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1.01899260985795</v>
+      </c>
+      <c r="G16" t="n">
+        <v>330.3561984983635</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.3206812265610493</v>
+      </c>
+      <c r="I16" t="n">
+        <v>705.0089515864252</v>
+      </c>
+      <c r="J16" t="n">
+        <v>1614123.97199986</v>
+      </c>
+      <c r="K16" t="n">
+        <v>34997.6155327829</v>
+      </c>
+      <c r="L16" t="n">
+        <v>32897.75860081593</v>
+      </c>
+      <c r="M16" t="n">
+        <v>29125.17071374985</v>
+      </c>
+      <c r="N16" t="n">
+        <v>32.70154930498601</v>
+      </c>
+      <c r="O16" t="n">
+        <v>737.7105008914111</v>
+      </c>
+      <c r="P16" t="n">
+        <v>737.7105008914111</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>1.151258948221676</v>
+      </c>
+      <c r="R16" t="n">
+        <v>1858274.666303953</v>
+      </c>
+      <c r="S16" t="n">
+        <v>1858274.666303953</v>
+      </c>
+      <c r="T16" t="n">
+        <v>486.1990348272283</v>
+      </c>
+      <c r="U16" t="n">
+        <v>497.3472941002998</v>
+      </c>
+      <c r="V16" t="n">
+        <v>0.7905694150420949</v>
+      </c>
+      <c r="W16" t="n">
+        <v>0.1924680917631673</v>
+      </c>
+      <c r="X16" t="n">
+        <v>1.163669370778668</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>150.8626639809193</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>0.3379099229908096</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>0.5080340262126917</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>0.05124625064326234</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>148.6602893242636</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>0.325513106422404</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>0.4911073006404607</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>0.04710328055450629</v>
+      </c>
+      <c r="AH16" t="n">
+        <v>0.6959190020712755</v>
+      </c>
+      <c r="AI16" t="n">
+        <v>0.9485785694002857</v>
+      </c>
+      <c r="AJ16" t="n">
+        <v>0.9746284682702154</v>
+      </c>
+      <c r="AK16" t="n">
+        <v>0.3208713199288842</v>
+      </c>
+      <c r="AL16" t="n">
+        <v>0.9542256000712814</v>
+      </c>
+      <c r="AM16" t="n">
+        <v>0.3671121342508658</v>
+      </c>
+      <c r="AN16" t="n">
+        <v>0.54614104169613</v>
+      </c>
+      <c r="AO16" t="n">
+        <v>0.04235675988127777</v>
+      </c>
+      <c r="AP16" t="n">
+        <v>0.8825989416561552</v>
+      </c>
+      <c r="AQ16" t="n">
+        <v>0.5357366647112239</v>
+      </c>
+      <c r="AR16" t="n">
+        <v>0.6521024943961845</v>
+      </c>
+      <c r="AS16" t="n">
+        <v>0.4533333333333334</v>
+      </c>
+      <c r="AT16" t="n">
+        <v>0.9176774782472779</v>
+      </c>
+      <c r="AU16" t="n">
+        <v>0.7022761781684479</v>
+      </c>
+      <c r="AV16" t="n">
+        <v>0.2655749838510933</v>
+      </c>
+      <c r="AW16" t="n">
+        <v>0.951367300855571</v>
+      </c>
+      <c r="AX16" t="n">
+        <v>0.2490911226871231</v>
+      </c>
+      <c r="AY16" t="n">
+        <v>163.7142166156229</v>
+      </c>
+      <c r="AZ16" t="n">
+        <v>8.280783401242548</v>
+      </c>
+      <c r="BA16" t="n">
+        <v>248.5959779538881</v>
+      </c>
+      <c r="BB16" t="n">
+        <v>149.7614766525915</v>
+      </c>
+      <c r="BC16" t="n">
+        <v>188.5707646676712</v>
+      </c>
+      <c r="BD16" t="n">
+        <v>231.8443672851328</v>
+      </c>
+      <c r="BE16" t="n">
+        <v>0.9809694806573909</v>
+      </c>
+      <c r="BF16" t="n">
+        <v>691.5922650965471</v>
+      </c>
+      <c r="BG16" t="n">
+        <v>527.5121456272326</v>
+      </c>
+      <c r="BH16" t="n">
+        <v>0.4712611453870844</v>
+      </c>
+      <c r="BI16" t="n">
+        <v>0.4661619154971754</v>
+      </c>
+      <c r="BJ16" t="n">
+        <v>737.7105008914111</v>
+      </c>
+      <c r="BK16" t="n">
+        <v>0.9637821780900007</v>
+      </c>
+      <c r="BL16" t="n">
+        <v>697.258860521273</v>
+      </c>
+      <c r="BM16" t="n">
+        <v>529.6688353295287</v>
+      </c>
+      <c r="BN16" t="n">
+        <v>0.4377157042681074</v>
+      </c>
+      <c r="BO16" t="n">
+        <v>0.3668220137585716</v>
+      </c>
+      <c r="BP16" t="n">
+        <v>0.1834110068792858</v>
+      </c>
+      <c r="BQ16" t="n">
+        <v>0.7469683953321788</v>
+      </c>
+      <c r="BR16" t="n">
+        <v>0.5799965296833545</v>
+      </c>
+      <c r="BS16" t="n">
+        <v>0.6475134422389898</v>
+      </c>
+      <c r="BT16" t="n">
+        <v>0.7150303547946251</v>
+      </c>
+      <c r="BU16" t="n">
+        <v>0.5480089019795173</v>
+      </c>
+      <c r="BV16" t="n">
+        <v>0.09281756276881292</v>
+      </c>
+      <c r="BW16" t="n">
+        <v>0.01886251272293382</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
returned to old type of calculation best parameters
</commit_message>
<xml_diff>
--- a/расчет_ступеней.xlsx
+++ b/расчет_ступеней.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BW16"/>
+  <dimension ref="A1:BW13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -795,3407 +795,2726 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.55</v>
+        <v>0.45</v>
       </c>
       <c r="B2" t="n">
-        <v>0.5433333333333333</v>
+        <v>0.4375</v>
       </c>
       <c r="C2" t="n">
         <v>0.99</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8749158980578627</v>
+        <v>0.884203297941869</v>
       </c>
       <c r="E2" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="F2" t="n">
-        <v>1.01899260985795</v>
+        <v>1.066429875635743</v>
       </c>
       <c r="G2" t="n">
-        <v>330.3561984983635</v>
+        <v>334.9958456714842</v>
       </c>
       <c r="H2" t="n">
-        <v>0.2595630893762285</v>
+        <v>0.3244400050544849</v>
       </c>
       <c r="I2" t="n">
         <v>288</v>
       </c>
       <c r="J2" t="n">
-        <v>100435.150625479</v>
+        <v>100674.7651178944</v>
       </c>
       <c r="K2" t="n">
-        <v>28327.47431431331</v>
+        <v>36409.37652649458</v>
       </c>
       <c r="L2" t="n">
-        <v>28044.19957117017</v>
+        <v>36045.28276122964</v>
       </c>
       <c r="M2" t="n">
-        <v>24536.31605312428</v>
+        <v>31871.35789272645</v>
       </c>
       <c r="N2" t="n">
-        <v>27.87693794350912</v>
+        <v>35.83030095549666</v>
       </c>
       <c r="O2" t="n">
-        <v>315.8769379435091</v>
+        <v>323.8303009554967</v>
       </c>
       <c r="P2" t="n">
-        <v>315.8769379435091</v>
+        <v>323.8303009554967</v>
       </c>
       <c r="Q2" t="n">
-        <v>1.329125860037873</v>
+        <v>1.440908707022073</v>
       </c>
       <c r="R2" t="n">
-        <v>133490.955953123</v>
+        <v>145063.1456357761</v>
       </c>
       <c r="S2" t="n">
-        <v>133490.955953123</v>
+        <v>145063.1456357761</v>
       </c>
       <c r="T2" t="n">
         <v>310.7513475433373</v>
       </c>
       <c r="U2" t="n">
-        <v>325.4436007858483</v>
+        <v>329.5152498904687</v>
       </c>
       <c r="V2" t="n">
-        <v>0.7905694150420949</v>
+        <v>0.7615773105863909</v>
       </c>
       <c r="W2" t="n">
-        <v>0.2311225957333003</v>
+        <v>0.1677833565897216</v>
       </c>
       <c r="X2" t="n">
-        <v>1.163669370778668</v>
+        <v>1.064577496794081</v>
       </c>
       <c r="Y2" t="n">
-        <v>181.6959091741</v>
+        <v>150.7481305521679</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.6367447812769583</v>
+        <v>0.5546733681375342</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.8432463363915963</v>
+        <v>0.7670768900816778</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.3171396294850015</v>
+        <v>0.3651710357190851</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.5433333333333333</v>
+        <v>0.4375</v>
       </c>
       <c r="AD2" t="n">
-        <v>179.4935345174442</v>
+        <v>146.5606824812743</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.6006290571014145</v>
+        <v>0.5085578472919455</v>
       </c>
       <c r="AF2" t="n">
-        <v>0.8113975363946587</v>
+        <v>0.7185450194326043</v>
       </c>
       <c r="AG2" t="n">
-        <v>0.2596975787927992</v>
+        <v>0.2868846230922911</v>
       </c>
       <c r="AH2" t="n">
-        <v>0.4594760190053363</v>
+        <v>0.4226367409601864</v>
       </c>
       <c r="AI2" t="n">
-        <v>0.6262928638025335</v>
+        <v>0.5681001461244793</v>
       </c>
       <c r="AJ2" t="n">
-        <v>0.8343388853607324</v>
+        <v>0.8132458964011607</v>
       </c>
       <c r="AK2" t="n">
-        <v>0.258758555424513</v>
+        <v>0.2029970421339847</v>
       </c>
       <c r="AL2" t="n">
-        <v>1.128380965431894</v>
+        <v>1.128936317318384</v>
       </c>
       <c r="AM2" t="n">
-        <v>0.6108874765005141</v>
+        <v>0.4903225573137425</v>
       </c>
       <c r="AN2" t="n">
-        <v>0.8201830387177463</v>
+        <v>0.7002124444906179</v>
       </c>
       <c r="AO2" t="n">
-        <v>0.2569157928083544</v>
+        <v>0.2943956776214189</v>
       </c>
       <c r="AP2" t="n">
-        <v>0.8124541502014136</v>
+        <v>0.7874116034937758</v>
       </c>
       <c r="AQ2" t="n">
-        <v>0.5443772360304509</v>
+        <v>0.5743120885198095</v>
       </c>
       <c r="AR2" t="n">
-        <v>0.7768834776589806</v>
+        <v>0.6484989891376707</v>
       </c>
       <c r="AS2" t="n">
-        <v>0.5466666666666666</v>
+        <v>0.44375</v>
       </c>
       <c r="AT2" t="n">
-        <v>1.114870585168517</v>
+        <v>1.123094102388967</v>
       </c>
       <c r="AU2" t="n">
-        <v>0.7874965457542674</v>
+        <v>0.657848686446533</v>
       </c>
       <c r="AV2" t="n">
-        <v>0.3379871075095369</v>
+        <v>0.474595113251296</v>
       </c>
       <c r="AW2" t="n">
-        <v>1.126334514505067</v>
+        <v>1.136366747647551</v>
       </c>
       <c r="AX2" t="n">
-        <v>0.3388379687507993</v>
+        <v>0.4785180612010175</v>
       </c>
       <c r="AY2" t="n">
-        <v>197.086657963137</v>
+        <v>160.8856583832313</v>
       </c>
       <c r="AZ2" t="n">
-        <v>1.252350556323866</v>
+        <v>1.407189122308089</v>
       </c>
       <c r="BA2" t="n">
-        <v>259.1729636003568</v>
+        <v>249.586801734187</v>
       </c>
       <c r="BB2" t="n">
-        <v>180.5947218457721</v>
+        <v>148.6544065167211</v>
       </c>
       <c r="BC2" t="n">
-        <v>201.1404516790544</v>
+        <v>164.9069462237893</v>
       </c>
       <c r="BD2" t="n">
-        <v>254.865261663562</v>
+        <v>243.1313991612655</v>
       </c>
       <c r="BE2" t="n">
-        <v>0.9324260139194265</v>
+        <v>0.9487229091131606</v>
       </c>
       <c r="BF2" t="n">
-        <v>268.5386920087948</v>
+        <v>273.2321978245902</v>
       </c>
       <c r="BG2" t="n">
-        <v>328.7084241644237</v>
+        <v>331.5685556814791</v>
       </c>
       <c r="BH2" t="n">
-        <v>0.7884585381685123</v>
+        <v>0.7527456915243563</v>
       </c>
       <c r="BI2" t="n">
-        <v>0.7831318884382398</v>
+        <v>0.7378456664511966</v>
       </c>
       <c r="BJ2" t="n">
-        <v>315.8769379435091</v>
+        <v>323.8303009554967</v>
       </c>
       <c r="BK2" t="n">
-        <v>0.8977840742185261</v>
+        <v>0.9092639620831983</v>
       </c>
       <c r="BL2" t="n">
-        <v>649.5118034080301</v>
+        <v>657.8170550648892</v>
       </c>
       <c r="BM2" t="n">
-        <v>511.2118633397067</v>
+        <v>514.4698924873144</v>
       </c>
       <c r="BN2" t="n">
-        <v>0.4985511486344378</v>
+        <v>0.4725862537568427</v>
       </c>
       <c r="BO2" t="n">
-        <v>0.3668220137585716</v>
+        <v>0.2975790404866964</v>
       </c>
       <c r="BP2" t="n">
-        <v>0.1834110068792858</v>
+        <v>0.2231842803650222</v>
       </c>
       <c r="BQ2" t="n">
-        <v>0.5658299146908039</v>
+        <v>0.4899327164348984</v>
       </c>
       <c r="BR2" t="n">
-        <v>0.5799965296833545</v>
+        <v>0.5665736133518423</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.5960521349267831</v>
+        <v>0.585792973589422</v>
       </c>
       <c r="BT2" t="n">
-        <v>0.6121077401702117</v>
+        <v>0.6050123338270017</v>
       </c>
       <c r="BU2" t="n">
-        <v>0.4151177375034429</v>
+        <v>0.3644842691493443</v>
       </c>
       <c r="BV2" t="n">
-        <v>0.1592631450068501</v>
+        <v>0.1897316660336983</v>
       </c>
       <c r="BW2" t="n">
-        <v>0.1370840042559034</v>
+        <v>0.1606554301282772</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.5433333333333333</v>
+        <v>0.4375</v>
       </c>
       <c r="B3" t="n">
-        <v>0.5366666666666667</v>
+        <v>0.425</v>
       </c>
       <c r="C3" t="n">
         <v>0.98</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8771926580212601</v>
+        <v>0.8813910730500205</v>
       </c>
       <c r="E3" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="F3" t="n">
-        <v>1.01899260985795</v>
+        <v>1.066429875635743</v>
       </c>
       <c r="G3" t="n">
-        <v>330.3561984983635</v>
+        <v>334.9958456714842</v>
       </c>
       <c r="H3" t="n">
-        <v>0.2643367262041065</v>
+        <v>0.3311958650192543</v>
       </c>
       <c r="I3" t="n">
-        <v>315.8769379435091</v>
+        <v>323.8303009554967</v>
       </c>
       <c r="J3" t="n">
-        <v>133490.955953123</v>
+        <v>145063.1456357761</v>
       </c>
       <c r="K3" t="n">
-        <v>28848.44620963379</v>
+        <v>37167.53410689608</v>
       </c>
       <c r="L3" t="n">
-        <v>28271.47728544112</v>
+        <v>36424.18342475816</v>
       </c>
       <c r="M3" t="n">
-        <v>24799.53230620377</v>
+        <v>32103.95011371837</v>
       </c>
       <c r="N3" t="n">
-        <v>28.10286012469296</v>
+        <v>36.20694177411348</v>
       </c>
       <c r="O3" t="n">
-        <v>343.9797980682021</v>
+        <v>360.0372427296102</v>
       </c>
       <c r="P3" t="n">
-        <v>343.9797980682021</v>
+        <v>360.0372427296102</v>
       </c>
       <c r="Q3" t="n">
-        <v>1.300842391209521</v>
+        <v>1.389521025919508</v>
       </c>
       <c r="R3" t="n">
-        <v>173650.6943469054</v>
+        <v>201568.2909469347</v>
       </c>
       <c r="S3" t="n">
-        <v>173650.6943469054</v>
+        <v>201568.2909469347</v>
       </c>
       <c r="T3" t="n">
-        <v>325.4436007858483</v>
+        <v>329.5152498904687</v>
       </c>
       <c r="U3" t="n">
-        <v>339.6121704124694</v>
+        <v>347.448539336746</v>
       </c>
       <c r="V3" t="n">
-        <v>0.7905694150420949</v>
+        <v>0.7615773105863909</v>
       </c>
       <c r="W3" t="n">
-        <v>0.2281034827135892</v>
+        <v>0.1633479172253532</v>
       </c>
       <c r="X3" t="n">
-        <v>1.163669370778668</v>
+        <v>1.064577496794081</v>
       </c>
       <c r="Y3" t="n">
-        <v>179.4935345174442</v>
+        <v>146.5606824812743</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.6006290571014145</v>
+        <v>0.5085578472919455</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.8113975363946587</v>
+        <v>0.7185450194326043</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.2596975787927993</v>
+        <v>0.2868846230922911</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.5366666666666667</v>
+        <v>0.425</v>
       </c>
       <c r="AD3" t="n">
-        <v>177.2911598607885</v>
+        <v>142.3732344103808</v>
       </c>
       <c r="AE3" t="n">
-        <v>0.5685086818351996</v>
+        <v>0.468528766832469</v>
       </c>
       <c r="AF3" t="n">
-        <v>0.7808554921734913</v>
+        <v>0.6733194447626319</v>
       </c>
       <c r="AG3" t="n">
-        <v>0.2164779885688478</v>
+        <v>0.2323217907867172</v>
       </c>
       <c r="AH3" t="n">
-        <v>0.5183324998489354</v>
+        <v>0.506480008400635</v>
       </c>
       <c r="AI3" t="n">
-        <v>0.7065177121432007</v>
+        <v>0.6808006472126222</v>
       </c>
       <c r="AJ3" t="n">
-        <v>0.8657849841537051</v>
+        <v>0.8554208090890487</v>
       </c>
       <c r="AK3" t="n">
-        <v>0.2775059382011241</v>
+        <v>0.2304275261048039</v>
       </c>
       <c r="AL3" t="n">
-        <v>1.096833439915491</v>
+        <v>1.073179621665038</v>
       </c>
       <c r="AM3" t="n">
-        <v>0.5877030380378492</v>
+        <v>0.4661209080755683</v>
       </c>
       <c r="AN3" t="n">
-        <v>0.7984193669688989</v>
+        <v>0.6707463493850978</v>
       </c>
       <c r="AO3" t="n">
-        <v>0.2117158391966206</v>
+        <v>0.233213016100909</v>
       </c>
       <c r="AP3" t="n">
-        <v>0.8281771995978999</v>
+        <v>0.8084990598377197</v>
       </c>
       <c r="AQ3" t="n">
-        <v>0.5369241791707747</v>
+        <v>0.5635107758827498</v>
       </c>
       <c r="AR3" t="n">
-        <v>0.7680978352575358</v>
+        <v>0.6314414656442968</v>
       </c>
       <c r="AS3" t="n">
-        <v>0.54</v>
+        <v>0.43125</v>
       </c>
       <c r="AT3" t="n">
-        <v>1.076160684397948</v>
+        <v>1.054171527737041</v>
       </c>
       <c r="AU3" t="n">
-        <v>0.7882542720494674</v>
+        <v>0.6532160462166496</v>
       </c>
       <c r="AV3" t="n">
-        <v>0.308062849140412</v>
+        <v>0.4227300620927443</v>
       </c>
       <c r="AW3" t="n">
-        <v>1.093568951179471</v>
+        <v>1.07397490693721</v>
       </c>
       <c r="AX3" t="n">
-        <v>0.3053146791300039</v>
+        <v>0.4207588607205606</v>
       </c>
       <c r="AY3" t="n">
-        <v>194.669887641445</v>
+        <v>156.4429853478237</v>
       </c>
       <c r="AZ3" t="n">
-        <v>1.51455275775179</v>
+        <v>1.776406807110386</v>
       </c>
       <c r="BA3" t="n">
-        <v>258.3501719836211</v>
+        <v>248.2779526487107</v>
       </c>
       <c r="BB3" t="n">
-        <v>178.3923471891163</v>
+        <v>144.4669584458276</v>
       </c>
       <c r="BC3" t="n">
-        <v>202.6859317515446</v>
+        <v>166.1511251787695</v>
       </c>
       <c r="BD3" t="n">
-        <v>251.5674000292789</v>
+        <v>237.7104076639635</v>
       </c>
       <c r="BE3" t="n">
-        <v>0.9398741226275776</v>
+        <v>0.9568948193262971</v>
       </c>
       <c r="BF3" t="n">
-        <v>296.8845599079414</v>
+        <v>309.8715373251904</v>
       </c>
       <c r="BG3" t="n">
-        <v>345.6218620466004</v>
+        <v>353.1004272981889</v>
       </c>
       <c r="BH3" t="n">
-        <v>0.7474937217622756</v>
+        <v>0.7031369362774604</v>
       </c>
       <c r="BI3" t="n">
-        <v>0.7407490718714309</v>
+        <v>0.6841600431469231</v>
       </c>
       <c r="BJ3" t="n">
-        <v>343.9797980682021</v>
+        <v>360.0372427296102</v>
       </c>
       <c r="BK3" t="n">
-        <v>0.9085484687536023</v>
+        <v>0.9219875058935334</v>
       </c>
       <c r="BL3" t="n">
-        <v>657.2994235138542</v>
+        <v>667.02204335028</v>
       </c>
       <c r="BM3" t="n">
-        <v>514.2674363062806</v>
+        <v>518.0569364099072</v>
       </c>
       <c r="BN3" t="n">
-        <v>0.4891762189652889</v>
+        <v>0.4588499660119938</v>
       </c>
       <c r="BO3" t="n">
-        <v>0.3668220137585716</v>
+        <v>0.2975790404866964</v>
       </c>
       <c r="BP3" t="n">
-        <v>0.1834110068792858</v>
+        <v>0.2231842803650222</v>
       </c>
       <c r="BQ3" t="n">
-        <v>0.6097171047851944</v>
+        <v>0.5543838557506463</v>
       </c>
       <c r="BR3" t="n">
-        <v>0.5799965296833545</v>
+        <v>0.5665736133518423</v>
       </c>
       <c r="BS3" t="n">
-        <v>0.6075872562108723</v>
+        <v>0.6014809361522618</v>
       </c>
       <c r="BT3" t="n">
-        <v>0.6351779827383902</v>
+        <v>0.6363882589526815</v>
       </c>
       <c r="BU3" t="n">
-        <v>0.447315312400702</v>
+        <v>0.412432539638981</v>
       </c>
       <c r="BV3" t="n">
-        <v>0.1431643575582206</v>
+        <v>0.1657575307888799</v>
       </c>
       <c r="BW3" t="n">
-        <v>0.1076557638341039</v>
+        <v>0.1187337964080529</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.5366666666666667</v>
+        <v>0.425</v>
       </c>
       <c r="B4" t="n">
-        <v>0.53</v>
+        <v>0.4125</v>
       </c>
       <c r="C4" t="n">
         <v>0.97</v>
       </c>
       <c r="D4" t="n">
-        <v>0.8792475775053105</v>
+        <v>0.8776400396808992</v>
       </c>
       <c r="E4" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="F4" t="n">
-        <v>1.01899260985795</v>
+        <v>1.066429875635743</v>
       </c>
       <c r="G4" t="n">
-        <v>330.3561984983635</v>
+        <v>334.9958456714842</v>
       </c>
       <c r="H4" t="n">
-        <v>0.2690626901699927</v>
+        <v>0.3375197589886442</v>
       </c>
       <c r="I4" t="n">
-        <v>343.9797980682021</v>
+        <v>360.0372427296102</v>
       </c>
       <c r="J4" t="n">
-        <v>173650.6943469054</v>
+        <v>201568.2909469347</v>
       </c>
       <c r="K4" t="n">
-        <v>29364.21531677354</v>
+        <v>37877.21550579287</v>
       </c>
       <c r="L4" t="n">
-        <v>28483.28885727033</v>
+        <v>36740.89904061908</v>
       </c>
       <c r="M4" t="n">
-        <v>25043.86272713894</v>
+        <v>32245.28409192084</v>
       </c>
       <c r="N4" t="n">
-        <v>28.31340840682935</v>
+        <v>36.52176843003885</v>
       </c>
       <c r="O4" t="n">
-        <v>372.2932064750314</v>
+        <v>396.559011159649</v>
       </c>
       <c r="P4" t="n">
-        <v>372.2932064750314</v>
+        <v>396.559011159649</v>
       </c>
       <c r="Q4" t="n">
-        <v>1.277053490892431</v>
+        <v>1.347829621392633</v>
       </c>
       <c r="R4" t="n">
-        <v>221761.22541161</v>
+        <v>271679.7132717671</v>
       </c>
       <c r="S4" t="n">
-        <v>221761.22541161</v>
+        <v>271679.7132717671</v>
       </c>
       <c r="T4" t="n">
-        <v>339.6121704124694</v>
+        <v>347.448539336746</v>
       </c>
       <c r="U4" t="n">
-        <v>353.3127681404651</v>
+        <v>364.6453570825088</v>
       </c>
       <c r="V4" t="n">
-        <v>0.7905694150420949</v>
+        <v>0.7615773105863909</v>
       </c>
       <c r="W4" t="n">
-        <v>0.2251145206591726</v>
+        <v>0.1591960774308347</v>
       </c>
       <c r="X4" t="n">
-        <v>1.163669370778668</v>
+        <v>1.064577496794081</v>
       </c>
       <c r="Y4" t="n">
-        <v>177.2911598607885</v>
+        <v>142.3732344103808</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.5685086818351996</v>
+        <v>0.468528766832469</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.7808554921734913</v>
+        <v>0.6733194447626319</v>
       </c>
       <c r="AB4" t="n">
-        <v>0.2164779885688478</v>
+        <v>0.2323217907867172</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.53</v>
+        <v>0.4125</v>
       </c>
       <c r="AD4" t="n">
-        <v>175.0887852041327</v>
+        <v>138.1857863394872</v>
       </c>
       <c r="AE4" t="n">
-        <v>0.5396749531487905</v>
+        <v>0.4333023913326854</v>
       </c>
       <c r="AF4" t="n">
-        <v>0.7517267294576299</v>
+        <v>0.6312866578179296</v>
       </c>
       <c r="AG4" t="n">
-        <v>0.1831856369214446</v>
+        <v>0.1929432963141447</v>
       </c>
       <c r="AH4" t="n">
-        <v>0.5589225687416454</v>
+        <v>0.558190666335634</v>
       </c>
       <c r="AI4" t="n">
-        <v>0.7618443656294672</v>
+        <v>0.750309115081092</v>
       </c>
       <c r="AJ4" t="n">
-        <v>0.8889338663369074</v>
+        <v>0.8840146401994062</v>
       </c>
       <c r="AK4" t="n">
-        <v>0.2904999969061935</v>
+        <v>0.2478040511669324</v>
       </c>
       <c r="AL4" t="n">
-        <v>1.073200018697416</v>
+        <v>1.032320478025595</v>
       </c>
       <c r="AM4" t="n">
-        <v>0.5651219377667424</v>
+        <v>0.4420825865074373</v>
       </c>
       <c r="AN4" t="n">
-        <v>0.7763585765325808</v>
+        <v>0.6411568471991366</v>
       </c>
       <c r="AO4" t="n">
-        <v>0.1773736310631089</v>
+        <v>0.1899730607426552</v>
       </c>
       <c r="AP4" t="n">
-        <v>0.8397516406895011</v>
+        <v>0.8227959753928986</v>
       </c>
       <c r="AQ4" t="n">
-        <v>0.5323375667571771</v>
+        <v>0.5575621335231457</v>
       </c>
       <c r="AR4" t="n">
-        <v>0.7592833643790334</v>
+        <v>0.614429921562137</v>
       </c>
       <c r="AS4" t="n">
-        <v>0.5333333333333334</v>
+        <v>0.41875</v>
       </c>
       <c r="AT4" t="n">
-        <v>1.047909504026529</v>
+        <v>1.006183457466621</v>
       </c>
       <c r="AU4" t="n">
-        <v>0.7863325665854001</v>
+        <v>0.6441646969371893</v>
       </c>
       <c r="AV4" t="n">
-        <v>0.2886261396474953</v>
+        <v>0.3917535359044838</v>
       </c>
       <c r="AW4" t="n">
-        <v>1.069402867446432</v>
+        <v>1.029835022076156</v>
       </c>
       <c r="AX4" t="n">
-        <v>0.2830703008610317</v>
+        <v>0.3856703251389664</v>
       </c>
       <c r="AY4" t="n">
-        <v>192.2569931323033</v>
+        <v>152.0336456146226</v>
       </c>
       <c r="AZ4" t="n">
-        <v>1.807707852097115</v>
+        <v>2.19436222248338</v>
       </c>
       <c r="BA4" t="n">
-        <v>257.5402235089658</v>
+        <v>246.9644608130197</v>
       </c>
       <c r="BB4" t="n">
-        <v>176.1899725324606</v>
+        <v>140.279510374934</v>
       </c>
       <c r="BC4" t="n">
-        <v>203.3631160598059</v>
+        <v>166.0513797701721</v>
       </c>
       <c r="BD4" t="n">
-        <v>248.9377491918774</v>
+        <v>233.5925564032956</v>
       </c>
       <c r="BE4" t="n">
-        <v>0.9461329797796673</v>
+        <v>0.9634134657750744</v>
       </c>
       <c r="BF4" t="n">
-        <v>325.4506313302762</v>
+        <v>346.8647278262354</v>
       </c>
       <c r="BG4" t="n">
-        <v>361.8678156759038</v>
+        <v>373.5833131821657</v>
       </c>
       <c r="BH4" t="n">
-        <v>0.7116969577079606</v>
+        <v>0.6610693039509383</v>
       </c>
       <c r="BI4" t="n">
-        <v>0.7045818086396137</v>
+        <v>0.6406020311687126</v>
       </c>
       <c r="BJ4" t="n">
-        <v>372.2932064750314</v>
+        <v>396.559011159649</v>
       </c>
       <c r="BK4" t="n">
-        <v>0.9172607458223552</v>
+        <v>0.93160483961042</v>
       </c>
       <c r="BL4" t="n">
-        <v>663.6024165755675</v>
+        <v>673.9798096393168</v>
       </c>
       <c r="BM4" t="n">
-        <v>516.7272668761979</v>
+        <v>520.7518758549752</v>
       </c>
       <c r="BN4" t="n">
-        <v>0.4817584926315107</v>
+        <v>0.4485678635718426</v>
       </c>
       <c r="BO4" t="n">
-        <v>0.3668220137585716</v>
+        <v>0.2975790404866964</v>
       </c>
       <c r="BP4" t="n">
-        <v>0.1834110068792858</v>
+        <v>0.2231842803650222</v>
       </c>
       <c r="BQ4" t="n">
-        <v>0.6405978739282687</v>
+        <v>0.5949675909202978</v>
       </c>
       <c r="BR4" t="n">
-        <v>0.5799965296833545</v>
+        <v>0.5665736133518423</v>
       </c>
       <c r="BS4" t="n">
-        <v>0.6160787757895745</v>
+        <v>0.6121170921843355</v>
       </c>
       <c r="BT4" t="n">
-        <v>0.6521610218957946</v>
+        <v>0.6576605710168285</v>
       </c>
       <c r="BU4" t="n">
-        <v>0.4699708042476542</v>
+        <v>0.4426247120668587</v>
       </c>
       <c r="BV4" t="n">
-        <v>0.1318366116347445</v>
+        <v>0.1506614445749411</v>
       </c>
       <c r="BW4" t="n">
-        <v>0.08736072938774891</v>
+        <v>0.09287846744055345</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.53</v>
+        <v>0.4125</v>
       </c>
       <c r="B5" t="n">
-        <v>0.5233333333333333</v>
+        <v>0.4</v>
       </c>
       <c r="C5" t="n">
         <v>0.96</v>
       </c>
       <c r="D5" t="n">
-        <v>0.8810742363872112</v>
+        <v>0.8729343479869782</v>
       </c>
       <c r="E5" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="F5" t="n">
-        <v>1.01899260985795</v>
+        <v>1.066429875635743</v>
       </c>
       <c r="G5" t="n">
-        <v>330.3561984983635</v>
+        <v>334.9958456714842</v>
       </c>
       <c r="H5" t="n">
-        <v>0.2737328478793182</v>
+        <v>0.3433570658223036</v>
       </c>
       <c r="I5" t="n">
-        <v>372.2932064750314</v>
+        <v>396.559011159649</v>
       </c>
       <c r="J5" t="n">
-        <v>221761.22541161</v>
+        <v>271679.7132717671</v>
       </c>
       <c r="K5" t="n">
-        <v>29873.89399594412</v>
+        <v>38532.29101774057</v>
       </c>
       <c r="L5" t="n">
-        <v>28678.93823610635</v>
+        <v>36990.99937703094</v>
       </c>
       <c r="M5" t="n">
-        <v>25268.2736067734</v>
+        <v>32290.71392257523</v>
       </c>
       <c r="N5" t="n">
-        <v>28.50789089076178</v>
+        <v>36.77037711434487</v>
       </c>
       <c r="O5" t="n">
-        <v>400.8010973657932</v>
+        <v>433.3293882739939</v>
       </c>
       <c r="P5" t="n">
-        <v>400.8010973657932</v>
+        <v>433.3293882739939</v>
       </c>
       <c r="Q5" t="n">
-        <v>1.256726699210606</v>
+        <v>1.313130303218921</v>
       </c>
       <c r="R5" t="n">
-        <v>278693.2528244318</v>
+        <v>356750.8642669851</v>
       </c>
       <c r="S5" t="n">
-        <v>278693.2528244318</v>
+        <v>356750.8642669851</v>
       </c>
       <c r="T5" t="n">
-        <v>353.3127681404651</v>
+        <v>364.6453570825088</v>
       </c>
       <c r="U5" t="n">
-        <v>366.5905180808015</v>
+        <v>381.1762635425639</v>
       </c>
       <c r="V5" t="n">
-        <v>0.7905694150420949</v>
+        <v>0.7615773105863909</v>
       </c>
       <c r="W5" t="n">
-        <v>0.22216085358044</v>
+        <v>0.1553636977416573</v>
       </c>
       <c r="X5" t="n">
-        <v>1.163669370778668</v>
+        <v>1.064577496794081</v>
       </c>
       <c r="Y5" t="n">
-        <v>175.0887852041327</v>
+        <v>138.1857863394872</v>
       </c>
       <c r="Z5" t="n">
-        <v>0.5396749531487905</v>
+        <v>0.4333023913326854</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.7517267294576299</v>
+        <v>0.6312866578179296</v>
       </c>
       <c r="AB5" t="n">
-        <v>0.1831856369214445</v>
+        <v>0.1929432963141447</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.5233333333333333</v>
+        <v>0.4</v>
       </c>
       <c r="AD5" t="n">
-        <v>172.8864105474769</v>
+        <v>133.9983382685937</v>
       </c>
       <c r="AE5" t="n">
-        <v>0.5135856672874103</v>
+        <v>0.4019499360408819</v>
       </c>
       <c r="AF5" t="n">
-        <v>0.7240261143390112</v>
+        <v>0.5922271443277999</v>
       </c>
       <c r="AG5" t="n">
-        <v>0.1570284104663461</v>
+        <v>0.1637251255561614</v>
       </c>
       <c r="AH5" t="n">
-        <v>0.5885102091982426</v>
+        <v>0.5931253835185788</v>
       </c>
       <c r="AI5" t="n">
-        <v>0.8021740614312992</v>
+        <v>0.7972676873324286</v>
       </c>
       <c r="AJ5" t="n">
-        <v>0.9064996483267894</v>
+        <v>0.9043328384130478</v>
       </c>
       <c r="AK5" t="n">
-        <v>0.2997257989200545</v>
+        <v>0.2594013382727521</v>
       </c>
       <c r="AL5" t="n">
-        <v>1.054667013070643</v>
+        <v>0.9997621798616013</v>
       </c>
       <c r="AM5" t="n">
-        <v>0.5434765911200543</v>
+        <v>0.4189892047782126</v>
       </c>
       <c r="AN5" t="n">
-        <v>0.754382910729652</v>
+        <v>0.6121999974112641</v>
       </c>
       <c r="AO5" t="n">
-        <v>0.1507094981258448</v>
+        <v>0.1583836392892018</v>
       </c>
       <c r="AP5" t="n">
-        <v>0.8485345316844422</v>
+        <v>0.8329550744997194</v>
       </c>
       <c r="AQ5" t="n">
-        <v>0.5295794185860807</v>
+        <v>0.5542658266274929</v>
       </c>
       <c r="AR5" t="n">
-        <v>0.7504449411331544</v>
+        <v>0.5974865025033296</v>
       </c>
       <c r="AS5" t="n">
-        <v>0.5266666666666666</v>
+        <v>0.40625</v>
       </c>
       <c r="AT5" t="n">
-        <v>1.026261321111047</v>
+        <v>0.9695253360656676</v>
       </c>
       <c r="AU5" t="n">
-        <v>0.7826405252138178</v>
+        <v>0.6325005241171194</v>
       </c>
       <c r="AV5" t="n">
-        <v>0.2758163799778928</v>
+        <v>0.372038833562338</v>
       </c>
       <c r="AW5" t="n">
-        <v>1.050673859882218</v>
+        <v>0.9954739554152893</v>
       </c>
       <c r="AX5" t="n">
-        <v>0.2680333346683998</v>
+        <v>0.3629734312981698</v>
       </c>
       <c r="AY5" t="n">
-        <v>189.8486237330193</v>
+        <v>147.6621745217523</v>
       </c>
       <c r="AZ5" t="n">
-        <v>2.132563514482126</v>
+        <v>2.659616017028643</v>
       </c>
       <c r="BA5" t="n">
-        <v>256.7418819150192</v>
+        <v>245.6347060214273</v>
       </c>
       <c r="BB5" t="n">
-        <v>173.9875978758048</v>
+        <v>136.0920623040405</v>
       </c>
       <c r="BC5" t="n">
-        <v>203.4066565885848</v>
+        <v>165.0366338893982</v>
       </c>
       <c r="BD5" t="n">
-        <v>246.7369691893362</v>
+        <v>230.2105659161242</v>
       </c>
       <c r="BE5" t="n">
-        <v>0.9514584908239752</v>
+        <v>0.9687081729442294</v>
       </c>
       <c r="BF5" t="n">
-        <v>354.221532376752</v>
+        <v>384.1499551650339</v>
       </c>
       <c r="BG5" t="n">
-        <v>377.5242717589293</v>
+        <v>393.1495592776405</v>
       </c>
       <c r="BH5" t="n">
-        <v>0.6800672198341821</v>
+        <v>0.6247869296171872</v>
       </c>
       <c r="BI5" t="n">
-        <v>0.6730587863566948</v>
+        <v>0.603947800360391</v>
       </c>
       <c r="BJ5" t="n">
-        <v>400.8010973657932</v>
+        <v>433.3293882739939</v>
       </c>
       <c r="BK5" t="n">
-        <v>0.9244986450180088</v>
+        <v>0.9392078424066409</v>
       </c>
       <c r="BL5" t="n">
-        <v>668.8387546823074</v>
+        <v>679.4802859780046</v>
       </c>
       <c r="BM5" t="n">
-        <v>518.761950545694</v>
+        <v>522.8725350083995</v>
       </c>
       <c r="BN5" t="n">
-        <v>0.4756265738645435</v>
+        <v>0.4402804708654778</v>
       </c>
       <c r="BO5" t="n">
-        <v>0.3668220137585716</v>
+        <v>0.2975790404866964</v>
       </c>
       <c r="BP5" t="n">
-        <v>0.1834110068792858</v>
+        <v>0.2231842803650222</v>
       </c>
       <c r="BQ5" t="n">
-        <v>0.663341317062243</v>
+        <v>0.6225980342642162</v>
       </c>
       <c r="BR5" t="n">
-        <v>0.5799965296833545</v>
+        <v>0.5665736133518423</v>
       </c>
       <c r="BS5" t="n">
-        <v>0.622522291312347</v>
+        <v>0.619674929595378</v>
       </c>
       <c r="BT5" t="n">
-        <v>0.6650480529413397</v>
+        <v>0.6727762458389134</v>
       </c>
       <c r="BU5" t="n">
-        <v>0.4866563954680702</v>
+        <v>0.4631803141131219</v>
       </c>
       <c r="BV5" t="n">
-        <v>0.1234938160245365</v>
+        <v>0.1403836435518095</v>
       </c>
       <c r="BW5" t="n">
-        <v>0.0725669091594503</v>
+        <v>0.07541110884908103</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.5233333333333333</v>
+        <v>0.4</v>
       </c>
       <c r="B6" t="n">
-        <v>0.5166666666666667</v>
+        <v>0.3875</v>
       </c>
       <c r="C6" t="n">
         <v>0.95</v>
       </c>
       <c r="D6" t="n">
-        <v>0.8826676089429577</v>
+        <v>0.8672584703581266</v>
       </c>
       <c r="E6" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="F6" t="n">
-        <v>1.01899260985795</v>
+        <v>1.066429875635743</v>
       </c>
       <c r="G6" t="n">
-        <v>330.3561984983635</v>
+        <v>334.9958456714842</v>
       </c>
       <c r="H6" t="n">
-        <v>0.2783389497856022</v>
+        <v>0.3486475855755174</v>
       </c>
       <c r="I6" t="n">
-        <v>400.8010973657932</v>
+        <v>433.3293882739939</v>
       </c>
       <c r="J6" t="n">
-        <v>278693.2528244318</v>
+        <v>356750.8642669851</v>
       </c>
       <c r="K6" t="n">
-        <v>30376.58193109288</v>
+        <v>39126.00487150306</v>
       </c>
       <c r="L6" t="n">
-        <v>28857.75283453823</v>
+        <v>37169.7046279279</v>
       </c>
       <c r="M6" t="n">
-        <v>25471.80369392872</v>
+        <v>32235.74117928013</v>
       </c>
       <c r="N6" t="n">
-        <v>28.68563900053502</v>
+        <v>36.94801652875537</v>
       </c>
       <c r="O6" t="n">
-        <v>429.4867363663282</v>
+        <v>470.2774048027492</v>
       </c>
       <c r="P6" t="n">
-        <v>429.4867363663282</v>
+        <v>470.2774048027492</v>
       </c>
       <c r="Q6" t="n">
-        <v>1.239121976574034</v>
+        <v>1.28363103095909</v>
       </c>
       <c r="R6" t="n">
-        <v>345334.934297657</v>
+        <v>457936.4796945766</v>
       </c>
       <c r="S6" t="n">
-        <v>345334.934297657</v>
+        <v>457936.4796945766</v>
       </c>
       <c r="T6" t="n">
-        <v>366.5905180808015</v>
+        <v>381.1762635425639</v>
       </c>
       <c r="U6" t="n">
-        <v>379.4824142218317</v>
+        <v>397.0944646181332</v>
       </c>
       <c r="V6" t="n">
-        <v>0.7905694150420949</v>
+        <v>0.7615773105863909</v>
       </c>
       <c r="W6" t="n">
-        <v>0.2192476989486998</v>
+        <v>0.1518903013578152</v>
       </c>
       <c r="X6" t="n">
-        <v>1.163669370778668</v>
+        <v>1.064577496794081</v>
       </c>
       <c r="Y6" t="n">
-        <v>172.8864105474769</v>
+        <v>133.9983382685937</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.5135856672874103</v>
+        <v>0.4019499360408819</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.7240261143390112</v>
+        <v>0.5922271443277999</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.1570284104663461</v>
+        <v>0.1637251255561614</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.5166666666666667</v>
+        <v>0.3875</v>
       </c>
       <c r="AD6" t="n">
-        <v>170.6840358908212</v>
+        <v>129.8108901977001</v>
       </c>
       <c r="AE6" t="n">
-        <v>0.4898177442230555</v>
+        <v>0.3737796859822607</v>
       </c>
       <c r="AF6" t="n">
-        <v>0.697718957219101</v>
+        <v>0.5558891806916422</v>
       </c>
       <c r="AG6" t="n">
-        <v>0.1361282651628454</v>
+        <v>0.1415608615306941</v>
       </c>
       <c r="AH6" t="n">
-        <v>0.6108958189145675</v>
+        <v>0.6180530627448302</v>
       </c>
       <c r="AI6" t="n">
-        <v>0.8326869653420473</v>
+        <v>0.8307749923973037</v>
       </c>
       <c r="AJ6" t="n">
-        <v>0.9201542213809998</v>
+        <v>0.9192896953607008</v>
       </c>
       <c r="AK6" t="n">
-        <v>0.3063566828539088</v>
+        <v>0.2674717268010952</v>
       </c>
       <c r="AL6" t="n">
-        <v>1.039595659752858</v>
+        <v>0.9720262250235825</v>
       </c>
       <c r="AM6" t="n">
-        <v>0.5229057101248068</v>
+        <v>0.3972152038601151</v>
       </c>
       <c r="AN6" t="n">
-        <v>0.7327403564424538</v>
+        <v>0.5843288480641364</v>
       </c>
       <c r="AO6" t="n">
-        <v>0.1296220010026499</v>
+        <v>0.1346710017740956</v>
       </c>
       <c r="AP6" t="n">
-        <v>0.8553618182115473</v>
+        <v>0.8404335029735459</v>
       </c>
       <c r="AQ6" t="n">
-        <v>0.5280449340574782</v>
+        <v>0.5524812982168491</v>
       </c>
       <c r="AR6" t="n">
-        <v>0.7415873974789472</v>
+        <v>0.5806335590240905</v>
       </c>
       <c r="AS6" t="n">
-        <v>0.52</v>
+        <v>0.39375</v>
       </c>
       <c r="AT6" t="n">
-        <v>1.008999437032235</v>
+        <v>0.9393663462540609</v>
       </c>
       <c r="AU6" t="n">
-        <v>0.7777221794859068</v>
+        <v>0.6191945916757878</v>
       </c>
       <c r="AV6" t="n">
-        <v>0.2674120395532883</v>
+        <v>0.3587327872299704</v>
       </c>
       <c r="AW6" t="n">
-        <v>1.035577946863965</v>
+        <v>0.9666442621479878</v>
       </c>
       <c r="AX6" t="n">
-        <v>0.2578557673780582</v>
+        <v>0.3474496704722</v>
       </c>
       <c r="AY6" t="n">
-        <v>187.4454377846733</v>
+        <v>143.3338608703159</v>
       </c>
       <c r="AZ6" t="n">
-        <v>2.489787201375131</v>
+        <v>3.169793873235574</v>
       </c>
       <c r="BA6" t="n">
-        <v>255.9538514603378</v>
+        <v>244.2756650661178</v>
       </c>
       <c r="BB6" t="n">
-        <v>171.7852232191491</v>
+        <v>131.9046142331469</v>
       </c>
       <c r="BC6" t="n">
-        <v>202.9840166499692</v>
+        <v>163.4132722977984</v>
       </c>
       <c r="BD6" t="n">
-        <v>244.8274784943593</v>
+        <v>227.2730542356306</v>
       </c>
       <c r="BE6" t="n">
-        <v>0.9560382937261576</v>
+        <v>0.9730727081527885</v>
       </c>
       <c r="BF6" t="n">
-        <v>383.1811972491644</v>
+        <v>421.6610013699664</v>
       </c>
       <c r="BG6" t="n">
-        <v>392.653519690291</v>
+        <v>411.8974635892041</v>
       </c>
       <c r="BH6" t="n">
-        <v>0.651856760795685</v>
+        <v>0.5930496947894299</v>
       </c>
       <c r="BI6" t="n">
-        <v>0.645161591997362</v>
+        <v>0.572340021043074</v>
       </c>
       <c r="BJ6" t="n">
-        <v>429.4867363663282</v>
+        <v>470.2774048027492</v>
       </c>
       <c r="BK6" t="n">
-        <v>0.9306277533685716</v>
+        <v>0.9454044833854023</v>
       </c>
       <c r="BL6" t="n">
-        <v>673.2729258069427</v>
+        <v>683.9633143283246</v>
       </c>
       <c r="BM6" t="n">
-        <v>520.4787165943305</v>
+        <v>524.5945855164201</v>
       </c>
       <c r="BN6" t="n">
-        <v>0.4703890297308387</v>
+        <v>0.4332356080494025</v>
       </c>
       <c r="BO6" t="n">
-        <v>0.3668220137585716</v>
+        <v>0.2975790404866964</v>
       </c>
       <c r="BP6" t="n">
-        <v>0.1834110068792858</v>
+        <v>0.2231842803650222</v>
       </c>
       <c r="BQ6" t="n">
-        <v>0.680652393008596</v>
+        <v>0.6423837994849889</v>
       </c>
       <c r="BR6" t="n">
-        <v>0.5799965296833545</v>
+        <v>0.5665736133518423</v>
       </c>
       <c r="BS6" t="n">
-        <v>0.6275310892971061</v>
+        <v>0.6252384885193522</v>
       </c>
       <c r="BT6" t="n">
-        <v>0.6750656489108576</v>
+        <v>0.6839033636868619</v>
       </c>
       <c r="BU6" t="n">
-        <v>0.4993565629460078</v>
+        <v>0.4778998866873533</v>
       </c>
       <c r="BV6" t="n">
-        <v>0.1171437322855677</v>
+        <v>0.1330238572646938</v>
       </c>
       <c r="BW6" t="n">
-        <v>0.06137410430128787</v>
+        <v>0.06294726923595534</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.5166666666666667</v>
+        <v>0.3875</v>
       </c>
       <c r="B7" t="n">
-        <v>0.51</v>
+        <v>0.375</v>
       </c>
       <c r="C7" t="n">
         <v>0.9399999999999999</v>
       </c>
       <c r="D7" t="n">
-        <v>0.8840297017740676</v>
+        <v>0.8605972014216101</v>
       </c>
       <c r="E7" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="F7" t="n">
-        <v>1.01899260985795</v>
+        <v>1.066429875635743</v>
       </c>
       <c r="G7" t="n">
-        <v>330.3561984983635</v>
+        <v>334.9958456714842</v>
       </c>
       <c r="H7" t="n">
-        <v>0.2828930011726652</v>
+        <v>0.3533255394992114</v>
       </c>
       <c r="I7" t="n">
-        <v>429.4867363663282</v>
+        <v>470.2774048027492</v>
       </c>
       <c r="J7" t="n">
-        <v>345334.934297657</v>
+        <v>457936.4796945766</v>
       </c>
       <c r="K7" t="n">
-        <v>30873.58932148536</v>
+        <v>39650.97523005291</v>
       </c>
       <c r="L7" t="n">
-        <v>29021.17396219624</v>
+        <v>37271.91671624973</v>
       </c>
       <c r="M7" t="n">
-        <v>25655.57976293367</v>
+        <v>32076.10721762385</v>
       </c>
       <c r="N7" t="n">
-        <v>28.84808544949924</v>
+        <v>37.04961900223631</v>
       </c>
       <c r="O7" t="n">
-        <v>458.3348218158275</v>
+        <v>507.3270238049855</v>
       </c>
       <c r="P7" t="n">
-        <v>458.3348218158275</v>
+        <v>507.3270238049855</v>
       </c>
       <c r="Q7" t="n">
-        <v>1.223714194449077</v>
+        <v>1.258098598953983</v>
       </c>
       <c r="R7" t="n">
-        <v>422591.2609391822</v>
+        <v>576129.2435136657</v>
       </c>
       <c r="S7" t="n">
-        <v>422591.2609391822</v>
+        <v>576129.2435136657</v>
       </c>
       <c r="T7" t="n">
-        <v>379.4824142218317</v>
+        <v>397.0944646181332</v>
       </c>
       <c r="U7" t="n">
-        <v>392.0199813209105</v>
+        <v>412.4399969472064</v>
       </c>
       <c r="V7" t="n">
-        <v>0.7905694150420949</v>
+        <v>0.7615773105863909</v>
       </c>
       <c r="W7" t="n">
-        <v>0.2163674639557862</v>
+        <v>0.1488190741438032</v>
       </c>
       <c r="X7" t="n">
-        <v>1.163669370778668</v>
+        <v>1.064577496794081</v>
       </c>
       <c r="Y7" t="n">
-        <v>170.6840358908212</v>
+        <v>129.8108901977001</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.4898177442230555</v>
+        <v>0.3737796859822607</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.697718957219101</v>
+        <v>0.5558891806916422</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.1361282651628454</v>
+        <v>0.1415608615306941</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.51</v>
+        <v>0.375</v>
       </c>
       <c r="AD7" t="n">
-        <v>168.4816612341654</v>
+        <v>125.6234421268066</v>
       </c>
       <c r="AE7" t="n">
-        <v>0.4680343173960578</v>
+        <v>0.3482637835623633</v>
       </c>
       <c r="AF7" t="n">
-        <v>0.6727435922915034</v>
+        <v>0.5220220244246978</v>
       </c>
       <c r="AG7" t="n">
-        <v>0.1191834119456657</v>
+        <v>0.1244499868451066</v>
       </c>
       <c r="AH7" t="n">
-        <v>0.6283067002390071</v>
+        <v>0.6365266021211494</v>
       </c>
       <c r="AI7" t="n">
-        <v>0.8564190215864946</v>
+        <v>0.8556067673047103</v>
       </c>
       <c r="AJ7" t="n">
-        <v>0.9309816165035615</v>
+        <v>0.9306081184520197</v>
       </c>
       <c r="AK7" t="n">
-        <v>0.3111452462475973</v>
+        <v>0.2733222986142951</v>
       </c>
       <c r="AL7" t="n">
-        <v>1.026946687773078</v>
+        <v>0.94708331955606</v>
       </c>
       <c r="AM7" t="n">
-        <v>0.503447796603768</v>
+        <v>0.3769042166111551</v>
       </c>
       <c r="AN7" t="n">
-        <v>0.7115932367921735</v>
+        <v>0.5577971839788439</v>
       </c>
       <c r="AO7" t="n">
-        <v>0.1126765581068928</v>
+        <v>0.1164682001603178</v>
       </c>
       <c r="AP7" t="n">
-        <v>0.8607755157728282</v>
+        <v>0.8460927145192053</v>
       </c>
       <c r="AQ7" t="n">
-        <v>0.5273692063357156</v>
+        <v>0.5515503936407113</v>
       </c>
       <c r="AR7" t="n">
-        <v>0.7327043540050766</v>
+        <v>0.5638932886886516</v>
       </c>
       <c r="AS7" t="n">
-        <v>0.5133333333333334</v>
+        <v>0.38125</v>
       </c>
       <c r="AT7" t="n">
-        <v>0.9947777367543102</v>
+        <v>0.913006188823837</v>
       </c>
       <c r="AU7" t="n">
-        <v>0.7719120599890752</v>
+        <v>0.6048180107391227</v>
       </c>
       <c r="AV7" t="n">
-        <v>0.2620733827492336</v>
+        <v>0.3491129001351854</v>
       </c>
       <c r="AW7" t="n">
-        <v>1.022991656980053</v>
+        <v>0.9409630125541549</v>
       </c>
       <c r="AX7" t="n">
-        <v>0.2510795969909776</v>
+        <v>0.3361450018150323</v>
       </c>
       <c r="AY7" t="n">
-        <v>185.0464595122539</v>
+        <v>139.0549019493772</v>
       </c>
       <c r="AZ7" t="n">
-        <v>2.879976293973698</v>
+        <v>3.721602002135425</v>
       </c>
       <c r="BA7" t="n">
-        <v>255.1779408559948</v>
+        <v>242.8728905954796</v>
       </c>
       <c r="BB7" t="n">
-        <v>169.5828485624933</v>
+        <v>127.7171661622534</v>
       </c>
       <c r="BC7" t="n">
-        <v>202.212234884853</v>
+        <v>161.3924812349645</v>
       </c>
       <c r="BD7" t="n">
-        <v>243.1272127708831</v>
+        <v>224.6120038691836</v>
       </c>
       <c r="BE7" t="n">
-        <v>0.9600130962407062</v>
+        <v>0.9767147910578338</v>
       </c>
       <c r="BF7" t="n">
-        <v>412.3128915733546</v>
+        <v>459.3268971711375</v>
       </c>
       <c r="BG7" t="n">
-        <v>407.3060459328526</v>
+        <v>429.900884327747</v>
       </c>
       <c r="BH7" t="n">
-        <v>0.626501726168982</v>
+        <v>0.5649508978686322</v>
       </c>
       <c r="BI7" t="n">
-        <v>0.6201908687196671</v>
+        <v>0.5445931663556255</v>
       </c>
       <c r="BJ7" t="n">
-        <v>458.3348218158275</v>
+        <v>507.3270238049855</v>
       </c>
       <c r="BK7" t="n">
-        <v>0.9358938810594575</v>
+        <v>0.9505697138597924</v>
       </c>
       <c r="BL7" t="n">
-        <v>677.0827640427808</v>
+        <v>687.7001573586039</v>
       </c>
       <c r="BM7" t="n">
-        <v>521.9492513073021</v>
+        <v>526.0256983406874</v>
       </c>
       <c r="BN7" t="n">
-        <v>0.4658062295557158</v>
+        <v>0.426998157271987</v>
       </c>
       <c r="BO7" t="n">
-        <v>0.3668220137585716</v>
+        <v>0.2975790404866964</v>
       </c>
       <c r="BP7" t="n">
-        <v>0.1834110068792858</v>
+        <v>0.2231842803650222</v>
       </c>
       <c r="BQ7" t="n">
-        <v>0.694167830649013</v>
+        <v>0.6570736359990065</v>
       </c>
       <c r="BR7" t="n">
-        <v>0.5799965296833545</v>
+        <v>0.5665736133518423</v>
       </c>
       <c r="BS7" t="n">
-        <v>0.6315028161797239</v>
+        <v>0.6294486453735235</v>
       </c>
       <c r="BT7" t="n">
-        <v>0.6830091026760933</v>
+        <v>0.6923236773952047</v>
       </c>
       <c r="BU7" t="n">
-        <v>0.5092720830501801</v>
+        <v>0.4888283553242228</v>
       </c>
       <c r="BV7" t="n">
-        <v>0.1121859722334815</v>
+        <v>0.127559622946259</v>
       </c>
       <c r="BW7" t="n">
-        <v>0.05266866363906803</v>
+        <v>0.05371049954779572</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.51</v>
+        <v>0.375</v>
       </c>
       <c r="B8" t="n">
-        <v>0.5033333333333334</v>
+        <v>0.3625</v>
       </c>
       <c r="C8" t="n">
         <v>0.9399999999999999</v>
       </c>
       <c r="D8" t="n">
-        <v>0.8851551928471313</v>
+        <v>0.8529356580420905</v>
       </c>
       <c r="E8" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="F8" t="n">
-        <v>1.01899260985795</v>
+        <v>1.066429875635743</v>
       </c>
       <c r="G8" t="n">
-        <v>330.3561984983635</v>
+        <v>334.9958456714842</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2873857616296107</v>
+        <v>0.3573195700399479</v>
       </c>
       <c r="I8" t="n">
-        <v>458.3348218158275</v>
+        <v>507.3270238049855</v>
       </c>
       <c r="J8" t="n">
-        <v>422591.2609391822</v>
+        <v>576129.2435136657</v>
       </c>
       <c r="K8" t="n">
-        <v>31363.90771286501</v>
+        <v>40099.19419057097</v>
       </c>
       <c r="L8" t="n">
-        <v>29482.07325009311</v>
+        <v>37693.24253913671</v>
       </c>
       <c r="M8" t="n">
-        <v>26096.21023321942</v>
+        <v>32149.91062885868</v>
       </c>
       <c r="N8" t="n">
-        <v>29.30623583508261</v>
+        <v>37.468431947452</v>
       </c>
       <c r="O8" t="n">
-        <v>487.6410576509101</v>
+        <v>544.7954557524375</v>
       </c>
       <c r="P8" t="n">
-        <v>487.6410576509101</v>
+        <v>544.7954557524375</v>
       </c>
       <c r="Q8" t="n">
-        <v>1.212504630046815</v>
+        <v>1.238387978501664</v>
       </c>
       <c r="R8" t="n">
-        <v>512393.8605060804</v>
+        <v>713471.5292305814</v>
       </c>
       <c r="S8" t="n">
-        <v>512393.8605060804</v>
+        <v>713471.5292305814</v>
       </c>
       <c r="T8" t="n">
-        <v>392.0199813209105</v>
+        <v>412.4399969472064</v>
       </c>
       <c r="U8" t="n">
-        <v>404.358809265175</v>
+        <v>427.3990130004892</v>
       </c>
       <c r="V8" t="n">
-        <v>0.7905694150420949</v>
+        <v>0.7615773105863909</v>
       </c>
       <c r="W8" t="n">
-        <v>0.2135259927506889</v>
+        <v>0.1461968646286187</v>
       </c>
       <c r="X8" t="n">
-        <v>1.163669370778668</v>
+        <v>1.064577496794081</v>
       </c>
       <c r="Y8" t="n">
-        <v>168.4816612341654</v>
+        <v>125.6234421268066</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.4680343173960578</v>
+        <v>0.3482637835623633</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.6727435922915034</v>
+        <v>0.5220220244246978</v>
       </c>
       <c r="AB8" t="n">
-        <v>0.1191834119456657</v>
+        <v>0.1244499868451067</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.5033333333333334</v>
+        <v>0.3625</v>
       </c>
       <c r="AD8" t="n">
-        <v>166.2792865775097</v>
+        <v>121.435994055913</v>
       </c>
       <c r="AE8" t="n">
-        <v>0.4478210551388968</v>
+        <v>0.3248720262443578</v>
       </c>
       <c r="AF8" t="n">
-        <v>0.6488550652132633</v>
+        <v>0.4902267786136445</v>
       </c>
       <c r="AG8" t="n">
-        <v>0.1051218473812989</v>
+        <v>0.1108926247734101</v>
       </c>
       <c r="AH8" t="n">
-        <v>0.6422872546996068</v>
+        <v>0.6507693397424607</v>
       </c>
       <c r="AI8" t="n">
-        <v>0.8754753403681166</v>
+        <v>0.874751580189404</v>
       </c>
       <c r="AJ8" t="n">
-        <v>0.9398023918868981</v>
+        <v>0.939465360469416</v>
       </c>
       <c r="AK8" t="n">
-        <v>0.3146515870937543</v>
+        <v>0.2778401656135346</v>
       </c>
       <c r="AL8" t="n">
-        <v>1.015946073443035</v>
+        <v>0.9235220626756799</v>
       </c>
       <c r="AM8" t="n">
-        <v>0.484956438220453</v>
+        <v>0.3579847479308438</v>
       </c>
       <c r="AN8" t="n">
-        <v>0.6908970018343493</v>
+        <v>0.532609775801597</v>
       </c>
       <c r="AO8" t="n">
-        <v>0.0987250530206893</v>
+        <v>0.1020682245887486</v>
       </c>
       <c r="AP8" t="n">
-        <v>0.8651859034644964</v>
+        <v>0.8505213355279034</v>
       </c>
       <c r="AQ8" t="n">
-        <v>0.5272772926466498</v>
+        <v>0.5510264886289833</v>
       </c>
       <c r="AR8" t="n">
-        <v>0.7238011676951294</v>
+        <v>0.5472873917189358</v>
       </c>
       <c r="AS8" t="n">
-        <v>0.5066666666666667</v>
+        <v>0.36875</v>
       </c>
       <c r="AT8" t="n">
-        <v>0.9826149747102656</v>
+        <v>0.8886668819554222</v>
       </c>
       <c r="AU8" t="n">
-        <v>0.7654668155981543</v>
+        <v>0.5897582525396874</v>
       </c>
       <c r="AV8" t="n">
-        <v>0.2588138070151362</v>
+        <v>0.3413794902364864</v>
       </c>
       <c r="AW8" t="n">
-        <v>1.012099504766793</v>
+        <v>0.9168465296054072</v>
       </c>
       <c r="AX8" t="n">
-        <v>0.2466326891686383</v>
+        <v>0.3270882770657199</v>
       </c>
       <c r="AY8" t="n">
-        <v>182.6524303501638</v>
+        <v>134.8326123950213</v>
       </c>
       <c r="AZ8" t="n">
-        <v>3.3082827805304</v>
+        <v>4.317328488730078</v>
       </c>
       <c r="BA8" t="n">
-        <v>254.4126923439285</v>
+        <v>241.4104959520961</v>
       </c>
       <c r="BB8" t="n">
-        <v>167.3804739058375</v>
+        <v>123.5297180913598</v>
       </c>
       <c r="BC8" t="n">
-        <v>201.1902719181625</v>
+        <v>159.1402078158146</v>
       </c>
       <c r="BD8" t="n">
-        <v>241.5743010493417</v>
+        <v>222.1117834262884</v>
       </c>
       <c r="BE8" t="n">
-        <v>0.9634906462899344</v>
+        <v>0.9797853895098045</v>
       </c>
       <c r="BF8" t="n">
-        <v>441.6013136885135</v>
+        <v>497.0716056276176</v>
       </c>
       <c r="BG8" t="n">
-        <v>421.5242633297759</v>
+        <v>447.2155310812989</v>
       </c>
       <c r="BH8" t="n">
-        <v>0.6035540880475745</v>
+        <v>0.5398079430926793</v>
       </c>
       <c r="BI8" t="n">
-        <v>0.5974255921080215</v>
+        <v>0.5196824902963315</v>
       </c>
       <c r="BJ8" t="n">
-        <v>487.6410576509101</v>
+        <v>544.7954557524375</v>
       </c>
       <c r="BK8" t="n">
-        <v>0.9405137769823967</v>
+        <v>0.9549883515465672</v>
       </c>
       <c r="BL8" t="n">
-        <v>680.4250787692673</v>
+        <v>690.896869591489</v>
       </c>
       <c r="BM8" t="n">
-        <v>523.2359264171396</v>
+        <v>527.2468723935984</v>
       </c>
       <c r="BN8" t="n">
-        <v>0.4616928785902046</v>
+        <v>0.4212671426915137</v>
       </c>
       <c r="BO8" t="n">
-        <v>0.3668220137585716</v>
+        <v>0.2975790404866964</v>
       </c>
       <c r="BP8" t="n">
-        <v>0.1834110068792858</v>
+        <v>0.2231842803650222</v>
       </c>
       <c r="BQ8" t="n">
-        <v>0.7050484345825851</v>
+        <v>0.6684108649448608</v>
       </c>
       <c r="BR8" t="n">
-        <v>0.5799965296833545</v>
+        <v>0.5665736133518423</v>
       </c>
       <c r="BS8" t="n">
-        <v>0.6347384707687515</v>
+        <v>0.6327433073496426</v>
       </c>
       <c r="BT8" t="n">
-        <v>0.6894804118541484</v>
+        <v>0.6989130013474428</v>
       </c>
       <c r="BU8" t="n">
-        <v>0.5172545731418249</v>
+        <v>0.4972626596029361</v>
       </c>
       <c r="BV8" t="n">
-        <v>0.1081947271876592</v>
+        <v>0.1233424708069024</v>
       </c>
       <c r="BW8" t="n">
-        <v>0.0456783864087682</v>
+        <v>0.04658913073714011</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.5033333333333334</v>
+        <v>0.3625</v>
       </c>
       <c r="B9" t="n">
-        <v>0.4966666666666667</v>
+        <v>0.35</v>
       </c>
       <c r="C9" t="n">
         <v>0.9399999999999999</v>
       </c>
       <c r="D9" t="n">
-        <v>0.886040204530712</v>
+        <v>0.8442592793216259</v>
       </c>
       <c r="E9" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="F9" t="n">
-        <v>1.01899260985795</v>
+        <v>1.066429875635743</v>
       </c>
       <c r="G9" t="n">
-        <v>330.3561984983635</v>
+        <v>334.9958456714842</v>
       </c>
       <c r="H9" t="n">
-        <v>0.2918079074728968</v>
+        <v>0.3605527408399267</v>
       </c>
       <c r="I9" t="n">
-        <v>487.6410576509101</v>
+        <v>544.7954557524375</v>
       </c>
       <c r="J9" t="n">
-        <v>512393.8605060804</v>
+        <v>713471.5292305814</v>
       </c>
       <c r="K9" t="n">
-        <v>31846.519562997</v>
+        <v>40462.02778444644</v>
       </c>
       <c r="L9" t="n">
-        <v>29935.72838921718</v>
+        <v>38034.30611737965</v>
       </c>
       <c r="M9" t="n">
-        <v>26524.25890475783</v>
+        <v>32110.81587215705</v>
       </c>
       <c r="N9" t="n">
-        <v>29.75718527755187</v>
+        <v>37.80746134928394</v>
       </c>
       <c r="O9" t="n">
-        <v>517.398242928462</v>
+        <v>582.6029171017215</v>
       </c>
       <c r="P9" t="n">
-        <v>517.398242928462</v>
+        <v>582.6029171017215</v>
       </c>
       <c r="Q9" t="n">
-        <v>1.202378070080593</v>
+        <v>1.220524649009106</v>
       </c>
       <c r="R9" t="n">
-        <v>616091.1411164453</v>
+        <v>870809.5877921456</v>
       </c>
       <c r="S9" t="n">
-        <v>616091.1411164453</v>
+        <v>870809.5877921456</v>
       </c>
       <c r="T9" t="n">
-        <v>404.358809265175</v>
+        <v>427.3990130004892</v>
       </c>
       <c r="U9" t="n">
-        <v>416.5136622656132</v>
+        <v>441.980495162634</v>
       </c>
       <c r="V9" t="n">
-        <v>0.7905694150420949</v>
+        <v>0.7615773105863909</v>
       </c>
       <c r="W9" t="n">
-        <v>0.2107291821486428</v>
+        <v>0.1440741840057616</v>
       </c>
       <c r="X9" t="n">
-        <v>1.163669370778668</v>
+        <v>1.064577496794081</v>
       </c>
       <c r="Y9" t="n">
-        <v>166.2792865775097</v>
+        <v>121.435994055913</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.4478210551388968</v>
+        <v>0.3248720262443578</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.6488550652132633</v>
+        <v>0.4902267786136445</v>
       </c>
       <c r="AB9" t="n">
-        <v>0.1051218473812989</v>
+        <v>0.1108926247734101</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.4966666666666667</v>
+        <v>0.35</v>
       </c>
       <c r="AD9" t="n">
-        <v>164.0769119208539</v>
+        <v>117.2485459850195</v>
       </c>
       <c r="AE9" t="n">
-        <v>0.4289942661294574</v>
+        <v>0.3033211971446864</v>
       </c>
       <c r="AF9" t="n">
-        <v>0.6260092288210374</v>
+        <v>0.4603395387699436</v>
       </c>
       <c r="AG9" t="n">
-        <v>0.0933428901700914</v>
+        <v>0.100056302624151</v>
       </c>
       <c r="AH9" t="n">
-        <v>0.6536884130678781</v>
+        <v>0.6619729934593227</v>
       </c>
       <c r="AI9" t="n">
-        <v>0.8910157904237872</v>
+        <v>0.8898113151741506</v>
       </c>
       <c r="AJ9" t="n">
-        <v>0.9470768550610151</v>
+        <v>0.946510479765531</v>
       </c>
       <c r="AK9" t="n">
-        <v>0.3171786054504727</v>
+        <v>0.281528605843333</v>
       </c>
       <c r="AL9" t="n">
-        <v>1.006182775046917</v>
+        <v>0.9005374717254715</v>
       </c>
       <c r="AM9" t="n">
-        <v>0.4674047518645908</v>
+        <v>0.3404490152611628</v>
       </c>
       <c r="AN9" t="n">
-        <v>0.670722061360207</v>
+        <v>0.5088534310976932</v>
       </c>
       <c r="AO9" t="n">
-        <v>0.08712030520183586</v>
+        <v>0.09051697283767492</v>
       </c>
       <c r="AP9" t="n">
-        <v>0.868823135051555</v>
+        <v>0.854043895175961</v>
       </c>
       <c r="AQ9" t="n">
-        <v>0.527614810474916</v>
+        <v>0.5506466038529215</v>
       </c>
       <c r="AR9" t="n">
-        <v>0.7148831019922585</v>
+        <v>0.5308367445217098</v>
       </c>
       <c r="AS9" t="n">
-        <v>0.5</v>
+        <v>0.35625</v>
       </c>
       <c r="AT9" t="n">
-        <v>0.9719690024117941</v>
+        <v>0.8653500475224741</v>
       </c>
       <c r="AU9" t="n">
-        <v>0.7585319039895938</v>
+        <v>0.5742398709033788</v>
       </c>
       <c r="AV9" t="n">
-        <v>0.2570859004195356</v>
+        <v>0.3345133030007643</v>
       </c>
       <c r="AW9" t="n">
-        <v>1.002466556264767</v>
+        <v>0.8933979759636368</v>
       </c>
       <c r="AX9" t="n">
-        <v>0.2439346522751727</v>
+        <v>0.319158105060258</v>
       </c>
       <c r="AY9" t="n">
-        <v>180.2640997302265</v>
+        <v>130.6757008041521</v>
       </c>
       <c r="AZ9" t="n">
-        <v>3.776266265917991</v>
+        <v>4.953187281049108</v>
       </c>
       <c r="BA9" t="n">
-        <v>253.6565891408028</v>
+        <v>239.8711457535123</v>
       </c>
       <c r="BB9" t="n">
-        <v>165.1780992491818</v>
+        <v>119.3422700204662</v>
       </c>
       <c r="BC9" t="n">
-        <v>199.9741661384299</v>
+        <v>156.7565726515706</v>
       </c>
       <c r="BD9" t="n">
-        <v>240.1345068725876</v>
+        <v>219.7035832877112</v>
       </c>
       <c r="BE9" t="n">
-        <v>0.9665760504290475</v>
+        <v>0.9824096944273142</v>
       </c>
       <c r="BF9" t="n">
-        <v>471.3421675312601</v>
+        <v>535.2123372111415</v>
       </c>
       <c r="BG9" t="n">
-        <v>435.4873528908478</v>
+        <v>464.0560698884079</v>
       </c>
       <c r="BH9" t="n">
-        <v>0.5824660290522381</v>
+        <v>0.5169012137072022</v>
       </c>
       <c r="BI9" t="n">
-        <v>0.5765345260618423</v>
+        <v>0.4970888663466193</v>
       </c>
       <c r="BJ9" t="n">
-        <v>517.398242928462</v>
+        <v>582.6029171017215</v>
       </c>
       <c r="BK9" t="n">
-        <v>0.9446013233764412</v>
+        <v>0.9588171098257054</v>
       </c>
       <c r="BL9" t="n">
-        <v>683.3822593499328</v>
+        <v>693.666827052431</v>
       </c>
       <c r="BM9" t="n">
-        <v>524.3717058271155</v>
+        <v>528.3027394712392</v>
       </c>
       <c r="BN9" t="n">
-        <v>0.4579471092815971</v>
+        <v>0.4158668257287578</v>
       </c>
       <c r="BO9" t="n">
-        <v>0.3668220137585716</v>
+        <v>0.2975790404866964</v>
       </c>
       <c r="BP9" t="n">
-        <v>0.1834110068792858</v>
+        <v>0.2231842803650222</v>
       </c>
       <c r="BQ9" t="n">
-        <v>0.7139378684462849</v>
+        <v>0.6773344445505896</v>
       </c>
       <c r="BR9" t="n">
-        <v>0.5799965296833545</v>
+        <v>0.5665736133518423</v>
       </c>
       <c r="BS9" t="n">
-        <v>0.6374069039992936</v>
+        <v>0.6353639071499578</v>
       </c>
       <c r="BT9" t="n">
-        <v>0.6948172783152328</v>
+        <v>0.7041542009480733</v>
       </c>
       <c r="BU9" t="n">
-        <v>0.5237762532039368</v>
+        <v>0.5039013352448847</v>
       </c>
       <c r="BV9" t="n">
-        <v>0.1049338871566032</v>
+        <v>0.1200231329859281</v>
       </c>
       <c r="BW9" t="n">
-        <v>0.03997780722463257</v>
+        <v>0.04098730387870908</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.4966666666666667</v>
+        <v>0.35</v>
       </c>
       <c r="B10" t="n">
-        <v>0.49</v>
+        <v>0.3375</v>
       </c>
       <c r="C10" t="n">
         <v>0.9399999999999999</v>
       </c>
       <c r="D10" t="n">
-        <v>0.8866846944514155</v>
+        <v>0.8345538265996715</v>
       </c>
       <c r="E10" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="F10" t="n">
-        <v>1.01899260985795</v>
+        <v>1.066429875635743</v>
       </c>
       <c r="G10" t="n">
-        <v>330.3561984983635</v>
+        <v>334.9958456714842</v>
       </c>
       <c r="H10" t="n">
-        <v>0.2961695371069186</v>
+        <v>0.3629425367369873</v>
       </c>
       <c r="I10" t="n">
-        <v>517.398242928462</v>
+        <v>582.6029171017215</v>
       </c>
       <c r="J10" t="n">
-        <v>616091.1411164453</v>
+        <v>870809.5877921456</v>
       </c>
       <c r="K10" t="n">
-        <v>32322.52696344526</v>
+        <v>40730.21597727716</v>
       </c>
       <c r="L10" t="n">
-        <v>30383.17534563854</v>
+        <v>38286.40301864053</v>
       </c>
       <c r="M10" t="n">
-        <v>26940.29654781129</v>
+        <v>31952.06414594367</v>
       </c>
       <c r="N10" t="n">
-        <v>30.20196356425303</v>
+        <v>38.05805469049754</v>
       </c>
       <c r="O10" t="n">
-        <v>547.600206492715</v>
+        <v>620.660971792219</v>
       </c>
       <c r="P10" t="n">
-        <v>547.600206492715</v>
+        <v>620.660971792219</v>
       </c>
       <c r="Q10" t="n">
-        <v>1.193179329499475</v>
+        <v>1.204167456353411</v>
       </c>
       <c r="R10" t="n">
-        <v>735107.2146678865</v>
+        <v>1048600.566299831</v>
       </c>
       <c r="S10" t="n">
-        <v>735107.2146678865</v>
+        <v>1048600.566299831</v>
       </c>
       <c r="T10" t="n">
-        <v>416.5136622656132</v>
+        <v>441.980495162634</v>
       </c>
       <c r="U10" t="n">
-        <v>428.4977820677807</v>
+        <v>456.1881452229234</v>
       </c>
       <c r="V10" t="n">
-        <v>0.7905694150420949</v>
+        <v>0.7615773105863909</v>
       </c>
       <c r="W10" t="n">
-        <v>0.2079706453579238</v>
+        <v>0.1425052061332324</v>
       </c>
       <c r="X10" t="n">
-        <v>1.163669370778668</v>
+        <v>1.064577496794081</v>
       </c>
       <c r="Y10" t="n">
-        <v>164.0769119208539</v>
+        <v>117.2485459850195</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.4289942661294574</v>
+        <v>0.3033211971446864</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.6260092288210374</v>
+        <v>0.4603395387699436</v>
       </c>
       <c r="AB10" t="n">
-        <v>0.09334289017009137</v>
+        <v>0.100056302624151</v>
       </c>
       <c r="AC10" t="n">
-        <v>0.49</v>
+        <v>0.3375</v>
       </c>
       <c r="AD10" t="n">
-        <v>161.8745372641982</v>
+        <v>113.0610979141259</v>
       </c>
       <c r="AE10" t="n">
-        <v>0.4113989955386405</v>
+        <v>0.2833789606329719</v>
       </c>
       <c r="AF10" t="n">
-        <v>0.6041564687702409</v>
+        <v>0.4322063770688386</v>
       </c>
       <c r="AG10" t="n">
-        <v>0.08339233905144858</v>
+        <v>0.09134516475091831</v>
       </c>
       <c r="AH10" t="n">
-        <v>0.6631087135010758</v>
+        <v>0.6709315018399133</v>
       </c>
       <c r="AI10" t="n">
-        <v>0.9038562144984964</v>
+        <v>0.9018531691514183</v>
       </c>
       <c r="AJ10" t="n">
-        <v>0.9531411376306114</v>
+        <v>0.9521919813536703</v>
       </c>
       <c r="AK10" t="n">
-        <v>0.318958052214398</v>
+        <v>0.2847475699273967</v>
       </c>
       <c r="AL10" t="n">
-        <v>0.9973423395446045</v>
+        <v>0.8775390029012443</v>
       </c>
       <c r="AM10" t="n">
-        <v>0.4507561511543577</v>
+        <v>0.3242639972996528</v>
       </c>
       <c r="AN10" t="n">
-        <v>0.651117799170164</v>
+        <v>0.4865739919422437</v>
       </c>
       <c r="AO10" t="n">
-        <v>0.07737773586903117</v>
+        <v>0.08113866210185122</v>
       </c>
       <c r="AP10" t="n">
-        <v>0.8718552763363532</v>
+        <v>0.8568846459700306</v>
       </c>
       <c r="AQ10" t="n">
-        <v>0.5282812194346006</v>
+        <v>0.5502155635368724</v>
       </c>
       <c r="AR10" t="n">
-        <v>0.7059448619703695</v>
+        <v>0.5145610942928165</v>
       </c>
       <c r="AS10" t="n">
-        <v>0.4933333333333334</v>
+        <v>0.34375</v>
       </c>
       <c r="AT10" t="n">
-        <v>0.9624677305416228</v>
+        <v>0.8423473256617744</v>
       </c>
       <c r="AU10" t="n">
-        <v>0.751203012861814</v>
+        <v>0.5584232149984406</v>
       </c>
       <c r="AV10" t="n">
-        <v>0.2565228685712533</v>
+        <v>0.3277862313689579</v>
       </c>
       <c r="AW10" t="n">
-        <v>0.9937642336736436</v>
+        <v>0.8699731692653212</v>
       </c>
       <c r="AX10" t="n">
-        <v>0.2425612208118296</v>
+        <v>0.3115499542668806</v>
       </c>
       <c r="AY10" t="n">
-        <v>177.8806523432204</v>
+        <v>126.5946303533889</v>
       </c>
       <c r="AZ10" t="n">
-        <v>4.285450887797291</v>
+        <v>5.624360949315135</v>
       </c>
       <c r="BA10" t="n">
-        <v>252.9111572103827</v>
+        <v>238.2360518720631</v>
       </c>
       <c r="BB10" t="n">
-        <v>162.975724592526</v>
+        <v>115.1548219495727</v>
       </c>
       <c r="BC10" t="n">
-        <v>198.6045059914631</v>
+        <v>154.3200418328142</v>
       </c>
       <c r="BD10" t="n">
-        <v>238.785798693533</v>
+        <v>217.3349232851236</v>
       </c>
       <c r="BE10" t="n">
-        <v>0.969327319938008</v>
+        <v>0.9846660418937857</v>
       </c>
       <c r="BF10" t="n">
-        <v>501.5282521584804</v>
+        <v>573.6693083783255</v>
       </c>
       <c r="BG10" t="n">
-        <v>449.2158807728041</v>
+        <v>480.4389481704237</v>
       </c>
       <c r="BH10" t="n">
-        <v>0.563005824227072</v>
+        <v>0.4958716456675673</v>
       </c>
       <c r="BI10" t="n">
-        <v>0.5572626246540556</v>
+        <v>0.4764151053923584</v>
       </c>
       <c r="BJ10" t="n">
-        <v>547.600206492715</v>
+        <v>620.660971792219</v>
       </c>
       <c r="BK10" t="n">
-        <v>0.9482430611939455</v>
+        <v>0.9621714412256647</v>
       </c>
       <c r="BL10" t="n">
-        <v>686.0169147924961</v>
+        <v>696.0935551481729</v>
       </c>
       <c r="BM10" t="n">
-        <v>525.3815431054927</v>
+        <v>529.226041356072</v>
       </c>
       <c r="BN10" t="n">
-        <v>0.4544997855883693</v>
+        <v>0.4106655876725784</v>
       </c>
       <c r="BO10" t="n">
-        <v>0.3668220137585716</v>
+        <v>0.2975790404866964</v>
       </c>
       <c r="BP10" t="n">
-        <v>0.1834110068792858</v>
+        <v>0.2231842803650222</v>
       </c>
       <c r="BQ10" t="n">
-        <v>0.721292760085028</v>
+        <v>0.6844724925067254</v>
       </c>
       <c r="BR10" t="n">
-        <v>0.5799965296833545</v>
+        <v>0.5665736133518423</v>
       </c>
       <c r="BS10" t="n">
-        <v>0.639631416343474</v>
+        <v>0.6374772768888605</v>
       </c>
       <c r="BT10" t="n">
-        <v>0.6992663030035934</v>
+        <v>0.7083809404258787</v>
       </c>
       <c r="BU10" t="n">
-        <v>0.5291721255277364</v>
+        <v>0.509211668899222</v>
       </c>
       <c r="BV10" t="n">
-        <v>0.1022359509947034</v>
+        <v>0.1173679661587594</v>
       </c>
       <c r="BW10" t="n">
-        <v>0.03526765700803369</v>
+        <v>0.03650804968841376</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.49</v>
+        <v>0.3375</v>
       </c>
       <c r="B11" t="n">
-        <v>0.4833333333333333</v>
+        <v>0.325</v>
       </c>
       <c r="C11" t="n">
         <v>0.9399999999999999</v>
       </c>
       <c r="D11" t="n">
-        <v>0.887084061455359</v>
+        <v>0.8238053834530781</v>
       </c>
       <c r="E11" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="F11" t="n">
-        <v>1.01899260985795</v>
+        <v>1.066429875635743</v>
       </c>
       <c r="G11" t="n">
-        <v>330.3561984983635</v>
+        <v>334.9958456714842</v>
       </c>
       <c r="H11" t="n">
-        <v>0.3004539467556255</v>
+        <v>0.3644008637646071</v>
       </c>
       <c r="I11" t="n">
-        <v>547.600206492715</v>
+        <v>620.660971792219</v>
       </c>
       <c r="J11" t="n">
-        <v>735107.2146678865</v>
+        <v>1048600.566299831</v>
       </c>
       <c r="K11" t="n">
-        <v>32790.10694397101</v>
+        <v>40893.87266886935</v>
       </c>
       <c r="L11" t="n">
-        <v>30822.70052733275</v>
+        <v>38440.24030873719</v>
       </c>
       <c r="M11" t="n">
-        <v>27342.32636880857</v>
+        <v>31667.27690756771</v>
       </c>
       <c r="N11" t="n">
-        <v>30.63886732339239</v>
+        <v>38.21097446196539</v>
       </c>
       <c r="O11" t="n">
-        <v>578.2390738161074</v>
+        <v>658.8719462541844</v>
       </c>
       <c r="P11" t="n">
-        <v>578.2390738161074</v>
+        <v>658.8719462541844</v>
       </c>
       <c r="Q11" t="n">
-        <v>1.184763652161305</v>
+        <v>1.189052302015514</v>
       </c>
       <c r="R11" t="n">
-        <v>870928.3083800498</v>
+        <v>1246840.917253586</v>
       </c>
       <c r="S11" t="n">
-        <v>870928.3083800498</v>
+        <v>1246840.917253586</v>
       </c>
       <c r="T11" t="n">
-        <v>428.4977820677807</v>
+        <v>456.1881452229234</v>
       </c>
       <c r="U11" t="n">
-        <v>440.3221110170835</v>
+        <v>470.021024613823</v>
       </c>
       <c r="V11" t="n">
-        <v>0.7905694150420949</v>
+        <v>0.7615773105863909</v>
       </c>
       <c r="W11" t="n">
-        <v>0.2052609467741006</v>
+        <v>0.141547767533534</v>
       </c>
       <c r="X11" t="n">
-        <v>1.163669370778668</v>
+        <v>1.064577496794081</v>
       </c>
       <c r="Y11" t="n">
-        <v>161.8745372641982</v>
+        <v>113.0610979141259</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.4113989955386405</v>
+        <v>0.2833789606329719</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.6041564687702409</v>
+        <v>0.4322063770688386</v>
       </c>
       <c r="AB11" t="n">
-        <v>0.08339233905144861</v>
+        <v>0.09134516475091832</v>
       </c>
       <c r="AC11" t="n">
-        <v>0.4833333333333333</v>
+        <v>0.325</v>
       </c>
       <c r="AD11" t="n">
-        <v>159.6721626075424</v>
+        <v>108.8736498432324</v>
       </c>
       <c r="AE11" t="n">
-        <v>0.3949044052960693</v>
+        <v>0.264852390566271</v>
       </c>
       <c r="AF11" t="n">
-        <v>0.5832461355531482</v>
+        <v>0.4056848070423067</v>
       </c>
       <c r="AG11" t="n">
-        <v>0.07492278450542181</v>
+        <v>0.08432577123228341</v>
       </c>
       <c r="AH11" t="n">
-        <v>0.6709790337886259</v>
+        <v>0.6781934296933768</v>
       </c>
       <c r="AI11" t="n">
-        <v>0.9145839243855182</v>
+        <v>0.9116145123449262</v>
       </c>
       <c r="AJ11" t="n">
-        <v>0.958244163755881</v>
+        <v>0.9568283595080879</v>
       </c>
       <c r="AK11" t="n">
-        <v>0.3201490716692275</v>
+        <v>0.2877665857908671</v>
       </c>
       <c r="AL11" t="n">
-        <v>0.9892092539638102</v>
+        <v>0.8540733970766762</v>
       </c>
       <c r="AM11" t="n">
-        <v>0.4349611283481297</v>
+        <v>0.3093872915612632</v>
       </c>
       <c r="AN11" t="n">
-        <v>0.6321077326660305</v>
+        <v>0.4657932677724579</v>
       </c>
       <c r="AO11" t="n">
-        <v>0.06913129245130799</v>
+        <v>0.07344392158062314</v>
       </c>
       <c r="AP11" t="n">
-        <v>0.874406789398988</v>
+        <v>0.8592028350472394</v>
       </c>
       <c r="AQ11" t="n">
-        <v>0.5291895934338091</v>
+        <v>0.5495796948299662</v>
       </c>
       <c r="AR11" t="n">
-        <v>0.696995567805058</v>
+        <v>0.4984787765891089</v>
       </c>
       <c r="AS11" t="n">
-        <v>0.4866666666666667</v>
+        <v>0.33125</v>
       </c>
       <c r="AT11" t="n">
-        <v>0.953822451893052</v>
+        <v>0.8191312917860756</v>
       </c>
       <c r="AU11" t="n">
-        <v>0.7435633897203713</v>
+        <v>0.5424268789629988</v>
       </c>
       <c r="AV11" t="n">
-        <v>0.256826884087994</v>
+        <v>0.3206525151969667</v>
       </c>
       <c r="AW11" t="n">
-        <v>0.9857691042117221</v>
+        <v>0.8460863486369866</v>
       </c>
       <c r="AX11" t="n">
-        <v>0.2422057144913509</v>
+        <v>0.3036594696739878</v>
       </c>
       <c r="AY11" t="n">
-        <v>175.5034385862216</v>
+        <v>122.6020817033145</v>
       </c>
       <c r="AZ11" t="n">
-        <v>4.837283589515337</v>
+        <v>6.325027396634392</v>
       </c>
       <c r="BA11" t="n">
-        <v>252.1736780466167</v>
+        <v>236.4849743786179</v>
       </c>
       <c r="BB11" t="n">
-        <v>160.7733499358703</v>
+        <v>110.9673738786792</v>
       </c>
       <c r="BC11" t="n">
-        <v>197.1148144606858</v>
+        <v>151.8950557315864</v>
       </c>
       <c r="BD11" t="n">
-        <v>237.5088922511478</v>
+        <v>214.9630528285631</v>
       </c>
       <c r="BE11" t="n">
-        <v>0.9717918110782996</v>
+        <v>0.9866160607784294</v>
       </c>
       <c r="BF11" t="n">
-        <v>532.1533964144063</v>
+        <v>612.3540830685511</v>
       </c>
       <c r="BG11" t="n">
-        <v>462.7280417062494</v>
+        <v>496.3736383647526</v>
       </c>
       <c r="BH11" t="n">
-        <v>0.5449716795134331</v>
+        <v>0.4764253298335728</v>
       </c>
       <c r="BI11" t="n">
-        <v>0.5393980595308624</v>
+        <v>0.45734773887015</v>
       </c>
       <c r="BJ11" t="n">
-        <v>578.2390738161074</v>
+        <v>658.8719462541844</v>
       </c>
       <c r="BK11" t="n">
-        <v>0.9515082888957234</v>
+        <v>0.9651388409583935</v>
       </c>
       <c r="BL11" t="n">
-        <v>688.3791798337485</v>
+        <v>698.2403532560753</v>
       </c>
       <c r="BM11" t="n">
-        <v>526.2853283133655</v>
+        <v>530.0414969944471</v>
       </c>
       <c r="BN11" t="n">
-        <v>0.4512930144040195</v>
+        <v>0.4055589119861215</v>
       </c>
       <c r="BO11" t="n">
-        <v>0.3668220137585716</v>
+        <v>0.2975790404866964</v>
       </c>
       <c r="BP11" t="n">
-        <v>0.1834110068792858</v>
+        <v>0.2231842803650222</v>
       </c>
       <c r="BQ11" t="n">
-        <v>0.7274437893707612</v>
+        <v>0.6902601129331082</v>
       </c>
       <c r="BR11" t="n">
-        <v>0.5799965296833545</v>
+        <v>0.5665736133518423</v>
       </c>
       <c r="BS11" t="n">
-        <v>0.6415033186630079</v>
+        <v>0.6392018880920168</v>
       </c>
       <c r="BT11" t="n">
-        <v>0.7030101076426614</v>
+        <v>0.7118301628321914</v>
       </c>
       <c r="BU11" t="n">
-        <v>0.5336847914262977</v>
+        <v>0.5135173552321824</v>
       </c>
       <c r="BV11" t="n">
-        <v>0.09997961804542277</v>
+        <v>0.1152151229922792</v>
       </c>
       <c r="BW11" t="n">
-        <v>0.03133249686425865</v>
+        <v>0.03287708576168202</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0.4833333333333333</v>
+        <v>0.325</v>
       </c>
       <c r="B12" t="n">
-        <v>0.4766666666666667</v>
+        <v>0.3125</v>
       </c>
       <c r="C12" t="n">
         <v>0.9399999999999999</v>
       </c>
       <c r="D12" t="n">
-        <v>0.8872368569202875</v>
+        <v>0.8120003556960932</v>
       </c>
       <c r="E12" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="F12" t="n">
-        <v>1.01899260985795</v>
+        <v>1.066429875635743</v>
       </c>
       <c r="G12" t="n">
-        <v>330.3561984983635</v>
+        <v>334.9958456714842</v>
       </c>
       <c r="H12" t="n">
-        <v>0.3046699184544066</v>
+        <v>0.3648340491519012</v>
       </c>
       <c r="I12" t="n">
-        <v>578.2390738161074</v>
+        <v>658.8719462541844</v>
       </c>
       <c r="J12" t="n">
-        <v>870928.3083800498</v>
+        <v>1246840.917253586</v>
       </c>
       <c r="K12" t="n">
-        <v>33250.21793391992</v>
+        <v>40942.48569323765</v>
       </c>
       <c r="L12" t="n">
-        <v>31255.20485788472</v>
+        <v>38485.93655164339</v>
       </c>
       <c r="M12" t="n">
-        <v>27730.76972050935</v>
+        <v>31250.59416923171</v>
       </c>
       <c r="N12" t="n">
-        <v>31.06879210525321</v>
+        <v>38.25639816266739</v>
       </c>
       <c r="O12" t="n">
-        <v>609.3078659213606</v>
+        <v>697.1283444168519</v>
       </c>
       <c r="P12" t="n">
-        <v>609.3078659213606</v>
+        <v>697.1283444168519</v>
       </c>
       <c r="Q12" t="n">
-        <v>1.177030148064128</v>
+        <v>1.174972243401005</v>
       </c>
       <c r="R12" t="n">
-        <v>1025108.875765811</v>
+        <v>1465003.469709612</v>
       </c>
       <c r="S12" t="n">
-        <v>1025108.875765811</v>
+        <v>1465003.469709612</v>
       </c>
       <c r="T12" t="n">
-        <v>440.3221110170835</v>
+        <v>470.021024613823</v>
       </c>
       <c r="U12" t="n">
-        <v>451.9966011414602</v>
+        <v>483.4740260685887</v>
       </c>
       <c r="V12" t="n">
-        <v>0.7905694150420949</v>
+        <v>0.7615773105863909</v>
       </c>
       <c r="W12" t="n">
-        <v>0.2025945321503091</v>
+        <v>0.1412633673936713</v>
       </c>
       <c r="X12" t="n">
-        <v>1.163669370778668</v>
+        <v>1.064577496794081</v>
       </c>
       <c r="Y12" t="n">
-        <v>159.6721626075424</v>
+        <v>108.8736498432324</v>
       </c>
       <c r="Z12" t="n">
-        <v>0.3949044052960693</v>
+        <v>0.264852390566271</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.5832461355531482</v>
+        <v>0.4056848070423067</v>
       </c>
       <c r="AB12" t="n">
-        <v>0.07492278450542178</v>
+        <v>0.08432577123228341</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.4766666666666667</v>
+        <v>0.3125</v>
       </c>
       <c r="AD12" t="n">
-        <v>157.4697879508866</v>
+        <v>104.6862017723388</v>
       </c>
       <c r="AE12" t="n">
-        <v>0.3793982636452001</v>
+        <v>0.2475795080404627</v>
       </c>
       <c r="AF12" t="n">
-        <v>0.5632271200850089</v>
+        <v>0.3806439700063695</v>
       </c>
       <c r="AG12" t="n">
-        <v>0.06766425569023406</v>
+        <v>0.07867891571681149</v>
       </c>
       <c r="AH12" t="n">
-        <v>0.6776186395344173</v>
+        <v>0.6841493266339539</v>
       </c>
       <c r="AI12" t="n">
-        <v>0.9236340978984978</v>
+        <v>0.9196203140046615</v>
       </c>
       <c r="AJ12" t="n">
-        <v>0.9625746586111572</v>
+        <v>0.9606512171256621</v>
       </c>
       <c r="AK12" t="n">
-        <v>0.3208808500673349</v>
+        <v>0.2907964460364127</v>
       </c>
       <c r="AL12" t="n">
-        <v>0.9816074212305465</v>
+        <v>0.8297807583132409</v>
       </c>
       <c r="AM12" t="n">
-        <v>0.419971480377387</v>
+        <v>0.2957759736655972</v>
       </c>
       <c r="AN12" t="n">
-        <v>0.6137058459021709</v>
+        <v>0.4465201903401176</v>
       </c>
       <c r="AO12" t="n">
-        <v>0.06209871409825427</v>
+        <v>0.06707122204581961</v>
       </c>
       <c r="AP12" t="n">
-        <v>0.8765720368266261</v>
+        <v>0.8611142638560265</v>
       </c>
       <c r="AQ12" t="n">
-        <v>0.5302872321937201</v>
+        <v>0.5486113102580497</v>
       </c>
       <c r="AR12" t="n">
-        <v>0.6880306120776167</v>
+        <v>0.4826064562566781</v>
       </c>
       <c r="AS12" t="n">
-        <v>0.48</v>
+        <v>0.31875</v>
       </c>
       <c r="AT12" t="n">
-        <v>0.9458343174188085</v>
+        <v>0.7952941051769974</v>
       </c>
       <c r="AU12" t="n">
-        <v>0.7356640262208594</v>
+        <v>0.5263410536891099</v>
       </c>
       <c r="AV12" t="n">
-        <v>0.2578037053411918</v>
+        <v>0.3126876489203193</v>
       </c>
       <c r="AW12" t="n">
-        <v>0.9783003714220208</v>
+        <v>0.8213575967455732</v>
       </c>
       <c r="AX12" t="n">
-        <v>0.2426363452011614</v>
+        <v>0.2950165430564633</v>
       </c>
       <c r="AY12" t="n">
-        <v>173.1317556491292</v>
+        <v>118.7135375702998</v>
       </c>
       <c r="AZ12" t="n">
-        <v>5.433149169660529</v>
+        <v>7.048422847999833</v>
       </c>
       <c r="BA12" t="n">
-        <v>251.4454667479009</v>
+        <v>234.596226942576</v>
       </c>
       <c r="BB12" t="n">
-        <v>158.5709752792145</v>
+        <v>106.7799258077856</v>
       </c>
       <c r="BC12" t="n">
-        <v>195.528779700271</v>
+        <v>149.5371544469267</v>
       </c>
       <c r="BD12" t="n">
-        <v>236.2923483443731</v>
+        <v>212.5510843845128</v>
       </c>
       <c r="BE12" t="n">
-        <v>0.9740084184462929</v>
+        <v>0.9883088685352219</v>
       </c>
       <c r="BF12" t="n">
-        <v>563.209725771476</v>
+        <v>651.1689877120725</v>
       </c>
       <c r="BG12" t="n">
-        <v>476.038932505957</v>
+        <v>511.8636086848034</v>
       </c>
       <c r="BH12" t="n">
-        <v>0.528203576594556</v>
+        <v>0.4583178467118498</v>
       </c>
       <c r="BI12" t="n">
-        <v>0.5227746132330348</v>
+        <v>0.4396328922008292</v>
       </c>
       <c r="BJ12" t="n">
-        <v>609.3078659213606</v>
+        <v>697.1283444168519</v>
       </c>
       <c r="BK12" t="n">
-        <v>0.9544511172931751</v>
+        <v>0.967787153349189</v>
       </c>
       <c r="BL12" t="n">
-        <v>690.5082015377847</v>
+        <v>700.1563041025308</v>
       </c>
       <c r="BM12" t="n">
-        <v>527.098548632742</v>
+        <v>530.7682079012403</v>
       </c>
       <c r="BN12" t="n">
-        <v>0.4482887478201174</v>
+        <v>0.4004593365246586</v>
       </c>
       <c r="BO12" t="n">
-        <v>0.3668220137585716</v>
+        <v>0.2975790404866964</v>
       </c>
       <c r="BP12" t="n">
-        <v>0.1834110068792858</v>
+        <v>0.2231842803650222</v>
       </c>
       <c r="BQ12" t="n">
-        <v>0.7326370666931614</v>
+        <v>0.6950075904856097</v>
       </c>
       <c r="BR12" t="n">
-        <v>0.5799965296833545</v>
+        <v>0.5665736133518423</v>
       </c>
       <c r="BS12" t="n">
-        <v>0.6430918395063915</v>
+        <v>0.6406238909692106</v>
       </c>
       <c r="BT12" t="n">
-        <v>0.7061871493294285</v>
+        <v>0.7146741685865788</v>
       </c>
       <c r="BU12" t="n">
-        <v>0.5374948083171168</v>
+        <v>0.5170492297691963</v>
       </c>
       <c r="BV12" t="n">
-        <v>0.09807460960001319</v>
+        <v>0.1134491857237723</v>
       </c>
       <c r="BW12" t="n">
-        <v>0.02801269399136297</v>
+        <v>0.02989913729139348</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.4766666666666667</v>
+        <v>0.3125</v>
       </c>
       <c r="B13" t="n">
-        <v>0.47</v>
+        <v>0.3</v>
       </c>
       <c r="C13" t="n">
         <v>0.9399999999999999</v>
       </c>
       <c r="D13" t="n">
-        <v>0.8871396719634219</v>
+        <v>0.7991254713803608</v>
       </c>
       <c r="E13" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="F13" t="n">
-        <v>1.01899260985795</v>
+        <v>1.066429875635743</v>
       </c>
       <c r="G13" t="n">
-        <v>330.3561984983635</v>
+        <v>334.9958456714842</v>
       </c>
       <c r="H13" t="n">
-        <v>0.3088064239835401</v>
+        <v>0.3641428413236223</v>
       </c>
       <c r="I13" t="n">
-        <v>609.3078659213606</v>
+        <v>697.1283444168519</v>
       </c>
       <c r="J13" t="n">
-        <v>1025108.875765811</v>
+        <v>1465003.469709612</v>
       </c>
       <c r="K13" t="n">
-        <v>33701.65636612976</v>
+        <v>40864.91681860507</v>
       </c>
       <c r="L13" t="n">
-        <v>31679.55698416197</v>
+        <v>38413.02180948877</v>
       </c>
       <c r="M13" t="n">
-        <v>28104.19179087598</v>
+        <v>30696.82416065179</v>
       </c>
       <c r="N13" t="n">
-        <v>31.49061330433595</v>
+        <v>38.18391829969062</v>
       </c>
       <c r="O13" t="n">
-        <v>640.7984792256966</v>
+        <v>735.3122627165425</v>
       </c>
       <c r="P13" t="n">
-        <v>640.7984792256966</v>
+        <v>735.3122627165425</v>
       </c>
       <c r="Q13" t="n">
-        <v>1.169883030704616</v>
+        <v>1.161763539474074</v>
       </c>
       <c r="R13" t="n">
-        <v>1199257.478383109</v>
+        <v>1701987.616311639</v>
       </c>
       <c r="S13" t="n">
-        <v>1199257.478383109</v>
+        <v>1701987.616311639</v>
       </c>
       <c r="T13" t="n">
-        <v>451.9966011414602</v>
+        <v>483.4740260685887</v>
       </c>
       <c r="U13" t="n">
-        <v>463.5296431560511</v>
+        <v>496.5382177525278</v>
       </c>
       <c r="V13" t="n">
-        <v>0.7905694150420949</v>
+        <v>0.7615773105863909</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1999783763451207</v>
+        <v>0.1417171675651513</v>
       </c>
       <c r="X13" t="n">
-        <v>1.163669370778668</v>
+        <v>1.064577496794081</v>
       </c>
       <c r="Y13" t="n">
-        <v>157.4697879508866</v>
+        <v>104.6862017723388</v>
       </c>
       <c r="Z13" t="n">
-        <v>0.3793982636452001</v>
+        <v>0.2475795080404627</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.5632271200850089</v>
+        <v>0.3806439700063695</v>
       </c>
       <c r="AB13" t="n">
-        <v>0.06766425569023406</v>
+        <v>0.07867891571681147</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.47</v>
+        <v>0.3</v>
       </c>
       <c r="AD13" t="n">
-        <v>155.2674132942309</v>
+        <v>100.4987537014453</v>
       </c>
       <c r="AE13" t="n">
-        <v>0.3647842428199741</v>
+        <v>0.2314229337341716</v>
       </c>
       <c r="AF13" t="n">
-        <v>0.5440499571377209</v>
+        <v>0.356964158557928</v>
       </c>
       <c r="AG13" t="n">
-        <v>0.06140503585093043</v>
+        <v>0.07416764671794335</v>
       </c>
       <c r="AH13" t="n">
-        <v>0.6832678985389423</v>
+        <v>0.6890844320072977</v>
       </c>
       <c r="AI13" t="n">
-        <v>0.9313343705002441</v>
+        <v>0.9262539873511073</v>
       </c>
       <c r="AJ13" t="n">
-        <v>0.9662773177703919</v>
+        <v>0.9638325708036187</v>
       </c>
       <c r="AK13" t="n">
-        <v>0.3212532171733763</v>
+        <v>0.2940089553983466</v>
       </c>
       <c r="AL13" t="n">
-        <v>0.9743997274875045</v>
+        <v>0.8043697733634284</v>
       </c>
       <c r="AM13" t="n">
-        <v>0.4057391306291831</v>
+        <v>0.2833915018027358</v>
       </c>
       <c r="AN13" t="n">
-        <v>0.5959162664950163</v>
+        <v>0.4287582016046487</v>
       </c>
       <c r="AO13" t="n">
-        <v>0.05606057260230587</v>
+        <v>0.0617485368298673</v>
       </c>
       <c r="AP13" t="n">
-        <v>0.8784233664062434</v>
+        <v>0.8627049406950048</v>
       </c>
       <c r="AQ13" t="n">
-        <v>0.531524125891526</v>
+        <v>0.5471991620698325</v>
       </c>
       <c r="AR13" t="n">
-        <v>0.6790558969686254</v>
+        <v>0.466958890421039</v>
       </c>
       <c r="AS13" t="n">
-        <v>0.4733333333333334</v>
+        <v>0.30625</v>
       </c>
       <c r="AT13" t="n">
-        <v>0.9383386323572477</v>
+        <v>0.7705127448541069</v>
       </c>
       <c r="AU13" t="n">
-        <v>0.7275532672972517</v>
+        <v>0.5102357395223244</v>
       </c>
       <c r="AV13" t="n">
-        <v>0.2592827353886222</v>
+        <v>0.3035538544330679</v>
       </c>
       <c r="AW13" t="n">
-        <v>0.9712183196685195</v>
+        <v>0.7954836030482841</v>
       </c>
       <c r="AX13" t="n">
-        <v>0.2436650523712678</v>
+        <v>0.2852478635259598</v>
       </c>
       <c r="AY13" t="n">
-        <v>170.7665041009618</v>
+        <v>114.9480074251195</v>
       </c>
       <c r="AZ13" t="n">
-        <v>6.074326617699174</v>
+        <v>7.786942573692805</v>
       </c>
       <c r="BA13" t="n">
-        <v>250.7246603128491</v>
+        <v>232.5466861290662</v>
       </c>
       <c r="BB13" t="n">
-        <v>156.3686006225587</v>
+        <v>102.5924777368921</v>
       </c>
       <c r="BC13" t="n">
-        <v>193.8668907052053</v>
+        <v>147.2964805650054</v>
       </c>
       <c r="BD13" t="n">
-        <v>235.1250548996557</v>
+        <v>210.0656314077421</v>
       </c>
       <c r="BE13" t="n">
-        <v>0.9760094929238345</v>
+        <v>0.9897840645330738</v>
       </c>
       <c r="BF13" t="n">
-        <v>594.690261252411</v>
+        <v>690.0065262381241</v>
       </c>
       <c r="BG13" t="n">
-        <v>489.1621137389118</v>
+        <v>526.9070372439256</v>
       </c>
       <c r="BH13" t="n">
-        <v>0.512559442505542</v>
+        <v>0.4413429119213136</v>
       </c>
       <c r="BI13" t="n">
-        <v>0.5072492307045374</v>
+        <v>0.4230603484230449</v>
       </c>
       <c r="BJ13" t="n">
-        <v>640.7984792256966</v>
+        <v>735.3122627165425</v>
       </c>
       <c r="BK13" t="n">
-        <v>0.9571163696582758</v>
+        <v>0.970169990265362</v>
       </c>
       <c r="BL13" t="n">
-        <v>692.4364077957325</v>
+        <v>701.8801937850227</v>
       </c>
       <c r="BM13" t="n">
-        <v>527.8339824610489</v>
+        <v>531.421221604239</v>
       </c>
       <c r="BN13" t="n">
-        <v>0.4454526663921389</v>
+        <v>0.3952902572720037</v>
       </c>
       <c r="BO13" t="n">
-        <v>0.3668220137585716</v>
+        <v>0.2975790404866964</v>
       </c>
       <c r="BP13" t="n">
-        <v>0.1834110068792858</v>
+        <v>0.2231842803650222</v>
       </c>
       <c r="BQ13" t="n">
-        <v>0.7370584924529089</v>
+        <v>0.6989417925686972</v>
       </c>
       <c r="BR13" t="n">
-        <v>0.5799965296833545</v>
+        <v>0.5665736133518423</v>
       </c>
       <c r="BS13" t="n">
-        <v>0.6444500563954436</v>
+        <v>0.6418072711878795</v>
       </c>
       <c r="BT13" t="n">
-        <v>0.7089035831075328</v>
+        <v>0.7170409290239167</v>
       </c>
       <c r="BU13" t="n">
-        <v>0.540738560918866</v>
+        <v>0.5199760699716112</v>
       </c>
       <c r="BV13" t="n">
-        <v>0.09645273329913862</v>
+        <v>0.1119857656225648</v>
       </c>
       <c r="BW13" t="n">
-        <v>0.02518806448910044</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="B14" t="n">
-        <v>0.4633333333333334</v>
-      </c>
-      <c r="C14" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="D14" t="n">
-        <v>0.8867906223057505</v>
-      </c>
-      <c r="E14" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F14" t="n">
-        <v>1.01899260985795</v>
-      </c>
-      <c r="G14" t="n">
-        <v>330.3561984983635</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0.3128524608067445</v>
-      </c>
-      <c r="I14" t="n">
-        <v>640.7984792256966</v>
-      </c>
-      <c r="J14" t="n">
-        <v>1199257.478383109</v>
-      </c>
-      <c r="K14" t="n">
-        <v>34143.22147640612</v>
-      </c>
-      <c r="L14" t="n">
-        <v>32094.62818782175</v>
-      </c>
-      <c r="M14" t="n">
-        <v>28461.21530335013</v>
-      </c>
-      <c r="N14" t="n">
-        <v>31.90320893421645</v>
-      </c>
-      <c r="O14" t="n">
-        <v>672.701688159913</v>
-      </c>
-      <c r="P14" t="n">
-        <v>672.701688159913</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>1.16324343509115</v>
-      </c>
-      <c r="R14" t="n">
-        <v>1395028.388713118</v>
-      </c>
-      <c r="S14" t="n">
-        <v>1395028.388713118</v>
-      </c>
-      <c r="T14" t="n">
-        <v>463.5296431560511</v>
-      </c>
-      <c r="U14" t="n">
-        <v>474.9282851547367</v>
-      </c>
-      <c r="V14" t="n">
-        <v>0.7905694150420949</v>
-      </c>
-      <c r="W14" t="n">
-        <v>0.1974194379734731</v>
-      </c>
-      <c r="X14" t="n">
-        <v>1.163669370778668</v>
-      </c>
-      <c r="Y14" t="n">
-        <v>155.2674132942309</v>
-      </c>
-      <c r="Z14" t="n">
-        <v>0.3647842428199741</v>
-      </c>
-      <c r="AA14" t="n">
-        <v>0.5440499571377209</v>
-      </c>
-      <c r="AB14" t="n">
-        <v>0.06140503585093043</v>
-      </c>
-      <c r="AC14" t="n">
-        <v>0.4633333333333334</v>
-      </c>
-      <c r="AD14" t="n">
-        <v>153.0650386375751</v>
-      </c>
-      <c r="AE14" t="n">
-        <v>0.3509790833065976</v>
-      </c>
-      <c r="AF14" t="n">
-        <v>0.525667382413151</v>
-      </c>
-      <c r="AG14" t="n">
-        <v>0.05597726199730441</v>
-      </c>
-      <c r="AH14" t="n">
-        <v>0.6881105248608028</v>
-      </c>
-      <c r="AI14" t="n">
-        <v>0.9379351552680958</v>
-      </c>
-      <c r="AJ14" t="n">
-        <v>0.9694643767276306</v>
-      </c>
-      <c r="AK14" t="n">
-        <v>0.3213353951078977</v>
-      </c>
-      <c r="AL14" t="n">
-        <v>0.9674905209827243</v>
-      </c>
-      <c r="AM14" t="n">
-        <v>0.3922139692006276</v>
-      </c>
-      <c r="AN14" t="n">
-        <v>0.578731489558265</v>
-      </c>
-      <c r="AO14" t="n">
-        <v>0.05084468586846386</v>
-      </c>
-      <c r="AP14" t="n">
-        <v>0.8800168958848628</v>
-      </c>
-      <c r="AQ14" t="n">
-        <v>0.532860485515865</v>
-      </c>
-      <c r="AR14" t="n">
-        <v>0.6700771141371021</v>
-      </c>
-      <c r="AS14" t="n">
-        <v>0.4666666666666667</v>
-      </c>
-      <c r="AT14" t="n">
-        <v>0.9312064177956002</v>
-      </c>
-      <c r="AU14" t="n">
-        <v>0.7192695921958087</v>
-      </c>
-      <c r="AV14" t="n">
-        <v>0.2611293036584981</v>
-      </c>
-      <c r="AW14" t="n">
-        <v>0.9644261057893925</v>
-      </c>
-      <c r="AX14" t="n">
-        <v>0.2451565135935838</v>
-      </c>
-      <c r="AY14" t="n">
-        <v>168.4085895407851</v>
-      </c>
-      <c r="AZ14" t="n">
-        <v>6.761980349845451</v>
-      </c>
-      <c r="BA14" t="n">
-        <v>250.0093488402438</v>
-      </c>
-      <c r="BB14" t="n">
-        <v>154.166225965903</v>
-      </c>
-      <c r="BC14" t="n">
-        <v>192.1456136513616</v>
-      </c>
-      <c r="BD14" t="n">
-        <v>233.9981012978615</v>
-      </c>
-      <c r="BE14" t="n">
-        <v>0.9778220760317097</v>
-      </c>
-      <c r="BF14" t="n">
-        <v>626.586899274433</v>
-      </c>
-      <c r="BG14" t="n">
-        <v>502.1090566720151</v>
-      </c>
-      <c r="BH14" t="n">
-        <v>0.4979184213431814</v>
-      </c>
-      <c r="BI14" t="n">
-        <v>0.4927019691438728</v>
-      </c>
-      <c r="BJ14" t="n">
-        <v>672.701688159913</v>
-      </c>
-      <c r="BK14" t="n">
-        <v>0.9595407949336251</v>
-      </c>
-      <c r="BL14" t="n">
-        <v>694.1903850359623</v>
-      </c>
-      <c r="BM14" t="n">
-        <v>528.5020750414039</v>
-      </c>
-      <c r="BN14" t="n">
-        <v>0.442757204462309</v>
-      </c>
-      <c r="BO14" t="n">
-        <v>0.3668220137585716</v>
-      </c>
-      <c r="BP14" t="n">
-        <v>0.1834110068792858</v>
-      </c>
-      <c r="BQ14" t="n">
-        <v>0.7408505072453273</v>
-      </c>
-      <c r="BR14" t="n">
-        <v>0.5799965296833545</v>
-      </c>
-      <c r="BS14" t="n">
-        <v>0.6456191397801052</v>
-      </c>
-      <c r="BT14" t="n">
-        <v>0.711241749876856</v>
-      </c>
-      <c r="BU14" t="n">
-        <v>0.5435205499235805</v>
-      </c>
-      <c r="BV14" t="n">
-        <v>0.09506173879678137</v>
-      </c>
-      <c r="BW14" t="n">
-        <v>0.02276675132817019</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>0.4633333333333334</v>
-      </c>
-      <c r="B15" t="n">
-        <v>0.4566666666666667</v>
-      </c>
-      <c r="C15" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0.8861860900624504</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F15" t="n">
-        <v>1.01899260985795</v>
-      </c>
-      <c r="G15" t="n">
-        <v>330.3561984983635</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0.3168147406662835</v>
-      </c>
-      <c r="I15" t="n">
-        <v>672.701688159913</v>
-      </c>
-      <c r="J15" t="n">
-        <v>1395028.388713118</v>
-      </c>
-      <c r="K15" t="n">
-        <v>34575.64575220337</v>
-      </c>
-      <c r="L15" t="n">
-        <v>32501.10700707116</v>
-      </c>
-      <c r="M15" t="n">
-        <v>28802.02894129771</v>
-      </c>
-      <c r="N15" t="n">
-        <v>32.30726342651209</v>
-      </c>
-      <c r="O15" t="n">
-        <v>705.0089515864252</v>
-      </c>
-      <c r="P15" t="n">
-        <v>705.0089515864252</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>1.157054569684315</v>
-      </c>
-      <c r="R15" t="n">
-        <v>1614123.97199986</v>
-      </c>
-      <c r="S15" t="n">
-        <v>1614123.97199986</v>
-      </c>
-      <c r="T15" t="n">
-        <v>474.9282851547367</v>
-      </c>
-      <c r="U15" t="n">
-        <v>486.1990348272283</v>
-      </c>
-      <c r="V15" t="n">
-        <v>0.7905694150420949</v>
-      </c>
-      <c r="W15" t="n">
-        <v>0.1949134721568421</v>
-      </c>
-      <c r="X15" t="n">
-        <v>1.163669370778668</v>
-      </c>
-      <c r="Y15" t="n">
-        <v>153.0650386375751</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>0.3509790833065976</v>
-      </c>
-      <c r="AA15" t="n">
-        <v>0.525667382413151</v>
-      </c>
-      <c r="AB15" t="n">
-        <v>0.05597726199730441</v>
-      </c>
-      <c r="AC15" t="n">
-        <v>0.4566666666666667</v>
-      </c>
-      <c r="AD15" t="n">
-        <v>150.8626639809193</v>
-      </c>
-      <c r="AE15" t="n">
-        <v>0.3379099229908096</v>
-      </c>
-      <c r="AF15" t="n">
-        <v>0.5080340262126917</v>
-      </c>
-      <c r="AG15" t="n">
-        <v>0.05124625064326233</v>
-      </c>
-      <c r="AH15" t="n">
-        <v>0.692289943098427</v>
-      </c>
-      <c r="AI15" t="n">
-        <v>0.9436319483732867</v>
-      </c>
-      <c r="AJ15" t="n">
-        <v>0.9722245764201718</v>
-      </c>
-      <c r="AK15" t="n">
-        <v>0.3211909139007521</v>
-      </c>
-      <c r="AL15" t="n">
-        <v>0.9607904300051596</v>
-      </c>
-      <c r="AM15" t="n">
-        <v>0.3793519973377993</v>
-      </c>
-      <c r="AN15" t="n">
-        <v>0.5621434959384141</v>
-      </c>
-      <c r="AO15" t="n">
-        <v>0.04631351110651925</v>
-      </c>
-      <c r="AP15" t="n">
-        <v>0.8813969957311334</v>
-      </c>
-      <c r="AQ15" t="n">
-        <v>0.5342738545897996</v>
-      </c>
-      <c r="AR15" t="n">
-        <v>0.6610906338160872</v>
-      </c>
-      <c r="AS15" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="AT15" t="n">
-        <v>0.9243478208701578</v>
-      </c>
-      <c r="AU15" t="n">
-        <v>0.7108350463555755</v>
-      </c>
-      <c r="AV15" t="n">
-        <v>0.2632571870540705</v>
-      </c>
-      <c r="AW15" t="n">
-        <v>0.9578337607810785</v>
-      </c>
-      <c r="AX15" t="n">
-        <v>0.246998714425503</v>
-      </c>
-      <c r="AY15" t="n">
-        <v>166.0574920583078</v>
-      </c>
-      <c r="AZ15" t="n">
-        <v>7.497165624283808</v>
-      </c>
-      <c r="BA15" t="n">
-        <v>249.3004942251385</v>
-      </c>
-      <c r="BB15" t="n">
-        <v>151.9638513092472</v>
-      </c>
-      <c r="BC15" t="n">
-        <v>190.3764767522471</v>
-      </c>
-      <c r="BD15" t="n">
-        <v>232.9066379252696</v>
-      </c>
-      <c r="BE15" t="n">
-        <v>0.97946894718021</v>
-      </c>
-      <c r="BF15" t="n">
-        <v>658.89041426834</v>
-      </c>
-      <c r="BG15" t="n">
-        <v>514.8894513242714</v>
-      </c>
-      <c r="BH15" t="n">
-        <v>0.4841825630413469</v>
-      </c>
-      <c r="BI15" t="n">
-        <v>0.4790355826354806</v>
-      </c>
-      <c r="BJ15" t="n">
-        <v>705.0089515864252</v>
-      </c>
-      <c r="BK15" t="n">
-        <v>0.9617541517615142</v>
-      </c>
-      <c r="BL15" t="n">
-        <v>695.7916624768873</v>
-      </c>
-      <c r="BM15" t="n">
-        <v>529.1112674232144</v>
-      </c>
-      <c r="BN15" t="n">
-        <v>0.4401846119428358</v>
-      </c>
-      <c r="BO15" t="n">
-        <v>0.3668220137585716</v>
-      </c>
-      <c r="BP15" t="n">
-        <v>0.1834110068792858</v>
-      </c>
-      <c r="BQ15" t="n">
-        <v>0.7441245380766146</v>
-      </c>
-      <c r="BR15" t="n">
-        <v>0.5799965296833545</v>
-      </c>
-      <c r="BS15" t="n">
-        <v>0.646631641789699</v>
-      </c>
-      <c r="BT15" t="n">
-        <v>0.7132667538960434</v>
-      </c>
-      <c r="BU15" t="n">
-        <v>0.5459225230888614</v>
-      </c>
-      <c r="BV15" t="n">
-        <v>0.09386075221414092</v>
-      </c>
-      <c r="BW15" t="n">
-        <v>0.02067704220935812</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>0.4566666666666667</v>
-      </c>
-      <c r="B16" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="C16" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="D16" t="n">
-        <v>0.8853238625511552</v>
-      </c>
-      <c r="E16" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F16" t="n">
-        <v>1.01899260985795</v>
-      </c>
-      <c r="G16" t="n">
-        <v>330.3561984983635</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0.3206812265610493</v>
-      </c>
-      <c r="I16" t="n">
-        <v>705.0089515864252</v>
-      </c>
-      <c r="J16" t="n">
-        <v>1614123.97199986</v>
-      </c>
-      <c r="K16" t="n">
-        <v>34997.6155327829</v>
-      </c>
-      <c r="L16" t="n">
-        <v>32897.75860081593</v>
-      </c>
-      <c r="M16" t="n">
-        <v>29125.17071374985</v>
-      </c>
-      <c r="N16" t="n">
-        <v>32.70154930498601</v>
-      </c>
-      <c r="O16" t="n">
-        <v>737.7105008914111</v>
-      </c>
-      <c r="P16" t="n">
-        <v>737.7105008914111</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>1.151258948221676</v>
-      </c>
-      <c r="R16" t="n">
-        <v>1858274.666303953</v>
-      </c>
-      <c r="S16" t="n">
-        <v>1858274.666303953</v>
-      </c>
-      <c r="T16" t="n">
-        <v>486.1990348272283</v>
-      </c>
-      <c r="U16" t="n">
-        <v>497.3472941002998</v>
-      </c>
-      <c r="V16" t="n">
-        <v>0.7905694150420949</v>
-      </c>
-      <c r="W16" t="n">
-        <v>0.1924680917631673</v>
-      </c>
-      <c r="X16" t="n">
-        <v>1.163669370778668</v>
-      </c>
-      <c r="Y16" t="n">
-        <v>150.8626639809193</v>
-      </c>
-      <c r="Z16" t="n">
-        <v>0.3379099229908096</v>
-      </c>
-      <c r="AA16" t="n">
-        <v>0.5080340262126917</v>
-      </c>
-      <c r="AB16" t="n">
-        <v>0.05124625064326234</v>
-      </c>
-      <c r="AC16" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="AD16" t="n">
-        <v>148.6602893242636</v>
-      </c>
-      <c r="AE16" t="n">
-        <v>0.325513106422404</v>
-      </c>
-      <c r="AF16" t="n">
-        <v>0.4911073006404607</v>
-      </c>
-      <c r="AG16" t="n">
-        <v>0.04710328055450629</v>
-      </c>
-      <c r="AH16" t="n">
-        <v>0.6959190020712755</v>
-      </c>
-      <c r="AI16" t="n">
-        <v>0.9485785694002857</v>
-      </c>
-      <c r="AJ16" t="n">
-        <v>0.9746284682702154</v>
-      </c>
-      <c r="AK16" t="n">
-        <v>0.3208713199288842</v>
-      </c>
-      <c r="AL16" t="n">
-        <v>0.9542256000712814</v>
-      </c>
-      <c r="AM16" t="n">
-        <v>0.3671121342508658</v>
-      </c>
-      <c r="AN16" t="n">
-        <v>0.54614104169613</v>
-      </c>
-      <c r="AO16" t="n">
-        <v>0.04235675988127777</v>
-      </c>
-      <c r="AP16" t="n">
-        <v>0.8825989416561552</v>
-      </c>
-      <c r="AQ16" t="n">
-        <v>0.5357366647112239</v>
-      </c>
-      <c r="AR16" t="n">
-        <v>0.6521024943961845</v>
-      </c>
-      <c r="AS16" t="n">
-        <v>0.4533333333333334</v>
-      </c>
-      <c r="AT16" t="n">
-        <v>0.9176774782472779</v>
-      </c>
-      <c r="AU16" t="n">
-        <v>0.7022761781684479</v>
-      </c>
-      <c r="AV16" t="n">
-        <v>0.2655749838510933</v>
-      </c>
-      <c r="AW16" t="n">
-        <v>0.951367300855571</v>
-      </c>
-      <c r="AX16" t="n">
-        <v>0.2490911226871231</v>
-      </c>
-      <c r="AY16" t="n">
-        <v>163.7142166156229</v>
-      </c>
-      <c r="AZ16" t="n">
-        <v>8.280783401242548</v>
-      </c>
-      <c r="BA16" t="n">
-        <v>248.5959779538881</v>
-      </c>
-      <c r="BB16" t="n">
-        <v>149.7614766525915</v>
-      </c>
-      <c r="BC16" t="n">
-        <v>188.5707646676712</v>
-      </c>
-      <c r="BD16" t="n">
-        <v>231.8443672851328</v>
-      </c>
-      <c r="BE16" t="n">
-        <v>0.9809694806573909</v>
-      </c>
-      <c r="BF16" t="n">
-        <v>691.5922650965471</v>
-      </c>
-      <c r="BG16" t="n">
-        <v>527.5121456272326</v>
-      </c>
-      <c r="BH16" t="n">
-        <v>0.4712611453870844</v>
-      </c>
-      <c r="BI16" t="n">
-        <v>0.4661619154971754</v>
-      </c>
-      <c r="BJ16" t="n">
-        <v>737.7105008914111</v>
-      </c>
-      <c r="BK16" t="n">
-        <v>0.9637821780900007</v>
-      </c>
-      <c r="BL16" t="n">
-        <v>697.258860521273</v>
-      </c>
-      <c r="BM16" t="n">
-        <v>529.6688353295287</v>
-      </c>
-      <c r="BN16" t="n">
-        <v>0.4377157042681074</v>
-      </c>
-      <c r="BO16" t="n">
-        <v>0.3668220137585716</v>
-      </c>
-      <c r="BP16" t="n">
-        <v>0.1834110068792858</v>
-      </c>
-      <c r="BQ16" t="n">
-        <v>0.7469683953321788</v>
-      </c>
-      <c r="BR16" t="n">
-        <v>0.5799965296833545</v>
-      </c>
-      <c r="BS16" t="n">
-        <v>0.6475134422389898</v>
-      </c>
-      <c r="BT16" t="n">
-        <v>0.7150303547946251</v>
-      </c>
-      <c r="BU16" t="n">
-        <v>0.5480089019795173</v>
-      </c>
-      <c r="BV16" t="n">
-        <v>0.09281756276881292</v>
-      </c>
-      <c r="BW16" t="n">
-        <v>0.01886251272293382</v>
+        <v>0.02743158460472156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
created new type of calculation
</commit_message>
<xml_diff>
--- a/расчет_ступеней.xlsx
+++ b/расчет_ступеней.xlsx
@@ -810,10 +810,10 @@
         <v>0.4</v>
       </c>
       <c r="F2" t="n">
-        <v>1.066429875635743</v>
+        <v>1.066314923944042</v>
       </c>
       <c r="G2" t="n">
-        <v>334.9958456714842</v>
+        <v>335.0078830645102</v>
       </c>
       <c r="H2" t="n">
         <v>0.3244400050544849</v>
@@ -822,40 +822,40 @@
         <v>288</v>
       </c>
       <c r="J2" t="n">
-        <v>100674.7651178944</v>
+        <v>100674.7250191952</v>
       </c>
       <c r="K2" t="n">
-        <v>36409.37652649458</v>
+        <v>36411.99316699915</v>
       </c>
       <c r="L2" t="n">
-        <v>36045.28276122964</v>
+        <v>36047.87323532916</v>
       </c>
       <c r="M2" t="n">
-        <v>31871.35789272645</v>
+        <v>31873.64839846847</v>
       </c>
       <c r="N2" t="n">
-        <v>35.83030095549666</v>
+        <v>35.83287597945244</v>
       </c>
       <c r="O2" t="n">
-        <v>323.8303009554967</v>
+        <v>323.8328759794524</v>
       </c>
       <c r="P2" t="n">
-        <v>323.8303009554967</v>
+        <v>323.8328759794524</v>
       </c>
       <c r="Q2" t="n">
-        <v>1.440908707022073</v>
+        <v>1.440944626051112</v>
       </c>
       <c r="R2" t="n">
-        <v>145063.1456357761</v>
+        <v>145066.7039955828</v>
       </c>
       <c r="S2" t="n">
-        <v>145063.1456357761</v>
+        <v>145066.7039955828</v>
       </c>
       <c r="T2" t="n">
         <v>310.7513475433373</v>
       </c>
       <c r="U2" t="n">
-        <v>329.5152498904687</v>
+        <v>329.5165600025443</v>
       </c>
       <c r="V2" t="n">
         <v>0.7615773105863909</v>
@@ -867,61 +867,61 @@
         <v>1.064577496794081</v>
       </c>
       <c r="Y2" t="n">
-        <v>150.7481305521679</v>
+        <v>150.7535473790296</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.5546733681375342</v>
+        <v>0.5546932991946492</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.7670768900816778</v>
+        <v>0.767097004253578</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.3651710357190851</v>
+        <v>0.3651616059552399</v>
       </c>
       <c r="AC2" t="n">
         <v>0.4375</v>
       </c>
       <c r="AD2" t="n">
-        <v>146.5606824812743</v>
+        <v>146.5659488407232</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.5085578472919455</v>
+        <v>0.5085740992537762</v>
       </c>
       <c r="AF2" t="n">
-        <v>0.7185450194326043</v>
+        <v>0.71856280975454</v>
       </c>
       <c r="AG2" t="n">
-        <v>0.2868846230922911</v>
+        <v>0.2868716240515501</v>
       </c>
       <c r="AH2" t="n">
-        <v>0.4226367409601864</v>
+        <v>0.4227095570019302</v>
       </c>
       <c r="AI2" t="n">
-        <v>0.5681001461244793</v>
+        <v>0.5681776077372761</v>
       </c>
       <c r="AJ2" t="n">
-        <v>0.8132458964011607</v>
+        <v>0.81327295354452</v>
       </c>
       <c r="AK2" t="n">
-        <v>0.2029970421339847</v>
+        <v>0.2030173452274385</v>
       </c>
       <c r="AL2" t="n">
-        <v>1.128936317318384</v>
+        <v>1.128903359239565</v>
       </c>
       <c r="AM2" t="n">
-        <v>0.4903225573137425</v>
+        <v>0.4903469147270716</v>
       </c>
       <c r="AN2" t="n">
-        <v>0.7002124444906179</v>
+        <v>0.7002387390779349</v>
       </c>
       <c r="AO2" t="n">
-        <v>0.2943956776214189</v>
+        <v>0.2943785722120517</v>
       </c>
       <c r="AP2" t="n">
-        <v>0.7874116034937758</v>
+        <v>0.7874251320654555</v>
       </c>
       <c r="AQ2" t="n">
-        <v>0.5743120885198095</v>
+        <v>0.5743022213947462</v>
       </c>
       <c r="AR2" t="n">
         <v>0.6484989891376707</v>
@@ -930,94 +930,94 @@
         <v>0.44375</v>
       </c>
       <c r="AT2" t="n">
-        <v>1.123094102388967</v>
+        <v>1.123051260722294</v>
       </c>
       <c r="AU2" t="n">
-        <v>0.657848686446533</v>
+        <v>0.6578569989227362</v>
       </c>
       <c r="AV2" t="n">
-        <v>0.474595113251296</v>
+        <v>0.4745522715846229</v>
       </c>
       <c r="AW2" t="n">
-        <v>1.136366747647551</v>
+        <v>1.136328562309924</v>
       </c>
       <c r="AX2" t="n">
-        <v>0.4785180612010175</v>
+        <v>0.4784715633871882</v>
       </c>
       <c r="AY2" t="n">
-        <v>160.8856583832313</v>
+        <v>160.8914394814964</v>
       </c>
       <c r="AZ2" t="n">
-        <v>1.407189122308089</v>
+        <v>1.407197860254812</v>
       </c>
       <c r="BA2" t="n">
-        <v>249.586801734187</v>
+        <v>249.5957701272743</v>
       </c>
       <c r="BB2" t="n">
-        <v>148.6544065167211</v>
+        <v>148.6597481098764</v>
       </c>
       <c r="BC2" t="n">
-        <v>164.9069462237893</v>
+        <v>164.916264892708</v>
       </c>
       <c r="BD2" t="n">
-        <v>243.1313991612655</v>
+        <v>243.1375198765841</v>
       </c>
       <c r="BE2" t="n">
-        <v>0.9487229091131606</v>
+        <v>0.9487192239714259</v>
       </c>
       <c r="BF2" t="n">
-        <v>273.2321978245902</v>
+        <v>273.2311365037707</v>
       </c>
       <c r="BG2" t="n">
-        <v>331.5685556814791</v>
+        <v>331.5679117219535</v>
       </c>
       <c r="BH2" t="n">
-        <v>0.7527456915243563</v>
+        <v>0.7527742019154753</v>
       </c>
       <c r="BI2" t="n">
-        <v>0.7378456664511966</v>
+        <v>0.7378613077130531</v>
       </c>
       <c r="BJ2" t="n">
-        <v>323.8303009554967</v>
+        <v>323.8328759794524</v>
       </c>
       <c r="BK2" t="n">
-        <v>0.9092639620831983</v>
+        <v>0.9092601150966639</v>
       </c>
       <c r="BL2" t="n">
-        <v>644.7761790602917</v>
+        <v>657.8142719199958</v>
       </c>
       <c r="BM2" t="n">
-        <v>509.3448177872226</v>
+        <v>514.4688041560241</v>
       </c>
       <c r="BN2" t="n">
-        <v>0.477341460383392</v>
+        <v>0.4725991506432472</v>
       </c>
       <c r="BO2" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.2975897333830798</v>
       </c>
       <c r="BP2" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.2231923000373098</v>
       </c>
       <c r="BQ2" t="n">
-        <v>0.4899327164348984</v>
+        <v>0.4899762006634609</v>
       </c>
       <c r="BR2" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5665939720200175</v>
       </c>
       <c r="BS2" t="n">
-        <v>0.585792973589422</v>
+        <v>0.5858240877762382</v>
       </c>
       <c r="BT2" t="n">
-        <v>0.6050123338270017</v>
+        <v>0.6050542035324588</v>
       </c>
       <c r="BU2" t="n">
-        <v>0.3644842691493443</v>
+        <v>0.3645297172987342</v>
       </c>
       <c r="BV2" t="n">
-        <v>0.1897316660336983</v>
+        <v>0.1897223080794826</v>
       </c>
       <c r="BW2" t="n">
-        <v>0.1606554301282772</v>
+        <v>0.1606323882278846</v>
       </c>
     </row>
     <row r="3">
@@ -1037,52 +1037,52 @@
         <v>0.4</v>
       </c>
       <c r="F3" t="n">
-        <v>1.066429875635743</v>
+        <v>1.066314923944042</v>
       </c>
       <c r="G3" t="n">
-        <v>334.9958456714842</v>
+        <v>335.0078830645102</v>
       </c>
       <c r="H3" t="n">
         <v>0.3311958650192543</v>
       </c>
       <c r="I3" t="n">
-        <v>323.8303009554967</v>
+        <v>323.8328759794524</v>
       </c>
       <c r="J3" t="n">
-        <v>145063.1456357761</v>
+        <v>145066.7039955828</v>
       </c>
       <c r="K3" t="n">
-        <v>37167.53410689608</v>
+        <v>37170.20523407476</v>
       </c>
       <c r="L3" t="n">
-        <v>36424.18342475816</v>
+        <v>36426.80112939327</v>
       </c>
       <c r="M3" t="n">
-        <v>32103.95011371837</v>
+        <v>32106.25733521563</v>
       </c>
       <c r="N3" t="n">
-        <v>36.20694177411348</v>
+        <v>36.20954386619609</v>
       </c>
       <c r="O3" t="n">
-        <v>360.0372427296102</v>
+        <v>360.0424198456485</v>
       </c>
       <c r="P3" t="n">
-        <v>360.0372427296102</v>
+        <v>360.0424198456485</v>
       </c>
       <c r="Q3" t="n">
-        <v>1.389521025919508</v>
+        <v>1.389548910431578</v>
       </c>
       <c r="R3" t="n">
-        <v>201568.2909469347</v>
+        <v>201577.2804769624</v>
       </c>
       <c r="S3" t="n">
-        <v>201568.2909469347</v>
+        <v>201577.2804769624</v>
       </c>
       <c r="T3" t="n">
-        <v>329.5152498904687</v>
+        <v>329.5165600025443</v>
       </c>
       <c r="U3" t="n">
-        <v>347.448539336746</v>
+        <v>347.4510373768453</v>
       </c>
       <c r="V3" t="n">
         <v>0.7615773105863909</v>
@@ -1094,61 +1094,61 @@
         <v>1.064577496794081</v>
       </c>
       <c r="Y3" t="n">
-        <v>146.5606824812743</v>
+        <v>146.5659488407232</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.5085578472919455</v>
+        <v>0.5085740992537762</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.7185450194326043</v>
+        <v>0.71856280975454</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.2868846230922911</v>
+        <v>0.2868716240515501</v>
       </c>
       <c r="AC3" t="n">
         <v>0.425</v>
       </c>
       <c r="AD3" t="n">
-        <v>142.3732344103808</v>
+        <v>142.3783503024168</v>
       </c>
       <c r="AE3" t="n">
-        <v>0.468528766832469</v>
+        <v>0.4685422337951722</v>
       </c>
       <c r="AF3" t="n">
-        <v>0.6733194447626319</v>
+        <v>0.6733351230940104</v>
       </c>
       <c r="AG3" t="n">
-        <v>0.2323217907867172</v>
+        <v>0.2323076911034632</v>
       </c>
       <c r="AH3" t="n">
-        <v>0.506480008400635</v>
+        <v>0.5065406265454202</v>
       </c>
       <c r="AI3" t="n">
-        <v>0.6808006472126222</v>
+        <v>0.6808576637196865</v>
       </c>
       <c r="AJ3" t="n">
-        <v>0.8554208090890487</v>
+        <v>0.8554434984982437</v>
       </c>
       <c r="AK3" t="n">
-        <v>0.2304275261048039</v>
+        <v>0.2304441034541804</v>
       </c>
       <c r="AL3" t="n">
-        <v>1.073179621665038</v>
+        <v>1.073152171295827</v>
       </c>
       <c r="AM3" t="n">
-        <v>0.4661209080755683</v>
+        <v>0.4661419243958083</v>
       </c>
       <c r="AN3" t="n">
-        <v>0.6707463493850978</v>
+        <v>0.6707701249956614</v>
       </c>
       <c r="AO3" t="n">
-        <v>0.233213016100909</v>
+        <v>0.2331960264119508</v>
       </c>
       <c r="AP3" t="n">
-        <v>0.8084990598377197</v>
+        <v>0.8085104045423173</v>
       </c>
       <c r="AQ3" t="n">
-        <v>0.5635107758827498</v>
+        <v>0.5635028689179736</v>
       </c>
       <c r="AR3" t="n">
         <v>0.6314414656442968</v>
@@ -1157,94 +1157,94 @@
         <v>0.43125</v>
       </c>
       <c r="AT3" t="n">
-        <v>1.054171527737041</v>
+        <v>1.054137778695374</v>
       </c>
       <c r="AU3" t="n">
-        <v>0.6532160462166496</v>
+        <v>0.6532228183453691</v>
       </c>
       <c r="AV3" t="n">
-        <v>0.4227300620927443</v>
+        <v>0.4226963130510768</v>
       </c>
       <c r="AW3" t="n">
-        <v>1.07397490693721</v>
+        <v>1.07394476316377</v>
       </c>
       <c r="AX3" t="n">
-        <v>0.4207588607205606</v>
+        <v>0.4207219448184006</v>
       </c>
       <c r="AY3" t="n">
-        <v>156.4429853478237</v>
+        <v>156.4486068076869</v>
       </c>
       <c r="AZ3" t="n">
-        <v>1.776406807110386</v>
+        <v>1.776445439543652</v>
       </c>
       <c r="BA3" t="n">
-        <v>248.2779526487107</v>
+        <v>248.2868740109734</v>
       </c>
       <c r="BB3" t="n">
-        <v>144.4669584458276</v>
+        <v>144.47214957157</v>
       </c>
       <c r="BC3" t="n">
-        <v>166.1511251787695</v>
+        <v>166.160281275451</v>
       </c>
       <c r="BD3" t="n">
-        <v>237.7104076639635</v>
+        <v>237.716845732129</v>
       </c>
       <c r="BE3" t="n">
-        <v>0.9568948193262971</v>
+        <v>0.9568920642613684</v>
       </c>
       <c r="BF3" t="n">
-        <v>309.8715373251904</v>
+        <v>309.8731091716739</v>
       </c>
       <c r="BG3" t="n">
-        <v>353.1004272981889</v>
+        <v>353.1013228611792</v>
       </c>
       <c r="BH3" t="n">
-        <v>0.7031369362774604</v>
+        <v>0.7031604186557712</v>
       </c>
       <c r="BI3" t="n">
-        <v>0.6841600431469231</v>
+        <v>0.684173653723478</v>
       </c>
       <c r="BJ3" t="n">
-        <v>360.0372427296102</v>
+        <v>360.0424198456485</v>
       </c>
       <c r="BK3" t="n">
-        <v>0.9219875058935334</v>
+        <v>0.9219844019251111</v>
       </c>
       <c r="BL3" t="n">
-        <v>653.7986833101451</v>
+        <v>667.0197977500453</v>
       </c>
       <c r="BM3" t="n">
-        <v>512.8961280967814</v>
+        <v>518.0560643624474</v>
       </c>
       <c r="BN3" t="n">
-        <v>0.4634669568398624</v>
+        <v>0.4588631657553867</v>
       </c>
       <c r="BO3" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.2975897333830798</v>
       </c>
       <c r="BP3" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.2231923000373098</v>
       </c>
       <c r="BQ3" t="n">
-        <v>0.5543838557506463</v>
+        <v>0.5544169446421737</v>
       </c>
       <c r="BR3" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5665939720200175</v>
       </c>
       <c r="BS3" t="n">
-        <v>0.6014809361522618</v>
+        <v>0.6015109893129853</v>
       </c>
       <c r="BT3" t="n">
-        <v>0.6363882589526815</v>
+        <v>0.6364280066059533</v>
       </c>
       <c r="BU3" t="n">
-        <v>0.412432539638981</v>
+        <v>0.4124719768478154</v>
       </c>
       <c r="BV3" t="n">
-        <v>0.1657575307888799</v>
+        <v>0.165751178304942</v>
       </c>
       <c r="BW3" t="n">
-        <v>0.1187337964080529</v>
+        <v>0.1187168534561396</v>
       </c>
     </row>
     <row r="4">
@@ -1264,52 +1264,52 @@
         <v>0.4</v>
       </c>
       <c r="F4" t="n">
-        <v>1.066429875635743</v>
+        <v>1.066314923944042</v>
       </c>
       <c r="G4" t="n">
-        <v>334.9958456714842</v>
+        <v>335.0078830645102</v>
       </c>
       <c r="H4" t="n">
         <v>0.3375197589886442</v>
       </c>
       <c r="I4" t="n">
-        <v>360.0372427296102</v>
+        <v>360.0424198456485</v>
       </c>
       <c r="J4" t="n">
-        <v>201568.2909469347</v>
+        <v>201577.2804769624</v>
       </c>
       <c r="K4" t="n">
-        <v>37877.21550579287</v>
+        <v>37879.93763579749</v>
       </c>
       <c r="L4" t="n">
-        <v>36740.89904061908</v>
+        <v>36743.53950672357</v>
       </c>
       <c r="M4" t="n">
-        <v>32245.28409192084</v>
+        <v>32247.60147069756</v>
       </c>
       <c r="N4" t="n">
-        <v>36.52176843003885</v>
+        <v>36.52439314783655</v>
       </c>
       <c r="O4" t="n">
-        <v>396.559011159649</v>
+        <v>396.5668129934851</v>
       </c>
       <c r="P4" t="n">
-        <v>396.559011159649</v>
+        <v>396.5668129934851</v>
       </c>
       <c r="Q4" t="n">
-        <v>1.347829621392633</v>
+        <v>1.347851790972096</v>
       </c>
       <c r="R4" t="n">
-        <v>271679.7132717671</v>
+        <v>271696.2985101583</v>
       </c>
       <c r="S4" t="n">
-        <v>271679.7132717671</v>
+        <v>271696.2985101583</v>
       </c>
       <c r="T4" t="n">
-        <v>347.448539336746</v>
+        <v>347.4510373768453</v>
       </c>
       <c r="U4" t="n">
-        <v>364.6453570825088</v>
+        <v>364.6489440499116</v>
       </c>
       <c r="V4" t="n">
         <v>0.7615773105863909</v>
@@ -1321,61 +1321,61 @@
         <v>1.064577496794081</v>
       </c>
       <c r="Y4" t="n">
-        <v>142.3732344103808</v>
+        <v>142.3783503024168</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.468528766832469</v>
+        <v>0.4685422337951722</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.6733194447626319</v>
+        <v>0.6733351230940104</v>
       </c>
       <c r="AB4" t="n">
-        <v>0.2323217907867172</v>
+        <v>0.2323076911034632</v>
       </c>
       <c r="AC4" t="n">
         <v>0.4125</v>
       </c>
       <c r="AD4" t="n">
-        <v>138.1857863394872</v>
+        <v>138.1907517641105</v>
       </c>
       <c r="AE4" t="n">
-        <v>0.4333023913326854</v>
+        <v>0.433313698722434</v>
       </c>
       <c r="AF4" t="n">
-        <v>0.6312866578179296</v>
+        <v>0.6313004709116813</v>
       </c>
       <c r="AG4" t="n">
-        <v>0.1929432963141447</v>
+        <v>0.1929291948039231</v>
       </c>
       <c r="AH4" t="n">
-        <v>0.558190666335634</v>
+        <v>0.5582446206577484</v>
       </c>
       <c r="AI4" t="n">
-        <v>0.750309115081092</v>
+        <v>0.7503546769728567</v>
       </c>
       <c r="AJ4" t="n">
-        <v>0.8840146401994062</v>
+        <v>0.8840339759463548</v>
       </c>
       <c r="AK4" t="n">
-        <v>0.2478040511669324</v>
+        <v>0.2478179666885366</v>
       </c>
       <c r="AL4" t="n">
-        <v>1.032320478025595</v>
+        <v>1.032297001042157</v>
       </c>
       <c r="AM4" t="n">
-        <v>0.4420825865074373</v>
+        <v>0.4421007066056573</v>
       </c>
       <c r="AN4" t="n">
-        <v>0.6411568471991366</v>
+        <v>0.6411782534948469</v>
       </c>
       <c r="AO4" t="n">
-        <v>0.1899730607426552</v>
+        <v>0.1899569906940193</v>
       </c>
       <c r="AP4" t="n">
-        <v>0.8227959753928986</v>
+        <v>0.8228056432663728</v>
       </c>
       <c r="AQ4" t="n">
-        <v>0.5575621335231457</v>
+        <v>0.5575555822309844</v>
       </c>
       <c r="AR4" t="n">
         <v>0.614429921562137</v>
@@ -1384,94 +1384,94 @@
         <v>0.41875</v>
       </c>
       <c r="AT4" t="n">
-        <v>1.006183457466621</v>
+        <v>1.006155815458483</v>
       </c>
       <c r="AU4" t="n">
-        <v>0.6441646969371893</v>
+        <v>0.6441703391036353</v>
       </c>
       <c r="AV4" t="n">
-        <v>0.3917535359044838</v>
+        <v>0.3917258938963463</v>
       </c>
       <c r="AW4" t="n">
-        <v>1.029835022076156</v>
+        <v>1.029810233725864</v>
       </c>
       <c r="AX4" t="n">
-        <v>0.3856703251389664</v>
+        <v>0.3856398946222284</v>
       </c>
       <c r="AY4" t="n">
-        <v>152.0336456146226</v>
+        <v>152.0391086338483</v>
       </c>
       <c r="AZ4" t="n">
-        <v>2.19436222248338</v>
+        <v>2.194437865938998</v>
       </c>
       <c r="BA4" t="n">
-        <v>246.9644608130197</v>
+        <v>246.9733349776299</v>
       </c>
       <c r="BB4" t="n">
-        <v>140.279510374934</v>
+        <v>140.2845510332637</v>
       </c>
       <c r="BC4" t="n">
-        <v>166.0513797701721</v>
+        <v>166.0602539824661</v>
       </c>
       <c r="BD4" t="n">
-        <v>233.5925564032956</v>
+        <v>233.5991951661016</v>
       </c>
       <c r="BE4" t="n">
-        <v>0.9634134657750744</v>
+        <v>0.9634113625250383</v>
       </c>
       <c r="BF4" t="n">
-        <v>346.8647278262354</v>
+        <v>346.8689582703082</v>
       </c>
       <c r="BG4" t="n">
-        <v>373.5833131821657</v>
+        <v>373.5855913303418</v>
       </c>
       <c r="BH4" t="n">
-        <v>0.6610693039509383</v>
+        <v>0.6610890267425882</v>
       </c>
       <c r="BI4" t="n">
-        <v>0.6406020311687126</v>
+        <v>0.6406139356161896</v>
       </c>
       <c r="BJ4" t="n">
-        <v>396.559011159649</v>
+        <v>396.5668129934851</v>
       </c>
       <c r="BK4" t="n">
-        <v>0.93160483961042</v>
+        <v>0.9316022975823894</v>
       </c>
       <c r="BL4" t="n">
-        <v>660.6185155539247</v>
+        <v>673.9779705810646</v>
       </c>
       <c r="BM4" t="n">
-        <v>515.5642209446628</v>
+        <v>520.7511653784341</v>
       </c>
       <c r="BN4" t="n">
-        <v>0.4530813949332761</v>
+        <v>0.4485812240023375</v>
       </c>
       <c r="BO4" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.2975897333830798</v>
       </c>
       <c r="BP4" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.2231923000373098</v>
       </c>
       <c r="BQ4" t="n">
-        <v>0.5949675909202978</v>
+        <v>0.5949943303780122</v>
       </c>
       <c r="BR4" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5665939720200175</v>
       </c>
       <c r="BS4" t="n">
-        <v>0.6121170921843355</v>
+        <v>0.6121462800143332</v>
       </c>
       <c r="BT4" t="n">
-        <v>0.6576605710168285</v>
+        <v>0.6576985880086491</v>
       </c>
       <c r="BU4" t="n">
-        <v>0.4426247120668587</v>
+        <v>0.4426605103540918</v>
       </c>
       <c r="BV4" t="n">
-        <v>0.1506614445749411</v>
+        <v>0.1506569115518038</v>
       </c>
       <c r="BW4" t="n">
-        <v>0.09287846744055345</v>
+        <v>0.09286485639997549</v>
       </c>
     </row>
     <row r="5">
@@ -1491,52 +1491,52 @@
         <v>0.4</v>
       </c>
       <c r="F5" t="n">
-        <v>1.066429875635743</v>
+        <v>1.066314923944042</v>
       </c>
       <c r="G5" t="n">
-        <v>334.9958456714842</v>
+        <v>335.0078830645102</v>
       </c>
       <c r="H5" t="n">
         <v>0.3433570658223036</v>
       </c>
       <c r="I5" t="n">
-        <v>396.559011159649</v>
+        <v>396.5668129934851</v>
       </c>
       <c r="J5" t="n">
-        <v>271679.7132717671</v>
+        <v>271696.2985101583</v>
       </c>
       <c r="K5" t="n">
-        <v>38532.29101774057</v>
+        <v>38535.0602261981</v>
       </c>
       <c r="L5" t="n">
-        <v>36990.99937703094</v>
+        <v>36993.65781715018</v>
       </c>
       <c r="M5" t="n">
-        <v>32290.71392257523</v>
+        <v>32293.03456626737</v>
       </c>
       <c r="N5" t="n">
-        <v>36.77037711434487</v>
+        <v>36.77301969895644</v>
       </c>
       <c r="O5" t="n">
-        <v>433.3293882739939</v>
+        <v>433.3398326924415</v>
       </c>
       <c r="P5" t="n">
-        <v>433.3293882739939</v>
+        <v>433.3398326924415</v>
       </c>
       <c r="Q5" t="n">
-        <v>1.313130303218921</v>
+        <v>1.313148265212468</v>
       </c>
       <c r="R5" t="n">
-        <v>356750.8642669851</v>
+        <v>356777.5230532631</v>
       </c>
       <c r="S5" t="n">
-        <v>356750.8642669851</v>
+        <v>356777.5230532631</v>
       </c>
       <c r="T5" t="n">
-        <v>364.6453570825088</v>
+        <v>364.6489440499116</v>
       </c>
       <c r="U5" t="n">
-        <v>381.1762635425639</v>
+        <v>381.1808572079344</v>
       </c>
       <c r="V5" t="n">
         <v>0.7615773105863909</v>
@@ -1548,61 +1548,61 @@
         <v>1.064577496794081</v>
       </c>
       <c r="Y5" t="n">
-        <v>138.1857863394872</v>
+        <v>138.1907517641105</v>
       </c>
       <c r="Z5" t="n">
-        <v>0.4333023913326854</v>
+        <v>0.433313698722434</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.6312866578179296</v>
+        <v>0.6313004709116813</v>
       </c>
       <c r="AB5" t="n">
-        <v>0.1929432963141447</v>
+        <v>0.1929291948039231</v>
       </c>
       <c r="AC5" t="n">
         <v>0.4</v>
       </c>
       <c r="AD5" t="n">
-        <v>133.9983382685937</v>
+        <v>134.0031532258041</v>
       </c>
       <c r="AE5" t="n">
-        <v>0.4019499360408819</v>
+        <v>0.4019595351621132</v>
       </c>
       <c r="AF5" t="n">
-        <v>0.5922271443277999</v>
+        <v>0.5922393305795842</v>
       </c>
       <c r="AG5" t="n">
-        <v>0.1637251255561614</v>
+        <v>0.1637114961067456</v>
       </c>
       <c r="AH5" t="n">
-        <v>0.5931253835185788</v>
+        <v>0.5931749205201829</v>
       </c>
       <c r="AI5" t="n">
-        <v>0.7972676873324286</v>
+        <v>0.7973056244606448</v>
       </c>
       <c r="AJ5" t="n">
-        <v>0.9043328384130478</v>
+        <v>0.9043495615072135</v>
       </c>
       <c r="AK5" t="n">
-        <v>0.2594013382727521</v>
+        <v>0.2594132644023123</v>
       </c>
       <c r="AL5" t="n">
-        <v>0.9997621798616013</v>
+        <v>0.9997416754265532</v>
       </c>
       <c r="AM5" t="n">
-        <v>0.4189892047782126</v>
+        <v>0.4190049139530834</v>
       </c>
       <c r="AN5" t="n">
-        <v>0.6121999974112641</v>
+        <v>0.612219282890097</v>
       </c>
       <c r="AO5" t="n">
-        <v>0.1583836392892018</v>
+        <v>0.1583687243641531</v>
       </c>
       <c r="AP5" t="n">
-        <v>0.8329550744997194</v>
+        <v>0.8329634360468021</v>
       </c>
       <c r="AQ5" t="n">
-        <v>0.5542658266274929</v>
+        <v>0.5542602627340431</v>
       </c>
       <c r="AR5" t="n">
         <v>0.5974865025033296</v>
@@ -1611,94 +1611,94 @@
         <v>0.40625</v>
       </c>
       <c r="AT5" t="n">
-        <v>0.9695253360656676</v>
+        <v>0.96950202760993</v>
       </c>
       <c r="AU5" t="n">
-        <v>0.6325005241171194</v>
+        <v>0.6325053104549879</v>
       </c>
       <c r="AV5" t="n">
-        <v>0.372038833562338</v>
+        <v>0.3720155251066004</v>
       </c>
       <c r="AW5" t="n">
-        <v>0.9954739554152893</v>
+        <v>0.9954529672207285</v>
       </c>
       <c r="AX5" t="n">
-        <v>0.3629734312981698</v>
+        <v>0.3629476567657406</v>
       </c>
       <c r="AY5" t="n">
-        <v>147.6621745217523</v>
+        <v>147.667480461073</v>
       </c>
       <c r="AZ5" t="n">
-        <v>2.659616017028643</v>
+        <v>2.659735625266538</v>
       </c>
       <c r="BA5" t="n">
-        <v>245.6347060214273</v>
+        <v>245.6435324040091</v>
       </c>
       <c r="BB5" t="n">
-        <v>136.0920623040405</v>
+        <v>136.0969524949573</v>
       </c>
       <c r="BC5" t="n">
-        <v>165.0366338893982</v>
+        <v>165.0452032127793</v>
       </c>
       <c r="BD5" t="n">
-        <v>230.2105659161242</v>
+        <v>230.2173346955283</v>
       </c>
       <c r="BE5" t="n">
-        <v>0.9687081729442294</v>
+        <v>0.9687065397499139</v>
       </c>
       <c r="BF5" t="n">
-        <v>384.1499551650339</v>
+        <v>384.1568651945702</v>
       </c>
       <c r="BG5" t="n">
-        <v>393.1495592776405</v>
+        <v>393.1530952182461</v>
       </c>
       <c r="BH5" t="n">
-        <v>0.6247869296171872</v>
+        <v>0.6248037606511738</v>
       </c>
       <c r="BI5" t="n">
-        <v>0.603947800360391</v>
+        <v>0.6039582794944622</v>
       </c>
       <c r="BJ5" t="n">
-        <v>433.3293882739939</v>
+        <v>433.3398326924415</v>
       </c>
       <c r="BK5" t="n">
-        <v>0.9392078424066409</v>
+        <v>0.9392057327716815</v>
       </c>
       <c r="BL5" t="n">
-        <v>666.0099478516489</v>
+        <v>679.478759739295</v>
       </c>
       <c r="BM5" t="n">
-        <v>517.6637543981512</v>
+        <v>522.871947773738</v>
       </c>
       <c r="BN5" t="n">
-        <v>0.4447106137144423</v>
+        <v>0.4402939107285023</v>
       </c>
       <c r="BO5" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.2975897333830798</v>
       </c>
       <c r="BP5" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.2231923000373098</v>
       </c>
       <c r="BQ5" t="n">
-        <v>0.6225980342642162</v>
+        <v>0.6226204072962837</v>
       </c>
       <c r="BR5" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5665939720200175</v>
       </c>
       <c r="BS5" t="n">
-        <v>0.619674929595378</v>
+        <v>0.6197034171275546</v>
       </c>
       <c r="BT5" t="n">
-        <v>0.6727762458389134</v>
+        <v>0.6728128622350918</v>
       </c>
       <c r="BU5" t="n">
-        <v>0.4631803141131219</v>
+        <v>0.4632136025154139</v>
       </c>
       <c r="BV5" t="n">
-        <v>0.1403836435518095</v>
+        <v>0.1403803654711427</v>
       </c>
       <c r="BW5" t="n">
-        <v>0.07541110884908103</v>
+        <v>0.07539970646875821</v>
       </c>
     </row>
     <row r="6">
@@ -1718,52 +1718,52 @@
         <v>0.4</v>
       </c>
       <c r="F6" t="n">
-        <v>1.066429875635743</v>
+        <v>1.066314923944042</v>
       </c>
       <c r="G6" t="n">
-        <v>334.9958456714842</v>
+        <v>335.0078830645102</v>
       </c>
       <c r="H6" t="n">
         <v>0.3486475855755174</v>
       </c>
       <c r="I6" t="n">
-        <v>433.3293882739939</v>
+        <v>433.3398326924415</v>
       </c>
       <c r="J6" t="n">
-        <v>356750.8642669851</v>
+        <v>356777.5230532631</v>
       </c>
       <c r="K6" t="n">
-        <v>39126.00487150306</v>
+        <v>39128.81674852199</v>
       </c>
       <c r="L6" t="n">
-        <v>37169.7046279279</v>
+        <v>37172.37591109589</v>
       </c>
       <c r="M6" t="n">
-        <v>32235.74117928013</v>
+        <v>32238.05787223429</v>
       </c>
       <c r="N6" t="n">
-        <v>36.94801652875537</v>
+        <v>36.95067187981698</v>
       </c>
       <c r="O6" t="n">
-        <v>470.2774048027492</v>
+        <v>470.2905045722585</v>
       </c>
       <c r="P6" t="n">
-        <v>470.2774048027492</v>
+        <v>470.2905045722585</v>
       </c>
       <c r="Q6" t="n">
-        <v>1.28363103095909</v>
+        <v>1.2836458064987</v>
       </c>
       <c r="R6" t="n">
-        <v>457936.4796945766</v>
+        <v>457975.9713203143</v>
       </c>
       <c r="S6" t="n">
-        <v>457936.4796945766</v>
+        <v>457975.9713203143</v>
       </c>
       <c r="T6" t="n">
-        <v>381.1762635425639</v>
+        <v>381.1808572079344</v>
       </c>
       <c r="U6" t="n">
-        <v>397.0944646181332</v>
+        <v>397.0999951940044</v>
       </c>
       <c r="V6" t="n">
         <v>0.7615773105863909</v>
@@ -1775,61 +1775,61 @@
         <v>1.064577496794081</v>
       </c>
       <c r="Y6" t="n">
-        <v>133.9983382685937</v>
+        <v>134.0031532258041</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.4019499360408819</v>
+        <v>0.4019595351621132</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.5922271443277999</v>
+        <v>0.5922393305795842</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.1637251255561614</v>
+        <v>0.1637114961067456</v>
       </c>
       <c r="AC6" t="n">
         <v>0.3875</v>
       </c>
       <c r="AD6" t="n">
-        <v>129.8108901977001</v>
+        <v>129.8155546874977</v>
       </c>
       <c r="AE6" t="n">
-        <v>0.3737796859822607</v>
+        <v>0.3737879110222118</v>
       </c>
       <c r="AF6" t="n">
-        <v>0.5558891806916422</v>
+        <v>0.5558999548939522</v>
       </c>
       <c r="AG6" t="n">
-        <v>0.1415608615306941</v>
+        <v>0.1415478825907238</v>
       </c>
       <c r="AH6" t="n">
-        <v>0.6180530627448302</v>
+        <v>0.6180994052132663</v>
       </c>
       <c r="AI6" t="n">
-        <v>0.8307749923973037</v>
+        <v>0.8308074316765526</v>
       </c>
       <c r="AJ6" t="n">
-        <v>0.9192896953607008</v>
+        <v>0.9193043534458514</v>
       </c>
       <c r="AK6" t="n">
-        <v>0.2674717268010952</v>
+        <v>0.2674821199975156</v>
       </c>
       <c r="AL6" t="n">
-        <v>0.9720262250235825</v>
+        <v>0.9720080062570743</v>
       </c>
       <c r="AM6" t="n">
-        <v>0.3972152038601151</v>
+        <v>0.3972289254972216</v>
       </c>
       <c r="AN6" t="n">
-        <v>0.5843288480641364</v>
+        <v>0.5843462737166659</v>
       </c>
       <c r="AO6" t="n">
-        <v>0.1346710017740956</v>
+        <v>0.1346572487697094</v>
       </c>
       <c r="AP6" t="n">
-        <v>0.8404335029735459</v>
+        <v>0.8404408320161212</v>
       </c>
       <c r="AQ6" t="n">
-        <v>0.5524812982168491</v>
+        <v>0.5524764803179532</v>
       </c>
       <c r="AR6" t="n">
         <v>0.5806335590240905</v>
@@ -1838,94 +1838,94 @@
         <v>0.39375</v>
       </c>
       <c r="AT6" t="n">
-        <v>0.9393663462540609</v>
+        <v>0.9393462467514107</v>
       </c>
       <c r="AU6" t="n">
-        <v>0.6191945916757878</v>
+        <v>0.619198713255527</v>
       </c>
       <c r="AV6" t="n">
-        <v>0.3587327872299704</v>
+        <v>0.3587126877273201</v>
       </c>
       <c r="AW6" t="n">
-        <v>0.9666442621479878</v>
+        <v>0.9666260963347023</v>
       </c>
       <c r="AX6" t="n">
-        <v>0.3474496704722</v>
+        <v>0.3474273830791753</v>
       </c>
       <c r="AY6" t="n">
-        <v>143.3338608703159</v>
+        <v>143.3390112805062</v>
       </c>
       <c r="AZ6" t="n">
-        <v>3.169793873235574</v>
+        <v>3.169964142308014</v>
       </c>
       <c r="BA6" t="n">
-        <v>244.2756650661178</v>
+        <v>244.2844426143324</v>
       </c>
       <c r="BB6" t="n">
-        <v>131.9046142331469</v>
+        <v>131.9093539566509</v>
       </c>
       <c r="BC6" t="n">
-        <v>163.4132722977984</v>
+        <v>163.4215463724512</v>
       </c>
       <c r="BD6" t="n">
-        <v>227.2730542356306</v>
+        <v>227.2799064491204</v>
       </c>
       <c r="BE6" t="n">
-        <v>0.9730727081527885</v>
+        <v>0.9730714220153763</v>
       </c>
       <c r="BF6" t="n">
-        <v>421.6610013699664</v>
+        <v>421.6706072139393</v>
       </c>
       <c r="BG6" t="n">
-        <v>411.8974635892041</v>
+        <v>411.9021552730704</v>
       </c>
       <c r="BH6" t="n">
-        <v>0.5930496947894299</v>
+        <v>0.5930642495725328</v>
       </c>
       <c r="BI6" t="n">
-        <v>0.572340021043074</v>
+        <v>0.5723493054641869</v>
       </c>
       <c r="BJ6" t="n">
-        <v>470.2774048027492</v>
+        <v>470.2905045722585</v>
       </c>
       <c r="BK6" t="n">
-        <v>0.9454044833854023</v>
+        <v>0.9454027120891105</v>
       </c>
       <c r="BL6" t="n">
-        <v>670.4041025304953</v>
+        <v>683.9620328644605</v>
       </c>
       <c r="BM6" t="n">
-        <v>519.368650087941</v>
+        <v>524.5940940797411</v>
       </c>
       <c r="BN6" t="n">
-        <v>0.437594864836659</v>
+        <v>0.4332490758360932</v>
       </c>
       <c r="BO6" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.2975897333830798</v>
       </c>
       <c r="BP6" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.2231923000373098</v>
       </c>
       <c r="BQ6" t="n">
-        <v>0.6423837994849889</v>
+        <v>0.6424029765185557</v>
       </c>
       <c r="BR6" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5665939720200175</v>
       </c>
       <c r="BS6" t="n">
-        <v>0.6252384885193522</v>
+        <v>0.625266407809828</v>
       </c>
       <c r="BT6" t="n">
-        <v>0.6839033636868619</v>
+        <v>0.6839388435996385</v>
       </c>
       <c r="BU6" t="n">
-        <v>0.4778998866873533</v>
+        <v>0.4779313262666346</v>
       </c>
       <c r="BV6" t="n">
-        <v>0.1330238572646938</v>
+        <v>0.1330215035955324</v>
       </c>
       <c r="BW6" t="n">
-        <v>0.06294726923595534</v>
+        <v>0.06293746412221651</v>
       </c>
     </row>
     <row r="7">
@@ -1945,52 +1945,52 @@
         <v>0.4</v>
       </c>
       <c r="F7" t="n">
-        <v>1.066429875635743</v>
+        <v>1.066314923944042</v>
       </c>
       <c r="G7" t="n">
-        <v>334.9958456714842</v>
+        <v>335.0078830645102</v>
       </c>
       <c r="H7" t="n">
         <v>0.3533255394992114</v>
       </c>
       <c r="I7" t="n">
-        <v>470.2774048027492</v>
+        <v>470.2905045722585</v>
       </c>
       <c r="J7" t="n">
-        <v>457936.4796945766</v>
+        <v>457975.9713203143</v>
       </c>
       <c r="K7" t="n">
-        <v>39650.97523005291</v>
+        <v>39653.82483522966</v>
       </c>
       <c r="L7" t="n">
-        <v>37271.91671624973</v>
+        <v>37274.59534511588</v>
       </c>
       <c r="M7" t="n">
-        <v>32076.10721762385</v>
+        <v>32078.4124381297</v>
       </c>
       <c r="N7" t="n">
-        <v>37.04961900223631</v>
+        <v>37.05228165518477</v>
       </c>
       <c r="O7" t="n">
-        <v>507.3270238049855</v>
+        <v>507.3427862274433</v>
       </c>
       <c r="P7" t="n">
-        <v>507.3270238049855</v>
+        <v>507.3427862274433</v>
       </c>
       <c r="Q7" t="n">
-        <v>1.258098598953983</v>
+        <v>1.258110903936187</v>
       </c>
       <c r="R7" t="n">
-        <v>576129.2435136657</v>
+        <v>576184.5632588541</v>
       </c>
       <c r="S7" t="n">
-        <v>576129.2435136657</v>
+        <v>576184.5632588541</v>
       </c>
       <c r="T7" t="n">
-        <v>397.0944646181332</v>
+        <v>397.0999951940044</v>
       </c>
       <c r="U7" t="n">
-        <v>412.4399969472064</v>
+        <v>412.4464040600448</v>
       </c>
       <c r="V7" t="n">
         <v>0.7615773105863909</v>
@@ -2002,61 +2002,61 @@
         <v>1.064577496794081</v>
       </c>
       <c r="Y7" t="n">
-        <v>129.8108901977001</v>
+        <v>129.8155546874977</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.3737796859822607</v>
+        <v>0.3737879110222118</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.5558891806916422</v>
+        <v>0.5558999548939522</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.1415608615306941</v>
+        <v>0.1415478825907238</v>
       </c>
       <c r="AC7" t="n">
         <v>0.375</v>
       </c>
       <c r="AD7" t="n">
-        <v>125.6234421268066</v>
+        <v>125.6279561491913</v>
       </c>
       <c r="AE7" t="n">
-        <v>0.3482637835623633</v>
+        <v>0.3482708874438034</v>
       </c>
       <c r="AF7" t="n">
-        <v>0.5220220244246978</v>
+        <v>0.5220315741413367</v>
       </c>
       <c r="AG7" t="n">
-        <v>0.1244499868451066</v>
+        <v>0.1244376950200846</v>
       </c>
       <c r="AH7" t="n">
-        <v>0.6365266021211494</v>
+        <v>0.6365705205435771</v>
       </c>
       <c r="AI7" t="n">
-        <v>0.8556067673047103</v>
+        <v>0.8556350560980354</v>
       </c>
       <c r="AJ7" t="n">
-        <v>0.9306081184520197</v>
+        <v>0.930621123020504</v>
       </c>
       <c r="AK7" t="n">
-        <v>0.2733222986142951</v>
+        <v>0.273331483665876</v>
       </c>
       <c r="AL7" t="n">
-        <v>0.94708331955606</v>
+        <v>0.9470668963058015</v>
       </c>
       <c r="AM7" t="n">
-        <v>0.3769042166111551</v>
+        <v>0.3769162990695156</v>
       </c>
       <c r="AN7" t="n">
-        <v>0.5577971839788439</v>
+        <v>0.5578129944380164</v>
       </c>
       <c r="AO7" t="n">
-        <v>0.1164682001603178</v>
+        <v>0.1164555262454946</v>
       </c>
       <c r="AP7" t="n">
-        <v>0.8460927145192053</v>
+        <v>0.8460992168034475</v>
       </c>
       <c r="AQ7" t="n">
-        <v>0.5515503936407113</v>
+        <v>0.5515461549682696</v>
       </c>
       <c r="AR7" t="n">
         <v>0.5638932886886516</v>
@@ -2065,94 +2065,94 @@
         <v>0.38125</v>
       </c>
       <c r="AT7" t="n">
-        <v>0.913006188823837</v>
+        <v>0.9129885463637443</v>
       </c>
       <c r="AU7" t="n">
-        <v>0.6048180107391227</v>
+        <v>0.6048216053748368</v>
       </c>
       <c r="AV7" t="n">
-        <v>0.3491129001351854</v>
+        <v>0.3490952576750926</v>
       </c>
       <c r="AW7" t="n">
-        <v>0.9409630125541549</v>
+        <v>0.9409470168595313</v>
       </c>
       <c r="AX7" t="n">
-        <v>0.3361450018150323</v>
+        <v>0.3361254114846945</v>
       </c>
       <c r="AY7" t="n">
-        <v>139.0549019493772</v>
+        <v>139.0598986038987</v>
       </c>
       <c r="AZ7" t="n">
-        <v>3.721602002135425</v>
+        <v>3.721829246247244</v>
       </c>
       <c r="BA7" t="n">
-        <v>242.8728905954796</v>
+        <v>242.8816177378524</v>
       </c>
       <c r="BB7" t="n">
-        <v>127.7171661622534</v>
+        <v>127.7217554183445</v>
       </c>
       <c r="BC7" t="n">
-        <v>161.3924812349645</v>
+        <v>161.400480464318</v>
       </c>
       <c r="BD7" t="n">
-        <v>224.6120038691836</v>
+        <v>224.618906754626</v>
       </c>
       <c r="BE7" t="n">
-        <v>0.9767147910578338</v>
+        <v>0.9767137662622751</v>
       </c>
       <c r="BF7" t="n">
-        <v>459.3268971711375</v>
+        <v>459.3392099581563</v>
       </c>
       <c r="BG7" t="n">
-        <v>429.900884327747</v>
+        <v>429.9066462835435</v>
       </c>
       <c r="BH7" t="n">
-        <v>0.5649508978686322</v>
+        <v>0.5649636260279184</v>
       </c>
       <c r="BI7" t="n">
-        <v>0.5445931663556255</v>
+        <v>0.544601442862684</v>
       </c>
       <c r="BJ7" t="n">
-        <v>507.3270238049855</v>
+        <v>507.3427862274433</v>
       </c>
       <c r="BK7" t="n">
-        <v>0.9505697138597924</v>
+        <v>0.9505682114053138</v>
       </c>
       <c r="BL7" t="n">
-        <v>674.066864619529</v>
+        <v>687.6990703913186</v>
       </c>
       <c r="BM7" t="n">
-        <v>520.7855063731264</v>
+        <v>526.0252826268438</v>
       </c>
       <c r="BN7" t="n">
-        <v>0.4312946522522004</v>
+        <v>0.4270116174510342</v>
       </c>
       <c r="BO7" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.2975897333830798</v>
       </c>
       <c r="BP7" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.2231923000373098</v>
       </c>
       <c r="BQ7" t="n">
-        <v>0.6570736359990065</v>
+        <v>0.6570903814170578</v>
       </c>
       <c r="BR7" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5665939720200175</v>
       </c>
       <c r="BS7" t="n">
-        <v>0.6294486453735235</v>
+        <v>0.6294761008604263</v>
       </c>
       <c r="BT7" t="n">
-        <v>0.6923236773952047</v>
+        <v>0.6923582297008352</v>
       </c>
       <c r="BU7" t="n">
-        <v>0.4888283553242228</v>
+        <v>0.488858378536221</v>
       </c>
       <c r="BV7" t="n">
-        <v>0.127559622946259</v>
+        <v>0.1275579774607392</v>
       </c>
       <c r="BW7" t="n">
-        <v>0.05371049954779572</v>
+        <v>0.05370190645706113</v>
       </c>
     </row>
     <row r="8">
@@ -2172,52 +2172,52 @@
         <v>0.4</v>
       </c>
       <c r="F8" t="n">
-        <v>1.066429875635743</v>
+        <v>1.066314923944042</v>
       </c>
       <c r="G8" t="n">
-        <v>334.9958456714842</v>
+        <v>335.0078830645102</v>
       </c>
       <c r="H8" t="n">
         <v>0.3573195700399479</v>
       </c>
       <c r="I8" t="n">
-        <v>507.3270238049855</v>
+        <v>507.3427862274433</v>
       </c>
       <c r="J8" t="n">
-        <v>576129.2435136657</v>
+        <v>576184.5632588541</v>
       </c>
       <c r="K8" t="n">
-        <v>40099.19419057097</v>
+        <v>40102.07600799629</v>
       </c>
       <c r="L8" t="n">
-        <v>37693.24253913671</v>
+        <v>37695.95144751651</v>
       </c>
       <c r="M8" t="n">
-        <v>32149.91062885868</v>
+        <v>32152.22115341019</v>
       </c>
       <c r="N8" t="n">
-        <v>37.468431947452</v>
+        <v>37.47112469932059</v>
       </c>
       <c r="O8" t="n">
-        <v>544.7954557524375</v>
+        <v>544.8139109267639</v>
       </c>
       <c r="P8" t="n">
-        <v>544.7954557524375</v>
+        <v>544.8139109267639</v>
       </c>
       <c r="Q8" t="n">
-        <v>1.238387978501664</v>
+        <v>1.238398457293167</v>
       </c>
       <c r="R8" t="n">
-        <v>713471.5292305814</v>
+        <v>713546.0742559022</v>
       </c>
       <c r="S8" t="n">
-        <v>713471.5292305814</v>
+        <v>713546.0742559022</v>
       </c>
       <c r="T8" t="n">
-        <v>412.4399969472064</v>
+        <v>412.4464040600448</v>
       </c>
       <c r="U8" t="n">
-        <v>427.3990130004892</v>
+        <v>427.406252099503</v>
       </c>
       <c r="V8" t="n">
         <v>0.7615773105863909</v>
@@ -2229,61 +2229,61 @@
         <v>1.064577496794081</v>
       </c>
       <c r="Y8" t="n">
-        <v>125.6234421268066</v>
+        <v>125.6279561491913</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.3482637835623633</v>
+        <v>0.3482708874438034</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.5220220244246978</v>
+        <v>0.5220315741413367</v>
       </c>
       <c r="AB8" t="n">
-        <v>0.1244499868451067</v>
+        <v>0.1244376950200846</v>
       </c>
       <c r="AC8" t="n">
         <v>0.3625</v>
       </c>
       <c r="AD8" t="n">
-        <v>121.435994055913</v>
+        <v>121.440357610885</v>
       </c>
       <c r="AE8" t="n">
-        <v>0.3248720262443578</v>
+        <v>0.3248781972126394</v>
       </c>
       <c r="AF8" t="n">
-        <v>0.4902267786136445</v>
+        <v>0.4902352568247675</v>
       </c>
       <c r="AG8" t="n">
-        <v>0.1108926247734101</v>
+        <v>0.1108810001132414</v>
       </c>
       <c r="AH8" t="n">
-        <v>0.6507693397424607</v>
+        <v>0.6508113381307393</v>
       </c>
       <c r="AI8" t="n">
-        <v>0.874751580189404</v>
+        <v>0.8747766002975195</v>
       </c>
       <c r="AJ8" t="n">
-        <v>0.939465360469416</v>
+        <v>0.9394770088799635</v>
       </c>
       <c r="AK8" t="n">
-        <v>0.2778401656135346</v>
+        <v>0.2778483690604185</v>
       </c>
       <c r="AL8" t="n">
-        <v>0.9235220626756799</v>
+        <v>0.9235070974918138</v>
       </c>
       <c r="AM8" t="n">
-        <v>0.3579847479308438</v>
+        <v>0.3579954594465656</v>
       </c>
       <c r="AN8" t="n">
-        <v>0.532609775801597</v>
+        <v>0.5326241746744999</v>
       </c>
       <c r="AO8" t="n">
-        <v>0.1020682245887486</v>
+        <v>0.1020565309502171</v>
       </c>
       <c r="AP8" t="n">
-        <v>0.8505213355279034</v>
+        <v>0.8505271597331772</v>
       </c>
       <c r="AQ8" t="n">
-        <v>0.5510264886289833</v>
+        <v>0.5510227153322175</v>
       </c>
       <c r="AR8" t="n">
         <v>0.5472873917189358</v>
@@ -2292,94 +2292,94 @@
         <v>0.36875</v>
       </c>
       <c r="AT8" t="n">
-        <v>0.8886668819554222</v>
+        <v>0.8886511998737473</v>
       </c>
       <c r="AU8" t="n">
-        <v>0.5897582525396874</v>
+        <v>0.5897614176634068</v>
       </c>
       <c r="AV8" t="n">
-        <v>0.3413794902364864</v>
+        <v>0.3413638081548115</v>
       </c>
       <c r="AW8" t="n">
-        <v>0.9168465296054072</v>
+        <v>0.9168322741071476</v>
       </c>
       <c r="AX8" t="n">
-        <v>0.3270882770657199</v>
+        <v>0.3270708564437408</v>
       </c>
       <c r="AY8" t="n">
-        <v>134.8326123950213</v>
+        <v>134.8374573301722</v>
       </c>
       <c r="AZ8" t="n">
-        <v>4.317328488730078</v>
+        <v>4.317619212606513</v>
       </c>
       <c r="BA8" t="n">
-        <v>241.4104959520961</v>
+        <v>241.4191705462976</v>
       </c>
       <c r="BB8" t="n">
-        <v>123.5297180913598</v>
+        <v>123.5341568800382</v>
       </c>
       <c r="BC8" t="n">
-        <v>159.1402078158146</v>
+        <v>159.1479532533926</v>
       </c>
       <c r="BD8" t="n">
-        <v>222.1117834262884</v>
+        <v>222.1187140127577</v>
       </c>
       <c r="BE8" t="n">
-        <v>0.9797853895098045</v>
+        <v>0.9797845648265177</v>
       </c>
       <c r="BF8" t="n">
-        <v>497.0716056276176</v>
+        <v>497.0866310217285</v>
       </c>
       <c r="BG8" t="n">
-        <v>447.2155310812989</v>
+        <v>447.2222902068978</v>
       </c>
       <c r="BH8" t="n">
-        <v>0.5398079430926793</v>
+        <v>0.5398191812724947</v>
       </c>
       <c r="BI8" t="n">
-        <v>0.5196824902963315</v>
+        <v>0.5196899037430248</v>
       </c>
       <c r="BJ8" t="n">
-        <v>544.7954557524375</v>
+        <v>544.8139109267639</v>
       </c>
       <c r="BK8" t="n">
-        <v>0.9549883515465672</v>
+        <v>0.9549870673245943</v>
       </c>
       <c r="BL8" t="n">
-        <v>677.2002037192149</v>
+        <v>690.8959405069201</v>
       </c>
       <c r="BM8" t="n">
-        <v>521.9945152666484</v>
+        <v>527.2465178854804</v>
       </c>
       <c r="BN8" t="n">
-        <v>0.4255059716725719</v>
+        <v>0.4212805708107162</v>
       </c>
       <c r="BO8" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.2975897333830798</v>
       </c>
       <c r="BP8" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.2231923000373098</v>
       </c>
       <c r="BQ8" t="n">
-        <v>0.6684108649448608</v>
+        <v>0.6684256868849153</v>
       </c>
       <c r="BR8" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5665939720200175</v>
       </c>
       <c r="BS8" t="n">
-        <v>0.6327433073496426</v>
+        <v>0.6327703767501607</v>
       </c>
       <c r="BT8" t="n">
-        <v>0.6989130013474428</v>
+        <v>0.698946781480304</v>
       </c>
       <c r="BU8" t="n">
-        <v>0.4972626596029361</v>
+        <v>0.4972915548662097</v>
       </c>
       <c r="BV8" t="n">
-        <v>0.1233424708069024</v>
+        <v>0.1233413892957448</v>
       </c>
       <c r="BW8" t="n">
-        <v>0.04658913073714011</v>
+        <v>0.04658149766348002</v>
       </c>
     </row>
     <row r="9">
@@ -2399,52 +2399,52 @@
         <v>0.4</v>
       </c>
       <c r="F9" t="n">
-        <v>1.066429875635743</v>
+        <v>1.066314923944042</v>
       </c>
       <c r="G9" t="n">
-        <v>334.9958456714842</v>
+        <v>335.0078830645102</v>
       </c>
       <c r="H9" t="n">
         <v>0.3605527408399267</v>
       </c>
       <c r="I9" t="n">
-        <v>544.7954557524375</v>
+        <v>544.8139109267639</v>
       </c>
       <c r="J9" t="n">
-        <v>713471.5292305814</v>
+        <v>713546.0742559022</v>
       </c>
       <c r="K9" t="n">
-        <v>40462.02778444644</v>
+        <v>40464.9356777118</v>
       </c>
       <c r="L9" t="n">
-        <v>38034.30611737965</v>
+        <v>38037.03953704909</v>
       </c>
       <c r="M9" t="n">
-        <v>32110.81587215705</v>
+        <v>32113.12358707725</v>
       </c>
       <c r="N9" t="n">
-        <v>37.80746134928394</v>
+        <v>37.81017846625158</v>
       </c>
       <c r="O9" t="n">
-        <v>582.6029171017215</v>
+        <v>582.6240893930155</v>
       </c>
       <c r="P9" t="n">
-        <v>582.6029171017215</v>
+        <v>582.6240893930155</v>
       </c>
       <c r="Q9" t="n">
-        <v>1.220524649009106</v>
+        <v>1.220533631218061</v>
       </c>
       <c r="R9" t="n">
-        <v>870809.5877921456</v>
+        <v>870906.9810529489</v>
       </c>
       <c r="S9" t="n">
-        <v>870809.5877921456</v>
+        <v>870906.9810529489</v>
       </c>
       <c r="T9" t="n">
-        <v>427.3990130004892</v>
+        <v>427.406252099503</v>
       </c>
       <c r="U9" t="n">
-        <v>441.980495162634</v>
+        <v>441.9885260654151</v>
       </c>
       <c r="V9" t="n">
         <v>0.7615773105863909</v>
@@ -2456,61 +2456,61 @@
         <v>1.064577496794081</v>
       </c>
       <c r="Y9" t="n">
-        <v>121.435994055913</v>
+        <v>121.440357610885</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.3248720262443578</v>
+        <v>0.3248781972126394</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.4902267786136445</v>
+        <v>0.4902352568247675</v>
       </c>
       <c r="AB9" t="n">
-        <v>0.1108926247734101</v>
+        <v>0.1108810001132414</v>
       </c>
       <c r="AC9" t="n">
         <v>0.35</v>
       </c>
       <c r="AD9" t="n">
-        <v>117.2485459850195</v>
+        <v>117.2527590725786</v>
       </c>
       <c r="AE9" t="n">
-        <v>0.3033211971446864</v>
+        <v>0.3033265848492985</v>
       </c>
       <c r="AF9" t="n">
-        <v>0.4603395387699436</v>
+        <v>0.4603470788060721</v>
       </c>
       <c r="AG9" t="n">
-        <v>0.100056302624151</v>
+        <v>0.1000452925335783</v>
       </c>
       <c r="AH9" t="n">
-        <v>0.6619729934593227</v>
+        <v>0.662013441433866</v>
       </c>
       <c r="AI9" t="n">
-        <v>0.8898113151741506</v>
+        <v>0.8898337101995019</v>
       </c>
       <c r="AJ9" t="n">
-        <v>0.946510479765531</v>
+        <v>0.9465210065834279</v>
       </c>
       <c r="AK9" t="n">
-        <v>0.281528605843333</v>
+        <v>0.2815360015571626</v>
       </c>
       <c r="AL9" t="n">
-        <v>0.9005374717254715</v>
+        <v>0.9005237062743279</v>
       </c>
       <c r="AM9" t="n">
-        <v>0.3404490152611628</v>
+        <v>0.3404585758986661</v>
       </c>
       <c r="AN9" t="n">
-        <v>0.5088534310976932</v>
+        <v>0.5088666015949554</v>
       </c>
       <c r="AO9" t="n">
-        <v>0.09051697283767492</v>
+        <v>0.09050615234283096</v>
       </c>
       <c r="AP9" t="n">
-        <v>0.854043895175961</v>
+        <v>0.8540491585849094</v>
       </c>
       <c r="AQ9" t="n">
-        <v>0.5506466038529215</v>
+        <v>0.550643210279808</v>
       </c>
       <c r="AR9" t="n">
         <v>0.5308367445217098</v>
@@ -2519,94 +2519,94 @@
         <v>0.35625</v>
       </c>
       <c r="AT9" t="n">
-        <v>0.8653500475224741</v>
+        <v>0.8653359629553143</v>
       </c>
       <c r="AU9" t="n">
-        <v>0.5742398709033788</v>
+        <v>0.5742426816295175</v>
       </c>
       <c r="AV9" t="n">
-        <v>0.3345133030007643</v>
+        <v>0.3344992184336045</v>
       </c>
       <c r="AW9" t="n">
-        <v>0.8933979759636368</v>
+        <v>0.893385146392757</v>
       </c>
       <c r="AX9" t="n">
-        <v>0.319158105060258</v>
+        <v>0.3191424647632395</v>
       </c>
       <c r="AY9" t="n">
-        <v>130.6757008041521</v>
+        <v>130.6803963691564</v>
       </c>
       <c r="AZ9" t="n">
-        <v>4.953187281049108</v>
+        <v>4.95354753872835</v>
       </c>
       <c r="BA9" t="n">
-        <v>239.8711457535123</v>
+        <v>239.8797650343014</v>
       </c>
       <c r="BB9" t="n">
-        <v>119.3422700204662</v>
+        <v>119.3465583417318</v>
       </c>
       <c r="BC9" t="n">
-        <v>156.7565726515706</v>
+        <v>156.7640857806538</v>
       </c>
       <c r="BD9" t="n">
-        <v>219.7035832877112</v>
+        <v>219.7105233637245</v>
       </c>
       <c r="BE9" t="n">
-        <v>0.9824096944273142</v>
+        <v>0.9824090261626442</v>
       </c>
       <c r="BF9" t="n">
-        <v>535.2123372111415</v>
+        <v>535.2301036734237</v>
       </c>
       <c r="BG9" t="n">
-        <v>464.0560698884079</v>
+        <v>464.0637720335846</v>
       </c>
       <c r="BH9" t="n">
-        <v>0.5169012137072022</v>
+        <v>0.5169112080934885</v>
       </c>
       <c r="BI9" t="n">
-        <v>0.4970888663466193</v>
+        <v>0.4970955362112884</v>
       </c>
       <c r="BJ9" t="n">
-        <v>582.6029171017215</v>
+        <v>582.6240893930155</v>
       </c>
       <c r="BK9" t="n">
-        <v>0.9588171098257054</v>
+        <v>0.9588160046464687</v>
       </c>
       <c r="BL9" t="n">
-        <v>679.9152482351244</v>
+        <v>693.6660274983068</v>
       </c>
       <c r="BM9" t="n">
-        <v>523.0398639490919</v>
+        <v>528.3024349974347</v>
       </c>
       <c r="BN9" t="n">
-        <v>0.4200513162206986</v>
+        <v>0.4158802019619527</v>
       </c>
       <c r="BO9" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.2975897333830798</v>
       </c>
       <c r="BP9" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.2231923000373098</v>
       </c>
       <c r="BQ9" t="n">
-        <v>0.6773344445505896</v>
+        <v>0.6773477176156892</v>
       </c>
       <c r="BR9" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5665939720200175</v>
       </c>
       <c r="BS9" t="n">
-        <v>0.6353639071499578</v>
+        <v>0.6353906534983169</v>
       </c>
       <c r="BT9" t="n">
-        <v>0.7041542009480733</v>
+        <v>0.7041873349766165</v>
       </c>
       <c r="BU9" t="n">
-        <v>0.5039013352448847</v>
+        <v>0.5039293167322264</v>
       </c>
       <c r="BV9" t="n">
-        <v>0.1200231329859281</v>
+        <v>0.1200225083627365</v>
       </c>
       <c r="BW9" t="n">
-        <v>0.04098730387870908</v>
+        <v>0.04098044601191669</v>
       </c>
     </row>
     <row r="10">
@@ -2626,52 +2626,52 @@
         <v>0.4</v>
       </c>
       <c r="F10" t="n">
-        <v>1.066429875635743</v>
+        <v>1.066314923944042</v>
       </c>
       <c r="G10" t="n">
-        <v>334.9958456714842</v>
+        <v>335.0078830645102</v>
       </c>
       <c r="H10" t="n">
         <v>0.3629425367369873</v>
       </c>
       <c r="I10" t="n">
-        <v>582.6029171017215</v>
+        <v>582.6240893930155</v>
       </c>
       <c r="J10" t="n">
-        <v>870809.5877921456</v>
+        <v>870906.9810529489</v>
       </c>
       <c r="K10" t="n">
-        <v>40730.21597727716</v>
+        <v>40733.14314448114</v>
       </c>
       <c r="L10" t="n">
-        <v>38286.40301864053</v>
+        <v>38289.15455581227</v>
       </c>
       <c r="M10" t="n">
-        <v>31952.06414594367</v>
+        <v>31954.36045181937</v>
       </c>
       <c r="N10" t="n">
-        <v>38.05805469049754</v>
+        <v>38.06078981691081</v>
       </c>
       <c r="O10" t="n">
-        <v>620.660971792219</v>
+        <v>620.6848792099263</v>
       </c>
       <c r="P10" t="n">
-        <v>620.660971792219</v>
+        <v>620.6848792099263</v>
       </c>
       <c r="Q10" t="n">
-        <v>1.204167456353411</v>
+        <v>1.204175196794033</v>
       </c>
       <c r="R10" t="n">
-        <v>1048600.566299831</v>
+        <v>1048724.585298731</v>
       </c>
       <c r="S10" t="n">
-        <v>1048600.566299831</v>
+        <v>1048724.585298731</v>
       </c>
       <c r="T10" t="n">
-        <v>441.980495162634</v>
+        <v>441.9885260654151</v>
       </c>
       <c r="U10" t="n">
-        <v>456.1881452229234</v>
+        <v>456.196931159218</v>
       </c>
       <c r="V10" t="n">
         <v>0.7615773105863909</v>
@@ -2683,61 +2683,61 @@
         <v>1.064577496794081</v>
       </c>
       <c r="Y10" t="n">
-        <v>117.2485459850195</v>
+        <v>117.2527590725786</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.3033211971446864</v>
+        <v>0.3033265848492985</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.4603395387699436</v>
+        <v>0.4603470788060721</v>
       </c>
       <c r="AB10" t="n">
-        <v>0.100056302624151</v>
+        <v>0.1000452925335783</v>
       </c>
       <c r="AC10" t="n">
         <v>0.3375</v>
       </c>
       <c r="AD10" t="n">
-        <v>113.0610979141259</v>
+        <v>113.0651605342722</v>
       </c>
       <c r="AE10" t="n">
-        <v>0.2833789606329719</v>
+        <v>0.2833836854623158</v>
       </c>
       <c r="AF10" t="n">
-        <v>0.4322063770688386</v>
+        <v>0.4322130945306098</v>
       </c>
       <c r="AG10" t="n">
-        <v>0.09134516475091831</v>
+        <v>0.0913347020509485</v>
       </c>
       <c r="AH10" t="n">
-        <v>0.6709315018399133</v>
+        <v>0.670970679725292</v>
       </c>
       <c r="AI10" t="n">
-        <v>0.9018531691514183</v>
+        <v>0.9018734243248485</v>
       </c>
       <c r="AJ10" t="n">
-        <v>0.9521919813536703</v>
+        <v>0.9522015735923325</v>
       </c>
       <c r="AK10" t="n">
-        <v>0.2847475699273967</v>
+        <v>0.2847542936424915</v>
       </c>
       <c r="AL10" t="n">
-        <v>0.8775390029012443</v>
+        <v>0.8775262364419676</v>
       </c>
       <c r="AM10" t="n">
-        <v>0.3242639972996528</v>
+        <v>0.3242725878026358</v>
       </c>
       <c r="AN10" t="n">
-        <v>0.4865739919422437</v>
+        <v>0.4865860970951499</v>
       </c>
       <c r="AO10" t="n">
-        <v>0.08113866210185122</v>
+        <v>0.08112861104568778</v>
       </c>
       <c r="AP10" t="n">
-        <v>0.8568846459700306</v>
+        <v>0.8568894420893617</v>
       </c>
       <c r="AQ10" t="n">
-        <v>0.5502155635368724</v>
+        <v>0.550212483910294</v>
       </c>
       <c r="AR10" t="n">
         <v>0.5145610942928165</v>
@@ -2746,94 +2746,94 @@
         <v>0.34375</v>
       </c>
       <c r="AT10" t="n">
-        <v>0.8423473256617744</v>
+        <v>0.8423345682187273</v>
       </c>
       <c r="AU10" t="n">
-        <v>0.5584232149984406</v>
+        <v>0.5584257301393467</v>
       </c>
       <c r="AV10" t="n">
-        <v>0.3277862313689579</v>
+        <v>0.3277734739259108</v>
       </c>
       <c r="AW10" t="n">
-        <v>0.8699731692653212</v>
+        <v>0.8699615314301051</v>
       </c>
       <c r="AX10" t="n">
-        <v>0.3115499542668806</v>
+        <v>0.3115358012907584</v>
       </c>
       <c r="AY10" t="n">
-        <v>126.5946303533889</v>
+        <v>126.5991792734434</v>
       </c>
       <c r="AZ10" t="n">
-        <v>5.624360949315135</v>
+        <v>5.624796194173435</v>
       </c>
       <c r="BA10" t="n">
-        <v>238.2360518720631</v>
+        <v>238.2446123990857</v>
       </c>
       <c r="BB10" t="n">
-        <v>115.1548219495727</v>
+        <v>115.1589598034254</v>
       </c>
       <c r="BC10" t="n">
-        <v>154.3200418328142</v>
+        <v>154.3273434635555</v>
       </c>
       <c r="BD10" t="n">
-        <v>217.3349232851236</v>
+        <v>217.3418577979388</v>
       </c>
       <c r="BE10" t="n">
-        <v>0.9846660418937857</v>
+        <v>0.9846654971539436</v>
       </c>
       <c r="BF10" t="n">
-        <v>573.6693083783255</v>
+        <v>573.6898386360373</v>
       </c>
       <c r="BG10" t="n">
-        <v>480.4389481704237</v>
+        <v>480.4475449761357</v>
       </c>
       <c r="BH10" t="n">
-        <v>0.4958716456675673</v>
+        <v>0.4958805906915801</v>
       </c>
       <c r="BI10" t="n">
-        <v>0.4764151053923584</v>
+        <v>0.4764211307727627</v>
       </c>
       <c r="BJ10" t="n">
-        <v>620.660971792219</v>
+        <v>620.6848792099263</v>
       </c>
       <c r="BK10" t="n">
-        <v>0.9621714412256647</v>
+        <v>0.962170484358867</v>
       </c>
       <c r="BL10" t="n">
-        <v>682.2938677268862</v>
+        <v>696.0928628923207</v>
       </c>
       <c r="BM10" t="n">
-        <v>523.9539680340154</v>
+        <v>529.2257782018504</v>
       </c>
       <c r="BN10" t="n">
-        <v>0.4147977428257859</v>
+        <v>0.4106788950009218</v>
       </c>
       <c r="BO10" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.2975897333830798</v>
       </c>
       <c r="BP10" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.2231923000373098</v>
       </c>
       <c r="BQ10" t="n">
-        <v>0.6844724925067254</v>
+        <v>0.6844845008679415</v>
       </c>
       <c r="BR10" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5665939720200175</v>
       </c>
       <c r="BS10" t="n">
-        <v>0.6374772768888605</v>
+        <v>0.6375037515253728</v>
       </c>
       <c r="BT10" t="n">
-        <v>0.7083809404258787</v>
+        <v>0.708413531030728</v>
       </c>
       <c r="BU10" t="n">
-        <v>0.509211668899222</v>
+        <v>0.5092389002953529</v>
       </c>
       <c r="BV10" t="n">
-        <v>0.1173679661587594</v>
+        <v>0.1173677165811732</v>
       </c>
       <c r="BW10" t="n">
-        <v>0.03650804968841376</v>
+        <v>0.03650182686620368</v>
       </c>
     </row>
     <row r="11">
@@ -2853,52 +2853,52 @@
         <v>0.4</v>
       </c>
       <c r="F11" t="n">
-        <v>1.066429875635743</v>
+        <v>1.066314923944042</v>
       </c>
       <c r="G11" t="n">
-        <v>334.9958456714842</v>
+        <v>335.0078830645102</v>
       </c>
       <c r="H11" t="n">
         <v>0.3644008637646071</v>
       </c>
       <c r="I11" t="n">
-        <v>620.660971792219</v>
+        <v>620.6848792099263</v>
       </c>
       <c r="J11" t="n">
-        <v>1048600.566299831</v>
+        <v>1048724.585298731</v>
       </c>
       <c r="K11" t="n">
-        <v>40893.87266886935</v>
+        <v>40896.81159762403</v>
       </c>
       <c r="L11" t="n">
-        <v>38440.24030873719</v>
+        <v>38443.00290176659</v>
       </c>
       <c r="M11" t="n">
-        <v>31667.27690756771</v>
+        <v>31669.55274657762</v>
       </c>
       <c r="N11" t="n">
-        <v>38.21097446196539</v>
+        <v>38.21372057829681</v>
       </c>
       <c r="O11" t="n">
-        <v>658.8719462541844</v>
+        <v>658.8985997882231</v>
       </c>
       <c r="P11" t="n">
-        <v>658.8719462541844</v>
+        <v>658.8985997882231</v>
       </c>
       <c r="Q11" t="n">
-        <v>1.189052302015514</v>
+        <v>1.189059000774152</v>
       </c>
       <c r="R11" t="n">
-        <v>1246840.917253586</v>
+        <v>1246995.407482597</v>
       </c>
       <c r="S11" t="n">
-        <v>1246840.917253586</v>
+        <v>1246995.407482597</v>
       </c>
       <c r="T11" t="n">
-        <v>456.1881452229234</v>
+        <v>456.196931159218</v>
       </c>
       <c r="U11" t="n">
-        <v>470.021024613823</v>
+        <v>470.0305314647031</v>
       </c>
       <c r="V11" t="n">
         <v>0.7615773105863909</v>
@@ -2910,61 +2910,61 @@
         <v>1.064577496794081</v>
       </c>
       <c r="Y11" t="n">
-        <v>113.0610979141259</v>
+        <v>113.0651605342722</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.2833789606329719</v>
+        <v>0.2833836854623158</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.4322063770688386</v>
+        <v>0.4322130945306098</v>
       </c>
       <c r="AB11" t="n">
-        <v>0.09134516475091832</v>
+        <v>0.09133470205094847</v>
       </c>
       <c r="AC11" t="n">
         <v>0.325</v>
       </c>
       <c r="AD11" t="n">
-        <v>108.8736498432324</v>
+        <v>108.8775619959658</v>
       </c>
       <c r="AE11" t="n">
-        <v>0.264852390566271</v>
+        <v>0.2648565503927191</v>
       </c>
       <c r="AF11" t="n">
-        <v>0.4056848070423067</v>
+        <v>0.4056908019310182</v>
       </c>
       <c r="AG11" t="n">
-        <v>0.08432577123228341</v>
+        <v>0.08431578356142674</v>
       </c>
       <c r="AH11" t="n">
-        <v>0.6781934296933768</v>
+        <v>0.6782315552914558</v>
       </c>
       <c r="AI11" t="n">
-        <v>0.9116145123449262</v>
+        <v>0.9116330023635398</v>
       </c>
       <c r="AJ11" t="n">
-        <v>0.9568283595080879</v>
+        <v>0.9568371677036699</v>
       </c>
       <c r="AK11" t="n">
-        <v>0.2877665857908671</v>
+        <v>0.2877727449012679</v>
       </c>
       <c r="AL11" t="n">
-        <v>0.8540733970766762</v>
+        <v>0.8540614720097621</v>
       </c>
       <c r="AM11" t="n">
-        <v>0.3093872915612632</v>
+        <v>0.3093950609732614</v>
       </c>
       <c r="AN11" t="n">
-        <v>0.4657932677724579</v>
+        <v>0.46580445200834</v>
       </c>
       <c r="AO11" t="n">
-        <v>0.07344392158062314</v>
+        <v>0.07343454469143831</v>
       </c>
       <c r="AP11" t="n">
-        <v>0.8592028350472394</v>
+        <v>0.8592072391450304</v>
       </c>
       <c r="AQ11" t="n">
-        <v>0.5495796948299662</v>
+        <v>0.5495768778114289</v>
       </c>
       <c r="AR11" t="n">
         <v>0.4984787765891089</v>
@@ -2973,94 +2973,94 @@
         <v>0.33125</v>
       </c>
       <c r="AT11" t="n">
-        <v>0.8191312917860756</v>
+        <v>0.819119657303519</v>
       </c>
       <c r="AU11" t="n">
-        <v>0.5424268789629988</v>
+        <v>0.5424291451639892</v>
       </c>
       <c r="AV11" t="n">
-        <v>0.3206525151969667</v>
+        <v>0.3206408807144101</v>
       </c>
       <c r="AW11" t="n">
-        <v>0.8460863486369866</v>
+        <v>0.8460757258958939</v>
       </c>
       <c r="AX11" t="n">
-        <v>0.3036594696739878</v>
+        <v>0.3036465807319046</v>
       </c>
       <c r="AY11" t="n">
-        <v>122.6020817033145</v>
+        <v>122.6064871592697</v>
       </c>
       <c r="AZ11" t="n">
-        <v>6.325027396634392</v>
+        <v>6.325542335235263</v>
       </c>
       <c r="BA11" t="n">
-        <v>236.4849743786179</v>
+        <v>236.4934719842393</v>
       </c>
       <c r="BB11" t="n">
-        <v>110.9673738786792</v>
+        <v>110.971361265119</v>
       </c>
       <c r="BC11" t="n">
-        <v>151.8950557315864</v>
+        <v>151.9021656994411</v>
       </c>
       <c r="BD11" t="n">
-        <v>214.9630528285631</v>
+        <v>214.9699688284873</v>
       </c>
       <c r="BE11" t="n">
-        <v>0.9866160607784294</v>
+        <v>0.9866156144689658</v>
       </c>
       <c r="BF11" t="n">
-        <v>612.3540830685511</v>
+        <v>612.3773934932973</v>
       </c>
       <c r="BG11" t="n">
-        <v>496.3736383647526</v>
+        <v>496.3830859789272</v>
       </c>
       <c r="BH11" t="n">
-        <v>0.4764253298335728</v>
+        <v>0.4764333811210463</v>
       </c>
       <c r="BI11" t="n">
-        <v>0.45734773887015</v>
+        <v>0.4573532024794233</v>
       </c>
       <c r="BJ11" t="n">
-        <v>658.8719462541844</v>
+        <v>658.8985997882231</v>
       </c>
       <c r="BK11" t="n">
-        <v>0.9651388409583935</v>
+        <v>0.9651380080303026</v>
       </c>
       <c r="BL11" t="n">
-        <v>684.3981066951061</v>
+        <v>698.2397506650492</v>
       </c>
       <c r="BM11" t="n">
-        <v>524.7613002211986</v>
+        <v>530.0412682778475</v>
       </c>
       <c r="BN11" t="n">
-        <v>0.4096396832959126</v>
+        <v>0.4055721350281731</v>
       </c>
       <c r="BO11" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.2975897333830798</v>
       </c>
       <c r="BP11" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.2231923000373098</v>
       </c>
       <c r="BQ11" t="n">
-        <v>0.6902601129331082</v>
+        <v>0.6902710768954838</v>
       </c>
       <c r="BR11" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5665939720200175</v>
       </c>
       <c r="BS11" t="n">
-        <v>0.6392018880920168</v>
+        <v>0.6392281330449541</v>
       </c>
       <c r="BT11" t="n">
-        <v>0.7118301628321914</v>
+        <v>0.7118622940698908</v>
       </c>
       <c r="BU11" t="n">
-        <v>0.5135173552321824</v>
+        <v>0.513543964338446</v>
       </c>
       <c r="BV11" t="n">
-        <v>0.1152151229922792</v>
+        <v>0.1152151845596267</v>
       </c>
       <c r="BW11" t="n">
-        <v>0.03287708576168202</v>
+        <v>0.03287138908312176</v>
       </c>
     </row>
     <row r="12">
@@ -3080,52 +3080,52 @@
         <v>0.4</v>
       </c>
       <c r="F12" t="n">
-        <v>1.066429875635743</v>
+        <v>1.066314923944042</v>
       </c>
       <c r="G12" t="n">
-        <v>334.9958456714842</v>
+        <v>335.0078830645102</v>
       </c>
       <c r="H12" t="n">
         <v>0.3648340491519012</v>
       </c>
       <c r="I12" t="n">
-        <v>658.8719462541844</v>
+        <v>658.8985997882231</v>
       </c>
       <c r="J12" t="n">
-        <v>1246840.917253586</v>
+        <v>1246995.407482597</v>
       </c>
       <c r="K12" t="n">
-        <v>40942.48569323765</v>
+        <v>40945.42811567503</v>
       </c>
       <c r="L12" t="n">
-        <v>38485.93655164339</v>
+        <v>38488.70242873453</v>
       </c>
       <c r="M12" t="n">
-        <v>31250.59416923171</v>
+        <v>31252.84006241352</v>
       </c>
       <c r="N12" t="n">
-        <v>38.25639816266739</v>
+        <v>38.25914754347369</v>
       </c>
       <c r="O12" t="n">
-        <v>697.1283444168519</v>
+        <v>697.1577473316968</v>
       </c>
       <c r="P12" t="n">
-        <v>697.1283444168519</v>
+        <v>697.1577473316968</v>
       </c>
       <c r="Q12" t="n">
-        <v>1.174972243401005</v>
+        <v>1.174978059777818</v>
       </c>
       <c r="R12" t="n">
-        <v>1465003.469709612</v>
+        <v>1465192.244435751</v>
       </c>
       <c r="S12" t="n">
-        <v>1465003.469709612</v>
+        <v>1465192.244435751</v>
       </c>
       <c r="T12" t="n">
-        <v>470.021024613823</v>
+        <v>470.0305314647031</v>
       </c>
       <c r="U12" t="n">
-        <v>483.4740260685887</v>
+        <v>483.4842217490845</v>
       </c>
       <c r="V12" t="n">
         <v>0.7615773105863909</v>
@@ -3137,61 +3137,61 @@
         <v>1.064577496794081</v>
       </c>
       <c r="Y12" t="n">
-        <v>108.8736498432324</v>
+        <v>108.8775619959658</v>
       </c>
       <c r="Z12" t="n">
-        <v>0.264852390566271</v>
+        <v>0.2648565503927191</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.4056848070423067</v>
+        <v>0.4056908019310182</v>
       </c>
       <c r="AB12" t="n">
-        <v>0.08432577123228341</v>
+        <v>0.08431578356142674</v>
       </c>
       <c r="AC12" t="n">
         <v>0.3125</v>
       </c>
       <c r="AD12" t="n">
-        <v>104.6862017723388</v>
+        <v>104.6899634576594</v>
       </c>
       <c r="AE12" t="n">
-        <v>0.2475795080404627</v>
+        <v>0.2475831831790785</v>
       </c>
       <c r="AF12" t="n">
-        <v>0.3806439700063695</v>
+        <v>0.3806493287854359</v>
       </c>
       <c r="AG12" t="n">
-        <v>0.07867891571681149</v>
+        <v>0.0786693302343812</v>
       </c>
       <c r="AH12" t="n">
-        <v>0.6841493266339539</v>
+        <v>0.6841865722433287</v>
       </c>
       <c r="AI12" t="n">
-        <v>0.9196203140046615</v>
+        <v>0.9196373335401227</v>
       </c>
       <c r="AJ12" t="n">
-        <v>0.9606512171256621</v>
+        <v>0.9606593634688591</v>
       </c>
       <c r="AK12" t="n">
-        <v>0.2907964460364127</v>
+        <v>0.290802126405799</v>
       </c>
       <c r="AL12" t="n">
-        <v>0.8297807583132409</v>
+        <v>0.8297695502434891</v>
       </c>
       <c r="AM12" t="n">
-        <v>0.2957759736655972</v>
+        <v>0.2957830455374672</v>
       </c>
       <c r="AN12" t="n">
-        <v>0.4465201903401176</v>
+        <v>0.446530581558673</v>
       </c>
       <c r="AO12" t="n">
-        <v>0.06707122204581961</v>
+        <v>0.0670624342126548</v>
       </c>
       <c r="AP12" t="n">
-        <v>0.8611142638560265</v>
+        <v>0.861118337027625</v>
       </c>
       <c r="AQ12" t="n">
-        <v>0.5486113102580497</v>
+        <v>0.548608715274397</v>
       </c>
       <c r="AR12" t="n">
         <v>0.4826064562566781</v>
@@ -3200,94 +3200,94 @@
         <v>0.31875</v>
       </c>
       <c r="AT12" t="n">
-        <v>0.7952941051769974</v>
+        <v>0.7952834384305292</v>
       </c>
       <c r="AU12" t="n">
-        <v>0.5263410536891099</v>
+        <v>0.5263431083424015</v>
       </c>
       <c r="AV12" t="n">
-        <v>0.3126876489203193</v>
+        <v>0.3126769821738511</v>
       </c>
       <c r="AW12" t="n">
-        <v>0.8213575967455732</v>
+        <v>0.8213478551650262</v>
       </c>
       <c r="AX12" t="n">
-        <v>0.2950165430564633</v>
+        <v>0.2950047468226247</v>
       </c>
       <c r="AY12" t="n">
-        <v>118.7135375702998</v>
+        <v>118.717803299346</v>
       </c>
       <c r="AZ12" t="n">
-        <v>7.048422847999833</v>
+        <v>7.049021303347698</v>
       </c>
       <c r="BA12" t="n">
-        <v>234.596226942576</v>
+        <v>234.6046566799074</v>
       </c>
       <c r="BB12" t="n">
-        <v>106.7799258077856</v>
+        <v>106.7837627268126</v>
       </c>
       <c r="BC12" t="n">
-        <v>149.5371544469267</v>
+        <v>149.5440916546002</v>
       </c>
       <c r="BD12" t="n">
-        <v>212.5510843845128</v>
+        <v>212.5579702993289</v>
       </c>
       <c r="BE12" t="n">
-        <v>0.9883088685352219</v>
+        <v>0.9883085012856782</v>
       </c>
       <c r="BF12" t="n">
-        <v>651.1689877120725</v>
+        <v>651.1950876559306</v>
       </c>
       <c r="BG12" t="n">
-        <v>511.8636086848034</v>
+        <v>511.8738667574661</v>
       </c>
       <c r="BH12" t="n">
-        <v>0.4583178467118498</v>
+        <v>0.4583251303022015</v>
       </c>
       <c r="BI12" t="n">
-        <v>0.4396328922008292</v>
+        <v>0.4396378635281316</v>
       </c>
       <c r="BJ12" t="n">
-        <v>697.1283444168519</v>
+        <v>697.1577473316968</v>
       </c>
       <c r="BK12" t="n">
-        <v>0.967787153349189</v>
+        <v>0.9677864248254033</v>
       </c>
       <c r="BL12" t="n">
-        <v>686.2760748270256</v>
+        <v>700.1557770439525</v>
       </c>
       <c r="BM12" t="n">
-        <v>525.4807717389875</v>
+        <v>530.7680081272841</v>
       </c>
       <c r="BN12" t="n">
-        <v>0.4044887954341541</v>
+        <v>0.4004724607447613</v>
       </c>
       <c r="BO12" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.2975897333830798</v>
       </c>
       <c r="BP12" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.2231923000373098</v>
       </c>
       <c r="BQ12" t="n">
-        <v>0.6950075904856097</v>
+        <v>0.6950176837537623</v>
       </c>
       <c r="BR12" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5665939720200175</v>
       </c>
       <c r="BS12" t="n">
-        <v>0.6406238909692106</v>
+        <v>0.6406499408183298</v>
       </c>
       <c r="BT12" t="n">
-        <v>0.7146741685865788</v>
+        <v>0.7147059096166422</v>
       </c>
       <c r="BU12" t="n">
-        <v>0.5170492297691963</v>
+        <v>0.5170753180120193</v>
       </c>
       <c r="BV12" t="n">
-        <v>0.1134491857237723</v>
+        <v>0.11344950772284</v>
       </c>
       <c r="BW12" t="n">
-        <v>0.02989913729139348</v>
+        <v>0.02989388060718534</v>
       </c>
     </row>
     <row r="13">
@@ -3307,52 +3307,52 @@
         <v>0.4</v>
       </c>
       <c r="F13" t="n">
-        <v>1.066429875635743</v>
+        <v>1.066314923944042</v>
       </c>
       <c r="G13" t="n">
-        <v>334.9958456714842</v>
+        <v>335.0078830645102</v>
       </c>
       <c r="H13" t="n">
         <v>0.3641428413236223</v>
       </c>
       <c r="I13" t="n">
-        <v>697.1283444168519</v>
+        <v>697.1577473316968</v>
       </c>
       <c r="J13" t="n">
-        <v>1465003.469709612</v>
+        <v>1465192.244435751</v>
       </c>
       <c r="K13" t="n">
-        <v>40864.91681860507</v>
+        <v>40867.85366638343</v>
       </c>
       <c r="L13" t="n">
-        <v>38413.02180948877</v>
+        <v>38415.78244640042</v>
       </c>
       <c r="M13" t="n">
-        <v>30696.82416065179</v>
+        <v>30699.03025592513</v>
       </c>
       <c r="N13" t="n">
-        <v>38.18391829969062</v>
+        <v>38.186662471571</v>
       </c>
       <c r="O13" t="n">
-        <v>735.3122627165425</v>
+        <v>735.3444098032678</v>
       </c>
       <c r="P13" t="n">
-        <v>735.3122627165425</v>
+        <v>735.3444098032678</v>
       </c>
       <c r="Q13" t="n">
-        <v>1.161763539474074</v>
+        <v>1.161768601873004</v>
       </c>
       <c r="R13" t="n">
-        <v>1701987.616311639</v>
+        <v>1702214.345293292</v>
       </c>
       <c r="S13" t="n">
-        <v>1701987.616311639</v>
+        <v>1702214.345293292</v>
       </c>
       <c r="T13" t="n">
-        <v>483.4740260685887</v>
+        <v>483.4842217490845</v>
       </c>
       <c r="U13" t="n">
-        <v>496.5382177525278</v>
+        <v>496.5490717009102</v>
       </c>
       <c r="V13" t="n">
         <v>0.7615773105863909</v>
@@ -3364,61 +3364,61 @@
         <v>1.064577496794081</v>
       </c>
       <c r="Y13" t="n">
-        <v>104.6862017723388</v>
+        <v>104.6899634576594</v>
       </c>
       <c r="Z13" t="n">
-        <v>0.2475795080404627</v>
+        <v>0.2475831831790785</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.3806439700063695</v>
+        <v>0.3806493287854359</v>
       </c>
       <c r="AB13" t="n">
-        <v>0.07867891571681147</v>
+        <v>0.07866933023438122</v>
       </c>
       <c r="AC13" t="n">
         <v>0.3</v>
       </c>
       <c r="AD13" t="n">
-        <v>100.4987537014453</v>
+        <v>100.5023649193531</v>
       </c>
       <c r="AE13" t="n">
-        <v>0.2314229337341716</v>
+        <v>0.2314261906448897</v>
       </c>
       <c r="AF13" t="n">
-        <v>0.356964158557928</v>
+        <v>0.3569689560278481</v>
       </c>
       <c r="AG13" t="n">
-        <v>0.07416764671794335</v>
+        <v>0.0741583922178526</v>
       </c>
       <c r="AH13" t="n">
-        <v>0.6890844320072977</v>
+        <v>0.6891209357936195</v>
       </c>
       <c r="AI13" t="n">
-        <v>0.9262539873511073</v>
+        <v>0.9262697714192063</v>
       </c>
       <c r="AJ13" t="n">
-        <v>0.9638325708036187</v>
+        <v>0.9638401551722643</v>
       </c>
       <c r="AK13" t="n">
-        <v>0.2940089553983466</v>
+        <v>0.2940142262079937</v>
       </c>
       <c r="AL13" t="n">
-        <v>0.8043697733634284</v>
+        <v>0.8043591841349204</v>
       </c>
       <c r="AM13" t="n">
-        <v>0.2833915018027358</v>
+        <v>0.2833979791330358</v>
       </c>
       <c r="AN13" t="n">
-        <v>0.4287582016046487</v>
+        <v>0.4287679133460001</v>
       </c>
       <c r="AO13" t="n">
-        <v>0.0617485368298673</v>
+        <v>0.06174026326766762</v>
       </c>
       <c r="AP13" t="n">
-        <v>0.8627049406950048</v>
+        <v>0.8627087328793276</v>
       </c>
       <c r="AQ13" t="n">
-        <v>0.5471991620698325</v>
+        <v>0.5471967567619866</v>
       </c>
       <c r="AR13" t="n">
         <v>0.466958890421039</v>
@@ -3427,94 +3427,94 @@
         <v>0.30625</v>
       </c>
       <c r="AT13" t="n">
-        <v>0.7705127448541069</v>
+        <v>0.7705029277862248</v>
       </c>
       <c r="AU13" t="n">
-        <v>0.5102357395223244</v>
+        <v>0.5102376128642553</v>
       </c>
       <c r="AV13" t="n">
-        <v>0.3035538544330679</v>
+        <v>0.3035440373651858</v>
       </c>
       <c r="AW13" t="n">
-        <v>0.7954836030482841</v>
+        <v>0.7954746412614898</v>
       </c>
       <c r="AX13" t="n">
-        <v>0.2852478635259598</v>
+        <v>0.2852370283972345</v>
       </c>
       <c r="AY13" t="n">
-        <v>114.9480074251195</v>
+        <v>114.9521378475137</v>
       </c>
       <c r="AZ13" t="n">
-        <v>7.786942573692805</v>
+        <v>7.78762736344407</v>
       </c>
       <c r="BA13" t="n">
-        <v>232.5466861290662</v>
+        <v>232.5550422203252</v>
       </c>
       <c r="BB13" t="n">
-        <v>102.5924777368921</v>
+        <v>102.5961641885063</v>
       </c>
       <c r="BC13" t="n">
-        <v>147.2964805650054</v>
+        <v>147.3032631620806</v>
       </c>
       <c r="BD13" t="n">
-        <v>210.0656314077421</v>
+        <v>210.0724765262511</v>
       </c>
       <c r="BE13" t="n">
-        <v>0.9897840645330738</v>
+        <v>0.9897837612344859</v>
       </c>
       <c r="BF13" t="n">
-        <v>690.0065262381241</v>
+        <v>690.0354173277282</v>
       </c>
       <c r="BG13" t="n">
-        <v>526.9070372439256</v>
+        <v>526.918068124433</v>
       </c>
       <c r="BH13" t="n">
-        <v>0.4413429119213136</v>
+        <v>0.4413495309585906</v>
       </c>
       <c r="BI13" t="n">
-        <v>0.4230603484230449</v>
+        <v>0.4230648862289798</v>
       </c>
       <c r="BJ13" t="n">
-        <v>735.3122627165425</v>
+        <v>735.3444098032678</v>
       </c>
       <c r="BK13" t="n">
-        <v>0.970169990265362</v>
+        <v>0.9701693503400101</v>
       </c>
       <c r="BL13" t="n">
-        <v>687.9657893062114</v>
+        <v>701.8797308239597</v>
       </c>
       <c r="BM13" t="n">
-        <v>526.127280213873</v>
+        <v>531.4210463411554</v>
       </c>
       <c r="BN13" t="n">
-        <v>0.3992677044276236</v>
+        <v>0.3953032684207831</v>
       </c>
       <c r="BO13" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.2975897333830798</v>
       </c>
       <c r="BP13" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.2231923000373098</v>
       </c>
       <c r="BQ13" t="n">
-        <v>0.6989417925686972</v>
+        <v>0.6989511539245858</v>
       </c>
       <c r="BR13" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5665939720200175</v>
       </c>
       <c r="BS13" t="n">
-        <v>0.6418072711878795</v>
+        <v>0.6418331545120342</v>
       </c>
       <c r="BT13" t="n">
-        <v>0.7170409290239167</v>
+        <v>0.7170723370040508</v>
       </c>
       <c r="BU13" t="n">
-        <v>0.5199760699716112</v>
+        <v>0.5200017188605336</v>
       </c>
       <c r="BV13" t="n">
-        <v>0.1119857656225648</v>
+        <v>0.1119863072985829</v>
       </c>
       <c r="BW13" t="n">
-        <v>0.02743158460472156</v>
+        <v>0.02742669883203991</v>
       </c>
     </row>
     <row r="14">
@@ -3534,52 +3534,52 @@
         <v>0.4</v>
       </c>
       <c r="F14" t="n">
-        <v>1.066429875635743</v>
+        <v>1.066314923944042</v>
       </c>
       <c r="G14" t="n">
-        <v>334.9958456714842</v>
+        <v>335.0078830645102</v>
       </c>
       <c r="H14" t="n">
         <v>0.3622224099001629</v>
       </c>
       <c r="I14" t="n">
-        <v>735.3122627165425</v>
+        <v>735.3444098032678</v>
       </c>
       <c r="J14" t="n">
-        <v>1701987.616311639</v>
+        <v>1702214.345293292</v>
       </c>
       <c r="K14" t="n">
-        <v>40649.40174740322</v>
+        <v>40652.32310671354</v>
       </c>
       <c r="L14" t="n">
-        <v>38210.43764255902</v>
+        <v>38213.18372031073</v>
       </c>
       <c r="M14" t="n">
-        <v>30001.60452701078</v>
+        <v>30003.76065878498</v>
       </c>
       <c r="N14" t="n">
-        <v>37.98254238822965</v>
+        <v>37.98527208778403</v>
       </c>
       <c r="O14" t="n">
-        <v>773.2948051047721</v>
+        <v>773.3296818910518</v>
       </c>
       <c r="P14" t="n">
-        <v>773.2948051047721</v>
+        <v>773.3296818910518</v>
       </c>
       <c r="Q14" t="n">
-        <v>1.149295676589019</v>
+        <v>1.149300089664899</v>
       </c>
       <c r="R14" t="n">
-        <v>1956087.009035017</v>
+        <v>1956355.099674458</v>
       </c>
       <c r="S14" t="n">
-        <v>1956087.009035017</v>
+        <v>1956355.099674458</v>
       </c>
       <c r="T14" t="n">
-        <v>496.5382177525278</v>
+        <v>496.5490717009102</v>
       </c>
       <c r="U14" t="n">
-        <v>509.2010881288747</v>
+        <v>509.2125708759257</v>
       </c>
       <c r="V14" t="n">
         <v>0.7615773105863909</v>
@@ -3591,61 +3591,61 @@
         <v>1.064577496794081</v>
       </c>
       <c r="Y14" t="n">
-        <v>100.4987537014453</v>
+        <v>100.5023649193531</v>
       </c>
       <c r="Z14" t="n">
-        <v>0.2314229337341716</v>
+        <v>0.2314261906448897</v>
       </c>
       <c r="AA14" t="n">
-        <v>0.356964158557928</v>
+        <v>0.3569689560278481</v>
       </c>
       <c r="AB14" t="n">
-        <v>0.07416764671794335</v>
+        <v>0.07415839221785263</v>
       </c>
       <c r="AC14" t="n">
         <v>0.3</v>
       </c>
       <c r="AD14" t="n">
-        <v>100.4987537014453</v>
+        <v>100.5023649193531</v>
       </c>
       <c r="AE14" t="n">
-        <v>0.2256678819868194</v>
+        <v>0.2256709019070894</v>
       </c>
       <c r="AF14" t="n">
-        <v>0.3484722271735652</v>
+        <v>0.3484766908783793</v>
       </c>
       <c r="AG14" t="n">
-        <v>0.06779158838817963</v>
+        <v>0.06778295878497693</v>
       </c>
       <c r="AH14" t="n">
-        <v>0.6942136754823024</v>
+        <v>0.6942493179570087</v>
       </c>
       <c r="AI14" t="n">
-        <v>0.9331486173850179</v>
+        <v>0.9331629960006975</v>
       </c>
       <c r="AJ14" t="n">
-        <v>0.9671520930359326</v>
+        <v>0.9671590296081088</v>
       </c>
       <c r="AK14" t="n">
-        <v>0.2963136642575243</v>
+        <v>0.2963184756102546</v>
       </c>
       <c r="AL14" t="n">
-        <v>0.7997749430087898</v>
+        <v>0.799765287469714</v>
       </c>
       <c r="AM14" t="n">
-        <v>0.2774074752935001</v>
+        <v>0.2774134119780806</v>
       </c>
       <c r="AN14" t="n">
-        <v>0.4205268857463317</v>
+        <v>0.4205358468463007</v>
       </c>
       <c r="AO14" t="n">
-        <v>0.05617592261036219</v>
+        <v>0.05616829421908321</v>
       </c>
       <c r="AP14" t="n">
-        <v>0.8643647018111618</v>
+        <v>0.8643681700972499</v>
       </c>
       <c r="AQ14" t="n">
-        <v>0.5450375333038594</v>
+        <v>0.5450353463352045</v>
       </c>
       <c r="AR14" t="n">
         <v>0.4515487103718533</v>
@@ -3654,94 +3654,94 @@
         <v>0.3</v>
       </c>
       <c r="AT14" t="n">
-        <v>0.7542015694605615</v>
+        <v>0.7541927318199282</v>
       </c>
       <c r="AU14" t="n">
-        <v>0.5031662314220492</v>
+        <v>0.5031679264631143</v>
       </c>
       <c r="AV14" t="n">
-        <v>0.3026528590887082</v>
+        <v>0.3026440214480749</v>
       </c>
       <c r="AW14" t="n">
-        <v>0.7915799583252537</v>
+        <v>0.7915718403290021</v>
       </c>
       <c r="AX14" t="n">
-        <v>0.2884137269032045</v>
+        <v>0.2884039138658878</v>
       </c>
       <c r="AY14" t="n">
-        <v>111.3289060246715</v>
+        <v>111.3329064020322</v>
       </c>
       <c r="AZ14" t="n">
-        <v>8.521985360920409</v>
+        <v>8.522757099108716</v>
       </c>
       <c r="BA14" t="n">
-        <v>230.3118040050343</v>
+        <v>230.3200797903587</v>
       </c>
       <c r="BB14" t="n">
-        <v>100.4987537014453</v>
+        <v>100.5023649193531</v>
       </c>
       <c r="BC14" t="n">
-        <v>146.7762958716887</v>
+        <v>146.7829507711086</v>
       </c>
       <c r="BD14" t="n">
-        <v>208.4163973905428</v>
+        <v>208.4232445623261</v>
       </c>
       <c r="BE14" t="n">
-        <v>0.9910739042903115</v>
+        <v>0.9910736530472659</v>
       </c>
       <c r="BF14" t="n">
-        <v>728.7487950830271</v>
+        <v>728.7804704716103</v>
       </c>
       <c r="BG14" t="n">
-        <v>541.4973362719403</v>
+        <v>541.5091043546332</v>
       </c>
       <c r="BH14" t="n">
-        <v>0.4253239832917139</v>
+        <v>0.4253300229639769</v>
       </c>
       <c r="BI14" t="n">
-        <v>0.409300769871478</v>
+        <v>0.4093049867245133</v>
       </c>
       <c r="BJ14" t="n">
-        <v>773.2948051047721</v>
+        <v>773.3296818910518</v>
       </c>
       <c r="BK14" t="n">
-        <v>0.9720788132971026</v>
+        <v>0.972078237973741</v>
       </c>
       <c r="BL14" t="n">
-        <v>689.3193716235928</v>
+        <v>703.2607366638852</v>
       </c>
       <c r="BM14" t="n">
-        <v>526.6446072699015</v>
+        <v>531.943596637915</v>
       </c>
       <c r="BN14" t="n">
-        <v>0.3957439125237845</v>
+        <v>0.3918145568057214</v>
       </c>
       <c r="BO14" t="n">
-        <v>0.2975790404866964</v>
+        <v>0.2975897333830798</v>
       </c>
       <c r="BP14" t="n">
-        <v>0.2231842803650222</v>
+        <v>0.2231923000373098</v>
       </c>
       <c r="BQ14" t="n">
-        <v>0.703031062951131</v>
+        <v>0.7030395913137015</v>
       </c>
       <c r="BR14" t="n">
-        <v>0.5665736133518423</v>
+        <v>0.5665939720200175</v>
       </c>
       <c r="BS14" t="n">
-        <v>0.6430420464888373</v>
+        <v>0.6430677332101528</v>
       </c>
       <c r="BT14" t="n">
-        <v>0.7195104796258323</v>
+        <v>0.7195414944002881</v>
       </c>
       <c r="BU14" t="n">
-        <v>0.5230182728633495</v>
+        <v>0.5230434113419845</v>
       </c>
       <c r="BV14" t="n">
-        <v>0.1104646641766957</v>
+        <v>0.1104654610578574</v>
       </c>
       <c r="BW14" t="n">
-        <v>0.02486696286721923</v>
+        <v>0.02486250775034532</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
again some little fixes and changed books positions
</commit_message>
<xml_diff>
--- a/расчет_ступеней.xlsx
+++ b/расчет_ступеней.xlsx
@@ -728,25 +728,25 @@
         <v>335.007893001304</v>
       </c>
       <c r="G2" t="n">
-        <v>36411.99532705859</v>
+        <v>36411.99532705869</v>
       </c>
       <c r="H2" t="n">
-        <v>36047.875373788</v>
+        <v>36047.87537378811</v>
       </c>
       <c r="I2" t="n">
-        <v>31873.65028930084</v>
+        <v>31873.6502893009</v>
       </c>
       <c r="J2" t="n">
-        <v>35832.87810515706</v>
+        <v>35.83287810515716</v>
       </c>
       <c r="K2" t="n">
-        <v>36120.87810515706</v>
+        <v>323.8328781051572</v>
       </c>
       <c r="L2" t="n">
-        <v>36120.87810515706</v>
+        <v>323.8328781051572</v>
       </c>
       <c r="M2" t="n">
-        <v>1.440944655702847</v>
+        <v>1.440944655702848</v>
       </c>
       <c r="N2" t="n">
         <v>145066.7069330656</v>
@@ -758,28 +758,28 @@
         <v>310.7513475433373</v>
       </c>
       <c r="Q2" t="n">
-        <v>3480.133679711048</v>
+        <v>329.5165610840511</v>
       </c>
       <c r="R2" t="n">
         <v>0.7615773105863909</v>
       </c>
       <c r="S2" t="n">
-        <v>0.1677833565897216</v>
+        <v>0.167783356589721</v>
       </c>
       <c r="T2" t="n">
-        <v>1.213910247893695</v>
+        <v>1.213910247893696</v>
       </c>
       <c r="U2" t="n">
         <v>150.7535518505868</v>
       </c>
       <c r="V2" t="n">
-        <v>0.5177497878149007</v>
+        <v>0.5177497878149004</v>
       </c>
       <c r="W2" t="n">
-        <v>0.7285310911802062</v>
+        <v>0.7285310911802059</v>
       </c>
       <c r="X2" t="n">
-        <v>0.3588841693639397</v>
+        <v>0.3588841693639396</v>
       </c>
       <c r="Y2" t="n">
         <v>0.4384615384615385</v>
@@ -788,41 +788,71 @@
         <v>146.8880761621102</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.04504597726235655</v>
+        <v>0.4757455045369876</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.07099730787528864</v>
+        <v>0.6816773513404401</v>
       </c>
       <c r="AC2" t="n">
-        <v>28.621745553666</v>
-      </c>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="inlineStr"/>
+        <v>0.2822542259235776</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>0.5922128766565673</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>0.8281605716505803</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>0.2135053003617265</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>1.117649652176082</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>0.4958084006661691</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>0.2731322398500622</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>0.1290558392935941</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>0.609671932167811</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>0.7948689411184856</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>0.5689239812174692</v>
+      </c>
       <c r="AN2" t="n">
-        <v>0.6484989891376707</v>
+        <v>0.6484989891376702</v>
       </c>
       <c r="AO2" t="n">
         <v>0.4442307692307692</v>
       </c>
-      <c r="AP2" t="inlineStr"/>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
+      <c r="AP2" t="n">
+        <v>1.100275974329452</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>0.662939786869682</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>0.4517769851917814</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>0.4547098653064001</v>
+      </c>
       <c r="AT2" t="n">
-        <v>249.5957775306275</v>
+        <v>249.5957775306276</v>
       </c>
       <c r="AU2" t="n">
         <v>148.8208140063485</v>
       </c>
-      <c r="AV2" t="inlineStr"/>
+      <c r="AV2" t="n">
+        <v>241.8133924165746</v>
+      </c>
       <c r="AW2" t="n">
         <v>0.9553225262029376</v>
       </c>
@@ -833,16 +863,26 @@
         <v>303.7302375370674</v>
       </c>
       <c r="AZ2" t="n">
-        <v>0.8217679594714923</v>
-      </c>
-      <c r="BA2" t="inlineStr"/>
+        <v>0.8217679594714927</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>0.7338429110241117</v>
+      </c>
       <c r="BB2" t="n">
-        <v>36120.87810515706</v>
-      </c>
-      <c r="BC2" t="inlineStr"/>
-      <c r="BD2" t="inlineStr"/>
-      <c r="BE2" t="inlineStr"/>
-      <c r="BF2" t="inlineStr"/>
+        <v>323.8328781051572</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>0.9102457636566097</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>668.0349528194652</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>473.2780574676653</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>0.5109330310186534</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -864,22 +904,22 @@
         <v>334.8608968769752</v>
       </c>
       <c r="G3" t="n">
-        <v>37081.05894345281</v>
+        <v>37081.05894345287</v>
       </c>
       <c r="H3" t="n">
-        <v>36339.43776458375</v>
+        <v>36339.43776458382</v>
       </c>
       <c r="I3" t="n">
-        <v>32038.30662392289</v>
+        <v>32038.30662392292</v>
       </c>
       <c r="J3" t="n">
-        <v>35979.64135107302</v>
+        <v>35.97964135107308</v>
       </c>
       <c r="K3" t="n">
-        <v>36301.94182320856</v>
+        <v>358.2801134866133</v>
       </c>
       <c r="L3" t="n">
-        <v>36301.94182320856</v>
+        <v>358.2801134866133</v>
       </c>
       <c r="M3" t="n">
         <v>1.390695899350074</v>
@@ -894,25 +934,25 @@
         <v>328.7359857196146</v>
       </c>
       <c r="Q3" t="n">
-        <v>3488.8452378003</v>
+        <v>346.5996567396763</v>
       </c>
       <c r="R3" t="n">
         <v>0.7725018866632134</v>
       </c>
       <c r="S3" t="n">
-        <v>0.1722115499736755</v>
+        <v>0.172211549973675</v>
       </c>
       <c r="T3" t="n">
-        <v>1.196544109661876</v>
+        <v>1.196544109661877</v>
       </c>
       <c r="U3" t="n">
         <v>146.8236240152891</v>
       </c>
       <c r="V3" t="n">
-        <v>0.4798450995388093</v>
+        <v>0.479845099538809</v>
       </c>
       <c r="W3" t="n">
-        <v>0.6863858064760087</v>
+        <v>0.6863858064760082</v>
       </c>
       <c r="X3" t="n">
         <v>0.1735963604307613</v>
@@ -924,41 +964,71 @@
         <v>142.9598444359394</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.04402351689456887</v>
+        <v>0.4431373034630462</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.06938843412514037</v>
+        <v>0.6432243354866706</v>
       </c>
       <c r="AC3" t="n">
-        <v>13.10461017038216</v>
-      </c>
-      <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr"/>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
-      <c r="AL3" t="inlineStr"/>
-      <c r="AM3" t="inlineStr"/>
+        <v>0.1404413998385572</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>0.8227608563817341</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>0.9228017710032826</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>0.2772675463787479</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>0.9948039683717862</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>0.4918175734636512</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>0.1290558392935941</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>0.09293479859248309</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>0.8385262173203589</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>0.847651828833248</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>0.5470706271897741</v>
+      </c>
       <c r="AN3" t="n">
-        <v>0.6308489453405539</v>
+        <v>0.6308489453405535</v>
       </c>
       <c r="AO3" t="n">
         <v>0.4326923076923077</v>
       </c>
-      <c r="AP3" t="inlineStr"/>
-      <c r="AQ3" t="inlineStr"/>
-      <c r="AR3" t="inlineStr"/>
-      <c r="AS3" t="inlineStr"/>
+      <c r="AP3" t="n">
+        <v>0.9636520867716827</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>0.6691833885527213</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>0.3328031414311292</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>0.3256205798190649</v>
+      </c>
       <c r="AT3" t="n">
-        <v>248.9251061897375</v>
+        <v>248.9251061897376</v>
       </c>
       <c r="AU3" t="n">
         <v>144.8917342256143</v>
       </c>
-      <c r="AV3" t="inlineStr"/>
+      <c r="AV3" t="n">
+        <v>233.5661127114676</v>
+      </c>
       <c r="AW3" t="n">
         <v>0.961624780074765</v>
       </c>
@@ -969,16 +1039,26 @@
         <v>322.366623658571</v>
       </c>
       <c r="AZ3" t="n">
-        <v>0.7721801449686746</v>
-      </c>
-      <c r="BA3" t="inlineStr"/>
+        <v>0.7721801449686749</v>
+      </c>
+      <c r="BA3" t="n">
+        <v>0.6738786613597089</v>
+      </c>
       <c r="BB3" t="n">
-        <v>36301.94182320856</v>
-      </c>
-      <c r="BC3" t="inlineStr"/>
-      <c r="BD3" t="inlineStr"/>
-      <c r="BE3" t="inlineStr"/>
-      <c r="BF3" t="inlineStr"/>
+        <v>358.2801134866133</v>
+      </c>
+      <c r="BC3" t="n">
+        <v>0.9243145916273412</v>
+      </c>
+      <c r="BD3" t="n">
+        <v>678.360152018303</v>
+      </c>
+      <c r="BE3" t="n">
+        <v>476.9215438326696</v>
+      </c>
+      <c r="BF3" t="n">
+        <v>0.4897369719020609</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1000,22 +1080,22 @@
         <v>334.7139007526465</v>
       </c>
       <c r="G4" t="n">
-        <v>37708.0443788087</v>
+        <v>37708.04437880874</v>
       </c>
       <c r="H4" t="n">
-        <v>36576.80304744444</v>
+        <v>36576.80304744447</v>
       </c>
       <c r="I4" t="n">
-        <v>32124.59638269979</v>
+        <v>32124.59638269978</v>
       </c>
       <c r="J4" t="n">
-        <v>36043.64141937289</v>
+        <v>36.04364141937292</v>
       </c>
       <c r="K4" t="n">
-        <v>36400.24236364396</v>
+        <v>392.6445856904533</v>
       </c>
       <c r="L4" t="n">
-        <v>36400.24236364396</v>
+        <v>392.6445856904533</v>
       </c>
       <c r="M4" t="n">
         <v>1.350089833806659</v>
@@ -1030,22 +1110,22 @@
         <v>345.7864899241919</v>
       </c>
       <c r="Q4" t="n">
-        <v>3493.565694892515</v>
+        <v>362.841190580685</v>
       </c>
       <c r="R4" t="n">
         <v>0.7842900694668242</v>
       </c>
       <c r="S4" t="n">
-        <v>0.177569699551567</v>
+        <v>0.1775696995515668</v>
       </c>
       <c r="T4" t="n">
-        <v>1.176633893900265</v>
+        <v>1.176633893900266</v>
       </c>
       <c r="U4" t="n">
         <v>142.8970883982452</v>
       </c>
       <c r="V4" t="n">
-        <v>0.4475729189884194</v>
+        <v>0.4475729189884193</v>
       </c>
       <c r="W4" t="n">
         <v>0.6485576489170397</v>
@@ -1060,41 +1140,71 @@
         <v>139.0350049280224</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.04310262147926873</v>
+        <v>0.415007567136801</v>
       </c>
       <c r="AB4" t="n">
-        <v>0.06793922069888089</v>
+        <v>0.6086768365849144</v>
       </c>
       <c r="AC4" t="n">
-        <v>8.852684035607712</v>
-      </c>
-      <c r="AD4" t="inlineStr"/>
-      <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr"/>
-      <c r="AI4" t="inlineStr"/>
-      <c r="AJ4" t="inlineStr"/>
-      <c r="AK4" t="inlineStr"/>
-      <c r="AL4" t="inlineStr"/>
-      <c r="AM4" t="inlineStr"/>
+        <v>0.1026257677193531</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>0.8740278426607593</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>0.9450442593643356</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>0.2903669344696717</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>0.9607206522143688</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>0.4675231842410476</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>0.09293479859248309</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>0.07707028988055241</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>0.8866889557871865</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>0.8646671644155799</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>0.5503213035612302</v>
+      </c>
       <c r="AN4" t="n">
-        <v>0.6131761582556861</v>
+        <v>0.6131761582556859</v>
       </c>
       <c r="AO4" t="n">
         <v>0.4211538461538462</v>
       </c>
-      <c r="AP4" t="inlineStr"/>
-      <c r="AQ4" t="inlineStr"/>
-      <c r="AR4" t="inlineStr"/>
-      <c r="AS4" t="inlineStr"/>
+      <c r="AP4" t="n">
+        <v>0.9296083408833998</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>0.653213338356202</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>0.3164321826277139</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>0.3075073138581668</v>
+      </c>
       <c r="AT4" t="n">
         <v>248.3146130188819</v>
       </c>
       <c r="AU4" t="n">
         <v>140.9660466631338</v>
       </c>
-      <c r="AV4" t="inlineStr"/>
+      <c r="AV4" t="n">
+        <v>231.9507197122134</v>
+      </c>
       <c r="AW4" t="n">
         <v>0.9666130803646976</v>
       </c>
@@ -1107,14 +1217,24 @@
       <c r="AZ4" t="n">
         <v>0.7304120392625181</v>
       </c>
-      <c r="BA4" t="inlineStr"/>
+      <c r="BA4" t="n">
+        <v>0.639262370793689</v>
+      </c>
       <c r="BB4" t="n">
-        <v>36400.24236364396</v>
-      </c>
-      <c r="BC4" t="inlineStr"/>
-      <c r="BD4" t="inlineStr"/>
-      <c r="BE4" t="inlineStr"/>
-      <c r="BF4" t="inlineStr"/>
+        <v>392.6445856904533</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>0.931890603547872</v>
+      </c>
+      <c r="BD4" t="n">
+        <v>683.9202336665388</v>
+      </c>
+      <c r="BE4" t="n">
+        <v>478.8720646982767</v>
+      </c>
+      <c r="BF4" t="n">
+        <v>0.4843688676188677</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1136,22 +1256,22 @@
         <v>334.5669046283177</v>
       </c>
       <c r="G5" t="n">
-        <v>38288.30593027177</v>
+        <v>38288.30593027178</v>
       </c>
       <c r="H5" t="n">
-        <v>36756.7736930609</v>
+        <v>36756.77369306091</v>
       </c>
       <c r="I5" t="n">
-        <v>32129.24271355218</v>
+        <v>32129.24271355215</v>
       </c>
       <c r="J5" t="n">
-        <v>36168.23999357074</v>
+        <v>36.16823999357076</v>
       </c>
       <c r="K5" t="n">
-        <v>36559.14140997736</v>
+        <v>427.0696564001913</v>
       </c>
       <c r="L5" t="n">
-        <v>36559.14140997736</v>
+        <v>427.0696564001913</v>
       </c>
       <c r="M5" t="n">
         <v>1.316368240203566</v>
@@ -1166,25 +1286,25 @@
         <v>362.0348669964536</v>
       </c>
       <c r="Q5" t="n">
-        <v>3501.182673721183</v>
+        <v>378.4130756078391</v>
       </c>
       <c r="R5" t="n">
         <v>0.7969035352526399</v>
       </c>
       <c r="S5" t="n">
-        <v>0.1838346066436046</v>
+        <v>0.1838346066436044</v>
       </c>
       <c r="T5" t="n">
         <v>1.154142696849574</v>
       </c>
       <c r="U5" t="n">
-        <v>138.9739449994551</v>
+        <v>138.973944999455</v>
       </c>
       <c r="V5" t="n">
-        <v>0.4197819976689975</v>
+        <v>0.4197819976689973</v>
       </c>
       <c r="W5" t="n">
-        <v>0.6146271972579198</v>
+        <v>0.6146271972579196</v>
       </c>
       <c r="X5" t="n">
         <v>0.1013539366335962</v>
@@ -1196,41 +1316,71 @@
         <v>135.1135576383591</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.04220121761521685</v>
+        <v>0.3904573637869123</v>
       </c>
       <c r="AB5" t="n">
-        <v>0.06652054161390027</v>
+        <v>0.5775401427632009</v>
       </c>
       <c r="AC5" t="n">
-        <v>6.87992327625264</v>
-      </c>
-      <c r="AD5" t="inlineStr"/>
-      <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr"/>
-      <c r="AI5" t="inlineStr"/>
-      <c r="AJ5" t="inlineStr"/>
-      <c r="AK5" t="inlineStr"/>
-      <c r="AL5" t="inlineStr"/>
-      <c r="AM5" t="inlineStr"/>
+        <v>0.08564629091578738</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>0.8960934288795586</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>0.954649477405116</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>0.294603227788098</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>0.9405489337121995</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>0.4419620774952459</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>0.07707028988055241</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>0.06855040237940825</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>0.9070343154587495</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>0.8757765063288779</v>
+      </c>
+      <c r="AM5" t="n">
+        <v>0.5578555636415101</v>
+      </c>
       <c r="AN5" t="n">
-        <v>0.5954991555222526</v>
+        <v>0.5954991555222525</v>
       </c>
       <c r="AO5" t="n">
         <v>0.4096153846153846</v>
       </c>
-      <c r="AP5" t="inlineStr"/>
-      <c r="AQ5" t="inlineStr"/>
-      <c r="AR5" t="inlineStr"/>
-      <c r="AS5" t="inlineStr"/>
+      <c r="AP5" t="n">
+        <v>0.9107712941505934</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>0.6333562460279528</v>
+      </c>
+      <c r="AR5" t="n">
+        <v>0.3152721386283409</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>0.3071926876842467</v>
+      </c>
       <c r="AT5" t="n">
         <v>247.7598137444</v>
       </c>
       <c r="AU5" t="n">
         <v>137.0437513189071</v>
       </c>
-      <c r="AV5" t="inlineStr"/>
+      <c r="AV5" t="n">
+        <v>231.5501733831518</v>
+      </c>
       <c r="AW5" t="n">
         <v>0.9706305124055044</v>
       </c>
@@ -1243,14 +1393,24 @@
       <c r="AZ5" t="n">
         <v>0.6946299383584459</v>
       </c>
-      <c r="BA5" t="inlineStr"/>
+      <c r="BA5" t="n">
+        <v>0.6118979187260279</v>
+      </c>
       <c r="BB5" t="n">
-        <v>36559.14140997736</v>
-      </c>
-      <c r="BC5" t="inlineStr"/>
-      <c r="BD5" t="inlineStr"/>
-      <c r="BE5" t="inlineStr"/>
-      <c r="BF5" t="inlineStr"/>
+        <v>427.0696564001913</v>
+      </c>
+      <c r="BC5" t="n">
+        <v>0.9375968228431258</v>
+      </c>
+      <c r="BD5" t="n">
+        <v>688.1080630307417</v>
+      </c>
+      <c r="BE5" t="n">
+        <v>480.3359590268125</v>
+      </c>
+      <c r="BF5" t="n">
+        <v>0.4820587945409821</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1278,16 +1438,16 @@
         <v>36875.92322328367</v>
       </c>
       <c r="I6" t="n">
-        <v>32049.09574441157</v>
+        <v>32049.09574441154</v>
       </c>
       <c r="J6" t="n">
-        <v>36116.59964737081</v>
+        <v>36.11659964737082</v>
       </c>
       <c r="K6" t="n">
-        <v>36541.80153591298</v>
+        <v>461.3184881895316</v>
       </c>
       <c r="L6" t="n">
-        <v>36541.80153591298</v>
+        <v>461.3184881895316</v>
       </c>
       <c r="M6" t="n">
         <v>1.287723328197106</v>
@@ -1302,13 +1462,13 @@
         <v>377.5846835190571</v>
       </c>
       <c r="Q6" t="n">
-        <v>3500.352275841908</v>
+        <v>393.2938965836489</v>
       </c>
       <c r="R6" t="n">
         <v>0.8103037450239648</v>
       </c>
       <c r="S6" t="n">
-        <v>0.190982577259829</v>
+        <v>0.1909825772598289</v>
       </c>
       <c r="T6" t="n">
         <v>1.129055245477055</v>
@@ -1323,7 +1483,7 @@
         <v>0.584211559070294</v>
       </c>
       <c r="X6" t="n">
-        <v>0.08880215565753605</v>
+        <v>0.08880215565753603</v>
       </c>
       <c r="Y6" t="n">
         <v>0.3923076923076923</v>
@@ -1332,41 +1492,71 @@
         <v>131.1955025669495</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.04146050473926558</v>
+        <v>0.3690023501058217</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.06535466559558402</v>
+        <v>0.5496154015473974</v>
       </c>
       <c r="AC6" t="n">
-        <v>5.714679499973112</v>
-      </c>
-      <c r="AD6" t="inlineStr"/>
-      <c r="AE6" t="inlineStr"/>
-      <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="inlineStr"/>
-      <c r="AI6" t="inlineStr"/>
-      <c r="AJ6" t="inlineStr"/>
-      <c r="AK6" t="inlineStr"/>
-      <c r="AL6" t="inlineStr"/>
-      <c r="AM6" t="inlineStr"/>
+        <v>0.07635105351990513</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>0.9079458936530936</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>0.9597681971993625</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>0.2958374898032921</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>0.924679206882428</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>0.4177978186232196</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>0.06855040237940825</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>0.06358754747461096</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>0.9177744737737201</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>0.8850359711116637</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>0.5670258362285011</v>
+      </c>
       <c r="AN6" t="n">
         <v>0.5778351468572825</v>
       </c>
       <c r="AO6" t="n">
         <v>0.3980769230769231</v>
       </c>
-      <c r="AP6" t="inlineStr"/>
-      <c r="AQ6" t="inlineStr"/>
-      <c r="AR6" t="inlineStr"/>
-      <c r="AS6" t="inlineStr"/>
+      <c r="AP6" t="n">
+        <v>0.896747206582462</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>0.6120962668994687</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>0.3189120597251794</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>0.3125829399829593</v>
+      </c>
       <c r="AT6" t="n">
         <v>247.256073758147</v>
       </c>
       <c r="AU6" t="n">
         <v>133.1248481929341</v>
       </c>
-      <c r="AV6" t="inlineStr"/>
+      <c r="AV6" t="n">
+        <v>231.6889353815089</v>
+      </c>
       <c r="AW6" t="n">
         <v>0.9739089868444597</v>
       </c>
@@ -1379,14 +1569,24 @@
       <c r="AZ6" t="n">
         <v>0.6635496323942373</v>
       </c>
-      <c r="BA6" t="inlineStr"/>
+      <c r="BA6" t="n">
+        <v>0.5890987309848359</v>
+      </c>
       <c r="BB6" t="n">
-        <v>36541.80153591298</v>
-      </c>
-      <c r="BC6" t="inlineStr"/>
-      <c r="BD6" t="inlineStr"/>
-      <c r="BE6" t="inlineStr"/>
-      <c r="BF6" t="inlineStr"/>
+        <v>461.3184881895316</v>
+      </c>
+      <c r="BC6" t="n">
+        <v>0.9421604475253427</v>
+      </c>
+      <c r="BD6" t="n">
+        <v>691.4573351954629</v>
+      </c>
+      <c r="BE6" t="n">
+        <v>481.5035248999105</v>
+      </c>
+      <c r="BF6" t="n">
+        <v>0.4811780670342335</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1408,22 +1608,22 @@
         <v>334.2729123796602</v>
       </c>
       <c r="G7" t="n">
-        <v>39287.89350685771</v>
+        <v>39287.89350685768</v>
       </c>
       <c r="H7" t="n">
-        <v>36930.61989644625</v>
+        <v>36930.61989644622</v>
       </c>
       <c r="I7" t="n">
-        <v>31881.19329867558</v>
+        <v>31881.19329867551</v>
       </c>
       <c r="J7" t="n">
-        <v>35976.50928166557</v>
+        <v>35.97650928166554</v>
       </c>
       <c r="K7" t="n">
-        <v>36436.01164234327</v>
+        <v>495.4788699593665</v>
       </c>
       <c r="L7" t="n">
-        <v>36436.01164234327</v>
+        <v>495.4788699593665</v>
       </c>
       <c r="M7" t="n">
         <v>1.262922611929034</v>
@@ -1438,25 +1638,25 @@
         <v>392.5189696501726</v>
       </c>
       <c r="Q7" t="n">
-        <v>3495.28177743622</v>
+        <v>407.5954674642195</v>
       </c>
       <c r="R7" t="n">
         <v>0.8244523377184381</v>
       </c>
       <c r="S7" t="n">
-        <v>0.1989900230881153</v>
+        <v>0.1989900230881154</v>
       </c>
       <c r="T7" t="n">
-        <v>1.101381881882768</v>
+        <v>1.101381881882767</v>
       </c>
       <c r="U7" t="n">
         <v>131.1378348566359</v>
       </c>
       <c r="V7" t="n">
-        <v>0.3746137054218504</v>
+        <v>0.3746137054218505</v>
       </c>
       <c r="W7" t="n">
-        <v>0.5569812067003773</v>
+        <v>0.5569812067003774</v>
       </c>
       <c r="X7" t="n">
         <v>0.08107434726661611</v>
@@ -1468,41 +1668,71 @@
         <v>127.2808397137937</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.0408316699655482</v>
+        <v>0.3501466610037778</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.06436481437757731</v>
+        <v>0.5245508609268315</v>
       </c>
       <c r="AC7" t="n">
-        <v>4.946753673599506</v>
-      </c>
-      <c r="AD7" t="inlineStr"/>
-      <c r="AE7" t="inlineStr"/>
-      <c r="AF7" t="inlineStr"/>
-      <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr"/>
-      <c r="AI7" t="inlineStr"/>
-      <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="inlineStr"/>
-      <c r="AL7" t="inlineStr"/>
-      <c r="AM7" t="inlineStr"/>
+        <v>0.07078290052051256</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>0.9149723790623341</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>0.9627373200998649</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>0.2957865509268111</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>0.9103544675172746</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>0.3954211232783114</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>0.06358754747461096</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>0.06056357647098572</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>0.9239731029776458</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>0.8935948289091515</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>0.5770667541588699</v>
+      </c>
       <c r="AN7" t="n">
-        <v>0.5602001159796426</v>
+        <v>0.5602001159796427</v>
       </c>
       <c r="AO7" t="n">
         <v>0.3865384615384615</v>
       </c>
-      <c r="AP7" t="inlineStr"/>
-      <c r="AQ7" t="inlineStr"/>
-      <c r="AR7" t="inlineStr"/>
-      <c r="AS7" t="inlineStr"/>
+      <c r="AP7" t="n">
+        <v>0.8846495783834111</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>0.5901916054573306</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>0.3244494624037684</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>0.3201628620599439</v>
+      </c>
       <c r="AT7" t="n">
         <v>246.7985679482697</v>
       </c>
       <c r="AU7" t="n">
         <v>129.2093372852148</v>
       </c>
-      <c r="AV7" t="inlineStr"/>
+      <c r="AV7" t="n">
+        <v>232.1736594147696</v>
+      </c>
       <c r="AW7" t="n">
         <v>0.9766107619516852</v>
       </c>
@@ -1515,14 +1745,24 @@
       <c r="AZ7" t="n">
         <v>0.636240385113307</v>
       </c>
-      <c r="BA7" t="inlineStr"/>
+      <c r="BA7" t="n">
+        <v>0.5696178636607405</v>
+      </c>
       <c r="BB7" t="n">
-        <v>36436.01164234327</v>
-      </c>
-      <c r="BC7" t="inlineStr"/>
-      <c r="BD7" t="inlineStr"/>
-      <c r="BE7" t="inlineStr"/>
-      <c r="BF7" t="inlineStr"/>
+        <v>495.4788699593665</v>
+      </c>
+      <c r="BC7" t="n">
+        <v>0.9459225815664291</v>
+      </c>
+      <c r="BD7" t="n">
+        <v>694.2183884592996</v>
+      </c>
+      <c r="BE7" t="n">
+        <v>482.4639112414556</v>
+      </c>
+      <c r="BF7" t="n">
+        <v>0.4812249248184184</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1544,43 +1784,43 @@
         <v>334.1259162553314</v>
       </c>
       <c r="G8" t="n">
-        <v>39695.3984833665</v>
+        <v>39695.39848336647</v>
       </c>
       <c r="H8" t="n">
-        <v>37313.67457436451</v>
+        <v>37313.67457436448</v>
       </c>
       <c r="I8" t="n">
-        <v>31962.7988129392</v>
+        <v>31962.79881293913</v>
       </c>
       <c r="J8" t="n">
-        <v>36121.36421242807</v>
+        <v>36.12136421242803</v>
       </c>
       <c r="K8" t="n">
-        <v>36615.16704524131</v>
+        <v>529.9241970256692</v>
       </c>
       <c r="L8" t="n">
-        <v>36615.16704524131</v>
+        <v>529.9241970256692</v>
       </c>
       <c r="M8" t="n">
-        <v>1.243895574934569</v>
+        <v>1.243895574934568</v>
       </c>
       <c r="N8" t="n">
-        <v>1129636.632014789</v>
+        <v>1129636.632014788</v>
       </c>
       <c r="O8" t="n">
-        <v>1129636.632014789</v>
+        <v>1129636.632014788</v>
       </c>
       <c r="P8" t="n">
         <v>406.9055048070495</v>
       </c>
       <c r="Q8" t="n">
-        <v>3503.864368132621</v>
+        <v>421.525305601819</v>
       </c>
       <c r="R8" t="n">
         <v>0.8393114668624276</v>
       </c>
       <c r="S8" t="n">
-        <v>0.2078358677458283</v>
+        <v>0.2078358677458284</v>
       </c>
       <c r="T8" t="n">
         <v>1.071159076681218</v>
@@ -1592,7 +1832,7 @@
         <v>0.3562086255178994</v>
       </c>
       <c r="W8" t="n">
-        <v>0.5326608273947991</v>
+        <v>0.5326608273947993</v>
       </c>
       <c r="X8" t="n">
         <v>0.07606035983189825</v>
@@ -1604,41 +1844,71 @@
         <v>123.3695690788916</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.04011314825615143</v>
+        <v>0.3334343846039873</v>
       </c>
       <c r="AB8" t="n">
-        <v>0.06323370877881927</v>
+        <v>0.501945251869729</v>
       </c>
       <c r="AC8" t="n">
-        <v>4.435374331513103</v>
-      </c>
-      <c r="AD8" t="inlineStr"/>
-      <c r="AE8" t="inlineStr"/>
-      <c r="AF8" t="inlineStr"/>
-      <c r="AG8" t="inlineStr"/>
-      <c r="AH8" t="inlineStr"/>
-      <c r="AI8" t="inlineStr"/>
-      <c r="AJ8" t="inlineStr"/>
-      <c r="AK8" t="inlineStr"/>
-      <c r="AL8" t="inlineStr"/>
-      <c r="AM8" t="inlineStr"/>
+        <v>0.06722006815433129</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>0.9194401671295115</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>0.9645419874248758</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>0.2952009644321385</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>0.8963587435290984</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>0.3747148934556732</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>0.06056357647098572</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>0.05888113047881129</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>0.9277297510649634</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>0.9019267271436517</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>0.5876361077145108</v>
+      </c>
       <c r="AN8" t="n">
         <v>0.5426102049201035</v>
       </c>
       <c r="AO8" t="n">
         <v>0.375</v>
       </c>
-      <c r="AP8" t="inlineStr"/>
-      <c r="AQ8" t="inlineStr"/>
-      <c r="AR8" t="inlineStr"/>
-      <c r="AS8" t="inlineStr"/>
+      <c r="AP8" t="n">
+        <v>0.8732466361975925</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>0.5679996810907018</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>0.330636431277489</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>0.3283590624383966</v>
+      </c>
       <c r="AT8" t="n">
         <v>246.3817046229869</v>
       </c>
       <c r="AU8" t="n">
         <v>125.2972185957493</v>
       </c>
-      <c r="AV8" t="inlineStr"/>
+      <c r="AV8" t="n">
+        <v>232.9174471314975</v>
+      </c>
       <c r="AW8" t="n">
         <v>0.9788525691844415</v>
       </c>
@@ -1651,14 +1921,24 @@
       <c r="AZ8" t="n">
         <v>0.61200680035082</v>
       </c>
-      <c r="BA8" t="inlineStr"/>
+      <c r="BA8" t="n">
+        <v>0.5525586341701532</v>
+      </c>
       <c r="BB8" t="n">
-        <v>36615.16704524131</v>
-      </c>
-      <c r="BC8" t="inlineStr"/>
-      <c r="BD8" t="inlineStr"/>
-      <c r="BE8" t="inlineStr"/>
-      <c r="BF8" t="inlineStr"/>
+        <v>529.9241970256692</v>
+      </c>
+      <c r="BC8" t="n">
+        <v>0.9491131593006692</v>
+      </c>
+      <c r="BD8" t="n">
+        <v>696.5599730414654</v>
+      </c>
+      <c r="BE8" t="n">
+        <v>483.2768967794792</v>
+      </c>
+      <c r="BF8" t="n">
+        <v>0.4819544420261797</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1680,43 +1960,43 @@
         <v>333.9789201310027</v>
       </c>
       <c r="G9" t="n">
-        <v>40033.66788134909</v>
+        <v>40033.66788134898</v>
       </c>
       <c r="H9" t="n">
-        <v>37631.64780846814</v>
+        <v>37631.64780846803</v>
       </c>
       <c r="I9" t="n">
-        <v>31951.43722511351</v>
+        <v>31951.43722511338</v>
       </c>
       <c r="J9" t="n">
-        <v>36197.47973519635</v>
+        <v>36.19747973519625</v>
       </c>
       <c r="K9" t="n">
-        <v>36725.58304014513</v>
+        <v>564.3007846839776</v>
       </c>
       <c r="L9" t="n">
-        <v>36725.58304014513</v>
+        <v>564.3007846839776</v>
       </c>
       <c r="M9" t="n">
-        <v>1.226798626151879</v>
+        <v>1.226798626151878</v>
       </c>
       <c r="N9" t="n">
-        <v>1279210.556326686</v>
+        <v>1279210.556326685</v>
       </c>
       <c r="O9" t="n">
-        <v>1279210.556326686</v>
+        <v>1279210.556326685</v>
       </c>
       <c r="P9" t="n">
         <v>420.8004730859109</v>
       </c>
       <c r="Q9" t="n">
-        <v>3509.143484293662</v>
+        <v>434.9828193211057</v>
       </c>
       <c r="R9" t="n">
         <v>0.8548440810533523</v>
       </c>
       <c r="S9" t="n">
-        <v>0.217494042091713</v>
+        <v>0.2174940420917135</v>
       </c>
       <c r="T9" t="n">
         <v>1.038469904488946</v>
@@ -1725,10 +2005,10 @@
         <v>123.3152935868318</v>
       </c>
       <c r="V9" t="n">
-        <v>0.3401109302577575</v>
+        <v>0.3401109302577576</v>
       </c>
       <c r="W9" t="n">
-        <v>0.5110190907706705</v>
+        <v>0.5110190907706706</v>
       </c>
       <c r="X9" t="n">
         <v>0.07274357402768651</v>
@@ -1740,41 +2020,71 @@
         <v>119.4616906622433</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.03951003349211687</v>
+        <v>0.318739891404164</v>
       </c>
       <c r="AB9" t="n">
-        <v>0.0622842151299508</v>
+        <v>0.4817789938534903</v>
       </c>
       <c r="AC9" t="n">
-        <v>4.057003568602814</v>
-      </c>
-      <c r="AD9" t="inlineStr"/>
-      <c r="AE9" t="inlineStr"/>
-      <c r="AF9" t="inlineStr"/>
-      <c r="AG9" t="inlineStr"/>
-      <c r="AH9" t="inlineStr"/>
-      <c r="AI9" t="inlineStr"/>
-      <c r="AJ9" t="inlineStr"/>
-      <c r="AK9" t="inlineStr"/>
-      <c r="AL9" t="inlineStr"/>
-      <c r="AM9" t="inlineStr"/>
+        <v>0.06501394252454777</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>0.9221957954528871</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>0.9655445893469043</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>0.2943757274641756</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>0.8821958879190526</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>0.3556826468593637</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>0.05888113047881129</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>0.05815806913968136</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>0.9298132651420739</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>0.9101943352001283</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>0.5985918471418362</v>
+      </c>
       <c r="AN9" t="n">
-        <v>0.5250761583694251</v>
+        <v>0.5250761583694254</v>
       </c>
       <c r="AO9" t="n">
         <v>0.3634615384615385</v>
       </c>
-      <c r="AP9" t="inlineStr"/>
-      <c r="AQ9" t="inlineStr"/>
-      <c r="AR9" t="inlineStr"/>
-      <c r="AS9" t="inlineStr"/>
+      <c r="AP9" t="n">
+        <v>0.8620685138187281</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>0.5456926176210596</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>0.3369923554493026</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>0.336503270297993</v>
+      </c>
       <c r="AT9" t="n">
-        <v>246.0013624874196</v>
+        <v>246.0013624874193</v>
       </c>
       <c r="AU9" t="n">
         <v>121.3884921245375</v>
       </c>
-      <c r="AV9" t="inlineStr"/>
+      <c r="AV9" t="n">
+        <v>233.8845791893684</v>
+      </c>
       <c r="AW9" t="n">
         <v>0.9807207591865338</v>
       </c>
@@ -1785,16 +2095,26 @@
         <v>416.7243746234115</v>
       </c>
       <c r="AZ9" t="n">
-        <v>0.5903215109740769</v>
-      </c>
-      <c r="BA9" t="inlineStr"/>
+        <v>0.5903215109740764</v>
+      </c>
+      <c r="BA9" t="n">
+        <v>0.5376869356688639</v>
+      </c>
       <c r="BB9" t="n">
-        <v>36725.58304014513</v>
-      </c>
-      <c r="BC9" t="inlineStr"/>
-      <c r="BD9" t="inlineStr"/>
-      <c r="BE9" t="inlineStr"/>
-      <c r="BF9" t="inlineStr"/>
+        <v>564.3007846839776</v>
+      </c>
+      <c r="BC9" t="n">
+        <v>0.9518154598685045</v>
+      </c>
+      <c r="BD9" t="n">
+        <v>698.5432080142774</v>
+      </c>
+      <c r="BE9" t="n">
+        <v>483.9643970863841</v>
+      </c>
+      <c r="BF9" t="n">
+        <v>0.4832681507098998</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1816,58 +2136,58 @@
         <v>333.8319240066739</v>
       </c>
       <c r="G10" t="n">
-        <v>40295.48134264065</v>
+        <v>40295.48134264052</v>
       </c>
       <c r="H10" t="n">
-        <v>37877.75246208221</v>
+        <v>37877.75246208208</v>
       </c>
       <c r="I10" t="n">
-        <v>31841.82633685333</v>
+        <v>31841.82633685318</v>
       </c>
       <c r="J10" t="n">
-        <v>36186.7862447195</v>
+        <v>36.18678624471938</v>
       </c>
       <c r="K10" t="n">
-        <v>36749.19002180382</v>
+        <v>598.5905633290409</v>
       </c>
       <c r="L10" t="n">
-        <v>36749.19002180382</v>
+        <v>598.5905633290409</v>
       </c>
       <c r="M10" t="n">
-        <v>1.211229011137438</v>
+        <v>1.211229011137437</v>
       </c>
       <c r="N10" t="n">
-        <v>1425980.856751485</v>
+        <v>1425980.856751484</v>
       </c>
       <c r="O10" t="n">
-        <v>1425980.856751485</v>
+        <v>1425980.856751484</v>
       </c>
       <c r="P10" t="n">
         <v>434.2510638517458</v>
       </c>
       <c r="Q10" t="n">
-        <v>3510.271131167908</v>
+        <v>448.0038123545685</v>
       </c>
       <c r="R10" t="n">
         <v>0.8710141506800956</v>
       </c>
       <c r="S10" t="n">
-        <v>0.2279462396392059</v>
+        <v>0.2279462396392065</v>
       </c>
       <c r="T10" t="n">
-        <v>1.003422927048463</v>
+        <v>1.003422927048462</v>
       </c>
       <c r="U10" t="n">
         <v>119.4091112793103</v>
       </c>
       <c r="V10" t="n">
-        <v>0.3260667458821139</v>
+        <v>0.3260667458821142</v>
       </c>
       <c r="W10" t="n">
-        <v>0.4918673171729251</v>
+        <v>0.4918673171729253</v>
       </c>
       <c r="X10" t="n">
-        <v>0.07057645739235101</v>
+        <v>0.07057645739235102</v>
       </c>
       <c r="Y10" t="n">
         <v>0.3461538461538461</v>
@@ -1876,43 +2196,73 @@
         <v>115.5572044638487</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.03903608894097606</v>
+        <v>0.3058618081016736</v>
       </c>
       <c r="AB10" t="n">
-        <v>0.06153803651945741</v>
+        <v>0.4638913822085473</v>
       </c>
       <c r="AC10" t="n">
-        <v>3.764763444764367</v>
-      </c>
-      <c r="AD10" t="inlineStr"/>
-      <c r="AE10" t="inlineStr"/>
-      <c r="AF10" t="inlineStr"/>
-      <c r="AG10" t="inlineStr"/>
-      <c r="AH10" t="inlineStr"/>
-      <c r="AI10" t="inlineStr"/>
-      <c r="AJ10" t="inlineStr"/>
-      <c r="AK10" t="inlineStr"/>
-      <c r="AL10" t="inlineStr"/>
-      <c r="AM10" t="inlineStr"/>
+        <v>0.06373912111679632</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>0.9237844025439431</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>0.9659751557909323</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>0.2935198956157492</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>0.8674957122980209</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>0.3381854374395047</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>0.05815806913968136</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>0.05818116247847879</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>0.9307072596744004</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>0.9184946532355139</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>0.6098252705029964</v>
+      </c>
       <c r="AN10" t="n">
-        <v>0.507612123231385</v>
+        <v>0.5076121232313855</v>
       </c>
       <c r="AO10" t="n">
         <v>0.3519230769230769</v>
       </c>
-      <c r="AP10" t="inlineStr"/>
-      <c r="AQ10" t="inlineStr"/>
-      <c r="AR10" t="inlineStr"/>
-      <c r="AS10" t="inlineStr"/>
+      <c r="AP10" t="n">
+        <v>0.8507819547078326</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>0.5234023357991608</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>0.3431698314764471</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>0.3440933764988601</v>
+      </c>
       <c r="AT10" t="n">
-        <v>245.6513333762859</v>
+        <v>245.6513333762857</v>
       </c>
       <c r="AU10" t="n">
         <v>117.4831578715795</v>
       </c>
-      <c r="AV10" t="inlineStr"/>
+      <c r="AV10" t="n">
+        <v>235.0462933011952</v>
+      </c>
       <c r="AW10" t="n">
-        <v>0.9822800795383082</v>
+        <v>0.9822800795383081</v>
       </c>
       <c r="AX10" t="n">
         <v>552.4380268870323</v>
@@ -1921,16 +2271,26 @@
         <v>430.3864198777907</v>
       </c>
       <c r="AZ10" t="n">
-        <v>0.5707692483560219</v>
-      </c>
-      <c r="BA10" t="inlineStr"/>
+        <v>0.5707692483560215</v>
+      </c>
+      <c r="BA10" t="n">
+        <v>0.5246524400447958</v>
+      </c>
       <c r="BB10" t="n">
-        <v>36749.19002180382</v>
-      </c>
-      <c r="BC10" t="inlineStr"/>
-      <c r="BD10" t="inlineStr"/>
-      <c r="BE10" t="inlineStr"/>
-      <c r="BF10" t="inlineStr"/>
+        <v>598.5905633290409</v>
+      </c>
+      <c r="BC10" t="n">
+        <v>0.9541233028591737</v>
+      </c>
+      <c r="BD10" t="n">
+        <v>700.2369481501206</v>
+      </c>
+      <c r="BE10" t="n">
+        <v>484.5507700073703</v>
+      </c>
+      <c r="BF10" t="n">
+        <v>0.4850808374478902</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1952,55 +2312,55 @@
         <v>333.6849278823452</v>
       </c>
       <c r="G11" t="n">
-        <v>40473.60344287158</v>
+        <v>40473.60344287136</v>
       </c>
       <c r="H11" t="n">
-        <v>38045.18723629928</v>
+        <v>38045.18723629908</v>
       </c>
       <c r="I11" t="n">
-        <v>31629.06019140607</v>
+        <v>31629.06019140586</v>
       </c>
       <c r="J11" t="n">
-        <v>36050.14175460383</v>
+        <v>36.05014175460364</v>
       </c>
       <c r="K11" t="n">
-        <v>36646.84600382369</v>
+        <v>632.7543909744653</v>
       </c>
       <c r="L11" t="n">
-        <v>36646.84600382369</v>
+        <v>632.7543909744653</v>
       </c>
       <c r="M11" t="n">
-        <v>1.19688358885424</v>
+        <v>1.196883588854239</v>
       </c>
       <c r="N11" t="n">
-        <v>1570166.486665584</v>
+        <v>1570166.486665582</v>
       </c>
       <c r="O11" t="n">
-        <v>1570166.486665584</v>
+        <v>1570166.486665582</v>
       </c>
       <c r="P11" t="n">
         <v>447.297367266363</v>
       </c>
       <c r="Q11" t="n">
-        <v>3505.37978899321</v>
+        <v>460.6110585881957</v>
       </c>
       <c r="R11" t="n">
         <v>0.8877868447582528</v>
       </c>
       <c r="S11" t="n">
-        <v>0.239173555716144</v>
+        <v>0.239173555716145</v>
       </c>
       <c r="T11" t="n">
-        <v>0.9661728705893988</v>
+        <v>0.9661728705893968</v>
       </c>
       <c r="U11" t="n">
         <v>115.5063211900426</v>
       </c>
       <c r="V11" t="n">
-        <v>0.313876903410737</v>
+        <v>0.3138769034107374</v>
       </c>
       <c r="W11" t="n">
-        <v>0.4750473884185649</v>
+        <v>0.4750473884185655</v>
       </c>
       <c r="X11" t="n">
         <v>0.06924046752817985</v>
@@ -2012,41 +2372,71 @@
         <v>111.6561104837078</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.03871661378398297</v>
+        <v>0.2946443271957259</v>
       </c>
       <c r="AB11" t="n">
-        <v>0.06103503510002987</v>
+        <v>0.44815339237128</v>
       </c>
       <c r="AC11" t="n">
-        <v>3.528617243442445</v>
-      </c>
-      <c r="AD11" t="inlineStr"/>
-      <c r="AE11" t="inlineStr"/>
-      <c r="AF11" t="inlineStr"/>
-      <c r="AG11" t="inlineStr"/>
-      <c r="AH11" t="inlineStr"/>
-      <c r="AI11" t="inlineStr"/>
-      <c r="AJ11" t="inlineStr"/>
-      <c r="AK11" t="inlineStr"/>
-      <c r="AL11" t="inlineStr"/>
-      <c r="AM11" t="inlineStr"/>
+        <v>0.06314752662728688</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>0.9245206853316195</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>0.9659614072042403</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>0.2927694518142698</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>0.8519985040338564</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>0.3220958597524807</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>0.05818116247847879</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>0.05884109942628889</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>0.9306787202982522</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>0.9268741259812465</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>0.6212605673260709</v>
+      </c>
       <c r="AN11" t="n">
-        <v>0.4902294708237513</v>
+        <v>0.4902294708237519</v>
       </c>
       <c r="AO11" t="n">
         <v>0.3403846153846154</v>
       </c>
-      <c r="AP11" t="inlineStr"/>
-      <c r="AQ11" t="inlineStr"/>
-      <c r="AR11" t="inlineStr"/>
-      <c r="AS11" t="inlineStr"/>
+      <c r="AP11" t="n">
+        <v>0.8391715906532821</v>
+      </c>
+      <c r="AQ11" t="n">
+        <v>0.5012244840821158</v>
+      </c>
+      <c r="AR11" t="n">
+        <v>0.3489421198295302</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>0.3507740199517405</v>
+      </c>
       <c r="AT11" t="n">
-        <v>245.3257589778895</v>
+        <v>245.3257589778892</v>
       </c>
       <c r="AU11" t="n">
         <v>113.5812158368752</v>
       </c>
-      <c r="AV11" t="inlineStr"/>
+      <c r="AV11" t="n">
+        <v>236.3814181777048</v>
+      </c>
       <c r="AW11" t="n">
         <v>0.9835802149175478</v>
       </c>
@@ -2057,16 +2447,26 @@
         <v>443.6099044591077</v>
       </c>
       <c r="AZ11" t="n">
-        <v>0.5530213742116838</v>
-      </c>
-      <c r="BA11" t="inlineStr"/>
+        <v>0.5530213742116832</v>
+      </c>
+      <c r="BA11" t="n">
+        <v>0.5131909314166924</v>
+      </c>
       <c r="BB11" t="n">
-        <v>36646.84600382369</v>
-      </c>
-      <c r="BC11" t="inlineStr"/>
-      <c r="BD11" t="inlineStr"/>
-      <c r="BE11" t="inlineStr"/>
-      <c r="BF11" t="inlineStr"/>
+        <v>632.7543909744653</v>
+      </c>
+      <c r="BC11" t="n">
+        <v>0.9561058446519446</v>
+      </c>
+      <c r="BD11" t="n">
+        <v>701.6919477402049</v>
+      </c>
+      <c r="BE11" t="n">
+        <v>485.0539249169011</v>
+      </c>
+      <c r="BF11" t="n">
+        <v>0.487330183377449</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -2088,58 +2488,58 @@
         <v>333.5379317580164</v>
       </c>
       <c r="G12" t="n">
-        <v>40560.37394973599</v>
+        <v>40560.37394973572</v>
       </c>
       <c r="H12" t="n">
-        <v>38126.75151275183</v>
+        <v>38126.75151275158</v>
       </c>
       <c r="I12" t="n">
-        <v>31308.56179011754</v>
+        <v>31308.56179011731</v>
       </c>
       <c r="J12" t="n">
-        <v>35873.16220184343</v>
+        <v>35.8731622018432</v>
       </c>
       <c r="K12" t="n">
-        <v>36504.16692319883</v>
+        <v>666.8778835572451</v>
       </c>
       <c r="L12" t="n">
-        <v>36504.16692319883</v>
+        <v>666.8778835572451</v>
       </c>
       <c r="M12" t="n">
-        <v>1.183530306631526</v>
+        <v>1.183530306631524</v>
       </c>
       <c r="N12" t="n">
-        <v>1711926.040961988</v>
+        <v>1711926.040961985</v>
       </c>
       <c r="O12" t="n">
-        <v>1711926.040961988</v>
+        <v>1711926.040961985</v>
       </c>
       <c r="P12" t="n">
         <v>459.9737851991853</v>
       </c>
       <c r="Q12" t="n">
-        <v>3498.549294971927</v>
+        <v>472.868009445283</v>
       </c>
       <c r="R12" t="n">
         <v>0.9051286626963524</v>
       </c>
       <c r="S12" t="n">
-        <v>0.2511589019127045</v>
+        <v>0.2511589019127057</v>
       </c>
       <c r="T12" t="n">
-        <v>0.9269178389038419</v>
+        <v>0.9269178389038394</v>
       </c>
       <c r="U12" t="n">
         <v>111.6069233190286</v>
       </c>
       <c r="V12" t="n">
-        <v>0.303382856793925</v>
+        <v>0.3033828567939255</v>
       </c>
       <c r="W12" t="n">
-        <v>0.4604258288065046</v>
+        <v>0.4604258288065053</v>
       </c>
       <c r="X12" t="n">
-        <v>0.06854017295532788</v>
+        <v>0.0685401729553279</v>
       </c>
       <c r="Y12" t="n">
         <v>0.323076923076923</v>
@@ -2148,61 +2548,101 @@
         <v>107.7584087218207</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.03851200714702566</v>
+        <v>0.2849339620378177</v>
       </c>
       <c r="AB12" t="n">
-        <v>0.06071288158424539</v>
+        <v>0.4344158747631086</v>
       </c>
       <c r="AC12" t="n">
-        <v>3.340408357251209</v>
-      </c>
-      <c r="AD12" t="inlineStr"/>
-      <c r="AE12" t="inlineStr"/>
-      <c r="AF12" t="inlineStr"/>
-      <c r="AG12" t="inlineStr"/>
-      <c r="AH12" t="inlineStr"/>
-      <c r="AI12" t="inlineStr"/>
-      <c r="AJ12" t="inlineStr"/>
-      <c r="AK12" t="inlineStr"/>
-      <c r="AL12" t="inlineStr"/>
-      <c r="AM12" t="inlineStr"/>
+        <v>0.06309960737010389</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>0.9245802986962449</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>0.9655684319411498</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>0.2922180220877941</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>0.8355091984621673</v>
+      </c>
+      <c r="AH12" t="n">
+        <v>0.3072692900787438</v>
+      </c>
+      <c r="AI12" t="n">
+        <v>0.05884109942628889</v>
+      </c>
+      <c r="AJ12" t="n">
+        <v>0.06007088836133104</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>0.9298627820934559</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>0.9353485473187511</v>
+      </c>
+      <c r="AM12" t="n">
+        <v>0.6328408556561717</v>
+      </c>
       <c r="AN12" t="n">
-        <v>0.4729383604313535</v>
+        <v>0.4729383604313542</v>
       </c>
       <c r="AO12" t="n">
         <v>0.3288461538461538</v>
       </c>
-      <c r="AP12" t="inlineStr"/>
-      <c r="AQ12" t="inlineStr"/>
-      <c r="AR12" t="inlineStr"/>
-      <c r="AS12" t="inlineStr"/>
+      <c r="AP12" t="n">
+        <v>0.8270914214257146</v>
+      </c>
+      <c r="AQ12" t="n">
+        <v>0.479231808360652</v>
+      </c>
+      <c r="AR12" t="n">
+        <v>0.3541530609943603</v>
+      </c>
+      <c r="AS12" t="n">
+        <v>0.3562773901015153</v>
+      </c>
       <c r="AT12" t="n">
-        <v>245.0184956066512</v>
+        <v>245.0184956066509</v>
       </c>
       <c r="AU12" t="n">
         <v>109.6826660204246</v>
       </c>
-      <c r="AV12" t="inlineStr"/>
+      <c r="AV12" t="n">
+        <v>237.8729631142037</v>
+      </c>
       <c r="AW12" t="n">
-        <v>0.9846598070339262</v>
+        <v>0.9846598070339261</v>
       </c>
       <c r="AX12" t="n">
-        <v>621.3249871673064</v>
+        <v>621.3249871673063</v>
       </c>
       <c r="AY12" t="n">
         <v>456.4321068868817</v>
       </c>
       <c r="AZ12" t="n">
-        <v>0.5368125771822062</v>
-      </c>
-      <c r="BA12" t="inlineStr"/>
+        <v>0.5368125771822055</v>
+      </c>
+      <c r="BA12" t="n">
+        <v>0.5030430444919507</v>
+      </c>
       <c r="BB12" t="n">
-        <v>36504.16692319883</v>
-      </c>
-      <c r="BC12" t="inlineStr"/>
-      <c r="BD12" t="inlineStr"/>
-      <c r="BE12" t="inlineStr"/>
-      <c r="BF12" t="inlineStr"/>
+        <v>666.8778835572451</v>
+      </c>
+      <c r="BC12" t="n">
+        <v>0.9578246158980449</v>
+      </c>
+      <c r="BD12" t="n">
+        <v>702.9533645071268</v>
+      </c>
+      <c r="BE12" t="n">
+        <v>485.4897147409403</v>
+      </c>
+      <c r="BF12" t="n">
+        <v>0.4899649897653008</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -2224,55 +2664,55 @@
         <v>333.3909356336877</v>
       </c>
       <c r="G13" t="n">
-        <v>40547.70978059008</v>
+        <v>40547.70978058977</v>
       </c>
       <c r="H13" t="n">
-        <v>38114.84719375468</v>
+        <v>38114.84719375438</v>
       </c>
       <c r="I13" t="n">
-        <v>30876.17615858889</v>
+        <v>30876.17615858862</v>
       </c>
       <c r="J13" t="n">
-        <v>35609.13417270093</v>
+        <v>35.60913417270066</v>
       </c>
       <c r="K13" t="n">
-        <v>36274.43936619188</v>
+        <v>700.9143276636428</v>
       </c>
       <c r="L13" t="n">
-        <v>36274.43936619188</v>
+        <v>700.9143276636428</v>
       </c>
       <c r="M13" t="n">
-        <v>1.170989670361084</v>
+        <v>1.170989670361082</v>
       </c>
       <c r="N13" t="n">
-        <v>1851376.294513946</v>
+        <v>1851376.294513944</v>
       </c>
       <c r="O13" t="n">
-        <v>1851376.294513946</v>
+        <v>1851376.294513944</v>
       </c>
       <c r="P13" t="n">
         <v>472.310100863313</v>
       </c>
       <c r="Q13" t="n">
-        <v>3487.523407732791</v>
+        <v>484.7850802836443</v>
       </c>
       <c r="R13" t="n">
         <v>0.9230075263024611</v>
       </c>
       <c r="S13" t="n">
-        <v>0.2638871209886917</v>
+        <v>0.2638871209886932</v>
       </c>
       <c r="T13" t="n">
-        <v>0.885899016419856</v>
+        <v>0.8858990164198532</v>
       </c>
       <c r="U13" t="n">
         <v>107.7109176662683</v>
       </c>
       <c r="V13" t="n">
-        <v>0.2944557473880431</v>
+        <v>0.2944557473880438</v>
       </c>
       <c r="W13" t="n">
-        <v>0.4478875986165669</v>
+        <v>0.4478875986165679</v>
       </c>
       <c r="X13" t="n">
         <v>0.06835157578026685</v>
@@ -2284,41 +2724,71 @@
         <v>103.8640991781873</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.03845349962267431</v>
+        <v>0.2766328533973357</v>
       </c>
       <c r="AB13" t="n">
-        <v>0.06062076021277094</v>
+        <v>0.4225907731006984</v>
       </c>
       <c r="AC13" t="n">
-        <v>3.184439660359877</v>
-      </c>
-      <c r="AD13" t="inlineStr"/>
-      <c r="AE13" t="inlineStr"/>
-      <c r="AF13" t="inlineStr"/>
-      <c r="AG13" t="inlineStr"/>
-      <c r="AH13" t="inlineStr"/>
-      <c r="AI13" t="inlineStr"/>
-      <c r="AJ13" t="inlineStr"/>
-      <c r="AK13" t="inlineStr"/>
-      <c r="AL13" t="inlineStr"/>
-      <c r="AM13" t="inlineStr"/>
+        <v>0.06349894451081993</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>0.9240833907064329</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>0.9648356976196854</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>0.29194404655797</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>0.8178556636542694</v>
+      </c>
+      <c r="AH13" t="n">
+        <v>0.2936182416907518</v>
+      </c>
+      <c r="AI13" t="n">
+        <v>0.06007088836133104</v>
+      </c>
+      <c r="AJ13" t="n">
+        <v>0.06184229672885735</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>0.9283403722786862</v>
+      </c>
+      <c r="AL13" t="n">
+        <v>0.9439216119610732</v>
+      </c>
+      <c r="AM13" t="n">
+        <v>0.6445165436780202</v>
+      </c>
       <c r="AN13" t="n">
-        <v>0.4557476825271521</v>
+        <v>0.455747682527153</v>
       </c>
       <c r="AO13" t="n">
         <v>0.3173076923076923</v>
       </c>
-      <c r="AP13" t="inlineStr"/>
-      <c r="AQ13" t="inlineStr"/>
-      <c r="AR13" t="inlineStr"/>
-      <c r="AS13" t="inlineStr"/>
+      <c r="AP13" t="n">
+        <v>0.8144191257089225</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>0.4574838896946357</v>
+      </c>
+      <c r="AR13" t="n">
+        <v>0.3586714431817695</v>
+      </c>
+      <c r="AS13" t="n">
+        <v>0.3603717739596337</v>
+      </c>
       <c r="AT13" t="n">
-        <v>244.723119303435</v>
+        <v>244.7231193034345</v>
       </c>
       <c r="AU13" t="n">
         <v>105.7875084222278</v>
       </c>
-      <c r="AV13" t="inlineStr"/>
+      <c r="AV13" t="n">
+        <v>239.5050749731142</v>
+      </c>
       <c r="AW13" t="n">
         <v>0.9855493021383581</v>
       </c>
@@ -2329,16 +2799,26 @@
         <v>468.8850770576346</v>
       </c>
       <c r="AZ13" t="n">
-        <v>0.5219255874789847</v>
-      </c>
-      <c r="BA13" t="inlineStr"/>
+        <v>0.5219255874789838</v>
+      </c>
+      <c r="BA13" t="n">
+        <v>0.4940438241890232</v>
+      </c>
       <c r="BB13" t="n">
-        <v>36274.43936619188</v>
-      </c>
-      <c r="BC13" t="inlineStr"/>
-      <c r="BD13" t="inlineStr"/>
-      <c r="BE13" t="inlineStr"/>
-      <c r="BF13" t="inlineStr"/>
+        <v>700.9143276636428</v>
+      </c>
+      <c r="BC13" t="n">
+        <v>0.9593201166301143</v>
+      </c>
+      <c r="BD13" t="n">
+        <v>704.0509216734201</v>
+      </c>
+      <c r="BE13" t="n">
+        <v>485.8685769187978</v>
+      </c>
+      <c r="BF13" t="n">
+        <v>0.4929420965890993</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -2360,58 +2840,58 @@
         <v>333.2439395093589</v>
       </c>
       <c r="G14" t="n">
-        <v>40427.22983054083</v>
+        <v>40427.22983054043</v>
       </c>
       <c r="H14" t="n">
-        <v>38001.59604070838</v>
+        <v>38001.596040708</v>
       </c>
       <c r="I14" t="n">
-        <v>30328.77244090705</v>
+        <v>30328.77244090673</v>
       </c>
       <c r="J14" t="n">
-        <v>35254.78155713555</v>
+        <v>35.25478155713519</v>
       </c>
       <c r="K14" t="n">
-        <v>35954.38722276203</v>
+        <v>734.8604471836175</v>
       </c>
       <c r="L14" t="n">
-        <v>35954.38722276203</v>
+        <v>734.8604471836175</v>
       </c>
       <c r="M14" t="n">
-        <v>1.159124662321262</v>
+        <v>1.159124662321261</v>
       </c>
       <c r="N14" t="n">
-        <v>1988610.271253235</v>
+        <v>1988610.271253233</v>
       </c>
       <c r="O14" t="n">
-        <v>1988610.271253235</v>
+        <v>1988610.271253233</v>
       </c>
       <c r="P14" t="n">
         <v>484.332302953829</v>
       </c>
       <c r="Q14" t="n">
-        <v>3472.103978251819</v>
+        <v>496.3856443740763</v>
       </c>
       <c r="R14" t="n">
         <v>0.9413928374782321</v>
       </c>
       <c r="S14" t="n">
-        <v>0.277344459001038</v>
+        <v>0.2773444590010399</v>
       </c>
       <c r="T14" t="n">
-        <v>0.8433989117289364</v>
+        <v>0.843398911728933</v>
       </c>
       <c r="U14" t="n">
         <v>103.8183042317618</v>
       </c>
       <c r="V14" t="n">
-        <v>0.2869879732052458</v>
+        <v>0.2869879732052466</v>
       </c>
       <c r="W14" t="n">
-        <v>0.4373303874026709</v>
+        <v>0.437330387402672</v>
       </c>
       <c r="X14" t="n">
-        <v>0.0685949079348202</v>
+        <v>0.06859490793482022</v>
       </c>
       <c r="Y14" t="n">
         <v>0.3</v>
@@ -2420,61 +2900,101 @@
         <v>99.97318185280768</v>
       </c>
       <c r="AA14" t="n">
-        <v>0.03854996554317704</v>
+        <v>0.2696481863264099</v>
       </c>
       <c r="AB14" t="n">
-        <v>0.06077264762793715</v>
+        <v>0.4125844983772042</v>
       </c>
       <c r="AC14" t="n">
-        <v>3.052899555073981</v>
-      </c>
-      <c r="AD14" t="inlineStr"/>
-      <c r="AE14" t="inlineStr"/>
-      <c r="AF14" t="inlineStr"/>
-      <c r="AG14" t="inlineStr"/>
-      <c r="AH14" t="inlineStr"/>
-      <c r="AI14" t="inlineStr"/>
-      <c r="AJ14" t="inlineStr"/>
-      <c r="AK14" t="inlineStr"/>
-      <c r="AL14" t="inlineStr"/>
-      <c r="AM14" t="inlineStr"/>
+        <v>0.06428864272086865</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>0.9230999564416354</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>0.9637792758337282</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>0.2920116907329444</v>
+      </c>
+      <c r="AG14" t="n">
+        <v>0.7988908437321858</v>
+      </c>
+      <c r="AH14" t="n">
+        <v>0.2810592386107025</v>
+      </c>
+      <c r="AI14" t="n">
+        <v>0.06184229672885735</v>
+      </c>
+      <c r="AJ14" t="n">
+        <v>0.06287462290091529</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>0.9261430694299728</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>0.9525860566559802</v>
+      </c>
+      <c r="AM14" t="n">
+        <v>0.6562455778871688</v>
+      </c>
       <c r="AN14" t="n">
-        <v>0.4386646551706975</v>
+        <v>0.4386646551706986</v>
       </c>
       <c r="AO14" t="n">
         <v>0.3057692307692308</v>
       </c>
-      <c r="AP14" t="inlineStr"/>
-      <c r="AQ14" t="inlineStr"/>
-      <c r="AR14" t="inlineStr"/>
-      <c r="AS14" t="inlineStr"/>
+      <c r="AP14" t="n">
+        <v>0.8010564084913128</v>
+      </c>
+      <c r="AQ14" t="n">
+        <v>0.4360279824188179</v>
+      </c>
+      <c r="AR14" t="n">
+        <v>0.3623917533206142</v>
+      </c>
+      <c r="AS14" t="n">
+        <v>0.3628628613133679</v>
+      </c>
       <c r="AT14" t="n">
-        <v>244.4331148181676</v>
+        <v>244.433114818167</v>
       </c>
       <c r="AU14" t="n">
         <v>101.8957430422848</v>
       </c>
-      <c r="AV14" t="inlineStr"/>
+      <c r="AV14" t="n">
+        <v>241.2633375449374</v>
+      </c>
       <c r="AW14" t="n">
-        <v>0.9862729838725909</v>
+        <v>0.9862729838725908</v>
       </c>
       <c r="AX14" t="n">
-        <v>690.0021673716008</v>
+        <v>690.0021673716006</v>
       </c>
       <c r="AY14" t="n">
         <v>480.9965974096883</v>
       </c>
       <c r="AZ14" t="n">
-        <v>0.5081805487492295</v>
-      </c>
-      <c r="BA14" t="inlineStr"/>
+        <v>0.5081805487492282</v>
+      </c>
+      <c r="BA14" t="n">
+        <v>0.4860401187652424</v>
+      </c>
       <c r="BB14" t="n">
-        <v>35954.38722276203</v>
-      </c>
-      <c r="BC14" t="inlineStr"/>
-      <c r="BD14" t="inlineStr"/>
-      <c r="BE14" t="inlineStr"/>
-      <c r="BF14" t="inlineStr"/>
+        <v>734.8604471836175</v>
+      </c>
+      <c r="BC14" t="n">
+        <v>0.9606275004917781</v>
+      </c>
+      <c r="BD14" t="n">
+        <v>705.0104187139062</v>
+      </c>
+      <c r="BE14" t="n">
+        <v>486.1995407183894</v>
+      </c>
+      <c r="BF14" t="n">
+        <v>0.4962228824577995</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -2496,103 +3016,133 @@
         <v>333.0969433850302</v>
       </c>
       <c r="G15" t="n">
-        <v>40189.87084991457</v>
+        <v>40189.87084991405</v>
       </c>
       <c r="H15" t="n">
-        <v>37778.47859891969</v>
+        <v>37778.4785989192</v>
       </c>
       <c r="I15" t="n">
-        <v>29662.44420332219</v>
+        <v>29662.4442033218</v>
       </c>
       <c r="J15" t="n">
-        <v>34750.41522806049</v>
+        <v>34.75041522806004</v>
       </c>
       <c r="K15" t="n">
-        <v>35484.32136582251</v>
+        <v>768.6565529900824</v>
       </c>
       <c r="L15" t="n">
-        <v>35484.32136582251</v>
+        <v>768.6565529900824</v>
       </c>
       <c r="M15" t="n">
-        <v>1.147820922348967</v>
+        <v>1.147820922348964</v>
       </c>
       <c r="N15" t="n">
-        <v>2123689.157522178</v>
+        <v>2123689.157522174</v>
       </c>
       <c r="O15" t="n">
-        <v>2123689.157522178</v>
+        <v>2123689.157522174</v>
       </c>
       <c r="P15" t="n">
         <v>496.0632298322525</v>
       </c>
       <c r="Q15" t="n">
-        <v>3449.332247545935</v>
+        <v>507.6716874295578</v>
       </c>
       <c r="R15" t="n">
         <v>0.9602555069185875</v>
       </c>
       <c r="S15" t="n">
-        <v>0.291520446711053</v>
+        <v>0.2915204467110554</v>
       </c>
       <c r="T15" t="n">
-        <v>0.799732363619133</v>
+        <v>0.799732363619129</v>
       </c>
       <c r="U15" t="n">
-        <v>99.92908301550906</v>
+        <v>99.92908301550905</v>
       </c>
       <c r="V15" t="n">
-        <v>0.280887875197627</v>
+        <v>0.280887875197628</v>
       </c>
       <c r="W15" t="n">
-        <v>0.4286613611154589</v>
+        <v>0.4286613611154603</v>
       </c>
       <c r="X15" t="n">
-        <v>0.06921949698481909</v>
+        <v>0.06921949698481912</v>
       </c>
       <c r="Y15" t="n">
         <v>0.3</v>
       </c>
       <c r="Z15" t="n">
-        <v>99.92908301550906</v>
+        <v>99.92908301550905</v>
       </c>
       <c r="AA15" t="n">
-        <v>0.04039568722044307</v>
+        <v>0.2744650726865439</v>
       </c>
       <c r="AB15" t="n">
-        <v>0.06367849486427389</v>
+        <v>0.4194906558197299</v>
       </c>
       <c r="AC15" t="n">
-        <v>2.822759275792766</v>
-      </c>
-      <c r="AD15" t="inlineStr"/>
-      <c r="AE15" t="inlineStr"/>
-      <c r="AF15" t="inlineStr"/>
-      <c r="AG15" t="inlineStr"/>
-      <c r="AH15" t="inlineStr"/>
-      <c r="AI15" t="inlineStr"/>
-      <c r="AJ15" t="inlineStr"/>
-      <c r="AK15" t="inlineStr"/>
-      <c r="AL15" t="inlineStr"/>
-      <c r="AM15" t="inlineStr"/>
+        <v>0.06306556002225917</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>0.9246226525464954</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>0.9631630890144903</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>0.2934643355010041</v>
+      </c>
+      <c r="AG15" t="n">
+        <v>0.7964104516033221</v>
+      </c>
+      <c r="AH15" t="n">
+        <v>0.275355442547742</v>
+      </c>
+      <c r="AI15" t="n">
+        <v>0.06287462290091529</v>
+      </c>
+      <c r="AJ15" t="n">
+        <v>0.06287462290091529</v>
+      </c>
+      <c r="AK15" t="n">
+        <v>0.9248601364962541</v>
+      </c>
+      <c r="AL15" t="n">
+        <v>0.9617092979665389</v>
+      </c>
+      <c r="AM15" t="n">
+        <v>0.6677241507299628</v>
+      </c>
       <c r="AN15" t="n">
-        <v>0.4216958620849969</v>
+        <v>0.4216958620849983</v>
       </c>
       <c r="AO15" t="n">
         <v>0.3</v>
       </c>
-      <c r="AP15" t="inlineStr"/>
-      <c r="AQ15" t="inlineStr"/>
-      <c r="AR15" t="inlineStr"/>
-      <c r="AS15" t="inlineStr"/>
+      <c r="AP15" t="n">
+        <v>0.7955240852555532</v>
+      </c>
+      <c r="AQ15" t="n">
+        <v>0.4222611100674148</v>
+      </c>
+      <c r="AR15" t="n">
+        <v>0.3738282231705549</v>
+      </c>
+      <c r="AS15" t="n">
+        <v>0.3741493415359073</v>
+      </c>
       <c r="AT15" t="n">
-        <v>244.1413319071562</v>
+        <v>244.1413319071554</v>
       </c>
       <c r="AU15" t="n">
-        <v>99.92908301550906</v>
-      </c>
-      <c r="AV15" t="inlineStr"/>
+        <v>99.92908301550905</v>
+      </c>
+      <c r="AV15" t="n">
+        <v>243.8341389321499</v>
+      </c>
       <c r="AW15" t="n">
-        <v>0.9868503335944937</v>
+        <v>0.9868503335944936</v>
       </c>
       <c r="AX15" t="n">
         <v>724.2555168774983</v>
@@ -2601,16 +3151,26 @@
         <v>492.7909037401413</v>
       </c>
       <c r="AZ15" t="n">
-        <v>0.4954258085005093</v>
-      </c>
-      <c r="BA15" t="inlineStr"/>
+        <v>0.4954258085005078</v>
+      </c>
+      <c r="BA15" t="n">
+        <v>0.4802988722233663</v>
+      </c>
       <c r="BB15" t="n">
-        <v>35484.32136582251</v>
-      </c>
-      <c r="BC15" t="inlineStr"/>
-      <c r="BD15" t="inlineStr"/>
-      <c r="BE15" t="inlineStr"/>
-      <c r="BF15" t="inlineStr"/>
+        <v>768.6565529900824</v>
+      </c>
+      <c r="BC15" t="n">
+        <v>0.9615521655568271</v>
+      </c>
+      <c r="BD15" t="n">
+        <v>705.6890360805198</v>
+      </c>
+      <c r="BE15" t="n">
+        <v>486.4334834258414</v>
+      </c>
+      <c r="BF15" t="n">
+        <v>0.5012692325677933</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
added calculation with loss function
</commit_message>
<xml_diff>
--- a/расчет_ступеней.xlsx
+++ b/расчет_ступеней.xlsx
@@ -728,25 +728,25 @@
         <v>335.007893001304</v>
       </c>
       <c r="G2" t="n">
-        <v>36411.99532705869</v>
+        <v>36411.99532705859</v>
       </c>
       <c r="H2" t="n">
-        <v>36047.87537378811</v>
+        <v>36047.875373788</v>
       </c>
       <c r="I2" t="n">
-        <v>31873.6502893009</v>
+        <v>31873.65028930084</v>
       </c>
       <c r="J2" t="n">
-        <v>35.83287810515716</v>
+        <v>35.83287810515706</v>
       </c>
       <c r="K2" t="n">
-        <v>323.8328781051572</v>
+        <v>323.8328781051571</v>
       </c>
       <c r="L2" t="n">
-        <v>323.8328781051572</v>
+        <v>323.8328781051571</v>
       </c>
       <c r="M2" t="n">
-        <v>1.440944655702848</v>
+        <v>1.440944655702847</v>
       </c>
       <c r="N2" t="n">
         <v>145066.7069330656</v>
@@ -764,22 +764,22 @@
         <v>0.7615773105863909</v>
       </c>
       <c r="S2" t="n">
-        <v>0.167783356589721</v>
+        <v>0.1677833565897216</v>
       </c>
       <c r="T2" t="n">
-        <v>1.213910247893696</v>
+        <v>1.213910247893695</v>
       </c>
       <c r="U2" t="n">
         <v>150.7535518505868</v>
       </c>
       <c r="V2" t="n">
-        <v>0.5177497878149004</v>
+        <v>0.5177497878149007</v>
       </c>
       <c r="W2" t="n">
-        <v>0.7285310911802059</v>
+        <v>0.7285310911802062</v>
       </c>
       <c r="X2" t="n">
-        <v>0.3588841693639396</v>
+        <v>0.3588841693639397</v>
       </c>
       <c r="Y2" t="n">
         <v>0.4384615384615385</v>
@@ -788,70 +788,70 @@
         <v>146.8880761621102</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.4757455045369876</v>
+        <v>0.475745504536988</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.6816773513404401</v>
+        <v>0.6816773513404407</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.2822542259235776</v>
+        <v>0.2822542259235777</v>
       </c>
       <c r="AD2" t="n">
         <v>0.5922128766565673</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.8281605716505803</v>
+        <v>0.8281605716505802</v>
       </c>
       <c r="AF2" t="n">
-        <v>0.2135053003617265</v>
+        <v>0.2135053003617271</v>
       </c>
       <c r="AG2" t="n">
-        <v>1.117649652176082</v>
+        <v>1.117649652176081</v>
       </c>
       <c r="AH2" t="n">
-        <v>0.4958084006661691</v>
+        <v>0.4958084006661695</v>
       </c>
       <c r="AI2" t="n">
-        <v>0.2731322398500622</v>
+        <v>0.2731322398500624</v>
       </c>
       <c r="AJ2" t="n">
-        <v>0.1290558392935941</v>
+        <v>0.1290558392935942</v>
       </c>
       <c r="AK2" t="n">
-        <v>0.609671932167811</v>
+        <v>0.6096719321678109</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.7948689411184856</v>
+        <v>0.7948689411184855</v>
       </c>
       <c r="AM2" t="n">
-        <v>0.5689239812174692</v>
+        <v>0.5689239812174688</v>
       </c>
       <c r="AN2" t="n">
-        <v>0.6484989891376702</v>
+        <v>0.6484989891376707</v>
       </c>
       <c r="AO2" t="n">
         <v>0.4442307692307692</v>
       </c>
       <c r="AP2" t="n">
-        <v>1.100275974329452</v>
+        <v>1.100275974329451</v>
       </c>
       <c r="AQ2" t="n">
-        <v>0.662939786869682</v>
+        <v>0.6629397868696824</v>
       </c>
       <c r="AR2" t="n">
-        <v>0.4517769851917814</v>
+        <v>0.4517769851917803</v>
       </c>
       <c r="AS2" t="n">
-        <v>0.4547098653064001</v>
+        <v>0.4547098653063985</v>
       </c>
       <c r="AT2" t="n">
-        <v>249.5957775306276</v>
+        <v>249.5957775306275</v>
       </c>
       <c r="AU2" t="n">
         <v>148.8208140063485</v>
       </c>
       <c r="AV2" t="n">
-        <v>241.8133924165746</v>
+        <v>241.8133924165745</v>
       </c>
       <c r="AW2" t="n">
         <v>0.9553225262029376</v>
@@ -863,13 +863,13 @@
         <v>303.7302375370674</v>
       </c>
       <c r="AZ2" t="n">
-        <v>0.8217679594714927</v>
+        <v>0.8217679594714923</v>
       </c>
       <c r="BA2" t="n">
-        <v>0.7338429110241117</v>
+        <v>0.7338429110241115</v>
       </c>
       <c r="BB2" t="n">
-        <v>323.8328781051572</v>
+        <v>323.8328781051571</v>
       </c>
       <c r="BC2" t="n">
         <v>0.9102457636566097</v>
@@ -881,7 +881,7 @@
         <v>473.2780574676653</v>
       </c>
       <c r="BF2" t="n">
-        <v>0.5109330310186534</v>
+        <v>0.5109330310186531</v>
       </c>
     </row>
     <row r="3">
@@ -904,22 +904,22 @@
         <v>334.8608968769752</v>
       </c>
       <c r="G3" t="n">
-        <v>37081.05894345287</v>
+        <v>37081.05894345281</v>
       </c>
       <c r="H3" t="n">
-        <v>36339.43776458382</v>
+        <v>36339.43776458375</v>
       </c>
       <c r="I3" t="n">
-        <v>32038.30662392292</v>
+        <v>32038.30662392289</v>
       </c>
       <c r="J3" t="n">
-        <v>35.97964135107308</v>
+        <v>35.97964135107302</v>
       </c>
       <c r="K3" t="n">
-        <v>358.2801134866133</v>
+        <v>358.2801134866132</v>
       </c>
       <c r="L3" t="n">
-        <v>358.2801134866133</v>
+        <v>358.2801134866132</v>
       </c>
       <c r="M3" t="n">
         <v>1.390695899350074</v>
@@ -940,19 +940,19 @@
         <v>0.7725018866632134</v>
       </c>
       <c r="S3" t="n">
-        <v>0.172211549973675</v>
+        <v>0.1722115499736755</v>
       </c>
       <c r="T3" t="n">
-        <v>1.196544109661877</v>
+        <v>1.196544109661876</v>
       </c>
       <c r="U3" t="n">
         <v>146.8236240152891</v>
       </c>
       <c r="V3" t="n">
-        <v>0.479845099538809</v>
+        <v>0.4798450995388093</v>
       </c>
       <c r="W3" t="n">
-        <v>0.6863858064760082</v>
+        <v>0.6863858064760087</v>
       </c>
       <c r="X3" t="n">
         <v>0.1735963604307613</v>
@@ -964,10 +964,10 @@
         <v>142.9598444359394</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.4431373034630462</v>
+        <v>0.4431373034630464</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.6432243354866706</v>
+        <v>0.6432243354866709</v>
       </c>
       <c r="AC3" t="n">
         <v>0.1404413998385572</v>
@@ -979,16 +979,16 @@
         <v>0.9228017710032826</v>
       </c>
       <c r="AF3" t="n">
-        <v>0.2772675463787479</v>
+        <v>0.2772675463787483</v>
       </c>
       <c r="AG3" t="n">
-        <v>0.9948039683717862</v>
+        <v>0.9948039683717855</v>
       </c>
       <c r="AH3" t="n">
-        <v>0.4918175734636512</v>
+        <v>0.4918175734636515</v>
       </c>
       <c r="AI3" t="n">
-        <v>0.1290558392935941</v>
+        <v>0.1290558392935942</v>
       </c>
       <c r="AJ3" t="n">
         <v>0.09293479859248309</v>
@@ -1000,28 +1000,28 @@
         <v>0.847651828833248</v>
       </c>
       <c r="AM3" t="n">
-        <v>0.5470706271897741</v>
+        <v>0.5470706271897736</v>
       </c>
       <c r="AN3" t="n">
-        <v>0.6308489453405535</v>
+        <v>0.6308489453405539</v>
       </c>
       <c r="AO3" t="n">
         <v>0.4326923076923077</v>
       </c>
       <c r="AP3" t="n">
-        <v>0.9636520867716827</v>
+        <v>0.963652086771682</v>
       </c>
       <c r="AQ3" t="n">
-        <v>0.6691833885527213</v>
+        <v>0.6691833885527217</v>
       </c>
       <c r="AR3" t="n">
-        <v>0.3328031414311292</v>
+        <v>0.3328031414311281</v>
       </c>
       <c r="AS3" t="n">
-        <v>0.3256205798190649</v>
+        <v>0.3256205798190638</v>
       </c>
       <c r="AT3" t="n">
-        <v>248.9251061897376</v>
+        <v>248.9251061897375</v>
       </c>
       <c r="AU3" t="n">
         <v>144.8917342256143</v>
@@ -1039,13 +1039,13 @@
         <v>322.366623658571</v>
       </c>
       <c r="AZ3" t="n">
-        <v>0.7721801449686749</v>
+        <v>0.7721801449686746</v>
       </c>
       <c r="BA3" t="n">
-        <v>0.6738786613597089</v>
+        <v>0.6738786613597086</v>
       </c>
       <c r="BB3" t="n">
-        <v>358.2801134866133</v>
+        <v>358.2801134866132</v>
       </c>
       <c r="BC3" t="n">
         <v>0.9243145916273412</v>
@@ -1057,7 +1057,7 @@
         <v>476.9215438326696</v>
       </c>
       <c r="BF3" t="n">
-        <v>0.4897369719020609</v>
+        <v>0.4897369719020607</v>
       </c>
     </row>
     <row r="4">
@@ -1080,16 +1080,16 @@
         <v>334.7139007526465</v>
       </c>
       <c r="G4" t="n">
-        <v>37708.04437880874</v>
+        <v>37708.0443788087</v>
       </c>
       <c r="H4" t="n">
-        <v>36576.80304744447</v>
+        <v>36576.80304744444</v>
       </c>
       <c r="I4" t="n">
-        <v>32124.59638269978</v>
+        <v>32124.59638269979</v>
       </c>
       <c r="J4" t="n">
-        <v>36.04364141937292</v>
+        <v>36.04364141937288</v>
       </c>
       <c r="K4" t="n">
         <v>392.6445856904533</v>
@@ -1116,16 +1116,16 @@
         <v>0.7842900694668242</v>
       </c>
       <c r="S4" t="n">
-        <v>0.1775696995515668</v>
+        <v>0.177569699551567</v>
       </c>
       <c r="T4" t="n">
-        <v>1.176633893900266</v>
+        <v>1.176633893900265</v>
       </c>
       <c r="U4" t="n">
         <v>142.8970883982452</v>
       </c>
       <c r="V4" t="n">
-        <v>0.4475729189884193</v>
+        <v>0.4475729189884194</v>
       </c>
       <c r="W4" t="n">
         <v>0.6485576489170397</v>
@@ -1140,10 +1140,10 @@
         <v>139.0350049280224</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.415007567136801</v>
+        <v>0.4150075671368011</v>
       </c>
       <c r="AB4" t="n">
-        <v>0.6086768365849144</v>
+        <v>0.6086768365849147</v>
       </c>
       <c r="AC4" t="n">
         <v>0.1026257677193531</v>
@@ -1155,10 +1155,10 @@
         <v>0.9450442593643356</v>
       </c>
       <c r="AF4" t="n">
-        <v>0.2903669344696717</v>
+        <v>0.2903669344696718</v>
       </c>
       <c r="AG4" t="n">
-        <v>0.9607206522143688</v>
+        <v>0.9607206522143685</v>
       </c>
       <c r="AH4" t="n">
         <v>0.4675231842410476</v>
@@ -1176,25 +1176,25 @@
         <v>0.8646671644155799</v>
       </c>
       <c r="AM4" t="n">
-        <v>0.5503213035612302</v>
+        <v>0.55032130356123</v>
       </c>
       <c r="AN4" t="n">
-        <v>0.6131761582556859</v>
+        <v>0.6131761582556861</v>
       </c>
       <c r="AO4" t="n">
         <v>0.4211538461538462</v>
       </c>
       <c r="AP4" t="n">
-        <v>0.9296083408833998</v>
+        <v>0.9296083408833995</v>
       </c>
       <c r="AQ4" t="n">
-        <v>0.653213338356202</v>
+        <v>0.6532133383562021</v>
       </c>
       <c r="AR4" t="n">
-        <v>0.3164321826277139</v>
+        <v>0.3164321826277134</v>
       </c>
       <c r="AS4" t="n">
-        <v>0.3075073138581668</v>
+        <v>0.3075073138581664</v>
       </c>
       <c r="AT4" t="n">
         <v>248.3146130188819</v>
@@ -1218,7 +1218,7 @@
         <v>0.7304120392625181</v>
       </c>
       <c r="BA4" t="n">
-        <v>0.639262370793689</v>
+        <v>0.6392623707936889</v>
       </c>
       <c r="BB4" t="n">
         <v>392.6445856904533</v>
@@ -1233,7 +1233,7 @@
         <v>478.8720646982767</v>
       </c>
       <c r="BF4" t="n">
-        <v>0.4843688676188677</v>
+        <v>0.4843688676188676</v>
       </c>
     </row>
     <row r="5">
@@ -1256,16 +1256,16 @@
         <v>334.5669046283177</v>
       </c>
       <c r="G5" t="n">
-        <v>38288.30593027178</v>
+        <v>38288.30593027177</v>
       </c>
       <c r="H5" t="n">
-        <v>36756.77369306091</v>
+        <v>36756.7736930609</v>
       </c>
       <c r="I5" t="n">
-        <v>32129.24271355215</v>
+        <v>32129.24271355218</v>
       </c>
       <c r="J5" t="n">
-        <v>36.16823999357076</v>
+        <v>36.16823999357074</v>
       </c>
       <c r="K5" t="n">
         <v>427.0696564001913</v>
@@ -1292,19 +1292,19 @@
         <v>0.7969035352526399</v>
       </c>
       <c r="S5" t="n">
-        <v>0.1838346066436044</v>
+        <v>0.1838346066436046</v>
       </c>
       <c r="T5" t="n">
         <v>1.154142696849574</v>
       </c>
       <c r="U5" t="n">
-        <v>138.973944999455</v>
+        <v>138.9739449994551</v>
       </c>
       <c r="V5" t="n">
-        <v>0.4197819976689973</v>
+        <v>0.4197819976689975</v>
       </c>
       <c r="W5" t="n">
-        <v>0.6146271972579196</v>
+        <v>0.6146271972579198</v>
       </c>
       <c r="X5" t="n">
         <v>0.1013539366335962</v>
@@ -1319,7 +1319,7 @@
         <v>0.3904573637869123</v>
       </c>
       <c r="AB5" t="n">
-        <v>0.5775401427632009</v>
+        <v>0.577540142763201</v>
       </c>
       <c r="AC5" t="n">
         <v>0.08564629091578738</v>
@@ -1331,19 +1331,19 @@
         <v>0.954649477405116</v>
       </c>
       <c r="AF5" t="n">
-        <v>0.294603227788098</v>
+        <v>0.2946032277880982</v>
       </c>
       <c r="AG5" t="n">
-        <v>0.9405489337121995</v>
+        <v>0.9405489337121993</v>
       </c>
       <c r="AH5" t="n">
-        <v>0.4419620774952459</v>
+        <v>0.4419620774952461</v>
       </c>
       <c r="AI5" t="n">
         <v>0.07707028988055241</v>
       </c>
       <c r="AJ5" t="n">
-        <v>0.06855040237940825</v>
+        <v>0.06855040237940827</v>
       </c>
       <c r="AK5" t="n">
         <v>0.9070343154587495</v>
@@ -1352,25 +1352,25 @@
         <v>0.8757765063288779</v>
       </c>
       <c r="AM5" t="n">
-        <v>0.5578555636415101</v>
+        <v>0.5578555636415099</v>
       </c>
       <c r="AN5" t="n">
-        <v>0.5954991555222525</v>
+        <v>0.5954991555222526</v>
       </c>
       <c r="AO5" t="n">
         <v>0.4096153846153846</v>
       </c>
       <c r="AP5" t="n">
-        <v>0.9107712941505934</v>
+        <v>0.9107712941505931</v>
       </c>
       <c r="AQ5" t="n">
-        <v>0.6333562460279528</v>
+        <v>0.633356246027953</v>
       </c>
       <c r="AR5" t="n">
-        <v>0.3152721386283409</v>
+        <v>0.3152721386283405</v>
       </c>
       <c r="AS5" t="n">
-        <v>0.3071926876842467</v>
+        <v>0.3071926876842462</v>
       </c>
       <c r="AT5" t="n">
         <v>247.7598137444</v>
@@ -1394,13 +1394,13 @@
         <v>0.6946299383584459</v>
       </c>
       <c r="BA5" t="n">
-        <v>0.6118979187260279</v>
+        <v>0.6118979187260278</v>
       </c>
       <c r="BB5" t="n">
         <v>427.0696564001913</v>
       </c>
       <c r="BC5" t="n">
-        <v>0.9375968228431258</v>
+        <v>0.937596822843126</v>
       </c>
       <c r="BD5" t="n">
         <v>688.1080630307417</v>
@@ -1409,7 +1409,7 @@
         <v>480.3359590268125</v>
       </c>
       <c r="BF5" t="n">
-        <v>0.4820587945409821</v>
+        <v>0.482058794540982</v>
       </c>
     </row>
     <row r="6">
@@ -1438,10 +1438,10 @@
         <v>36875.92322328367</v>
       </c>
       <c r="I6" t="n">
-        <v>32049.09574441154</v>
+        <v>32049.09574441157</v>
       </c>
       <c r="J6" t="n">
-        <v>36.11659964737082</v>
+        <v>36.11659964737081</v>
       </c>
       <c r="K6" t="n">
         <v>461.3184881895316</v>
@@ -1468,7 +1468,7 @@
         <v>0.8103037450239648</v>
       </c>
       <c r="S6" t="n">
-        <v>0.1909825772598289</v>
+        <v>0.190982577259829</v>
       </c>
       <c r="T6" t="n">
         <v>1.129055245477055</v>
@@ -1483,7 +1483,7 @@
         <v>0.584211559070294</v>
       </c>
       <c r="X6" t="n">
-        <v>0.08880215565753603</v>
+        <v>0.08880215565753605</v>
       </c>
       <c r="Y6" t="n">
         <v>0.3923076923076923</v>
@@ -1492,13 +1492,13 @@
         <v>131.1955025669495</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.3690023501058217</v>
+        <v>0.3690023501058218</v>
       </c>
       <c r="AB6" t="n">
         <v>0.5496154015473974</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.07635105351990513</v>
+        <v>0.07635105351990515</v>
       </c>
       <c r="AD6" t="n">
         <v>0.9079458936530936</v>
@@ -1516,13 +1516,13 @@
         <v>0.4177978186232196</v>
       </c>
       <c r="AI6" t="n">
-        <v>0.06855040237940825</v>
+        <v>0.06855040237940827</v>
       </c>
       <c r="AJ6" t="n">
         <v>0.06358754747461096</v>
       </c>
       <c r="AK6" t="n">
-        <v>0.9177744737737201</v>
+        <v>0.91777447377372</v>
       </c>
       <c r="AL6" t="n">
         <v>0.8850359711116637</v>
@@ -1608,16 +1608,16 @@
         <v>334.2729123796602</v>
       </c>
       <c r="G7" t="n">
-        <v>39287.89350685768</v>
+        <v>39287.89350685771</v>
       </c>
       <c r="H7" t="n">
-        <v>36930.61989644622</v>
+        <v>36930.61989644625</v>
       </c>
       <c r="I7" t="n">
-        <v>31881.19329867551</v>
+        <v>31881.19329867558</v>
       </c>
       <c r="J7" t="n">
-        <v>35.97650928166554</v>
+        <v>35.97650928166557</v>
       </c>
       <c r="K7" t="n">
         <v>495.4788699593665</v>
@@ -1644,19 +1644,19 @@
         <v>0.8244523377184381</v>
       </c>
       <c r="S7" t="n">
-        <v>0.1989900230881154</v>
+        <v>0.1989900230881153</v>
       </c>
       <c r="T7" t="n">
-        <v>1.101381881882767</v>
+        <v>1.101381881882768</v>
       </c>
       <c r="U7" t="n">
         <v>131.1378348566359</v>
       </c>
       <c r="V7" t="n">
-        <v>0.3746137054218505</v>
+        <v>0.3746137054218504</v>
       </c>
       <c r="W7" t="n">
-        <v>0.5569812067003774</v>
+        <v>0.5569812067003773</v>
       </c>
       <c r="X7" t="n">
         <v>0.08107434726661611</v>
@@ -1671,10 +1671,10 @@
         <v>0.3501466610037778</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.5245508609268315</v>
+        <v>0.5245508609268316</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.07078290052051256</v>
+        <v>0.07078290052051253</v>
       </c>
       <c r="AD7" t="n">
         <v>0.9149723790623341</v>
@@ -1683,19 +1683,19 @@
         <v>0.9627373200998649</v>
       </c>
       <c r="AF7" t="n">
-        <v>0.2957865509268111</v>
+        <v>0.2957865509268109</v>
       </c>
       <c r="AG7" t="n">
-        <v>0.9103544675172746</v>
+        <v>0.9103544675172747</v>
       </c>
       <c r="AH7" t="n">
-        <v>0.3954211232783114</v>
+        <v>0.3954211232783115</v>
       </c>
       <c r="AI7" t="n">
         <v>0.06358754747461096</v>
       </c>
       <c r="AJ7" t="n">
-        <v>0.06056357647098572</v>
+        <v>0.0605635764709857</v>
       </c>
       <c r="AK7" t="n">
         <v>0.9239731029776458</v>
@@ -1704,25 +1704,25 @@
         <v>0.8935948289091515</v>
       </c>
       <c r="AM7" t="n">
-        <v>0.5770667541588699</v>
+        <v>0.57706675415887</v>
       </c>
       <c r="AN7" t="n">
-        <v>0.5602001159796427</v>
+        <v>0.5602001159796426</v>
       </c>
       <c r="AO7" t="n">
         <v>0.3865384615384615</v>
       </c>
       <c r="AP7" t="n">
-        <v>0.8846495783834111</v>
+        <v>0.8846495783834112</v>
       </c>
       <c r="AQ7" t="n">
-        <v>0.5901916054573306</v>
+        <v>0.5901916054573305</v>
       </c>
       <c r="AR7" t="n">
-        <v>0.3244494624037684</v>
+        <v>0.3244494624037686</v>
       </c>
       <c r="AS7" t="n">
-        <v>0.3201628620599439</v>
+        <v>0.3201628620599442</v>
       </c>
       <c r="AT7" t="n">
         <v>246.7985679482697</v>
@@ -1731,7 +1731,7 @@
         <v>129.2093372852148</v>
       </c>
       <c r="AV7" t="n">
-        <v>232.1736594147696</v>
+        <v>232.1736594147697</v>
       </c>
       <c r="AW7" t="n">
         <v>0.9766107619516852</v>
@@ -1746,22 +1746,22 @@
         <v>0.636240385113307</v>
       </c>
       <c r="BA7" t="n">
-        <v>0.5696178636607405</v>
+        <v>0.5696178636607407</v>
       </c>
       <c r="BB7" t="n">
         <v>495.4788699593665</v>
       </c>
       <c r="BC7" t="n">
-        <v>0.9459225815664291</v>
+        <v>0.9459225815664289</v>
       </c>
       <c r="BD7" t="n">
-        <v>694.2183884592996</v>
+        <v>694.2183884592995</v>
       </c>
       <c r="BE7" t="n">
         <v>482.4639112414556</v>
       </c>
       <c r="BF7" t="n">
-        <v>0.4812249248184184</v>
+        <v>0.4812249248184186</v>
       </c>
     </row>
     <row r="8">
@@ -1784,16 +1784,16 @@
         <v>334.1259162553314</v>
       </c>
       <c r="G8" t="n">
-        <v>39695.39848336647</v>
+        <v>39695.3984833665</v>
       </c>
       <c r="H8" t="n">
-        <v>37313.67457436448</v>
+        <v>37313.67457436451</v>
       </c>
       <c r="I8" t="n">
-        <v>31962.79881293913</v>
+        <v>31962.7988129392</v>
       </c>
       <c r="J8" t="n">
-        <v>36.12136421242803</v>
+        <v>36.12136421242806</v>
       </c>
       <c r="K8" t="n">
         <v>529.9241970256692</v>
@@ -1802,13 +1802,13 @@
         <v>529.9241970256692</v>
       </c>
       <c r="M8" t="n">
-        <v>1.243895574934568</v>
+        <v>1.243895574934569</v>
       </c>
       <c r="N8" t="n">
-        <v>1129636.632014788</v>
+        <v>1129636.632014789</v>
       </c>
       <c r="O8" t="n">
-        <v>1129636.632014788</v>
+        <v>1129636.632014789</v>
       </c>
       <c r="P8" t="n">
         <v>406.9055048070495</v>
@@ -1820,7 +1820,7 @@
         <v>0.8393114668624276</v>
       </c>
       <c r="S8" t="n">
-        <v>0.2078358677458284</v>
+        <v>0.2078358677458283</v>
       </c>
       <c r="T8" t="n">
         <v>1.071159076681218</v>
@@ -1832,7 +1832,7 @@
         <v>0.3562086255178994</v>
       </c>
       <c r="W8" t="n">
-        <v>0.5326608273947993</v>
+        <v>0.5326608273947991</v>
       </c>
       <c r="X8" t="n">
         <v>0.07606035983189825</v>
@@ -1847,10 +1847,10 @@
         <v>0.3334343846039873</v>
       </c>
       <c r="AB8" t="n">
-        <v>0.501945251869729</v>
+        <v>0.5019452518697289</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.06722006815433129</v>
+        <v>0.06722006815433125</v>
       </c>
       <c r="AD8" t="n">
         <v>0.9194401671295115</v>
@@ -1859,19 +1859,19 @@
         <v>0.9645419874248758</v>
       </c>
       <c r="AF8" t="n">
-        <v>0.2952009644321385</v>
+        <v>0.2952009644321383</v>
       </c>
       <c r="AG8" t="n">
-        <v>0.8963587435290984</v>
+        <v>0.8963587435290988</v>
       </c>
       <c r="AH8" t="n">
-        <v>0.3747148934556732</v>
+        <v>0.374714893455673</v>
       </c>
       <c r="AI8" t="n">
-        <v>0.06056357647098572</v>
+        <v>0.0605635764709857</v>
       </c>
       <c r="AJ8" t="n">
-        <v>0.05888113047881129</v>
+        <v>0.05888113047881122</v>
       </c>
       <c r="AK8" t="n">
         <v>0.9277297510649634</v>
@@ -1880,7 +1880,7 @@
         <v>0.9019267271436517</v>
       </c>
       <c r="AM8" t="n">
-        <v>0.5876361077145108</v>
+        <v>0.587636107714511</v>
       </c>
       <c r="AN8" t="n">
         <v>0.5426102049201035</v>
@@ -1889,16 +1889,16 @@
         <v>0.375</v>
       </c>
       <c r="AP8" t="n">
-        <v>0.8732466361975925</v>
+        <v>0.8732466361975928</v>
       </c>
       <c r="AQ8" t="n">
-        <v>0.5679996810907018</v>
+        <v>0.5679996810907016</v>
       </c>
       <c r="AR8" t="n">
-        <v>0.330636431277489</v>
+        <v>0.3306364312774893</v>
       </c>
       <c r="AS8" t="n">
-        <v>0.3283590624383966</v>
+        <v>0.3283590624383972</v>
       </c>
       <c r="AT8" t="n">
         <v>246.3817046229869</v>
@@ -1922,22 +1922,22 @@
         <v>0.61200680035082</v>
       </c>
       <c r="BA8" t="n">
-        <v>0.5525586341701532</v>
+        <v>0.5525586341701533</v>
       </c>
       <c r="BB8" t="n">
         <v>529.9241970256692</v>
       </c>
       <c r="BC8" t="n">
-        <v>0.9491131593006692</v>
+        <v>0.9491131593006691</v>
       </c>
       <c r="BD8" t="n">
-        <v>696.5599730414654</v>
+        <v>696.5599730414652</v>
       </c>
       <c r="BE8" t="n">
-        <v>483.2768967794792</v>
+        <v>483.2768967794791</v>
       </c>
       <c r="BF8" t="n">
-        <v>0.4819544420261797</v>
+        <v>0.4819544420261798</v>
       </c>
     </row>
     <row r="9">
@@ -1960,43 +1960,43 @@
         <v>333.9789201310027</v>
       </c>
       <c r="G9" t="n">
-        <v>40033.66788134898</v>
+        <v>40033.66788134909</v>
       </c>
       <c r="H9" t="n">
-        <v>37631.64780846803</v>
+        <v>37631.64780846814</v>
       </c>
       <c r="I9" t="n">
-        <v>31951.43722511338</v>
+        <v>31951.43722511351</v>
       </c>
       <c r="J9" t="n">
-        <v>36.19747973519625</v>
+        <v>36.19747973519635</v>
       </c>
       <c r="K9" t="n">
-        <v>564.3007846839776</v>
+        <v>564.3007846839777</v>
       </c>
       <c r="L9" t="n">
-        <v>564.3007846839776</v>
+        <v>564.3007846839777</v>
       </c>
       <c r="M9" t="n">
-        <v>1.226798626151878</v>
+        <v>1.226798626151879</v>
       </c>
       <c r="N9" t="n">
-        <v>1279210.556326685</v>
+        <v>1279210.556326686</v>
       </c>
       <c r="O9" t="n">
-        <v>1279210.556326685</v>
+        <v>1279210.556326686</v>
       </c>
       <c r="P9" t="n">
         <v>420.8004730859109</v>
       </c>
       <c r="Q9" t="n">
-        <v>434.9828193211057</v>
+        <v>434.9828193211058</v>
       </c>
       <c r="R9" t="n">
         <v>0.8548440810533523</v>
       </c>
       <c r="S9" t="n">
-        <v>0.2174940420917135</v>
+        <v>0.217494042091713</v>
       </c>
       <c r="T9" t="n">
         <v>1.038469904488946</v>
@@ -2005,10 +2005,10 @@
         <v>123.3152935868318</v>
       </c>
       <c r="V9" t="n">
-        <v>0.3401109302577576</v>
+        <v>0.3401109302577575</v>
       </c>
       <c r="W9" t="n">
-        <v>0.5110190907706706</v>
+        <v>0.5110190907706705</v>
       </c>
       <c r="X9" t="n">
         <v>0.07274357402768651</v>
@@ -2020,31 +2020,31 @@
         <v>119.4616906622433</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.318739891404164</v>
+        <v>0.3187398914041639</v>
       </c>
       <c r="AB9" t="n">
-        <v>0.4817789938534903</v>
+        <v>0.4817789938534902</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.06501394252454777</v>
+        <v>0.06501394252454772</v>
       </c>
       <c r="AD9" t="n">
-        <v>0.9221957954528871</v>
+        <v>0.9221957954528872</v>
       </c>
       <c r="AE9" t="n">
         <v>0.9655445893469043</v>
       </c>
       <c r="AF9" t="n">
-        <v>0.2943757274641756</v>
+        <v>0.2943757274641752</v>
       </c>
       <c r="AG9" t="n">
-        <v>0.8821958879190526</v>
+        <v>0.8821958879190533</v>
       </c>
       <c r="AH9" t="n">
-        <v>0.3556826468593637</v>
+        <v>0.3556826468593636</v>
       </c>
       <c r="AI9" t="n">
-        <v>0.05888113047881129</v>
+        <v>0.05888113047881122</v>
       </c>
       <c r="AJ9" t="n">
         <v>0.05815806913968136</v>
@@ -2056,34 +2056,34 @@
         <v>0.9101943352001283</v>
       </c>
       <c r="AM9" t="n">
-        <v>0.5985918471418362</v>
+        <v>0.5985918471418368</v>
       </c>
       <c r="AN9" t="n">
-        <v>0.5250761583694254</v>
+        <v>0.5250761583694251</v>
       </c>
       <c r="AO9" t="n">
         <v>0.3634615384615385</v>
       </c>
       <c r="AP9" t="n">
-        <v>0.8620685138187281</v>
+        <v>0.8620685138187288</v>
       </c>
       <c r="AQ9" t="n">
-        <v>0.5456926176210596</v>
+        <v>0.5456926176210593</v>
       </c>
       <c r="AR9" t="n">
-        <v>0.3369923554493026</v>
+        <v>0.3369923554493037</v>
       </c>
       <c r="AS9" t="n">
-        <v>0.336503270297993</v>
+        <v>0.3365032702979941</v>
       </c>
       <c r="AT9" t="n">
-        <v>246.0013624874193</v>
+        <v>246.0013624874196</v>
       </c>
       <c r="AU9" t="n">
         <v>121.3884921245375</v>
       </c>
       <c r="AV9" t="n">
-        <v>233.8845791893684</v>
+        <v>233.8845791893686</v>
       </c>
       <c r="AW9" t="n">
         <v>0.9807207591865338</v>
@@ -2095,13 +2095,13 @@
         <v>416.7243746234115</v>
       </c>
       <c r="AZ9" t="n">
-        <v>0.5903215109740764</v>
+        <v>0.5903215109740769</v>
       </c>
       <c r="BA9" t="n">
-        <v>0.5376869356688639</v>
+        <v>0.5376869356688643</v>
       </c>
       <c r="BB9" t="n">
-        <v>564.3007846839776</v>
+        <v>564.3007846839777</v>
       </c>
       <c r="BC9" t="n">
         <v>0.9518154598685045</v>
@@ -2113,7 +2113,7 @@
         <v>483.9643970863841</v>
       </c>
       <c r="BF9" t="n">
-        <v>0.4832681507098998</v>
+        <v>0.4832681507099002</v>
       </c>
     </row>
     <row r="10">
@@ -2136,31 +2136,31 @@
         <v>333.8319240066739</v>
       </c>
       <c r="G10" t="n">
-        <v>40295.48134264052</v>
+        <v>40295.48134264065</v>
       </c>
       <c r="H10" t="n">
-        <v>37877.75246208208</v>
+        <v>37877.75246208221</v>
       </c>
       <c r="I10" t="n">
-        <v>31841.82633685318</v>
+        <v>31841.82633685333</v>
       </c>
       <c r="J10" t="n">
-        <v>36.18678624471938</v>
+        <v>36.1867862447195</v>
       </c>
       <c r="K10" t="n">
-        <v>598.5905633290409</v>
+        <v>598.5905633290411</v>
       </c>
       <c r="L10" t="n">
-        <v>598.5905633290409</v>
+        <v>598.5905633290411</v>
       </c>
       <c r="M10" t="n">
-        <v>1.211229011137437</v>
+        <v>1.211229011137438</v>
       </c>
       <c r="N10" t="n">
-        <v>1425980.856751484</v>
+        <v>1425980.856751485</v>
       </c>
       <c r="O10" t="n">
-        <v>1425980.856751484</v>
+        <v>1425980.856751485</v>
       </c>
       <c r="P10" t="n">
         <v>434.2510638517458</v>
@@ -2172,22 +2172,22 @@
         <v>0.8710141506800956</v>
       </c>
       <c r="S10" t="n">
-        <v>0.2279462396392065</v>
+        <v>0.2279462396392059</v>
       </c>
       <c r="T10" t="n">
-        <v>1.003422927048462</v>
+        <v>1.003422927048463</v>
       </c>
       <c r="U10" t="n">
         <v>119.4091112793103</v>
       </c>
       <c r="V10" t="n">
-        <v>0.3260667458821142</v>
+        <v>0.3260667458821139</v>
       </c>
       <c r="W10" t="n">
-        <v>0.4918673171729253</v>
+        <v>0.4918673171729251</v>
       </c>
       <c r="X10" t="n">
-        <v>0.07057645739235102</v>
+        <v>0.07057645739235101</v>
       </c>
       <c r="Y10" t="n">
         <v>0.3461538461538461</v>
@@ -2196,13 +2196,13 @@
         <v>115.5572044638487</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.3058618081016736</v>
+        <v>0.3058618081016733</v>
       </c>
       <c r="AB10" t="n">
-        <v>0.4638913822085473</v>
+        <v>0.4638913822085468</v>
       </c>
       <c r="AC10" t="n">
-        <v>0.06373912111679632</v>
+        <v>0.0637391211167963</v>
       </c>
       <c r="AD10" t="n">
         <v>0.9237844025439431</v>
@@ -2211,19 +2211,19 @@
         <v>0.9659751557909323</v>
       </c>
       <c r="AF10" t="n">
-        <v>0.2935198956157492</v>
+        <v>0.2935198956157486</v>
       </c>
       <c r="AG10" t="n">
-        <v>0.8674957122980209</v>
+        <v>0.8674957122980219</v>
       </c>
       <c r="AH10" t="n">
-        <v>0.3381854374395047</v>
+        <v>0.3381854374395044</v>
       </c>
       <c r="AI10" t="n">
         <v>0.05815806913968136</v>
       </c>
       <c r="AJ10" t="n">
-        <v>0.05818116247847879</v>
+        <v>0.05818116247847869</v>
       </c>
       <c r="AK10" t="n">
         <v>0.9307072596744004</v>
@@ -2232,37 +2232,37 @@
         <v>0.9184946532355139</v>
       </c>
       <c r="AM10" t="n">
-        <v>0.6098252705029964</v>
+        <v>0.6098252705029971</v>
       </c>
       <c r="AN10" t="n">
-        <v>0.5076121232313855</v>
+        <v>0.507612123231385</v>
       </c>
       <c r="AO10" t="n">
         <v>0.3519230769230769</v>
       </c>
       <c r="AP10" t="n">
-        <v>0.8507819547078326</v>
+        <v>0.8507819547078337</v>
       </c>
       <c r="AQ10" t="n">
-        <v>0.5234023357991608</v>
+        <v>0.5234023357991604</v>
       </c>
       <c r="AR10" t="n">
-        <v>0.3431698314764471</v>
+        <v>0.3431698314764486</v>
       </c>
       <c r="AS10" t="n">
-        <v>0.3440933764988601</v>
+        <v>0.3440933764988615</v>
       </c>
       <c r="AT10" t="n">
-        <v>245.6513333762857</v>
+        <v>245.6513333762859</v>
       </c>
       <c r="AU10" t="n">
         <v>117.4831578715795</v>
       </c>
       <c r="AV10" t="n">
-        <v>235.0462933011952</v>
+        <v>235.0462933011954</v>
       </c>
       <c r="AW10" t="n">
-        <v>0.9822800795383081</v>
+        <v>0.9822800795383082</v>
       </c>
       <c r="AX10" t="n">
         <v>552.4380268870323</v>
@@ -2271,25 +2271,25 @@
         <v>430.3864198777907</v>
       </c>
       <c r="AZ10" t="n">
-        <v>0.5707692483560215</v>
+        <v>0.5707692483560219</v>
       </c>
       <c r="BA10" t="n">
-        <v>0.5246524400447958</v>
+        <v>0.5246524400447963</v>
       </c>
       <c r="BB10" t="n">
-        <v>598.5905633290409</v>
+        <v>598.5905633290411</v>
       </c>
       <c r="BC10" t="n">
-        <v>0.9541233028591737</v>
+        <v>0.9541233028591736</v>
       </c>
       <c r="BD10" t="n">
-        <v>700.2369481501206</v>
+        <v>700.2369481501205</v>
       </c>
       <c r="BE10" t="n">
         <v>484.5507700073703</v>
       </c>
       <c r="BF10" t="n">
-        <v>0.4850808374478902</v>
+        <v>0.4850808374478907</v>
       </c>
     </row>
     <row r="11">
@@ -2312,55 +2312,55 @@
         <v>333.6849278823452</v>
       </c>
       <c r="G11" t="n">
-        <v>40473.60344287136</v>
+        <v>40473.60344287158</v>
       </c>
       <c r="H11" t="n">
-        <v>38045.18723629908</v>
+        <v>38045.18723629928</v>
       </c>
       <c r="I11" t="n">
-        <v>31629.06019140586</v>
+        <v>31629.06019140607</v>
       </c>
       <c r="J11" t="n">
-        <v>36.05014175460364</v>
+        <v>36.05014175460383</v>
       </c>
       <c r="K11" t="n">
-        <v>632.7543909744653</v>
+        <v>632.7543909744655</v>
       </c>
       <c r="L11" t="n">
-        <v>632.7543909744653</v>
+        <v>632.7543909744655</v>
       </c>
       <c r="M11" t="n">
-        <v>1.196883588854239</v>
+        <v>1.19688358885424</v>
       </c>
       <c r="N11" t="n">
-        <v>1570166.486665582</v>
+        <v>1570166.486665584</v>
       </c>
       <c r="O11" t="n">
-        <v>1570166.486665582</v>
+        <v>1570166.486665584</v>
       </c>
       <c r="P11" t="n">
         <v>447.297367266363</v>
       </c>
       <c r="Q11" t="n">
-        <v>460.6110585881957</v>
+        <v>460.6110585881958</v>
       </c>
       <c r="R11" t="n">
         <v>0.8877868447582528</v>
       </c>
       <c r="S11" t="n">
-        <v>0.239173555716145</v>
+        <v>0.239173555716144</v>
       </c>
       <c r="T11" t="n">
-        <v>0.9661728705893968</v>
+        <v>0.9661728705893988</v>
       </c>
       <c r="U11" t="n">
         <v>115.5063211900426</v>
       </c>
       <c r="V11" t="n">
-        <v>0.3138769034107374</v>
+        <v>0.313876903410737</v>
       </c>
       <c r="W11" t="n">
-        <v>0.4750473884185655</v>
+        <v>0.4750473884185649</v>
       </c>
       <c r="X11" t="n">
         <v>0.06924046752817985</v>
@@ -2372,70 +2372,70 @@
         <v>111.6561104837078</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.2946443271957259</v>
+        <v>0.2946443271957255</v>
       </c>
       <c r="AB11" t="n">
-        <v>0.44815339237128</v>
+        <v>0.4481533923712796</v>
       </c>
       <c r="AC11" t="n">
-        <v>0.06314752662728688</v>
+        <v>0.06314752662728677</v>
       </c>
       <c r="AD11" t="n">
         <v>0.9245206853316195</v>
       </c>
       <c r="AE11" t="n">
-        <v>0.9659614072042403</v>
+        <v>0.9659614072042404</v>
       </c>
       <c r="AF11" t="n">
-        <v>0.2927694518142698</v>
+        <v>0.2927694518142688</v>
       </c>
       <c r="AG11" t="n">
-        <v>0.8519985040338564</v>
+        <v>0.8519985040338579</v>
       </c>
       <c r="AH11" t="n">
-        <v>0.3220958597524807</v>
+        <v>0.3220958597524803</v>
       </c>
       <c r="AI11" t="n">
-        <v>0.05818116247847879</v>
+        <v>0.05818116247847869</v>
       </c>
       <c r="AJ11" t="n">
-        <v>0.05884109942628889</v>
+        <v>0.05884109942628883</v>
       </c>
       <c r="AK11" t="n">
-        <v>0.9306787202982522</v>
+        <v>0.9306787202982524</v>
       </c>
       <c r="AL11" t="n">
         <v>0.9268741259812465</v>
       </c>
       <c r="AM11" t="n">
-        <v>0.6212605673260709</v>
+        <v>0.621260567326072</v>
       </c>
       <c r="AN11" t="n">
-        <v>0.4902294708237519</v>
+        <v>0.4902294708237513</v>
       </c>
       <c r="AO11" t="n">
         <v>0.3403846153846154</v>
       </c>
       <c r="AP11" t="n">
-        <v>0.8391715906532821</v>
+        <v>0.8391715906532838</v>
       </c>
       <c r="AQ11" t="n">
-        <v>0.5012244840821158</v>
+        <v>0.5012244840821152</v>
       </c>
       <c r="AR11" t="n">
-        <v>0.3489421198295302</v>
+        <v>0.3489421198295325</v>
       </c>
       <c r="AS11" t="n">
-        <v>0.3507740199517405</v>
+        <v>0.3507740199517427</v>
       </c>
       <c r="AT11" t="n">
-        <v>245.3257589778892</v>
+        <v>245.3257589778895</v>
       </c>
       <c r="AU11" t="n">
         <v>113.5812158368752</v>
       </c>
       <c r="AV11" t="n">
-        <v>236.3814181777048</v>
+        <v>236.3814181777051</v>
       </c>
       <c r="AW11" t="n">
         <v>0.9835802149175478</v>
@@ -2447,25 +2447,25 @@
         <v>443.6099044591077</v>
       </c>
       <c r="AZ11" t="n">
-        <v>0.5530213742116832</v>
+        <v>0.5530213742116838</v>
       </c>
       <c r="BA11" t="n">
-        <v>0.5131909314166924</v>
+        <v>0.513190931416693</v>
       </c>
       <c r="BB11" t="n">
-        <v>632.7543909744653</v>
+        <v>632.7543909744655</v>
       </c>
       <c r="BC11" t="n">
-        <v>0.9561058446519446</v>
+        <v>0.9561058446519445</v>
       </c>
       <c r="BD11" t="n">
-        <v>701.6919477402049</v>
+        <v>701.6919477402048</v>
       </c>
       <c r="BE11" t="n">
         <v>485.0539249169011</v>
       </c>
       <c r="BF11" t="n">
-        <v>0.487330183377449</v>
+        <v>0.4873301833774498</v>
       </c>
     </row>
     <row r="12">
@@ -2488,58 +2488,58 @@
         <v>333.5379317580164</v>
       </c>
       <c r="G12" t="n">
-        <v>40560.37394973572</v>
+        <v>40560.37394973599</v>
       </c>
       <c r="H12" t="n">
-        <v>38126.75151275158</v>
+        <v>38126.75151275183</v>
       </c>
       <c r="I12" t="n">
-        <v>31308.56179011731</v>
+        <v>31308.56179011754</v>
       </c>
       <c r="J12" t="n">
-        <v>35.8731622018432</v>
+        <v>35.87316220184343</v>
       </c>
       <c r="K12" t="n">
-        <v>666.8778835572451</v>
+        <v>666.8778835572454</v>
       </c>
       <c r="L12" t="n">
-        <v>666.8778835572451</v>
+        <v>666.8778835572454</v>
       </c>
       <c r="M12" t="n">
-        <v>1.183530306631524</v>
+        <v>1.183530306631526</v>
       </c>
       <c r="N12" t="n">
-        <v>1711926.040961985</v>
+        <v>1711926.040961988</v>
       </c>
       <c r="O12" t="n">
-        <v>1711926.040961985</v>
+        <v>1711926.040961988</v>
       </c>
       <c r="P12" t="n">
         <v>459.9737851991853</v>
       </c>
       <c r="Q12" t="n">
-        <v>472.868009445283</v>
+        <v>472.8680094452831</v>
       </c>
       <c r="R12" t="n">
         <v>0.9051286626963524</v>
       </c>
       <c r="S12" t="n">
-        <v>0.2511589019127057</v>
+        <v>0.2511589019127045</v>
       </c>
       <c r="T12" t="n">
-        <v>0.9269178389038394</v>
+        <v>0.9269178389038419</v>
       </c>
       <c r="U12" t="n">
         <v>111.6069233190286</v>
       </c>
       <c r="V12" t="n">
-        <v>0.3033828567939255</v>
+        <v>0.303382856793925</v>
       </c>
       <c r="W12" t="n">
-        <v>0.4604258288065053</v>
+        <v>0.4604258288065046</v>
       </c>
       <c r="X12" t="n">
-        <v>0.0685401729553279</v>
+        <v>0.06854017295532788</v>
       </c>
       <c r="Y12" t="n">
         <v>0.323076923076923</v>
@@ -2548,100 +2548,100 @@
         <v>107.7584087218207</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.2849339620378177</v>
+        <v>0.2849339620378171</v>
       </c>
       <c r="AB12" t="n">
-        <v>0.4344158747631086</v>
+        <v>0.4344158747631079</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.06309960737010389</v>
+        <v>0.0630996073701038</v>
       </c>
       <c r="AD12" t="n">
-        <v>0.9245802986962449</v>
+        <v>0.924580298696245</v>
       </c>
       <c r="AE12" t="n">
-        <v>0.9655684319411498</v>
+        <v>0.9655684319411499</v>
       </c>
       <c r="AF12" t="n">
-        <v>0.2922180220877941</v>
+        <v>0.2922180220877929</v>
       </c>
       <c r="AG12" t="n">
-        <v>0.8355091984621673</v>
+        <v>0.8355091984621694</v>
       </c>
       <c r="AH12" t="n">
-        <v>0.3072692900787438</v>
+        <v>0.3072692900787432</v>
       </c>
       <c r="AI12" t="n">
-        <v>0.05884109942628889</v>
+        <v>0.05884109942628883</v>
       </c>
       <c r="AJ12" t="n">
-        <v>0.06007088836133104</v>
+        <v>0.06007088836133092</v>
       </c>
       <c r="AK12" t="n">
-        <v>0.9298627820934559</v>
+        <v>0.929862782093456</v>
       </c>
       <c r="AL12" t="n">
-        <v>0.9353485473187511</v>
+        <v>0.9353485473187512</v>
       </c>
       <c r="AM12" t="n">
-        <v>0.6328408556561717</v>
+        <v>0.6328408556561728</v>
       </c>
       <c r="AN12" t="n">
-        <v>0.4729383604313542</v>
+        <v>0.4729383604313535</v>
       </c>
       <c r="AO12" t="n">
         <v>0.3288461538461538</v>
       </c>
       <c r="AP12" t="n">
-        <v>0.8270914214257146</v>
+        <v>0.8270914214257162</v>
       </c>
       <c r="AQ12" t="n">
-        <v>0.479231808360652</v>
+        <v>0.4792318083606513</v>
       </c>
       <c r="AR12" t="n">
-        <v>0.3541530609943603</v>
+        <v>0.3541530609943628</v>
       </c>
       <c r="AS12" t="n">
-        <v>0.3562773901015153</v>
+        <v>0.3562773901015182</v>
       </c>
       <c r="AT12" t="n">
-        <v>245.0184956066509</v>
+        <v>245.0184956066512</v>
       </c>
       <c r="AU12" t="n">
         <v>109.6826660204246</v>
       </c>
       <c r="AV12" t="n">
-        <v>237.8729631142037</v>
+        <v>237.872963114204</v>
       </c>
       <c r="AW12" t="n">
-        <v>0.9846598070339261</v>
+        <v>0.9846598070339262</v>
       </c>
       <c r="AX12" t="n">
-        <v>621.3249871673063</v>
+        <v>621.3249871673064</v>
       </c>
       <c r="AY12" t="n">
         <v>456.4321068868817</v>
       </c>
       <c r="AZ12" t="n">
-        <v>0.5368125771822055</v>
+        <v>0.5368125771822062</v>
       </c>
       <c r="BA12" t="n">
-        <v>0.5030430444919507</v>
+        <v>0.5030430444919513</v>
       </c>
       <c r="BB12" t="n">
-        <v>666.8778835572451</v>
+        <v>666.8778835572454</v>
       </c>
       <c r="BC12" t="n">
-        <v>0.9578246158980449</v>
+        <v>0.9578246158980448</v>
       </c>
       <c r="BD12" t="n">
-        <v>702.9533645071268</v>
+        <v>702.9533645071267</v>
       </c>
       <c r="BE12" t="n">
         <v>485.4897147409403</v>
       </c>
       <c r="BF12" t="n">
-        <v>0.4899649897653008</v>
+        <v>0.4899649897653016</v>
       </c>
     </row>
     <row r="13">
@@ -2664,31 +2664,31 @@
         <v>333.3909356336877</v>
       </c>
       <c r="G13" t="n">
-        <v>40547.70978058977</v>
+        <v>40547.70978059008</v>
       </c>
       <c r="H13" t="n">
-        <v>38114.84719375438</v>
+        <v>38114.84719375468</v>
       </c>
       <c r="I13" t="n">
-        <v>30876.17615858862</v>
+        <v>30876.17615858889</v>
       </c>
       <c r="J13" t="n">
-        <v>35.60913417270066</v>
+        <v>35.60913417270093</v>
       </c>
       <c r="K13" t="n">
-        <v>700.9143276636428</v>
+        <v>700.914327663643</v>
       </c>
       <c r="L13" t="n">
-        <v>700.9143276636428</v>
+        <v>700.914327663643</v>
       </c>
       <c r="M13" t="n">
-        <v>1.170989670361082</v>
+        <v>1.170989670361084</v>
       </c>
       <c r="N13" t="n">
-        <v>1851376.294513944</v>
+        <v>1851376.294513946</v>
       </c>
       <c r="O13" t="n">
-        <v>1851376.294513944</v>
+        <v>1851376.294513946</v>
       </c>
       <c r="P13" t="n">
         <v>472.310100863313</v>
@@ -2700,19 +2700,19 @@
         <v>0.9230075263024611</v>
       </c>
       <c r="S13" t="n">
-        <v>0.2638871209886932</v>
+        <v>0.2638871209886917</v>
       </c>
       <c r="T13" t="n">
-        <v>0.8858990164198532</v>
+        <v>0.885899016419856</v>
       </c>
       <c r="U13" t="n">
         <v>107.7109176662683</v>
       </c>
       <c r="V13" t="n">
-        <v>0.2944557473880438</v>
+        <v>0.2944557473880431</v>
       </c>
       <c r="W13" t="n">
-        <v>0.4478875986165679</v>
+        <v>0.4478875986165669</v>
       </c>
       <c r="X13" t="n">
         <v>0.06835157578026685</v>
@@ -2724,34 +2724,34 @@
         <v>103.8640991781873</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.2766328533973357</v>
+        <v>0.2766328533973351</v>
       </c>
       <c r="AB13" t="n">
-        <v>0.4225907731006984</v>
+        <v>0.4225907731006975</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.06349894451081993</v>
+        <v>0.06349894451081982</v>
       </c>
       <c r="AD13" t="n">
-        <v>0.9240833907064329</v>
+        <v>0.924083390706433</v>
       </c>
       <c r="AE13" t="n">
         <v>0.9648356976196854</v>
       </c>
       <c r="AF13" t="n">
-        <v>0.29194404655797</v>
+        <v>0.2919440465579686</v>
       </c>
       <c r="AG13" t="n">
-        <v>0.8178556636542694</v>
+        <v>0.8178556636542718</v>
       </c>
       <c r="AH13" t="n">
-        <v>0.2936182416907518</v>
+        <v>0.2936182416907512</v>
       </c>
       <c r="AI13" t="n">
-        <v>0.06007088836133104</v>
+        <v>0.06007088836133092</v>
       </c>
       <c r="AJ13" t="n">
-        <v>0.06184229672885735</v>
+        <v>0.06184229672885732</v>
       </c>
       <c r="AK13" t="n">
         <v>0.9283403722786862</v>
@@ -2760,34 +2760,34 @@
         <v>0.9439216119610732</v>
       </c>
       <c r="AM13" t="n">
-        <v>0.6445165436780202</v>
+        <v>0.6445165436780217</v>
       </c>
       <c r="AN13" t="n">
-        <v>0.455747682527153</v>
+        <v>0.4557476825271521</v>
       </c>
       <c r="AO13" t="n">
         <v>0.3173076923076923</v>
       </c>
       <c r="AP13" t="n">
-        <v>0.8144191257089225</v>
+        <v>0.8144191257089248</v>
       </c>
       <c r="AQ13" t="n">
-        <v>0.4574838896946357</v>
+        <v>0.4574838896946348</v>
       </c>
       <c r="AR13" t="n">
-        <v>0.3586714431817695</v>
+        <v>0.3586714431817727</v>
       </c>
       <c r="AS13" t="n">
-        <v>0.3603717739596337</v>
+        <v>0.3603717739596369</v>
       </c>
       <c r="AT13" t="n">
-        <v>244.7231193034345</v>
+        <v>244.723119303435</v>
       </c>
       <c r="AU13" t="n">
         <v>105.7875084222278</v>
       </c>
       <c r="AV13" t="n">
-        <v>239.5050749731142</v>
+        <v>239.5050749731147</v>
       </c>
       <c r="AW13" t="n">
         <v>0.9855493021383581</v>
@@ -2799,25 +2799,25 @@
         <v>468.8850770576346</v>
       </c>
       <c r="AZ13" t="n">
-        <v>0.5219255874789838</v>
+        <v>0.5219255874789847</v>
       </c>
       <c r="BA13" t="n">
-        <v>0.4940438241890232</v>
+        <v>0.494043824189024</v>
       </c>
       <c r="BB13" t="n">
-        <v>700.9143276636428</v>
+        <v>700.914327663643</v>
       </c>
       <c r="BC13" t="n">
-        <v>0.9593201166301143</v>
+        <v>0.9593201166301142</v>
       </c>
       <c r="BD13" t="n">
-        <v>704.0509216734201</v>
+        <v>704.05092167342</v>
       </c>
       <c r="BE13" t="n">
         <v>485.8685769187978</v>
       </c>
       <c r="BF13" t="n">
-        <v>0.4929420965890993</v>
+        <v>0.4929420965891002</v>
       </c>
     </row>
     <row r="14">
@@ -2840,58 +2840,58 @@
         <v>333.2439395093589</v>
       </c>
       <c r="G14" t="n">
-        <v>40427.22983054043</v>
+        <v>40427.22983054083</v>
       </c>
       <c r="H14" t="n">
-        <v>38001.596040708</v>
+        <v>38001.59604070838</v>
       </c>
       <c r="I14" t="n">
-        <v>30328.77244090673</v>
+        <v>30328.77244090705</v>
       </c>
       <c r="J14" t="n">
-        <v>35.25478155713519</v>
+        <v>35.25478155713554</v>
       </c>
       <c r="K14" t="n">
-        <v>734.8604471836175</v>
+        <v>734.8604471836178</v>
       </c>
       <c r="L14" t="n">
-        <v>734.8604471836175</v>
+        <v>734.8604471836178</v>
       </c>
       <c r="M14" t="n">
-        <v>1.159124662321261</v>
+        <v>1.159124662321262</v>
       </c>
       <c r="N14" t="n">
-        <v>1988610.271253233</v>
+        <v>1988610.271253235</v>
       </c>
       <c r="O14" t="n">
-        <v>1988610.271253233</v>
+        <v>1988610.271253235</v>
       </c>
       <c r="P14" t="n">
         <v>484.332302953829</v>
       </c>
       <c r="Q14" t="n">
-        <v>496.3856443740763</v>
+        <v>496.3856443740764</v>
       </c>
       <c r="R14" t="n">
         <v>0.9413928374782321</v>
       </c>
       <c r="S14" t="n">
-        <v>0.2773444590010399</v>
+        <v>0.277344459001038</v>
       </c>
       <c r="T14" t="n">
-        <v>0.843398911728933</v>
+        <v>0.8433989117289364</v>
       </c>
       <c r="U14" t="n">
         <v>103.8183042317618</v>
       </c>
       <c r="V14" t="n">
-        <v>0.2869879732052466</v>
+        <v>0.2869879732052458</v>
       </c>
       <c r="W14" t="n">
-        <v>0.437330387402672</v>
+        <v>0.4373303874026709</v>
       </c>
       <c r="X14" t="n">
-        <v>0.06859490793482022</v>
+        <v>0.0685949079348202</v>
       </c>
       <c r="Y14" t="n">
         <v>0.3</v>
@@ -2900,100 +2900,100 @@
         <v>99.97318185280768</v>
       </c>
       <c r="AA14" t="n">
-        <v>0.2696481863264099</v>
+        <v>0.269648186326409</v>
       </c>
       <c r="AB14" t="n">
-        <v>0.4125844983772042</v>
+        <v>0.4125844983772029</v>
       </c>
       <c r="AC14" t="n">
-        <v>0.06428864272086865</v>
+        <v>0.06428864272086859</v>
       </c>
       <c r="AD14" t="n">
         <v>0.9230999564416354</v>
       </c>
       <c r="AE14" t="n">
-        <v>0.9637792758337282</v>
+        <v>0.9637792758337284</v>
       </c>
       <c r="AF14" t="n">
-        <v>0.2920116907329444</v>
+        <v>0.2920116907329426</v>
       </c>
       <c r="AG14" t="n">
-        <v>0.7988908437321858</v>
+        <v>0.7988908437321889</v>
       </c>
       <c r="AH14" t="n">
-        <v>0.2810592386107025</v>
+        <v>0.2810592386107015</v>
       </c>
       <c r="AI14" t="n">
-        <v>0.06184229672885735</v>
+        <v>0.06184229672885732</v>
       </c>
       <c r="AJ14" t="n">
-        <v>0.06287462290091529</v>
+        <v>0.06287462290091517</v>
       </c>
       <c r="AK14" t="n">
-        <v>0.9261430694299728</v>
+        <v>0.9261430694299729</v>
       </c>
       <c r="AL14" t="n">
-        <v>0.9525860566559802</v>
+        <v>0.9525860566559803</v>
       </c>
       <c r="AM14" t="n">
-        <v>0.6562455778871688</v>
+        <v>0.6562455778871705</v>
       </c>
       <c r="AN14" t="n">
-        <v>0.4386646551706986</v>
+        <v>0.4386646551706975</v>
       </c>
       <c r="AO14" t="n">
         <v>0.3057692307692308</v>
       </c>
       <c r="AP14" t="n">
-        <v>0.8010564084913128</v>
+        <v>0.8010564084913155</v>
       </c>
       <c r="AQ14" t="n">
-        <v>0.4360279824188179</v>
+        <v>0.4360279824188169</v>
       </c>
       <c r="AR14" t="n">
-        <v>0.3623917533206142</v>
+        <v>0.3623917533206181</v>
       </c>
       <c r="AS14" t="n">
-        <v>0.3628628613133679</v>
+        <v>0.362862861313372</v>
       </c>
       <c r="AT14" t="n">
-        <v>244.433114818167</v>
+        <v>244.4331148181676</v>
       </c>
       <c r="AU14" t="n">
         <v>101.8957430422848</v>
       </c>
       <c r="AV14" t="n">
-        <v>241.2633375449374</v>
+        <v>241.263337544938</v>
       </c>
       <c r="AW14" t="n">
-        <v>0.9862729838725908</v>
+        <v>0.9862729838725909</v>
       </c>
       <c r="AX14" t="n">
-        <v>690.0021673716006</v>
+        <v>690.0021673716008</v>
       </c>
       <c r="AY14" t="n">
         <v>480.9965974096883</v>
       </c>
       <c r="AZ14" t="n">
-        <v>0.5081805487492282</v>
+        <v>0.5081805487492295</v>
       </c>
       <c r="BA14" t="n">
-        <v>0.4860401187652424</v>
+        <v>0.4860401187652434</v>
       </c>
       <c r="BB14" t="n">
-        <v>734.8604471836175</v>
+        <v>734.8604471836178</v>
       </c>
       <c r="BC14" t="n">
-        <v>0.9606275004917781</v>
+        <v>0.960627500491778</v>
       </c>
       <c r="BD14" t="n">
-        <v>705.0104187139062</v>
+        <v>705.0104187139061</v>
       </c>
       <c r="BE14" t="n">
         <v>486.1995407183894</v>
       </c>
       <c r="BF14" t="n">
-        <v>0.4962228824577995</v>
+        <v>0.4962228824578006</v>
       </c>
     </row>
     <row r="15">
@@ -3016,133 +3016,133 @@
         <v>333.0969433850302</v>
       </c>
       <c r="G15" t="n">
-        <v>40189.87084991405</v>
+        <v>40189.87084991457</v>
       </c>
       <c r="H15" t="n">
-        <v>37778.4785989192</v>
+        <v>37778.47859891969</v>
       </c>
       <c r="I15" t="n">
-        <v>29662.4442033218</v>
+        <v>29662.44420332219</v>
       </c>
       <c r="J15" t="n">
-        <v>34.75041522806004</v>
+        <v>34.75041522806048</v>
       </c>
       <c r="K15" t="n">
-        <v>768.6565529900824</v>
+        <v>768.6565529900829</v>
       </c>
       <c r="L15" t="n">
-        <v>768.6565529900824</v>
+        <v>768.6565529900829</v>
       </c>
       <c r="M15" t="n">
-        <v>1.147820922348964</v>
+        <v>1.147820922348967</v>
       </c>
       <c r="N15" t="n">
-        <v>2123689.157522174</v>
+        <v>2123689.157522178</v>
       </c>
       <c r="O15" t="n">
-        <v>2123689.157522174</v>
+        <v>2123689.157522178</v>
       </c>
       <c r="P15" t="n">
         <v>496.0632298322525</v>
       </c>
       <c r="Q15" t="n">
-        <v>507.6716874295578</v>
+        <v>507.6716874295579</v>
       </c>
       <c r="R15" t="n">
         <v>0.9602555069185875</v>
       </c>
       <c r="S15" t="n">
-        <v>0.2915204467110554</v>
+        <v>0.291520446711053</v>
       </c>
       <c r="T15" t="n">
-        <v>0.799732363619129</v>
+        <v>0.799732363619133</v>
       </c>
       <c r="U15" t="n">
-        <v>99.92908301550905</v>
+        <v>99.92908301550906</v>
       </c>
       <c r="V15" t="n">
-        <v>0.280887875197628</v>
+        <v>0.280887875197627</v>
       </c>
       <c r="W15" t="n">
-        <v>0.4286613611154603</v>
+        <v>0.4286613611154589</v>
       </c>
       <c r="X15" t="n">
-        <v>0.06921949698481912</v>
+        <v>0.06921949698481909</v>
       </c>
       <c r="Y15" t="n">
         <v>0.3</v>
       </c>
       <c r="Z15" t="n">
-        <v>99.92908301550905</v>
+        <v>99.92908301550906</v>
       </c>
       <c r="AA15" t="n">
-        <v>0.2744650726865439</v>
+        <v>0.2744650726865429</v>
       </c>
       <c r="AB15" t="n">
-        <v>0.4194906558197299</v>
+        <v>0.4194906558197284</v>
       </c>
       <c r="AC15" t="n">
-        <v>0.06306556002225917</v>
+        <v>0.06306556002225903</v>
       </c>
       <c r="AD15" t="n">
-        <v>0.9246226525464954</v>
+        <v>0.9246226525464956</v>
       </c>
       <c r="AE15" t="n">
         <v>0.9631630890144903</v>
       </c>
       <c r="AF15" t="n">
-        <v>0.2934643355010041</v>
+        <v>0.2934643355010018</v>
       </c>
       <c r="AG15" t="n">
-        <v>0.7964104516033221</v>
+        <v>0.7964104516033261</v>
       </c>
       <c r="AH15" t="n">
-        <v>0.275355442547742</v>
+        <v>0.2753554425477409</v>
       </c>
       <c r="AI15" t="n">
-        <v>0.06287462290091529</v>
+        <v>0.06287462290091517</v>
       </c>
       <c r="AJ15" t="n">
-        <v>0.06287462290091529</v>
+        <v>0.06287462290091517</v>
       </c>
       <c r="AK15" t="n">
-        <v>0.9248601364962541</v>
+        <v>0.9248601364962542</v>
       </c>
       <c r="AL15" t="n">
         <v>0.9617092979665389</v>
       </c>
       <c r="AM15" t="n">
-        <v>0.6677241507299628</v>
+        <v>0.6677241507299653</v>
       </c>
       <c r="AN15" t="n">
-        <v>0.4216958620849983</v>
+        <v>0.4216958620849969</v>
       </c>
       <c r="AO15" t="n">
         <v>0.3</v>
       </c>
       <c r="AP15" t="n">
-        <v>0.7955240852555532</v>
+        <v>0.7955240852555574</v>
       </c>
       <c r="AQ15" t="n">
-        <v>0.4222611100674148</v>
+        <v>0.4222611100674134</v>
       </c>
       <c r="AR15" t="n">
-        <v>0.3738282231705549</v>
+        <v>0.3738282231705605</v>
       </c>
       <c r="AS15" t="n">
-        <v>0.3741493415359073</v>
+        <v>0.3741493415359127</v>
       </c>
       <c r="AT15" t="n">
-        <v>244.1413319071554</v>
+        <v>244.1413319071562</v>
       </c>
       <c r="AU15" t="n">
-        <v>99.92908301550905</v>
+        <v>99.92908301550906</v>
       </c>
       <c r="AV15" t="n">
-        <v>243.8341389321499</v>
+        <v>243.8341389321507</v>
       </c>
       <c r="AW15" t="n">
-        <v>0.9868503335944936</v>
+        <v>0.9868503335944937</v>
       </c>
       <c r="AX15" t="n">
         <v>724.2555168774983</v>
@@ -3151,25 +3151,25 @@
         <v>492.7909037401413</v>
       </c>
       <c r="AZ15" t="n">
-        <v>0.4954258085005078</v>
+        <v>0.4954258085005093</v>
       </c>
       <c r="BA15" t="n">
-        <v>0.4802988722233663</v>
+        <v>0.4802988722233676</v>
       </c>
       <c r="BB15" t="n">
-        <v>768.6565529900824</v>
+        <v>768.6565529900829</v>
       </c>
       <c r="BC15" t="n">
-        <v>0.9615521655568271</v>
+        <v>0.9615521655568269</v>
       </c>
       <c r="BD15" t="n">
-        <v>705.6890360805198</v>
+        <v>705.6890360805196</v>
       </c>
       <c r="BE15" t="n">
-        <v>486.4334834258414</v>
+        <v>486.4334834258413</v>
       </c>
       <c r="BF15" t="n">
-        <v>0.5012692325677933</v>
+        <v>0.501269232567795</v>
       </c>
     </row>
   </sheetData>

</xml_diff>